<commit_message>
Costeo: precios de venta directa ajustados por el equipo (unidad S/4.00, pack de 6 S/23.50, pack de 12 S/44.00)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Kfbf7cfV7pXUcNjjyaPCzV
</commit_message>
<xml_diff>
--- a/04-reformulacion/Costeo-presentaciones-AndiBite.xlsx
+++ b/04-reformulacion/Costeo-presentaciones-AndiBite.xlsx
@@ -379,7 +379,7 @@
     <t xml:space="preserve">Pack de 6</t>
   </si>
   <si>
-    <t xml:space="preserve">Unidad = caja degustación de 3 (S/13.50) o unidades agregadas al pedido</t>
+    <t xml:space="preserve">Precios ajustados por el equipo (9-oct-2026). Unidad = caja degustación de 3 (S/12.00) o unidades agregadas al pedido</t>
   </si>
   <si>
     <t xml:space="preserve">La unidad suelta cuesta más que dentro del pack para empujar el pack</t>
@@ -1455,11 +1455,11 @@
       </c>
       <c r="D5" s="6" t="n">
         <f aca="false">Costeo!B19</f>
-        <v>4.5</v>
+        <v>4</v>
       </c>
       <c r="E5" s="7" t="n">
         <f aca="false">Costeo!B22</f>
-        <v>0.555992222222222</v>
+        <v>0.50049125</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1476,11 +1476,11 @@
       </c>
       <c r="D6" s="6" t="n">
         <f aca="false">Costeo!C19</f>
-        <v>27</v>
+        <v>23.5</v>
       </c>
       <c r="E6" s="7" t="n">
         <f aca="false">Costeo!C22</f>
-        <v>0.567464444444445</v>
+        <v>0.503044255319149</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1497,11 +1497,11 @@
       </c>
       <c r="D7" s="6" t="n">
         <f aca="false">Costeo!D19</f>
-        <v>27</v>
+        <v>23.5</v>
       </c>
       <c r="E7" s="7" t="n">
         <f aca="false">Costeo!D22</f>
-        <v>0.589491111111111</v>
+        <v>0.528351489361702</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1518,11 +1518,11 @@
       </c>
       <c r="D8" s="6" t="n">
         <f aca="false">Costeo!E19</f>
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="E8" s="7" t="n">
         <f aca="false">Costeo!E22</f>
-        <v>0.550636734693878</v>
+        <v>0.499572727272727</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1557,11 +1557,11 @@
       </c>
       <c r="B13" s="9" t="n">
         <f aca="false">Proyeccion!I17</f>
-        <v>322971.33</v>
+        <v>291304.38</v>
       </c>
       <c r="C13" s="9" t="n">
         <f aca="false">Proyeccion!I17</f>
-        <v>322971.33</v>
+        <v>291304.38</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1570,11 +1570,11 @@
       </c>
       <c r="B14" s="9" t="n">
         <f aca="false">Proyeccion!J17</f>
-        <v>273704.516949153</v>
+        <v>246868.118644068</v>
       </c>
       <c r="C14" s="9" t="n">
         <f aca="false">Proyeccion!J17</f>
-        <v>273704.516949153</v>
+        <v>246868.118644068</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1583,11 +1583,11 @@
       </c>
       <c r="B15" s="9" t="n">
         <f aca="false">Proyeccion!P17</f>
-        <v>82183.262079661</v>
+        <v>56565.2362576271</v>
       </c>
       <c r="C15" s="9" t="n">
         <f aca="false">Proyeccion!Q17</f>
-        <v>85628.505279661</v>
+        <v>60010.4794576271</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1609,11 +1609,11 @@
       </c>
       <c r="B17" s="11" t="n">
         <f aca="false">B15-B16</f>
-        <v>47903.222079661</v>
+        <v>22285.1962576271</v>
       </c>
       <c r="C17" s="11" t="n">
         <f aca="false">C15-C16</f>
-        <v>51348.465279661</v>
+        <v>25730.4394576271</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1622,11 +1622,11 @@
       </c>
       <c r="B18" s="12" t="n">
         <f aca="false">IF(B14=0,0,B17/B14)</f>
-        <v>0.175018018020361</v>
+        <v>0.0902716656165623</v>
       </c>
       <c r="C18" s="12" t="n">
         <f aca="false">IF(C14=0,0,C17/C14)</f>
-        <v>0.187605472690099</v>
+        <v>0.10422747011219</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1635,11 +1635,11 @@
       </c>
       <c r="B19" s="13" t="n">
         <f aca="false">IF(B12=0,0,B15/B12)</f>
-        <v>1.07661311429437</v>
+        <v>0.741013116625757</v>
       </c>
       <c r="C19" s="13" t="n">
         <f aca="false">IF(C12=0,0,C15/C12)</f>
-        <v>1.12174631924623</v>
+        <v>0.786146321577613</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1648,11 +1648,11 @@
       </c>
       <c r="B20" s="14" t="n">
         <f aca="false">IF(B19&lt;=0,"No alcanza",Supuestos!$B$58/B19)</f>
-        <v>2653.38584684833</v>
+        <v>3855.0869558261</v>
       </c>
       <c r="C20" s="14" t="n">
         <f aca="false">IF(C19&lt;=0,"No alcanza",Supuestos!$B$58/C19)</f>
-        <v>2546.62747805544</v>
+        <v>3633.76374294715</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1661,11 +1661,11 @@
       </c>
       <c r="B21" s="15" t="n">
         <f aca="false">IF(ISNUMBER(B20),B20/6,"No alcanza")</f>
-        <v>442.230974474722</v>
+        <v>642.514492637684</v>
       </c>
       <c r="C21" s="15" t="n">
         <f aca="false">IF(ISNUMBER(C20),C20/6,"No alcanza")</f>
-        <v>424.43791300924</v>
+        <v>605.627290491191</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2142,13 +2142,13 @@
         <v>100</v>
       </c>
       <c r="B39" s="24" t="n">
-        <v>4.5</v>
+        <v>4</v>
       </c>
       <c r="C39" s="24" t="n">
-        <v>27</v>
+        <v>23.5</v>
       </c>
       <c r="D39" s="24" t="n">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="E39" s="4" t="s">
         <v>110</v>
@@ -2740,19 +2740,19 @@
       </c>
       <c r="B19" s="6" t="n">
         <f aca="false">Supuestos!B39</f>
-        <v>4.5</v>
+        <v>4</v>
       </c>
       <c r="C19" s="6" t="n">
         <f aca="false">Supuestos!C39</f>
-        <v>27</v>
+        <v>23.5</v>
       </c>
       <c r="D19" s="6" t="n">
         <f aca="false">Supuestos!C39</f>
-        <v>27</v>
+        <v>23.5</v>
       </c>
       <c r="E19" s="6" t="n">
         <f aca="false">Supuestos!D39</f>
-        <v>49</v>
+        <v>44</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2761,19 +2761,19 @@
       </c>
       <c r="B20" s="13" t="n">
         <f aca="false">B19/(1+Supuestos!$B$26)</f>
-        <v>3.8135593220339</v>
+        <v>3.38983050847458</v>
       </c>
       <c r="C20" s="13" t="n">
         <f aca="false">C19/(1+Supuestos!$B$26)</f>
-        <v>22.8813559322034</v>
+        <v>19.9152542372881</v>
       </c>
       <c r="D20" s="13" t="n">
         <f aca="false">D19/(1+Supuestos!$B$26)</f>
-        <v>22.8813559322034</v>
+        <v>19.9152542372881</v>
       </c>
       <c r="E20" s="13" t="n">
         <f aca="false">E19/(1+Supuestos!$B$26)</f>
-        <v>41.5254237288136</v>
+        <v>37.2881355932203</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2782,19 +2782,19 @@
       </c>
       <c r="B21" s="13" t="n">
         <f aca="false">B20-B15</f>
-        <v>2.1203093220339</v>
+        <v>1.69658050847458</v>
       </c>
       <c r="C21" s="13" t="n">
         <f aca="false">C20-C15</f>
-        <v>12.9843559322034</v>
+        <v>10.0182542372881</v>
       </c>
       <c r="D21" s="13" t="n">
         <f aca="false">D20-D15</f>
-        <v>13.4883559322034</v>
+        <v>10.5222542372881</v>
       </c>
       <c r="E21" s="13" t="n">
         <f aca="false">E20-E15</f>
-        <v>22.8654237288136</v>
+        <v>18.6281355932203</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2803,19 +2803,19 @@
       </c>
       <c r="B22" s="12" t="n">
         <f aca="false">IF(B20=0,0,B21/B20)</f>
-        <v>0.555992222222222</v>
+        <v>0.50049125</v>
       </c>
       <c r="C22" s="12" t="n">
         <f aca="false">IF(C20=0,0,C21/C20)</f>
-        <v>0.567464444444445</v>
+        <v>0.503044255319149</v>
       </c>
       <c r="D22" s="12" t="n">
         <f aca="false">IF(D20=0,0,D21/D20)</f>
-        <v>0.589491111111111</v>
+        <v>0.528351489361702</v>
       </c>
       <c r="E22" s="12" t="n">
         <f aca="false">IF(E20=0,0,E21/E20)</f>
-        <v>0.550636734693878</v>
+        <v>0.499572727272727</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2950,15 +2950,15 @@
       </c>
       <c r="H5" s="6" t="n">
         <f aca="false">Supuestos!B39</f>
-        <v>4.5</v>
+        <v>4</v>
       </c>
       <c r="I5" s="29" t="n">
         <f aca="false">G5*H5</f>
-        <v>27143.1</v>
+        <v>24127.2</v>
       </c>
       <c r="J5" s="29" t="n">
         <f aca="false">I5/(1+Supuestos!$B$26)</f>
-        <v>23002.6271186441</v>
+        <v>20446.779661017</v>
       </c>
       <c r="K5" s="6" t="n">
         <f aca="false">Costeo!B15</f>
@@ -2970,31 +2970,31 @@
       </c>
       <c r="M5" s="13" t="n">
         <f aca="false">IF(H5=0,0,C5*Supuestos!$B$32+H5*Supuestos!$B$27*Supuestos!$C$32+H5/(1+Supuestos!$B$26)*Supuestos!$B$28)</f>
-        <v>0.973135593220339</v>
+        <v>0.953898305084746</v>
       </c>
       <c r="N5" s="13" t="n">
         <f aca="false">IF(H5=0,0,H5/(1+Supuestos!$B$26)-K5-M5)</f>
-        <v>1.14717372881356</v>
+        <v>0.742682203389831</v>
       </c>
       <c r="O5" s="13" t="n">
         <f aca="false">IF(H5=0,0,H5/(1+Supuestos!$B$26)-L5-M5)</f>
-        <v>1.14717372881356</v>
+        <v>0.742682203389831</v>
       </c>
       <c r="P5" s="29" t="n">
         <f aca="false">G5*N5</f>
-        <v>6919.52249745763</v>
+        <v>4479.71051440678</v>
       </c>
       <c r="Q5" s="29" t="n">
         <f aca="false">G5*O5</f>
-        <v>6919.52249745763</v>
+        <v>4479.71051440678</v>
       </c>
       <c r="R5" s="12" t="n">
         <f aca="false">IF(H5=0,0,N5/(H5/(1+Supuestos!$B$26)))</f>
-        <v>0.300814444444444</v>
+        <v>0.21909125</v>
       </c>
       <c r="S5" s="12" t="n">
         <f aca="false">IF(H5=0,0,O5/(H5/(1+Supuestos!$B$26)))</f>
-        <v>0.300814444444444</v>
+        <v>0.21909125</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3026,15 +3026,15 @@
       </c>
       <c r="H6" s="6" t="n">
         <f aca="false">Supuestos!C39</f>
-        <v>27</v>
+        <v>23.5</v>
       </c>
       <c r="I6" s="29" t="n">
         <f aca="false">G6*H6</f>
-        <v>162858.6</v>
+        <v>141747.3</v>
       </c>
       <c r="J6" s="29" t="n">
         <f aca="false">I6/(1+Supuestos!$B$26)</f>
-        <v>138015.762711864</v>
+        <v>120124.830508475</v>
       </c>
       <c r="K6" s="6" t="n">
         <f aca="false">Costeo!C15</f>
@@ -3046,31 +3046,31 @@
       </c>
       <c r="M6" s="13" t="n">
         <f aca="false">IF(H6=0,0,C6*Supuestos!$B$32+H6*Supuestos!$B$27*Supuestos!$C$32+H6/(1+Supuestos!$B$26)*Supuestos!$B$28)</f>
-        <v>5.83881355932203</v>
+        <v>5.70415254237288</v>
       </c>
       <c r="N6" s="13" t="n">
         <f aca="false">IF(H6=0,0,H6/(1+Supuestos!$B$26)-K6-M6)</f>
-        <v>7.14554237288136</v>
+        <v>4.31410169491525</v>
       </c>
       <c r="O6" s="13" t="n">
         <f aca="false">IF(H6=0,0,H6/(1+Supuestos!$B$26)-L6-M6)</f>
-        <v>7.64954237288136</v>
+        <v>4.81810169491525</v>
       </c>
       <c r="P6" s="29" t="n">
         <f aca="false">G6*N6</f>
-        <v>43100.4824847458</v>
+        <v>26021.7986033898</v>
       </c>
       <c r="Q6" s="29" t="n">
         <f aca="false">G6*O6</f>
-        <v>46140.5096847458</v>
+        <v>29061.8258033898</v>
       </c>
       <c r="R6" s="12" t="n">
         <f aca="false">IF(H6=0,0,N6/(H6/(1+Supuestos!$B$26)))</f>
-        <v>0.312286666666667</v>
+        <v>0.216622978723404</v>
       </c>
       <c r="S6" s="12" t="n">
         <f aca="false">IF(H6=0,0,O6/(H6/(1+Supuestos!$B$26)))</f>
-        <v>0.334313333333333</v>
+        <v>0.241930212765957</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3102,15 +3102,15 @@
       </c>
       <c r="H7" s="6" t="n">
         <f aca="false">Supuestos!D39</f>
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="I7" s="29" t="n">
         <f aca="false">G7*H7</f>
-        <v>73889.55</v>
+        <v>66349.8</v>
       </c>
       <c r="J7" s="29" t="n">
         <f aca="false">I7/(1+Supuestos!$B$26)</f>
-        <v>62618.2627118644</v>
+        <v>56228.6440677966</v>
       </c>
       <c r="K7" s="6" t="n">
         <f aca="false">Costeo!E15</f>
@@ -3122,31 +3122,31 @@
       </c>
       <c r="M7" s="13" t="n">
         <f aca="false">IF(H7=0,0,C7*Supuestos!$B$32+H7*Supuestos!$B$27*Supuestos!$C$32+H7/(1+Supuestos!$B$26)*Supuestos!$B$28)</f>
-        <v>11.4852542372881</v>
+        <v>11.2928813559322</v>
       </c>
       <c r="N7" s="13" t="n">
         <f aca="false">IF(H7=0,0,H7/(1+Supuestos!$B$26)-K7-M7)</f>
-        <v>11.3801694915254</v>
+        <v>7.33525423728814</v>
       </c>
       <c r="O7" s="13" t="n">
         <f aca="false">IF(H7=0,0,H7/(1+Supuestos!$B$26)-L7-M7)</f>
-        <v>11.3801694915254</v>
+        <v>7.33525423728814</v>
       </c>
       <c r="P7" s="29" t="n">
         <f aca="false">G7*N7</f>
-        <v>17160.7265847458</v>
+        <v>11061.1966271186</v>
       </c>
       <c r="Q7" s="29" t="n">
         <f aca="false">G7*O7</f>
-        <v>17160.7265847458</v>
+        <v>11061.1966271186</v>
       </c>
       <c r="R7" s="12" t="n">
         <f aca="false">IF(H7=0,0,N7/(H7/(1+Supuestos!$B$26)))</f>
-        <v>0.27405306122449</v>
+        <v>0.196718181818182</v>
       </c>
       <c r="S7" s="12" t="n">
         <f aca="false">IF(H7=0,0,O7/(H7/(1+Supuestos!$B$26)))</f>
-        <v>0.27405306122449</v>
+        <v>0.196718181818182</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3843,19 +3843,19 @@
       </c>
       <c r="I17" s="11" t="n">
         <f aca="false">SUM(I5:I16)</f>
-        <v>322971.33</v>
+        <v>291304.38</v>
       </c>
       <c r="J17" s="11" t="n">
         <f aca="false">SUM(J5:J16)</f>
-        <v>273704.516949153</v>
+        <v>246868.118644068</v>
       </c>
       <c r="P17" s="11" t="n">
         <f aca="false">SUM(P5:P16)</f>
-        <v>82183.262079661</v>
+        <v>56565.2362576271</v>
       </c>
       <c r="Q17" s="11" t="n">
         <f aca="false">SUM(Q5:Q16)</f>
-        <v>85628.505279661</v>
+        <v>60010.4794576271</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3906,27 +3906,27 @@
       </c>
       <c r="C22" s="29" t="n">
         <f aca="false">SUMIF($A$5:$A$16,A22,$P$5:$P$16)</f>
-        <v>67180.7315669492</v>
+        <v>41562.7057449153</v>
       </c>
       <c r="D22" s="29" t="n">
         <f aca="false">SUMIF($A$5:$A$16,A22,$Q$5:$Q$16)</f>
-        <v>70220.7587669492</v>
+        <v>44602.7329449152</v>
       </c>
       <c r="E22" s="29" t="n">
         <f aca="false">SUMIF($A$5:$A$16,A22,$I$5:$I$16)</f>
-        <v>263891.25</v>
+        <v>232224.3</v>
       </c>
       <c r="F22" s="13" t="n">
         <f aca="false">IF(B22=0,0,C22/B22)</f>
-        <v>1.11377584745763</v>
+        <v>0.689059745762712</v>
       </c>
       <c r="G22" s="13" t="n">
         <f aca="false">IF(B22=0,0,D22/B22)</f>
-        <v>1.16417584745763</v>
+        <v>0.739459745762712</v>
       </c>
       <c r="H22" s="13" t="n">
         <f aca="false">IF(B22=0,0,E22/B22)</f>
-        <v>4.375</v>
+        <v>3.85</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4038,27 +4038,27 @@
       </c>
       <c r="C26" s="11" t="n">
         <f aca="false">SUM(C22:C25)</f>
-        <v>82183.262079661</v>
+        <v>56565.2362576271</v>
       </c>
       <c r="D26" s="11" t="n">
         <f aca="false">SUM(D22:D25)</f>
-        <v>85628.505279661</v>
+        <v>60010.4794576271</v>
       </c>
       <c r="E26" s="11" t="n">
         <f aca="false">SUM(E22:E25)</f>
-        <v>322971.33</v>
+        <v>291304.38</v>
       </c>
       <c r="F26" s="27" t="n">
         <f aca="false">IF(B26=0,0,C26/B26)</f>
-        <v>1.07661311429437</v>
+        <v>0.741013116625757</v>
       </c>
       <c r="G26" s="27" t="n">
         <f aca="false">IF(B26=0,0,D26/B26)</f>
-        <v>1.12174631924623</v>
+        <v>0.786146321577613</v>
       </c>
       <c r="H26" s="27" t="n">
         <f aca="false">IF(B26=0,0,E26/B26)</f>
-        <v>4.23097307919041</v>
+        <v>3.81613126350953</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4111,15 +4111,15 @@
       </c>
       <c r="D30" s="29" t="n">
         <f aca="false">SUMIF($B$5:$B$16,A30,$I$5:$I$16)</f>
-        <v>68618.1</v>
+        <v>65602.2</v>
       </c>
       <c r="E30" s="29" t="n">
         <f aca="false">SUMIF($B$5:$B$16,A30,$P$5:$P$16)</f>
-        <v>17499.0972813559</v>
+        <v>15059.2852983051</v>
       </c>
       <c r="F30" s="29" t="n">
         <f aca="false">SUMIF($B$5:$B$16,A30,$Q$5:$Q$16)</f>
-        <v>17499.0972813559</v>
+        <v>15059.2852983051</v>
       </c>
       <c r="G30" s="12" t="n">
         <f aca="false">IF($F$17=0,0,B30/$F$17)</f>
@@ -4140,15 +4140,15 @@
       </c>
       <c r="D31" s="29" t="n">
         <f aca="false">SUMIF($B$5:$B$16,A31,$I$5:$I$16)</f>
-        <v>180463.68</v>
+        <v>159352.38</v>
       </c>
       <c r="E31" s="29" t="n">
         <f aca="false">SUMIF($B$5:$B$16,A31,$P$5:$P$16)</f>
-        <v>47523.4382135593</v>
+        <v>30444.7543322034</v>
       </c>
       <c r="F31" s="29" t="n">
         <f aca="false">SUMIF($B$5:$B$16,A31,$Q$5:$Q$16)</f>
-        <v>50968.6814135593</v>
+        <v>33889.9975322034</v>
       </c>
       <c r="G31" s="12" t="n">
         <f aca="false">IF($F$17=0,0,B31/$F$17)</f>
@@ -4169,15 +4169,15 @@
       </c>
       <c r="D32" s="29" t="n">
         <f aca="false">SUMIF($B$5:$B$16,A32,$I$5:$I$16)</f>
-        <v>73889.55</v>
+        <v>66349.8</v>
       </c>
       <c r="E32" s="29" t="n">
         <f aca="false">SUMIF($B$5:$B$16,A32,$P$5:$P$16)</f>
-        <v>17160.7265847458</v>
+        <v>11061.1966271186</v>
       </c>
       <c r="F32" s="29" t="n">
         <f aca="false">SUMIF($B$5:$B$16,A32,$Q$5:$Q$16)</f>
-        <v>17160.7265847458</v>
+        <v>11061.1966271186</v>
       </c>
       <c r="G32" s="12" t="n">
         <f aca="false">IF($F$17=0,0,B32/$F$17)</f>
@@ -4896,55 +4896,55 @@
       </c>
       <c r="B19" s="9" t="n">
         <f aca="false">SUMPRODUCT(B$5:B$8,Proyeccion!$H$22:$H$25)</f>
-        <v>11778</v>
+        <v>10644</v>
       </c>
       <c r="C19" s="9" t="n">
         <f aca="false">SUMPRODUCT(C$5:C$8,Proyeccion!$H$22:$H$25)</f>
-        <v>17346</v>
+        <v>15582</v>
       </c>
       <c r="D19" s="9" t="n">
         <f aca="false">SUMPRODUCT(D$5:D$8,Proyeccion!$H$22:$H$25)</f>
-        <v>22510.8</v>
+        <v>20242.8</v>
       </c>
       <c r="E19" s="9" t="n">
         <f aca="false">SUMPRODUCT(E$5:E$8,Proyeccion!$H$22:$H$25)</f>
-        <v>26695.2</v>
+        <v>23986.2</v>
       </c>
       <c r="F19" s="9" t="n">
         <f aca="false">SUMPRODUCT(F$5:F$8,Proyeccion!$H$22:$H$25)</f>
-        <v>24693.6</v>
+        <v>22274.4</v>
       </c>
       <c r="G19" s="9" t="n">
         <f aca="false">SUMPRODUCT(G$5:G$8,Proyeccion!$H$22:$H$25)</f>
-        <v>29813.25</v>
+        <v>26975.1</v>
       </c>
       <c r="H19" s="9" t="n">
         <f aca="false">SUMPRODUCT(H$5:H$8,Proyeccion!$H$22:$H$25)</f>
-        <v>36944.4</v>
+        <v>33290.4</v>
       </c>
       <c r="I19" s="9" t="n">
         <f aca="false">SUMPRODUCT(I$5:I$8,Proyeccion!$H$22:$H$25)</f>
-        <v>39569.4</v>
+        <v>35600.4</v>
       </c>
       <c r="J19" s="9" t="n">
         <f aca="false">SUMPRODUCT(J$5:J$8,Proyeccion!$H$22:$H$25)</f>
-        <v>43867.8</v>
+        <v>39583.8</v>
       </c>
       <c r="K19" s="9" t="n">
         <f aca="false">SUMPRODUCT(K$5:K$8,Proyeccion!$H$22:$H$25)</f>
-        <v>33448.2</v>
+        <v>30361.2</v>
       </c>
       <c r="L19" s="9" t="n">
         <f aca="false">SUMPRODUCT(L$5:L$8,Proyeccion!$H$22:$H$25)</f>
-        <v>15894.84</v>
+        <v>14395.44</v>
       </c>
       <c r="M19" s="9" t="n">
         <f aca="false">SUMPRODUCT(M$5:M$8,Proyeccion!$H$22:$H$25)</f>
-        <v>20409.84</v>
+        <v>18368.64</v>
       </c>
       <c r="N19" s="29" t="n">
         <f aca="false">SUM(B19:M19)</f>
-        <v>322971.33</v>
+        <v>291304.38</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4953,55 +4953,55 @@
       </c>
       <c r="B20" s="29" t="n">
         <f aca="false">B19/(1+Supuestos!$B$26)</f>
-        <v>9981.35593220339</v>
+        <v>9020.33898305085</v>
       </c>
       <c r="C20" s="29" t="n">
         <f aca="false">C19/(1+Supuestos!$B$26)</f>
-        <v>14700</v>
+        <v>13205.0847457627</v>
       </c>
       <c r="D20" s="29" t="n">
         <f aca="false">D19/(1+Supuestos!$B$26)</f>
-        <v>19076.9491525424</v>
+        <v>17154.9152542373</v>
       </c>
       <c r="E20" s="29" t="n">
         <f aca="false">E19/(1+Supuestos!$B$26)</f>
-        <v>22623.0508474576</v>
+        <v>20327.2881355932</v>
       </c>
       <c r="F20" s="29" t="n">
         <f aca="false">F19/(1+Supuestos!$B$26)</f>
-        <v>20926.779661017</v>
+        <v>18876.6101694915</v>
       </c>
       <c r="G20" s="29" t="n">
         <f aca="false">G19/(1+Supuestos!$B$26)</f>
-        <v>25265.4661016949</v>
+        <v>22860.2542372881</v>
       </c>
       <c r="H20" s="29" t="n">
         <f aca="false">H19/(1+Supuestos!$B$26)</f>
-        <v>31308.813559322</v>
+        <v>28212.2033898305</v>
       </c>
       <c r="I20" s="29" t="n">
         <f aca="false">I19/(1+Supuestos!$B$26)</f>
-        <v>33533.3898305085</v>
+        <v>30169.8305084746</v>
       </c>
       <c r="J20" s="29" t="n">
         <f aca="false">J19/(1+Supuestos!$B$26)</f>
-        <v>37176.1016949153</v>
+        <v>33545.593220339</v>
       </c>
       <c r="K20" s="29" t="n">
         <f aca="false">K19/(1+Supuestos!$B$26)</f>
-        <v>28345.9322033898</v>
+        <v>25729.8305084746</v>
       </c>
       <c r="L20" s="29" t="n">
         <f aca="false">L19/(1+Supuestos!$B$26)</f>
-        <v>13470.2033898305</v>
+        <v>12199.5254237288</v>
       </c>
       <c r="M20" s="29" t="n">
         <f aca="false">M19/(1+Supuestos!$B$26)</f>
-        <v>17296.4745762712</v>
+        <v>15566.6440677966</v>
       </c>
       <c r="N20" s="29" t="n">
         <f aca="false">SUM(B20:M20)</f>
-        <v>273704.516949153</v>
+        <v>246868.118644068</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5010,55 +5010,55 @@
       </c>
       <c r="B21" s="9" t="n">
         <f aca="false">SUMPRODUCT(B$5:B$8,Proyeccion!$F$22:$F$25)</f>
-        <v>3002.60837288136</v>
+        <v>2085.22159322034</v>
       </c>
       <c r="C21" s="9" t="n">
         <f aca="false">SUMPRODUCT(C$5:C$8,Proyeccion!$F$22:$F$25)</f>
-        <v>4407.036</v>
+        <v>2979.98989830509</v>
       </c>
       <c r="D21" s="9" t="n">
         <f aca="false">SUMPRODUCT(D$5:D$8,Proyeccion!$F$22:$F$25)</f>
-        <v>5730.69666101695</v>
+        <v>3895.92310169492</v>
       </c>
       <c r="E21" s="9" t="n">
         <f aca="false">SUMPRODUCT(E$5:E$8,Proyeccion!$F$22:$F$25)</f>
-        <v>6786.77633898305</v>
+        <v>4595.24125423729</v>
       </c>
       <c r="F21" s="9" t="n">
         <f aca="false">SUMPRODUCT(F$5:F$8,Proyeccion!$F$22:$F$25)</f>
-        <v>6286.95266440678</v>
+        <v>4329.86086779661</v>
       </c>
       <c r="G21" s="9" t="n">
         <f aca="false">SUMPRODUCT(G$5:G$8,Proyeccion!$F$22:$F$25)</f>
-        <v>7583.82454067797</v>
+        <v>5287.80929491526</v>
       </c>
       <c r="H21" s="9" t="n">
         <f aca="false">SUMPRODUCT(H$5:H$8,Proyeccion!$F$22:$F$25)</f>
-        <v>9383.62642372882</v>
+        <v>6427.60235593221</v>
       </c>
       <c r="I21" s="9" t="n">
         <f aca="false">SUMPRODUCT(I$5:I$8,Proyeccion!$F$22:$F$25)</f>
-        <v>10051.8919322034</v>
+        <v>6841.03820338983</v>
       </c>
       <c r="J21" s="9" t="n">
         <f aca="false">SUMPRODUCT(J$5:J$8,Proyeccion!$F$22:$F$25)</f>
-        <v>11139.0916779661</v>
+        <v>7673.4082881356</v>
       </c>
       <c r="K21" s="9" t="n">
         <f aca="false">SUMPRODUCT(K$5:K$8,Proyeccion!$F$22:$F$25)</f>
-        <v>8516.50088135593</v>
+        <v>6019.17020338983</v>
       </c>
       <c r="L21" s="9" t="n">
         <f aca="false">SUMPRODUCT(L$5:L$8,Proyeccion!$F$22:$F$25)</f>
-        <v>4072.4199559322</v>
+        <v>2859.43076949153</v>
       </c>
       <c r="M21" s="9" t="n">
         <f aca="false">SUMPRODUCT(M$5:M$8,Proyeccion!$F$22:$F$25)</f>
-        <v>5221.83663050848</v>
+        <v>3570.54042711865</v>
       </c>
       <c r="N21" s="29" t="n">
         <f aca="false">SUM(B21:M21)</f>
-        <v>82183.262079661</v>
+        <v>56565.2362576271</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5067,55 +5067,55 @@
       </c>
       <c r="B22" s="9" t="n">
         <f aca="false">SUMPRODUCT(B$5:B$8,Proyeccion!$G$22:$G$25)</f>
-        <v>3123.56837288136</v>
+        <v>2206.18159322034</v>
       </c>
       <c r="C22" s="9" t="n">
         <f aca="false">SUMPRODUCT(C$5:C$8,Proyeccion!$G$22:$G$25)</f>
-        <v>4585.452</v>
+        <v>3158.40589830508</v>
       </c>
       <c r="D22" s="9" t="n">
         <f aca="false">SUMPRODUCT(D$5:D$8,Proyeccion!$G$22:$G$25)</f>
-        <v>5970.60066101695</v>
+        <v>4135.82710169492</v>
       </c>
       <c r="E22" s="9" t="n">
         <f aca="false">SUMPRODUCT(E$5:E$8,Proyeccion!$G$22:$G$25)</f>
-        <v>7071.03233898305</v>
+        <v>4879.49725423729</v>
       </c>
       <c r="F22" s="9" t="n">
         <f aca="false">SUMPRODUCT(F$5:F$8,Proyeccion!$G$22:$G$25)</f>
-        <v>6551.45186440678</v>
+        <v>4594.36006779661</v>
       </c>
       <c r="G22" s="9" t="n">
         <f aca="false">SUMPRODUCT(G$5:G$8,Proyeccion!$G$22:$G$25)</f>
-        <v>7896.60694067797</v>
+        <v>5600.59169491525</v>
       </c>
       <c r="H22" s="9" t="n">
         <f aca="false">SUMPRODUCT(H$5:H$8,Proyeccion!$G$22:$G$25)</f>
-        <v>9773.72242372882</v>
+        <v>6817.6983559322</v>
       </c>
       <c r="I22" s="9" t="n">
         <f aca="false">SUMPRODUCT(I$5:I$8,Proyeccion!$G$22:$G$25)</f>
-        <v>10472.2279322034</v>
+        <v>7261.37420338983</v>
       </c>
       <c r="J22" s="9" t="n">
         <f aca="false">SUMPRODUCT(J$5:J$8,Proyeccion!$G$22:$G$25)</f>
-        <v>11597.7316779661</v>
+        <v>8132.04828813559</v>
       </c>
       <c r="K22" s="9" t="n">
         <f aca="false">SUMPRODUCT(K$5:K$8,Proyeccion!$G$22:$G$25)</f>
-        <v>8871.31688135593</v>
+        <v>6373.98620338983</v>
       </c>
       <c r="L22" s="9" t="n">
         <f aca="false">SUMPRODUCT(L$5:L$8,Proyeccion!$G$22:$G$25)</f>
-        <v>4256.6823559322</v>
+        <v>3043.69316949152</v>
       </c>
       <c r="M22" s="9" t="n">
         <f aca="false">SUMPRODUCT(M$5:M$8,Proyeccion!$G$22:$G$25)</f>
-        <v>5458.11183050848</v>
+        <v>3806.81562711864</v>
       </c>
       <c r="N22" s="29" t="n">
         <f aca="false">SUM(B22:M22)</f>
-        <v>85628.505279661</v>
+        <v>60010.4794576271</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5181,55 +5181,55 @@
       </c>
       <c r="B24" s="11" t="n">
         <f aca="false">B21-B23</f>
-        <v>145.938372881356</v>
+        <v>-771.448406779661</v>
       </c>
       <c r="C24" s="11" t="n">
         <f aca="false">C21-C23</f>
-        <v>1550.366</v>
+        <v>123.319898305085</v>
       </c>
       <c r="D24" s="11" t="n">
         <f aca="false">D21-D23</f>
-        <v>2874.02666101695</v>
+        <v>1039.25310169492</v>
       </c>
       <c r="E24" s="11" t="n">
         <f aca="false">E21-E23</f>
-        <v>3930.10633898305</v>
+        <v>1738.57125423729</v>
       </c>
       <c r="F24" s="11" t="n">
         <f aca="false">F21-F23</f>
-        <v>3430.28266440678</v>
+        <v>1473.19086779661</v>
       </c>
       <c r="G24" s="11" t="n">
         <f aca="false">G21-G23</f>
-        <v>4727.15454067797</v>
+        <v>2431.13929491526</v>
       </c>
       <c r="H24" s="11" t="n">
         <f aca="false">H21-H23</f>
-        <v>6526.95642372882</v>
+        <v>3570.9323559322</v>
       </c>
       <c r="I24" s="11" t="n">
         <f aca="false">I21-I23</f>
-        <v>7195.22193220339</v>
+        <v>3984.36820338983</v>
       </c>
       <c r="J24" s="11" t="n">
         <f aca="false">J21-J23</f>
-        <v>8282.4216779661</v>
+        <v>4816.7382881356</v>
       </c>
       <c r="K24" s="11" t="n">
         <f aca="false">K21-K23</f>
-        <v>5659.83088135593</v>
+        <v>3162.50020338983</v>
       </c>
       <c r="L24" s="11" t="n">
         <f aca="false">L21-L23</f>
-        <v>1215.7499559322</v>
+        <v>2.76076949152593</v>
       </c>
       <c r="M24" s="11" t="n">
         <f aca="false">M21-M23</f>
-        <v>2365.16663050848</v>
+        <v>713.870427118645</v>
       </c>
       <c r="N24" s="11" t="n">
         <f aca="false">SUM(B24:M24)</f>
-        <v>47903.222079661</v>
+        <v>22285.1962576271</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5238,55 +5238,55 @@
       </c>
       <c r="B25" s="11" t="n">
         <f aca="false">B22-B23</f>
-        <v>266.898372881356</v>
+        <v>-650.488406779662</v>
       </c>
       <c r="C25" s="11" t="n">
         <f aca="false">C22-C23</f>
-        <v>1728.782</v>
+        <v>301.735898305084</v>
       </c>
       <c r="D25" s="11" t="n">
         <f aca="false">D22-D23</f>
-        <v>3113.93066101695</v>
+        <v>1279.15710169491</v>
       </c>
       <c r="E25" s="11" t="n">
         <f aca="false">E22-E23</f>
-        <v>4214.36233898305</v>
+        <v>2022.82725423729</v>
       </c>
       <c r="F25" s="11" t="n">
         <f aca="false">F22-F23</f>
-        <v>3694.78186440678</v>
+        <v>1737.69006779661</v>
       </c>
       <c r="G25" s="11" t="n">
         <f aca="false">G22-G23</f>
-        <v>5039.93694067797</v>
+        <v>2743.92169491525</v>
       </c>
       <c r="H25" s="11" t="n">
         <f aca="false">H22-H23</f>
-        <v>6917.05242372882</v>
+        <v>3961.0283559322</v>
       </c>
       <c r="I25" s="11" t="n">
         <f aca="false">I22-I23</f>
-        <v>7615.55793220339</v>
+        <v>4404.70420338983</v>
       </c>
       <c r="J25" s="11" t="n">
         <f aca="false">J22-J23</f>
-        <v>8741.06167796611</v>
+        <v>5275.37828813559</v>
       </c>
       <c r="K25" s="11" t="n">
         <f aca="false">K22-K23</f>
-        <v>6014.64688135593</v>
+        <v>3517.31620338983</v>
       </c>
       <c r="L25" s="11" t="n">
         <f aca="false">L22-L23</f>
-        <v>1400.0123559322</v>
+        <v>187.023169491525</v>
       </c>
       <c r="M25" s="11" t="n">
         <f aca="false">M22-M23</f>
-        <v>2601.44183050848</v>
+        <v>950.145627118643</v>
       </c>
       <c r="N25" s="11" t="n">
         <f aca="false">SUM(B25:M25)</f>
-        <v>51348.465279661</v>
+        <v>25730.4394576271</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5295,51 +5295,51 @@
       </c>
       <c r="B26" s="29" t="n">
         <f aca="false">B24</f>
-        <v>145.938372881356</v>
+        <v>-771.448406779661</v>
       </c>
       <c r="C26" s="29" t="n">
         <f aca="false">B26+C24</f>
-        <v>1696.30437288136</v>
+        <v>-648.128508474576</v>
       </c>
       <c r="D26" s="29" t="n">
         <f aca="false">C26+D24</f>
-        <v>4570.33103389831</v>
+        <v>391.124593220341</v>
       </c>
       <c r="E26" s="29" t="n">
         <f aca="false">D26+E24</f>
-        <v>8500.43737288136</v>
+        <v>2129.69584745763</v>
       </c>
       <c r="F26" s="29" t="n">
         <f aca="false">E26+F24</f>
-        <v>11930.7200372881</v>
+        <v>3602.88671525424</v>
       </c>
       <c r="G26" s="29" t="n">
         <f aca="false">F26+G24</f>
-        <v>16657.8745779661</v>
+        <v>6034.0260101695</v>
       </c>
       <c r="H26" s="29" t="n">
         <f aca="false">G26+H24</f>
-        <v>23184.8310016949</v>
+        <v>9604.9583661017</v>
       </c>
       <c r="I26" s="29" t="n">
         <f aca="false">H26+I24</f>
-        <v>30380.0529338983</v>
+        <v>13589.3265694915</v>
       </c>
       <c r="J26" s="29" t="n">
         <f aca="false">I26+J24</f>
-        <v>38662.4746118644</v>
+        <v>18406.0648576271</v>
       </c>
       <c r="K26" s="29" t="n">
         <f aca="false">J26+K24</f>
-        <v>44322.3054932204</v>
+        <v>21568.565061017</v>
       </c>
       <c r="L26" s="29" t="n">
         <f aca="false">K26+L24</f>
-        <v>45538.0554491526</v>
+        <v>21571.3258305085</v>
       </c>
       <c r="M26" s="29" t="n">
         <f aca="false">L26+M24</f>
-        <v>47903.222079661</v>
+        <v>22285.1962576271</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5348,51 +5348,51 @@
       </c>
       <c r="B27" s="29" t="n">
         <f aca="false">B25</f>
-        <v>266.898372881356</v>
+        <v>-650.488406779662</v>
       </c>
       <c r="C27" s="29" t="n">
         <f aca="false">B27+C25</f>
-        <v>1995.68037288136</v>
+        <v>-348.752508474578</v>
       </c>
       <c r="D27" s="29" t="n">
         <f aca="false">C27+D25</f>
-        <v>5109.61103389831</v>
+        <v>930.404593220337</v>
       </c>
       <c r="E27" s="29" t="n">
         <f aca="false">D27+E25</f>
-        <v>9323.97337288136</v>
+        <v>2953.23184745762</v>
       </c>
       <c r="F27" s="29" t="n">
         <f aca="false">E27+F25</f>
-        <v>13018.7552372881</v>
+        <v>4690.92191525423</v>
       </c>
       <c r="G27" s="29" t="n">
         <f aca="false">F27+G25</f>
-        <v>18058.6921779661</v>
+        <v>7434.84361016949</v>
       </c>
       <c r="H27" s="29" t="n">
         <f aca="false">G27+H25</f>
-        <v>24975.7446016949</v>
+        <v>11395.8719661017</v>
       </c>
       <c r="I27" s="29" t="n">
         <f aca="false">H27+I25</f>
-        <v>32591.3025338983</v>
+        <v>15800.5761694915</v>
       </c>
       <c r="J27" s="29" t="n">
         <f aca="false">I27+J25</f>
-        <v>41332.3642118644</v>
+        <v>21075.9544576271</v>
       </c>
       <c r="K27" s="29" t="n">
         <f aca="false">J27+K25</f>
-        <v>47347.0110932204</v>
+        <v>24593.2706610169</v>
       </c>
       <c r="L27" s="29" t="n">
         <f aca="false">K27+L25</f>
-        <v>48747.0234491526</v>
+        <v>24780.2938305085</v>
       </c>
       <c r="M27" s="29" t="n">
         <f aca="false">L27+M25</f>
-        <v>51348.465279661</v>
+        <v>25730.4394576271</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Costeo: precios de ferias (S/5, S/25, S/42) y tienda naturista (S/24) ajustados por el equipo
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Kfbf7cfV7pXUcNjjyaPCzV
</commit_message>
<xml_diff>
--- a/04-reformulacion/Costeo-presentaciones-AndiBite.xlsx
+++ b/04-reformulacion/Costeo-presentaciones-AndiBite.xlsx
@@ -382,13 +382,13 @@
     <t xml:space="preserve">Precios ajustados por el equipo (9-oct-2026). Unidad = caja degustación de 3 (S/12.00) o unidades agregadas al pedido</t>
   </si>
   <si>
-    <t xml:space="preserve">La unidad suelta cuesta más que dentro del pack para empujar el pack</t>
+    <t xml:space="preserve">Precios ajustados por el equipo (9-oct-2026). La unidad suelta cuesta más que dentro del pack</t>
   </si>
   <si>
     <t xml:space="preserve">El alumno paga S/4.00; el concesionario se queda 25 %</t>
   </si>
   <si>
-    <t xml:space="preserve">Precio en anaquel S/31.90; la tienda se queda 40 %</t>
+    <t xml:space="preserve">Precio ajustado por el equipo (9-oct-2026): lo que cobra AndiBite a la tienda. Con 40 % para la tienda, el anaquel quedaría en S/40.00</t>
   </si>
   <si>
     <t xml:space="preserve">6. Mezcla de presentaciones por canal (% de las unidades que vende cada canal)</t>
@@ -1557,11 +1557,11 @@
       </c>
       <c r="B13" s="9" t="n">
         <f aca="false">Proyeccion!I17</f>
-        <v>291304.38</v>
+        <v>293277.3</v>
       </c>
       <c r="C13" s="9" t="n">
         <f aca="false">Proyeccion!I17</f>
-        <v>291304.38</v>
+        <v>293277.3</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1570,11 +1570,11 @@
       </c>
       <c r="B14" s="9" t="n">
         <f aca="false">Proyeccion!J17</f>
-        <v>246868.118644068</v>
+        <v>248540.084745763</v>
       </c>
       <c r="C14" s="9" t="n">
         <f aca="false">Proyeccion!J17</f>
-        <v>246868.118644068</v>
+        <v>248540.084745763</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1583,11 +1583,11 @@
       </c>
       <c r="B15" s="9" t="n">
         <f aca="false">Proyeccion!P17</f>
-        <v>56565.2362576271</v>
+        <v>58237.4026983051</v>
       </c>
       <c r="C15" s="9" t="n">
         <f aca="false">Proyeccion!Q17</f>
-        <v>60010.4794576271</v>
+        <v>61682.6458983051</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1609,11 +1609,11 @@
       </c>
       <c r="B17" s="11" t="n">
         <f aca="false">B15-B16</f>
-        <v>22285.1962576271</v>
+        <v>23957.3626983051</v>
       </c>
       <c r="C17" s="11" t="n">
         <f aca="false">C15-C16</f>
-        <v>25730.4394576271</v>
+        <v>27402.6058983051</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1622,11 +1622,11 @@
       </c>
       <c r="B18" s="12" t="n">
         <f aca="false">IF(B14=0,0,B17/B14)</f>
-        <v>0.0902716656165623</v>
+        <v>0.0963923494385689</v>
       </c>
       <c r="C18" s="12" t="n">
         <f aca="false">IF(C14=0,0,C17/C14)</f>
-        <v>0.10422747011219</v>
+        <v>0.11025427116248</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1635,11 +1635,11 @@
       </c>
       <c r="B19" s="13" t="n">
         <f aca="false">IF(B12=0,0,B15/B12)</f>
-        <v>0.741013116625757</v>
+        <v>0.762918748913409</v>
       </c>
       <c r="C19" s="13" t="n">
         <f aca="false">IF(C12=0,0,C15/C12)</f>
-        <v>0.786146321577613</v>
+        <v>0.808051953865266</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1648,11 +1648,11 @@
       </c>
       <c r="B20" s="14" t="n">
         <f aca="false">IF(B19&lt;=0,"No alcanza",Supuestos!$B$58/B19)</f>
-        <v>3855.0869558261</v>
+        <v>3744.39611566582</v>
       </c>
       <c r="C20" s="14" t="n">
         <f aca="false">IF(C19&lt;=0,"No alcanza",Supuestos!$B$58/C19)</f>
-        <v>3633.76374294715</v>
+        <v>3535.25535868739</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1661,11 +1661,11 @@
       </c>
       <c r="B21" s="15" t="n">
         <f aca="false">IF(ISNUMBER(B20),B20/6,"No alcanza")</f>
-        <v>642.514492637684</v>
+        <v>624.066019277637</v>
       </c>
       <c r="C21" s="15" t="n">
         <f aca="false">IF(ISNUMBER(C20),C20/6,"No alcanza")</f>
-        <v>605.627290491191</v>
+        <v>589.209226447899</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2162,10 +2162,10 @@
         <v>5</v>
       </c>
       <c r="C40" s="24" t="n">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="D40" s="24" t="n">
-        <v>49</v>
+        <v>42</v>
       </c>
       <c r="E40" s="4" t="s">
         <v>111</v>
@@ -2196,7 +2196,7 @@
         <v>0</v>
       </c>
       <c r="C42" s="24" t="n">
-        <v>19.14</v>
+        <v>24</v>
       </c>
       <c r="D42" s="24" t="n">
         <v>0</v>
@@ -3254,15 +3254,15 @@
       </c>
       <c r="H9" s="6" t="n">
         <f aca="false">Supuestos!C40</f>
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="I9" s="29" t="n">
         <f aca="false">G9*H9</f>
-        <v>7614</v>
+        <v>7050</v>
       </c>
       <c r="J9" s="29" t="n">
         <f aca="false">I9/(1+Supuestos!$B$26)</f>
-        <v>6452.54237288136</v>
+        <v>5974.57627118644</v>
       </c>
       <c r="K9" s="6" t="n">
         <f aca="false">Costeo!C15</f>
@@ -3274,31 +3274,31 @@
       </c>
       <c r="M9" s="13" t="n">
         <f aca="false">IF(H9=0,0,C9*Supuestos!$B$33+H9*Supuestos!$B$27*Supuestos!$C$33+H9/(1+Supuestos!$B$26)*Supuestos!$B$28)</f>
-        <v>7.03881355932203</v>
+        <v>6.96186440677966</v>
       </c>
       <c r="N9" s="13" t="n">
         <f aca="false">IF(H9=0,0,H9/(1+Supuestos!$B$26)-K9-M9)</f>
-        <v>5.94554237288136</v>
+        <v>4.32757627118644</v>
       </c>
       <c r="O9" s="13" t="n">
         <f aca="false">IF(H9=0,0,H9/(1+Supuestos!$B$26)-L9-M9)</f>
-        <v>6.44954237288136</v>
+        <v>4.83157627118644</v>
       </c>
       <c r="P9" s="29" t="n">
         <f aca="false">G9*N9</f>
-        <v>1676.64294915254</v>
+        <v>1220.37650847458</v>
       </c>
       <c r="Q9" s="29" t="n">
         <f aca="false">G9*O9</f>
-        <v>1818.77094915254</v>
+        <v>1362.50450847458</v>
       </c>
       <c r="R9" s="12" t="n">
         <f aca="false">IF(H9=0,0,N9/(H9/(1+Supuestos!$B$26)))</f>
-        <v>0.259842222222222</v>
+        <v>0.2042616</v>
       </c>
       <c r="S9" s="12" t="n">
         <f aca="false">IF(H9=0,0,O9/(H9/(1+Supuestos!$B$26)))</f>
-        <v>0.281868888888889</v>
+        <v>0.2280504</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3330,7 +3330,7 @@
       </c>
       <c r="H10" s="6" t="n">
         <f aca="false">Supuestos!D40</f>
-        <v>49</v>
+        <v>42</v>
       </c>
       <c r="I10" s="29" t="n">
         <f aca="false">G10*H10</f>
@@ -3350,15 +3350,15 @@
       </c>
       <c r="M10" s="13" t="n">
         <f aca="false">IF(H10=0,0,C10*Supuestos!$B$33+H10*Supuestos!$B$27*Supuestos!$C$33+H10/(1+Supuestos!$B$26)*Supuestos!$B$28)</f>
-        <v>13.8852542372881</v>
+        <v>13.6159322033898</v>
       </c>
       <c r="N10" s="13" t="n">
         <f aca="false">IF(H10=0,0,H10/(1+Supuestos!$B$26)-K10-M10)</f>
-        <v>8.98016949152543</v>
+        <v>3.31728813559323</v>
       </c>
       <c r="O10" s="13" t="n">
         <f aca="false">IF(H10=0,0,H10/(1+Supuestos!$B$26)-L10-M10)</f>
-        <v>8.98016949152543</v>
+        <v>3.31728813559323</v>
       </c>
       <c r="P10" s="29" t="n">
         <f aca="false">G10*N10</f>
@@ -3370,11 +3370,11 @@
       </c>
       <c r="R10" s="12" t="n">
         <f aca="false">IF(H10=0,0,N10/(H10/(1+Supuestos!$B$26)))</f>
-        <v>0.216257142857143</v>
+        <v>0.0932000000000001</v>
       </c>
       <c r="S10" s="12" t="n">
         <f aca="false">IF(H10=0,0,O10/(H10/(1+Supuestos!$B$26)))</f>
-        <v>0.216257142857143</v>
+        <v>0.0932000000000001</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3710,15 +3710,15 @@
       </c>
       <c r="H15" s="6" t="n">
         <f aca="false">Supuestos!C42</f>
-        <v>19.14</v>
+        <v>24</v>
       </c>
       <c r="I15" s="29" t="n">
         <f aca="false">G15*H15</f>
-        <v>9991.08</v>
+        <v>12528</v>
       </c>
       <c r="J15" s="29" t="n">
         <f aca="false">I15/(1+Supuestos!$B$26)</f>
-        <v>8467.01694915254</v>
+        <v>10616.9491525424</v>
       </c>
       <c r="K15" s="6" t="n">
         <f aca="false">Costeo!C15</f>
@@ -3730,31 +3730,31 @@
       </c>
       <c r="M15" s="13" t="n">
         <f aca="false">IF(H15=0,0,C15*Supuestos!$B$35+H15*Supuestos!$B$27*Supuestos!$C$35+H15/(1+Supuestos!$B$26)*Supuestos!$B$28)</f>
-        <v>1.06220338983051</v>
+        <v>1.10338983050847</v>
       </c>
       <c r="N15" s="13" t="n">
         <f aca="false">IF(H15=0,0,H15/(1+Supuestos!$B$26)-K15-M15)</f>
-        <v>5.26113559322034</v>
+        <v>9.33859322033899</v>
       </c>
       <c r="O15" s="13" t="n">
         <f aca="false">IF(H15=0,0,H15/(1+Supuestos!$B$26)-L15-M15)</f>
-        <v>5.76513559322034</v>
+        <v>9.84259322033899</v>
       </c>
       <c r="P15" s="29" t="n">
         <f aca="false">G15*N15</f>
-        <v>2746.31277966102</v>
+        <v>4874.74566101695</v>
       </c>
       <c r="Q15" s="29" t="n">
         <f aca="false">G15*O15</f>
-        <v>3009.40077966102</v>
+        <v>5137.83366101695</v>
       </c>
       <c r="R15" s="12" t="n">
         <f aca="false">IF(H15=0,0,N15/(H15/(1+Supuestos!$B$26)))</f>
-        <v>0.324354231974922</v>
+        <v>0.4591475</v>
       </c>
       <c r="S15" s="12" t="n">
         <f aca="false">IF(H15=0,0,O15/(H15/(1+Supuestos!$B$26)))</f>
-        <v>0.355426332288401</v>
+        <v>0.4839275</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3843,19 +3843,19 @@
       </c>
       <c r="I17" s="11" t="n">
         <f aca="false">SUM(I5:I16)</f>
-        <v>291304.38</v>
+        <v>293277.3</v>
       </c>
       <c r="J17" s="11" t="n">
         <f aca="false">SUM(J5:J16)</f>
-        <v>246868.118644068</v>
+        <v>248540.084745763</v>
       </c>
       <c r="P17" s="11" t="n">
         <f aca="false">SUM(P5:P16)</f>
-        <v>56565.2362576271</v>
+        <v>58237.4026983051</v>
       </c>
       <c r="Q17" s="11" t="n">
         <f aca="false">SUM(Q5:Q16)</f>
-        <v>60010.4794576271</v>
+        <v>61682.6458983051</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3939,27 +3939,27 @@
       </c>
       <c r="C23" s="29" t="n">
         <f aca="false">SUMIF($A$5:$A$16,A23,$P$5:$P$16)</f>
-        <v>7013.01737288136</v>
+        <v>6556.75093220339</v>
       </c>
       <c r="D23" s="29" t="n">
         <f aca="false">SUMIF($A$5:$A$16,A23,$Q$5:$Q$16)</f>
-        <v>7155.14537288136</v>
+        <v>6698.87893220339</v>
       </c>
       <c r="E23" s="29" t="n">
         <f aca="false">SUMIF($A$5:$A$16,A23,$I$5:$I$16)</f>
-        <v>27354</v>
+        <v>26790</v>
       </c>
       <c r="F23" s="13" t="n">
         <f aca="false">IF(B23=0,0,C23/B23)</f>
-        <v>1.24344279661017</v>
+        <v>1.16254449152542</v>
       </c>
       <c r="G23" s="13" t="n">
         <f aca="false">IF(B23=0,0,D23/B23)</f>
-        <v>1.26864279661017</v>
+        <v>1.18774449152542</v>
       </c>
       <c r="H23" s="13" t="n">
         <f aca="false">IF(B23=0,0,E23/B23)</f>
-        <v>4.85</v>
+        <v>4.75</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4005,27 +4005,27 @@
       </c>
       <c r="C25" s="29" t="n">
         <f aca="false">SUMIF($A$5:$A$16,A25,$P$5:$P$16)</f>
-        <v>2746.31277966102</v>
+        <v>4874.74566101695</v>
       </c>
       <c r="D25" s="29" t="n">
         <f aca="false">SUMIF($A$5:$A$16,A25,$Q$5:$Q$16)</f>
-        <v>3009.40077966102</v>
+        <v>5137.83366101695</v>
       </c>
       <c r="E25" s="29" t="n">
         <f aca="false">SUMIF($A$5:$A$16,A25,$I$5:$I$16)</f>
-        <v>9991.08</v>
+        <v>12528</v>
       </c>
       <c r="F25" s="13" t="n">
         <f aca="false">IF(B25=0,0,C25/B25)</f>
-        <v>0.87685593220339</v>
+        <v>1.55643220338983</v>
       </c>
       <c r="G25" s="13" t="n">
         <f aca="false">IF(B25=0,0,D25/B25)</f>
-        <v>0.96085593220339</v>
+        <v>1.64043220338983</v>
       </c>
       <c r="H25" s="13" t="n">
         <f aca="false">IF(B25=0,0,E25/B25)</f>
-        <v>3.19</v>
+        <v>4</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4038,27 +4038,27 @@
       </c>
       <c r="C26" s="11" t="n">
         <f aca="false">SUM(C22:C25)</f>
-        <v>56565.2362576271</v>
+        <v>58237.4026983051</v>
       </c>
       <c r="D26" s="11" t="n">
         <f aca="false">SUM(D22:D25)</f>
-        <v>60010.4794576271</v>
+        <v>61682.6458983051</v>
       </c>
       <c r="E26" s="11" t="n">
         <f aca="false">SUM(E22:E25)</f>
-        <v>291304.38</v>
+        <v>293277.3</v>
       </c>
       <c r="F26" s="27" t="n">
         <f aca="false">IF(B26=0,0,C26/B26)</f>
-        <v>0.741013116625757</v>
+        <v>0.762918748913409</v>
       </c>
       <c r="G26" s="27" t="n">
         <f aca="false">IF(B26=0,0,D26/B26)</f>
-        <v>0.786146321577613</v>
+        <v>0.808051953865266</v>
       </c>
       <c r="H26" s="27" t="n">
         <f aca="false">IF(B26=0,0,E26/B26)</f>
-        <v>3.81613126350953</v>
+        <v>3.84197681273335</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4140,15 +4140,15 @@
       </c>
       <c r="D31" s="29" t="n">
         <f aca="false">SUMIF($B$5:$B$16,A31,$I$5:$I$16)</f>
-        <v>159352.38</v>
+        <v>161325.3</v>
       </c>
       <c r="E31" s="29" t="n">
         <f aca="false">SUMIF($B$5:$B$16,A31,$P$5:$P$16)</f>
-        <v>30444.7543322034</v>
+        <v>32116.9207728814</v>
       </c>
       <c r="F31" s="29" t="n">
         <f aca="false">SUMIF($B$5:$B$16,A31,$Q$5:$Q$16)</f>
-        <v>33889.9975322034</v>
+        <v>35562.1639728813</v>
       </c>
       <c r="G31" s="12" t="n">
         <f aca="false">IF($F$17=0,0,B31/$F$17)</f>
@@ -4896,55 +4896,55 @@
       </c>
       <c r="B19" s="9" t="n">
         <f aca="false">SUMPRODUCT(B$5:B$8,Proyeccion!$H$22:$H$25)</f>
-        <v>10644</v>
+        <v>10596</v>
       </c>
       <c r="C19" s="9" t="n">
         <f aca="false">SUMPRODUCT(C$5:C$8,Proyeccion!$H$22:$H$25)</f>
-        <v>15582</v>
+        <v>15546</v>
       </c>
       <c r="D19" s="9" t="n">
         <f aca="false">SUMPRODUCT(D$5:D$8,Proyeccion!$H$22:$H$25)</f>
-        <v>20242.8</v>
+        <v>20292</v>
       </c>
       <c r="E19" s="9" t="n">
         <f aca="false">SUMPRODUCT(E$5:E$8,Proyeccion!$H$22:$H$25)</f>
-        <v>23986.2</v>
+        <v>24096</v>
       </c>
       <c r="F19" s="9" t="n">
         <f aca="false">SUMPRODUCT(F$5:F$8,Proyeccion!$H$22:$H$25)</f>
-        <v>22274.4</v>
+        <v>22420.8</v>
       </c>
       <c r="G19" s="9" t="n">
         <f aca="false">SUMPRODUCT(G$5:G$8,Proyeccion!$H$22:$H$25)</f>
-        <v>26975.1</v>
+        <v>27158.1</v>
       </c>
       <c r="H19" s="9" t="n">
         <f aca="false">SUMPRODUCT(H$5:H$8,Proyeccion!$H$22:$H$25)</f>
-        <v>33290.4</v>
+        <v>33546</v>
       </c>
       <c r="I19" s="9" t="n">
         <f aca="false">SUMPRODUCT(I$5:I$8,Proyeccion!$H$22:$H$25)</f>
-        <v>35600.4</v>
+        <v>35856</v>
       </c>
       <c r="J19" s="9" t="n">
         <f aca="false">SUMPRODUCT(J$5:J$8,Proyeccion!$H$22:$H$25)</f>
-        <v>39583.8</v>
+        <v>39876</v>
       </c>
       <c r="K19" s="9" t="n">
         <f aca="false">SUMPRODUCT(K$5:K$8,Proyeccion!$H$22:$H$25)</f>
-        <v>30361.2</v>
+        <v>30678</v>
       </c>
       <c r="L19" s="9" t="n">
         <f aca="false">SUMPRODUCT(L$5:L$8,Proyeccion!$H$22:$H$25)</f>
-        <v>14395.44</v>
+        <v>14619.6</v>
       </c>
       <c r="M19" s="9" t="n">
         <f aca="false">SUMPRODUCT(M$5:M$8,Proyeccion!$H$22:$H$25)</f>
-        <v>18368.64</v>
+        <v>18592.8</v>
       </c>
       <c r="N19" s="29" t="n">
         <f aca="false">SUM(B19:M19)</f>
-        <v>291304.38</v>
+        <v>293277.3</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4953,55 +4953,55 @@
       </c>
       <c r="B20" s="29" t="n">
         <f aca="false">B19/(1+Supuestos!$B$26)</f>
-        <v>9020.33898305085</v>
+        <v>8979.66101694915</v>
       </c>
       <c r="C20" s="29" t="n">
         <f aca="false">C19/(1+Supuestos!$B$26)</f>
-        <v>13205.0847457627</v>
+        <v>13174.5762711864</v>
       </c>
       <c r="D20" s="29" t="n">
         <f aca="false">D19/(1+Supuestos!$B$26)</f>
-        <v>17154.9152542373</v>
+        <v>17196.6101694915</v>
       </c>
       <c r="E20" s="29" t="n">
         <f aca="false">E19/(1+Supuestos!$B$26)</f>
-        <v>20327.2881355932</v>
+        <v>20420.3389830509</v>
       </c>
       <c r="F20" s="29" t="n">
         <f aca="false">F19/(1+Supuestos!$B$26)</f>
-        <v>18876.6101694915</v>
+        <v>19000.6779661017</v>
       </c>
       <c r="G20" s="29" t="n">
         <f aca="false">G19/(1+Supuestos!$B$26)</f>
-        <v>22860.2542372881</v>
+        <v>23015.3389830509</v>
       </c>
       <c r="H20" s="29" t="n">
         <f aca="false">H19/(1+Supuestos!$B$26)</f>
-        <v>28212.2033898305</v>
+        <v>28428.813559322</v>
       </c>
       <c r="I20" s="29" t="n">
         <f aca="false">I19/(1+Supuestos!$B$26)</f>
-        <v>30169.8305084746</v>
+        <v>30386.4406779661</v>
       </c>
       <c r="J20" s="29" t="n">
         <f aca="false">J19/(1+Supuestos!$B$26)</f>
-        <v>33545.593220339</v>
+        <v>33793.2203389831</v>
       </c>
       <c r="K20" s="29" t="n">
         <f aca="false">K19/(1+Supuestos!$B$26)</f>
-        <v>25729.8305084746</v>
+        <v>25998.3050847458</v>
       </c>
       <c r="L20" s="29" t="n">
         <f aca="false">L19/(1+Supuestos!$B$26)</f>
-        <v>12199.5254237288</v>
+        <v>12389.4915254237</v>
       </c>
       <c r="M20" s="29" t="n">
         <f aca="false">M19/(1+Supuestos!$B$26)</f>
-        <v>15566.6440677966</v>
+        <v>15756.6101694915</v>
       </c>
       <c r="N20" s="29" t="n">
         <f aca="false">SUM(B20:M20)</f>
-        <v>246868.118644068</v>
+        <v>248540.084745763</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5010,55 +5010,55 @@
       </c>
       <c r="B21" s="9" t="n">
         <f aca="false">SUMPRODUCT(B$5:B$8,Proyeccion!$F$22:$F$25)</f>
-        <v>2085.22159322034</v>
+        <v>2046.39040677966</v>
       </c>
       <c r="C21" s="9" t="n">
         <f aca="false">SUMPRODUCT(C$5:C$8,Proyeccion!$F$22:$F$25)</f>
-        <v>2979.98989830509</v>
+        <v>2950.86650847458</v>
       </c>
       <c r="D21" s="9" t="n">
         <f aca="false">SUMPRODUCT(D$5:D$8,Proyeccion!$F$22:$F$25)</f>
-        <v>3895.92310169492</v>
+        <v>3938.64106779661</v>
       </c>
       <c r="E21" s="9" t="n">
         <f aca="false">SUMPRODUCT(E$5:E$8,Proyeccion!$F$22:$F$25)</f>
-        <v>4595.24125423729</v>
+        <v>4688.44159322034</v>
       </c>
       <c r="F21" s="9" t="n">
         <f aca="false">SUMPRODUCT(F$5:F$8,Proyeccion!$F$22:$F$25)</f>
-        <v>4329.86086779661</v>
+        <v>4454.12798644068</v>
       </c>
       <c r="G21" s="9" t="n">
         <f aca="false">SUMPRODUCT(G$5:G$8,Proyeccion!$F$22:$F$25)</f>
-        <v>5287.80929491526</v>
+        <v>5443.14319322034</v>
       </c>
       <c r="H21" s="9" t="n">
         <f aca="false">SUMPRODUCT(H$5:H$8,Proyeccion!$F$22:$F$25)</f>
-        <v>6427.60235593221</v>
+        <v>6643.12642372882</v>
       </c>
       <c r="I21" s="9" t="n">
         <f aca="false">SUMPRODUCT(I$5:I$8,Proyeccion!$F$22:$F$25)</f>
-        <v>6841.03820338983</v>
+        <v>7056.56227118644</v>
       </c>
       <c r="J21" s="9" t="n">
         <f aca="false">SUMPRODUCT(J$5:J$8,Proyeccion!$F$22:$F$25)</f>
-        <v>7673.4082881356</v>
+        <v>7919.99913559322</v>
       </c>
       <c r="K21" s="9" t="n">
         <f aca="false">SUMPRODUCT(K$5:K$8,Proyeccion!$F$22:$F$25)</f>
-        <v>6019.17020338983</v>
+        <v>6287.12003389831</v>
       </c>
       <c r="L21" s="9" t="n">
         <f aca="false">SUMPRODUCT(L$5:L$8,Proyeccion!$F$22:$F$25)</f>
-        <v>2859.43076949153</v>
+        <v>3048.93721016949</v>
       </c>
       <c r="M21" s="9" t="n">
         <f aca="false">SUMPRODUCT(M$5:M$8,Proyeccion!$F$22:$F$25)</f>
-        <v>3570.54042711865</v>
+        <v>3760.04686779661</v>
       </c>
       <c r="N21" s="29" t="n">
         <f aca="false">SUM(B21:M21)</f>
-        <v>56565.2362576271</v>
+        <v>58237.4026983051</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5067,55 +5067,55 @@
       </c>
       <c r="B22" s="9" t="n">
         <f aca="false">SUMPRODUCT(B$5:B$8,Proyeccion!$G$22:$G$25)</f>
-        <v>2206.18159322034</v>
+        <v>2167.35040677966</v>
       </c>
       <c r="C22" s="9" t="n">
         <f aca="false">SUMPRODUCT(C$5:C$8,Proyeccion!$G$22:$G$25)</f>
-        <v>3158.40589830508</v>
+        <v>3129.28250847458</v>
       </c>
       <c r="D22" s="9" t="n">
         <f aca="false">SUMPRODUCT(D$5:D$8,Proyeccion!$G$22:$G$25)</f>
-        <v>4135.82710169492</v>
+        <v>4178.54506779661</v>
       </c>
       <c r="E22" s="9" t="n">
         <f aca="false">SUMPRODUCT(E$5:E$8,Proyeccion!$G$22:$G$25)</f>
-        <v>4879.49725423729</v>
+        <v>4972.69759322034</v>
       </c>
       <c r="F22" s="9" t="n">
         <f aca="false">SUMPRODUCT(F$5:F$8,Proyeccion!$G$22:$G$25)</f>
-        <v>4594.36006779661</v>
+        <v>4718.62718644068</v>
       </c>
       <c r="G22" s="9" t="n">
         <f aca="false">SUMPRODUCT(G$5:G$8,Proyeccion!$G$22:$G$25)</f>
-        <v>5600.59169491525</v>
+        <v>5755.92559322034</v>
       </c>
       <c r="H22" s="9" t="n">
         <f aca="false">SUMPRODUCT(H$5:H$8,Proyeccion!$G$22:$G$25)</f>
-        <v>6817.6983559322</v>
+        <v>7033.22242372881</v>
       </c>
       <c r="I22" s="9" t="n">
         <f aca="false">SUMPRODUCT(I$5:I$8,Proyeccion!$G$22:$G$25)</f>
-        <v>7261.37420338983</v>
+        <v>7476.89827118644</v>
       </c>
       <c r="J22" s="9" t="n">
         <f aca="false">SUMPRODUCT(J$5:J$8,Proyeccion!$G$22:$G$25)</f>
-        <v>8132.04828813559</v>
+        <v>8378.63913559322</v>
       </c>
       <c r="K22" s="9" t="n">
         <f aca="false">SUMPRODUCT(K$5:K$8,Proyeccion!$G$22:$G$25)</f>
-        <v>6373.98620338983</v>
+        <v>6641.9360338983</v>
       </c>
       <c r="L22" s="9" t="n">
         <f aca="false">SUMPRODUCT(L$5:L$8,Proyeccion!$G$22:$G$25)</f>
-        <v>3043.69316949152</v>
+        <v>3233.19961016949</v>
       </c>
       <c r="M22" s="9" t="n">
         <f aca="false">SUMPRODUCT(M$5:M$8,Proyeccion!$G$22:$G$25)</f>
-        <v>3806.81562711864</v>
+        <v>3996.32206779661</v>
       </c>
       <c r="N22" s="29" t="n">
         <f aca="false">SUM(B22:M22)</f>
-        <v>60010.4794576271</v>
+        <v>61682.6458983051</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5181,55 +5181,55 @@
       </c>
       <c r="B24" s="11" t="n">
         <f aca="false">B21-B23</f>
-        <v>-771.448406779661</v>
+        <v>-810.279593220339</v>
       </c>
       <c r="C24" s="11" t="n">
         <f aca="false">C21-C23</f>
-        <v>123.319898305085</v>
+        <v>94.1965084745771</v>
       </c>
       <c r="D24" s="11" t="n">
         <f aca="false">D21-D23</f>
-        <v>1039.25310169492</v>
+        <v>1081.97106779661</v>
       </c>
       <c r="E24" s="11" t="n">
         <f aca="false">E21-E23</f>
-        <v>1738.57125423729</v>
+        <v>1831.77159322034</v>
       </c>
       <c r="F24" s="11" t="n">
         <f aca="false">F21-F23</f>
-        <v>1473.19086779661</v>
+        <v>1597.45798644068</v>
       </c>
       <c r="G24" s="11" t="n">
         <f aca="false">G21-G23</f>
-        <v>2431.13929491526</v>
+        <v>2586.47319322034</v>
       </c>
       <c r="H24" s="11" t="n">
         <f aca="false">H21-H23</f>
-        <v>3570.9323559322</v>
+        <v>3786.45642372882</v>
       </c>
       <c r="I24" s="11" t="n">
         <f aca="false">I21-I23</f>
-        <v>3984.36820338983</v>
+        <v>4199.89227118644</v>
       </c>
       <c r="J24" s="11" t="n">
         <f aca="false">J21-J23</f>
-        <v>4816.7382881356</v>
+        <v>5063.32913559322</v>
       </c>
       <c r="K24" s="11" t="n">
         <f aca="false">K21-K23</f>
-        <v>3162.50020338983</v>
+        <v>3430.45003389831</v>
       </c>
       <c r="L24" s="11" t="n">
         <f aca="false">L21-L23</f>
-        <v>2.76076949152593</v>
+        <v>192.267210169492</v>
       </c>
       <c r="M24" s="11" t="n">
         <f aca="false">M21-M23</f>
-        <v>713.870427118645</v>
+        <v>903.376867796611</v>
       </c>
       <c r="N24" s="11" t="n">
         <f aca="false">SUM(B24:M24)</f>
-        <v>22285.1962576271</v>
+        <v>23957.3626983051</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5238,55 +5238,55 @@
       </c>
       <c r="B25" s="11" t="n">
         <f aca="false">B22-B23</f>
-        <v>-650.488406779662</v>
+        <v>-689.319593220339</v>
       </c>
       <c r="C25" s="11" t="n">
         <f aca="false">C22-C23</f>
-        <v>301.735898305084</v>
+        <v>272.612508474575</v>
       </c>
       <c r="D25" s="11" t="n">
         <f aca="false">D22-D23</f>
-        <v>1279.15710169491</v>
+        <v>1321.87506779661</v>
       </c>
       <c r="E25" s="11" t="n">
         <f aca="false">E22-E23</f>
-        <v>2022.82725423729</v>
+        <v>2116.02759322034</v>
       </c>
       <c r="F25" s="11" t="n">
         <f aca="false">F22-F23</f>
-        <v>1737.69006779661</v>
+        <v>1861.95718644068</v>
       </c>
       <c r="G25" s="11" t="n">
         <f aca="false">G22-G23</f>
-        <v>2743.92169491525</v>
+        <v>2899.25559322034</v>
       </c>
       <c r="H25" s="11" t="n">
         <f aca="false">H22-H23</f>
-        <v>3961.0283559322</v>
+        <v>4176.55242372881</v>
       </c>
       <c r="I25" s="11" t="n">
         <f aca="false">I22-I23</f>
-        <v>4404.70420338983</v>
+        <v>4620.22827118644</v>
       </c>
       <c r="J25" s="11" t="n">
         <f aca="false">J22-J23</f>
-        <v>5275.37828813559</v>
+        <v>5521.96913559322</v>
       </c>
       <c r="K25" s="11" t="n">
         <f aca="false">K22-K23</f>
-        <v>3517.31620338983</v>
+        <v>3785.2660338983</v>
       </c>
       <c r="L25" s="11" t="n">
         <f aca="false">L22-L23</f>
-        <v>187.023169491525</v>
+        <v>376.529610169491</v>
       </c>
       <c r="M25" s="11" t="n">
         <f aca="false">M22-M23</f>
-        <v>950.145627118643</v>
+        <v>1139.65206779661</v>
       </c>
       <c r="N25" s="11" t="n">
         <f aca="false">SUM(B25:M25)</f>
-        <v>25730.4394576271</v>
+        <v>27402.6058983051</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5295,51 +5295,51 @@
       </c>
       <c r="B26" s="29" t="n">
         <f aca="false">B24</f>
-        <v>-771.448406779661</v>
+        <v>-810.279593220339</v>
       </c>
       <c r="C26" s="29" t="n">
         <f aca="false">B26+C24</f>
-        <v>-648.128508474576</v>
+        <v>-716.083084745762</v>
       </c>
       <c r="D26" s="29" t="n">
         <f aca="false">C26+D24</f>
-        <v>391.124593220341</v>
+        <v>365.887983050849</v>
       </c>
       <c r="E26" s="29" t="n">
         <f aca="false">D26+E24</f>
-        <v>2129.69584745763</v>
+        <v>2197.65957627119</v>
       </c>
       <c r="F26" s="29" t="n">
         <f aca="false">E26+F24</f>
-        <v>3602.88671525424</v>
+        <v>3795.11756271187</v>
       </c>
       <c r="G26" s="29" t="n">
         <f aca="false">F26+G24</f>
-        <v>6034.0260101695</v>
+        <v>6381.59075593221</v>
       </c>
       <c r="H26" s="29" t="n">
         <f aca="false">G26+H24</f>
-        <v>9604.9583661017</v>
+        <v>10168.047179661</v>
       </c>
       <c r="I26" s="29" t="n">
         <f aca="false">H26+I24</f>
-        <v>13589.3265694915</v>
+        <v>14367.9394508475</v>
       </c>
       <c r="J26" s="29" t="n">
         <f aca="false">I26+J24</f>
-        <v>18406.0648576271</v>
+        <v>19431.2685864407</v>
       </c>
       <c r="K26" s="29" t="n">
         <f aca="false">J26+K24</f>
-        <v>21568.565061017</v>
+        <v>22861.718620339</v>
       </c>
       <c r="L26" s="29" t="n">
         <f aca="false">K26+L24</f>
-        <v>21571.3258305085</v>
+        <v>23053.9858305085</v>
       </c>
       <c r="M26" s="29" t="n">
         <f aca="false">L26+M24</f>
-        <v>22285.1962576271</v>
+        <v>23957.3626983051</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5348,51 +5348,51 @@
       </c>
       <c r="B27" s="29" t="n">
         <f aca="false">B25</f>
-        <v>-650.488406779662</v>
+        <v>-689.319593220339</v>
       </c>
       <c r="C27" s="29" t="n">
         <f aca="false">B27+C25</f>
-        <v>-348.752508474578</v>
+        <v>-416.707084745764</v>
       </c>
       <c r="D27" s="29" t="n">
         <f aca="false">C27+D25</f>
-        <v>930.404593220337</v>
+        <v>905.167983050845</v>
       </c>
       <c r="E27" s="29" t="n">
         <f aca="false">D27+E25</f>
-        <v>2953.23184745762</v>
+        <v>3021.19557627118</v>
       </c>
       <c r="F27" s="29" t="n">
         <f aca="false">E27+F25</f>
-        <v>4690.92191525423</v>
+        <v>4883.15276271186</v>
       </c>
       <c r="G27" s="29" t="n">
         <f aca="false">F27+G25</f>
-        <v>7434.84361016949</v>
+        <v>7782.4083559322</v>
       </c>
       <c r="H27" s="29" t="n">
         <f aca="false">G27+H25</f>
-        <v>11395.8719661017</v>
+        <v>11958.960779661</v>
       </c>
       <c r="I27" s="29" t="n">
         <f aca="false">H27+I25</f>
-        <v>15800.5761694915</v>
+        <v>16579.1890508475</v>
       </c>
       <c r="J27" s="29" t="n">
         <f aca="false">I27+J25</f>
-        <v>21075.9544576271</v>
+        <v>22101.1581864407</v>
       </c>
       <c r="K27" s="29" t="n">
         <f aca="false">J27+K25</f>
-        <v>24593.2706610169</v>
+        <v>25886.424220339</v>
       </c>
       <c r="L27" s="29" t="n">
         <f aca="false">K27+L25</f>
-        <v>24780.2938305085</v>
+        <v>26262.9538305085</v>
       </c>
       <c r="M27" s="29" t="n">
         <f aca="false">L27+M25</f>
-        <v>25730.4394576271</v>
+        <v>27402.6058983051</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Costeo: precios intermedios recomendados (pack 6 S/24.90, pack 12 S/46.90, ferias S/26/S/48, naturista S/17.34 a tienda)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Kfbf7cfV7pXUcNjjyaPCzV
</commit_message>
<xml_diff>
--- a/04-reformulacion/Costeo-presentaciones-AndiBite.xlsx
+++ b/04-reformulacion/Costeo-presentaciones-AndiBite.xlsx
@@ -379,16 +379,16 @@
     <t xml:space="preserve">Pack de 6</t>
   </si>
   <si>
-    <t xml:space="preserve">Precios ajustados por el equipo (9-oct-2026). Unidad = caja degustación de 3 (S/12.00) o unidades agregadas al pedido</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Precios ajustados por el equipo (9-oct-2026). La unidad suelta cuesta más que dentro del pack</t>
+    <t xml:space="preserve">Precio intermedio recomendado (9-oct-2026). S/4.15 por brownie en el pack de 6, a la par de Fika (S/4.00) y Mamalama (S/4.10) por 20 g. Unidad = caja degustación de 3 (S/12.00)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Precio intermedio recomendado (9-oct-2026). En feria se cobra algo más que por WhatsApp porque el stand cuesta cerca de S/1 por brownie</t>
   </si>
   <si>
     <t xml:space="preserve">El alumno paga S/4.00; el concesionario se queda 25 %</t>
   </si>
   <si>
-    <t xml:space="preserve">Precio ajustado por el equipo (9-oct-2026): lo que cobra AndiBite a la tienda. Con 40 % para la tienda, el anaquel quedaría en S/40.00</t>
+    <t xml:space="preserve">Precio intermedio recomendado (9-oct-2026): AndiBite cobra S/17.34 a la tienda; con 40 % para la tienda, el anaquel queda en S/28.90</t>
   </si>
   <si>
     <t xml:space="preserve">6. Mezcla de presentaciones por canal (% de las unidades que vende cada canal)</t>
@@ -1476,11 +1476,11 @@
       </c>
       <c r="D6" s="6" t="n">
         <f aca="false">Costeo!C19</f>
-        <v>23.5</v>
+        <v>24.9</v>
       </c>
       <c r="E6" s="7" t="n">
         <f aca="false">Costeo!C22</f>
-        <v>0.503044255319149</v>
+        <v>0.530985542168675</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1497,11 +1497,11 @@
       </c>
       <c r="D7" s="6" t="n">
         <f aca="false">Costeo!D19</f>
-        <v>23.5</v>
+        <v>24.9</v>
       </c>
       <c r="E7" s="7" t="n">
         <f aca="false">Costeo!D22</f>
-        <v>0.528351489361702</v>
+        <v>0.554869879518072</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1518,11 +1518,11 @@
       </c>
       <c r="D8" s="6" t="n">
         <f aca="false">Costeo!E19</f>
-        <v>44</v>
+        <v>46.9</v>
       </c>
       <c r="E8" s="7" t="n">
         <f aca="false">Costeo!E22</f>
-        <v>0.499572727272727</v>
+        <v>0.530515991471215</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1557,11 +1557,11 @@
       </c>
       <c r="B13" s="9" t="n">
         <f aca="false">Proyeccion!I17</f>
-        <v>293277.3</v>
+        <v>302900.355</v>
       </c>
       <c r="C13" s="9" t="n">
         <f aca="false">Proyeccion!I17</f>
-        <v>293277.3</v>
+        <v>302900.355</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1570,11 +1570,11 @@
       </c>
       <c r="B14" s="9" t="n">
         <f aca="false">Proyeccion!J17</f>
-        <v>248540.084745763</v>
+        <v>256695.216101695</v>
       </c>
       <c r="C14" s="9" t="n">
         <f aca="false">Proyeccion!J17</f>
-        <v>248540.084745763</v>
+        <v>256695.216101695</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1583,11 +1583,11 @@
       </c>
       <c r="B15" s="9" t="n">
         <f aca="false">Proyeccion!P17</f>
-        <v>58237.4026983051</v>
+        <v>65917.995490678</v>
       </c>
       <c r="C15" s="9" t="n">
         <f aca="false">Proyeccion!Q17</f>
-        <v>61682.6458983051</v>
+        <v>69363.238690678</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1609,11 +1609,11 @@
       </c>
       <c r="B17" s="11" t="n">
         <f aca="false">B15-B16</f>
-        <v>23957.3626983051</v>
+        <v>31637.955490678</v>
       </c>
       <c r="C17" s="11" t="n">
         <f aca="false">C15-C16</f>
-        <v>27402.6058983051</v>
+        <v>35083.198690678</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1622,11 +1622,11 @@
       </c>
       <c r="B18" s="12" t="n">
         <f aca="false">IF(B14=0,0,B17/B14)</f>
-        <v>0.0963923494385689</v>
+        <v>0.123251052244558</v>
       </c>
       <c r="C18" s="12" t="n">
         <f aca="false">IF(C14=0,0,C17/C14)</f>
-        <v>0.11025427116248</v>
+        <v>0.136672584801031</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1635,11 +1635,11 @@
       </c>
       <c r="B19" s="13" t="n">
         <f aca="false">IF(B12=0,0,B15/B12)</f>
-        <v>0.762918748913409</v>
+        <v>0.863535671588105</v>
       </c>
       <c r="C19" s="13" t="n">
         <f aca="false">IF(C12=0,0,C15/C12)</f>
-        <v>0.808051953865266</v>
+        <v>0.908668876539962</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1648,11 +1648,11 @@
       </c>
       <c r="B20" s="14" t="n">
         <f aca="false">IF(B19&lt;=0,"No alcanza",Supuestos!$B$58/B19)</f>
-        <v>3744.39611566582</v>
+        <v>3308.10885292831</v>
       </c>
       <c r="C20" s="14" t="n">
         <f aca="false">IF(C19&lt;=0,"No alcanza",Supuestos!$B$58/C19)</f>
-        <v>3535.25535868739</v>
+        <v>3143.79646288498</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1661,11 +1661,11 @@
       </c>
       <c r="B21" s="15" t="n">
         <f aca="false">IF(ISNUMBER(B20),B20/6,"No alcanza")</f>
-        <v>624.066019277637</v>
+        <v>551.351475488051</v>
       </c>
       <c r="C21" s="15" t="n">
         <f aca="false">IF(ISNUMBER(C20),C20/6,"No alcanza")</f>
-        <v>589.209226447899</v>
+        <v>523.966077147497</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2145,10 +2145,10 @@
         <v>4</v>
       </c>
       <c r="C39" s="24" t="n">
-        <v>23.5</v>
+        <v>24.9</v>
       </c>
       <c r="D39" s="24" t="n">
-        <v>44</v>
+        <v>46.9</v>
       </c>
       <c r="E39" s="4" t="s">
         <v>110</v>
@@ -2162,10 +2162,10 @@
         <v>5</v>
       </c>
       <c r="C40" s="24" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D40" s="24" t="n">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="E40" s="4" t="s">
         <v>111</v>
@@ -2196,7 +2196,7 @@
         <v>0</v>
       </c>
       <c r="C42" s="24" t="n">
-        <v>24</v>
+        <v>17.34</v>
       </c>
       <c r="D42" s="24" t="n">
         <v>0</v>
@@ -2744,15 +2744,15 @@
       </c>
       <c r="C19" s="6" t="n">
         <f aca="false">Supuestos!C39</f>
-        <v>23.5</v>
+        <v>24.9</v>
       </c>
       <c r="D19" s="6" t="n">
         <f aca="false">Supuestos!C39</f>
-        <v>23.5</v>
+        <v>24.9</v>
       </c>
       <c r="E19" s="6" t="n">
         <f aca="false">Supuestos!D39</f>
-        <v>44</v>
+        <v>46.9</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2765,15 +2765,15 @@
       </c>
       <c r="C20" s="13" t="n">
         <f aca="false">C19/(1+Supuestos!$B$26)</f>
-        <v>19.9152542372881</v>
+        <v>21.1016949152542</v>
       </c>
       <c r="D20" s="13" t="n">
         <f aca="false">D19/(1+Supuestos!$B$26)</f>
-        <v>19.9152542372881</v>
+        <v>21.1016949152542</v>
       </c>
       <c r="E20" s="13" t="n">
         <f aca="false">E19/(1+Supuestos!$B$26)</f>
-        <v>37.2881355932203</v>
+        <v>39.7457627118644</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2786,15 +2786,15 @@
       </c>
       <c r="C21" s="13" t="n">
         <f aca="false">C20-C15</f>
-        <v>10.0182542372881</v>
+        <v>11.2046949152542</v>
       </c>
       <c r="D21" s="13" t="n">
         <f aca="false">D20-D15</f>
-        <v>10.5222542372881</v>
+        <v>11.7086949152542</v>
       </c>
       <c r="E21" s="13" t="n">
         <f aca="false">E20-E15</f>
-        <v>18.6281355932203</v>
+        <v>21.0857627118644</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2807,15 +2807,15 @@
       </c>
       <c r="C22" s="12" t="n">
         <f aca="false">IF(C20=0,0,C21/C20)</f>
-        <v>0.503044255319149</v>
+        <v>0.530985542168675</v>
       </c>
       <c r="D22" s="12" t="n">
         <f aca="false">IF(D20=0,0,D21/D20)</f>
-        <v>0.528351489361702</v>
+        <v>0.554869879518072</v>
       </c>
       <c r="E22" s="12" t="n">
         <f aca="false">IF(E20=0,0,E21/E20)</f>
-        <v>0.499572727272727</v>
+        <v>0.530515991471215</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3026,15 +3026,15 @@
       </c>
       <c r="H6" s="6" t="n">
         <f aca="false">Supuestos!C39</f>
-        <v>23.5</v>
+        <v>24.9</v>
       </c>
       <c r="I6" s="29" t="n">
         <f aca="false">G6*H6</f>
-        <v>141747.3</v>
+        <v>150191.82</v>
       </c>
       <c r="J6" s="29" t="n">
         <f aca="false">I6/(1+Supuestos!$B$26)</f>
-        <v>120124.830508475</v>
+        <v>127281.203389831</v>
       </c>
       <c r="K6" s="6" t="n">
         <f aca="false">Costeo!C15</f>
@@ -3046,31 +3046,31 @@
       </c>
       <c r="M6" s="13" t="n">
         <f aca="false">IF(H6=0,0,C6*Supuestos!$B$32+H6*Supuestos!$B$27*Supuestos!$C$32+H6/(1+Supuestos!$B$26)*Supuestos!$B$28)</f>
-        <v>5.70415254237288</v>
+        <v>5.75801694915254</v>
       </c>
       <c r="N6" s="13" t="n">
         <f aca="false">IF(H6=0,0,H6/(1+Supuestos!$B$26)-K6-M6)</f>
-        <v>4.31410169491525</v>
+        <v>5.4466779661017</v>
       </c>
       <c r="O6" s="13" t="n">
         <f aca="false">IF(H6=0,0,H6/(1+Supuestos!$B$26)-L6-M6)</f>
-        <v>4.81810169491525</v>
+        <v>5.9506779661017</v>
       </c>
       <c r="P6" s="29" t="n">
         <f aca="false">G6*N6</f>
-        <v>26021.7986033898</v>
+        <v>32853.2721559322</v>
       </c>
       <c r="Q6" s="29" t="n">
         <f aca="false">G6*O6</f>
-        <v>29061.8258033898</v>
+        <v>35893.2993559322</v>
       </c>
       <c r="R6" s="12" t="n">
         <f aca="false">IF(H6=0,0,N6/(H6/(1+Supuestos!$B$26)))</f>
-        <v>0.216622978723404</v>
+        <v>0.258115662650603</v>
       </c>
       <c r="S6" s="12" t="n">
         <f aca="false">IF(H6=0,0,O6/(H6/(1+Supuestos!$B$26)))</f>
-        <v>0.241930212765957</v>
+        <v>0.282</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3102,15 +3102,15 @@
       </c>
       <c r="H7" s="6" t="n">
         <f aca="false">Supuestos!D39</f>
-        <v>44</v>
+        <v>46.9</v>
       </c>
       <c r="I7" s="29" t="n">
         <f aca="false">G7*H7</f>
-        <v>66349.8</v>
+        <v>70722.855</v>
       </c>
       <c r="J7" s="29" t="n">
         <f aca="false">I7/(1+Supuestos!$B$26)</f>
-        <v>56228.6440677966</v>
+        <v>59934.6228813559</v>
       </c>
       <c r="K7" s="6" t="n">
         <f aca="false">Costeo!E15</f>
@@ -3122,31 +3122,31 @@
       </c>
       <c r="M7" s="13" t="n">
         <f aca="false">IF(H7=0,0,C7*Supuestos!$B$32+H7*Supuestos!$B$27*Supuestos!$C$32+H7/(1+Supuestos!$B$26)*Supuestos!$B$28)</f>
-        <v>11.2928813559322</v>
+        <v>11.4044576271186</v>
       </c>
       <c r="N7" s="13" t="n">
         <f aca="false">IF(H7=0,0,H7/(1+Supuestos!$B$26)-K7-M7)</f>
-        <v>7.33525423728814</v>
+        <v>9.68130508474577</v>
       </c>
       <c r="O7" s="13" t="n">
         <f aca="false">IF(H7=0,0,H7/(1+Supuestos!$B$26)-L7-M7)</f>
-        <v>7.33525423728814</v>
+        <v>9.68130508474577</v>
       </c>
       <c r="P7" s="29" t="n">
         <f aca="false">G7*N7</f>
-        <v>11061.1966271186</v>
+        <v>14598.9240025424</v>
       </c>
       <c r="Q7" s="29" t="n">
         <f aca="false">G7*O7</f>
-        <v>11061.1966271186</v>
+        <v>14598.9240025424</v>
       </c>
       <c r="R7" s="12" t="n">
         <f aca="false">IF(H7=0,0,N7/(H7/(1+Supuestos!$B$26)))</f>
-        <v>0.196718181818182</v>
+        <v>0.243580810234542</v>
       </c>
       <c r="S7" s="12" t="n">
         <f aca="false">IF(H7=0,0,O7/(H7/(1+Supuestos!$B$26)))</f>
-        <v>0.196718181818182</v>
+        <v>0.243580810234542</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3254,15 +3254,15 @@
       </c>
       <c r="H9" s="6" t="n">
         <f aca="false">Supuestos!C40</f>
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="I9" s="29" t="n">
         <f aca="false">G9*H9</f>
-        <v>7050</v>
+        <v>7332</v>
       </c>
       <c r="J9" s="29" t="n">
         <f aca="false">I9/(1+Supuestos!$B$26)</f>
-        <v>5974.57627118644</v>
+        <v>6213.5593220339</v>
       </c>
       <c r="K9" s="6" t="n">
         <f aca="false">Costeo!C15</f>
@@ -3274,31 +3274,31 @@
       </c>
       <c r="M9" s="13" t="n">
         <f aca="false">IF(H9=0,0,C9*Supuestos!$B$33+H9*Supuestos!$B$27*Supuestos!$C$33+H9/(1+Supuestos!$B$26)*Supuestos!$B$28)</f>
-        <v>6.96186440677966</v>
+        <v>7.00033898305085</v>
       </c>
       <c r="N9" s="13" t="n">
         <f aca="false">IF(H9=0,0,H9/(1+Supuestos!$B$26)-K9-M9)</f>
-        <v>4.32757627118644</v>
+        <v>5.1365593220339</v>
       </c>
       <c r="O9" s="13" t="n">
         <f aca="false">IF(H9=0,0,H9/(1+Supuestos!$B$26)-L9-M9)</f>
-        <v>4.83157627118644</v>
+        <v>5.6405593220339</v>
       </c>
       <c r="P9" s="29" t="n">
         <f aca="false">G9*N9</f>
-        <v>1220.37650847458</v>
+        <v>1448.50972881356</v>
       </c>
       <c r="Q9" s="29" t="n">
         <f aca="false">G9*O9</f>
-        <v>1362.50450847458</v>
+        <v>1590.63772881356</v>
       </c>
       <c r="R9" s="12" t="n">
         <f aca="false">IF(H9=0,0,N9/(H9/(1+Supuestos!$B$26)))</f>
-        <v>0.2042616</v>
+        <v>0.233120769230769</v>
       </c>
       <c r="S9" s="12" t="n">
         <f aca="false">IF(H9=0,0,O9/(H9/(1+Supuestos!$B$26)))</f>
-        <v>0.2280504</v>
+        <v>0.255994615384615</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3330,7 +3330,7 @@
       </c>
       <c r="H10" s="6" t="n">
         <f aca="false">Supuestos!D40</f>
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="I10" s="29" t="n">
         <f aca="false">G10*H10</f>
@@ -3350,15 +3350,15 @@
       </c>
       <c r="M10" s="13" t="n">
         <f aca="false">IF(H10=0,0,C10*Supuestos!$B$33+H10*Supuestos!$B$27*Supuestos!$C$33+H10/(1+Supuestos!$B$26)*Supuestos!$B$28)</f>
-        <v>13.6159322033898</v>
+        <v>13.846779661017</v>
       </c>
       <c r="N10" s="13" t="n">
         <f aca="false">IF(H10=0,0,H10/(1+Supuestos!$B$26)-K10-M10)</f>
-        <v>3.31728813559323</v>
+        <v>8.17118644067798</v>
       </c>
       <c r="O10" s="13" t="n">
         <f aca="false">IF(H10=0,0,H10/(1+Supuestos!$B$26)-L10-M10)</f>
-        <v>3.31728813559323</v>
+        <v>8.17118644067798</v>
       </c>
       <c r="P10" s="29" t="n">
         <f aca="false">G10*N10</f>
@@ -3370,11 +3370,11 @@
       </c>
       <c r="R10" s="12" t="n">
         <f aca="false">IF(H10=0,0,N10/(H10/(1+Supuestos!$B$26)))</f>
-        <v>0.0932000000000001</v>
+        <v>0.200875</v>
       </c>
       <c r="S10" s="12" t="n">
         <f aca="false">IF(H10=0,0,O10/(H10/(1+Supuestos!$B$26)))</f>
-        <v>0.0932000000000001</v>
+        <v>0.200875</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3710,15 +3710,15 @@
       </c>
       <c r="H15" s="6" t="n">
         <f aca="false">Supuestos!C42</f>
-        <v>24</v>
+        <v>17.34</v>
       </c>
       <c r="I15" s="29" t="n">
         <f aca="false">G15*H15</f>
-        <v>12528</v>
+        <v>9051.48</v>
       </c>
       <c r="J15" s="29" t="n">
         <f aca="false">I15/(1+Supuestos!$B$26)</f>
-        <v>10616.9491525424</v>
+        <v>7670.74576271187</v>
       </c>
       <c r="K15" s="6" t="n">
         <f aca="false">Costeo!C15</f>
@@ -3730,31 +3730,31 @@
       </c>
       <c r="M15" s="13" t="n">
         <f aca="false">IF(H15=0,0,C15*Supuestos!$B$35+H15*Supuestos!$B$27*Supuestos!$C$35+H15/(1+Supuestos!$B$26)*Supuestos!$B$28)</f>
-        <v>1.10338983050847</v>
+        <v>1.04694915254237</v>
       </c>
       <c r="N15" s="13" t="n">
         <f aca="false">IF(H15=0,0,H15/(1+Supuestos!$B$26)-K15-M15)</f>
-        <v>9.33859322033899</v>
+        <v>3.75096610169492</v>
       </c>
       <c r="O15" s="13" t="n">
         <f aca="false">IF(H15=0,0,H15/(1+Supuestos!$B$26)-L15-M15)</f>
-        <v>9.84259322033899</v>
+        <v>4.25496610169492</v>
       </c>
       <c r="P15" s="29" t="n">
         <f aca="false">G15*N15</f>
-        <v>4874.74566101695</v>
+        <v>1958.00430508475</v>
       </c>
       <c r="Q15" s="29" t="n">
         <f aca="false">G15*O15</f>
-        <v>5137.83366101695</v>
+        <v>2221.09230508475</v>
       </c>
       <c r="R15" s="12" t="n">
         <f aca="false">IF(H15=0,0,N15/(H15/(1+Supuestos!$B$26)))</f>
-        <v>0.4591475</v>
+        <v>0.255256055363322</v>
       </c>
       <c r="S15" s="12" t="n">
         <f aca="false">IF(H15=0,0,O15/(H15/(1+Supuestos!$B$26)))</f>
-        <v>0.4839275</v>
+        <v>0.289553633217993</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3843,19 +3843,19 @@
       </c>
       <c r="I17" s="11" t="n">
         <f aca="false">SUM(I5:I16)</f>
-        <v>293277.3</v>
+        <v>302900.355</v>
       </c>
       <c r="J17" s="11" t="n">
         <f aca="false">SUM(J5:J16)</f>
-        <v>248540.084745763</v>
+        <v>256695.216101695</v>
       </c>
       <c r="P17" s="11" t="n">
         <f aca="false">SUM(P5:P16)</f>
-        <v>58237.4026983051</v>
+        <v>65917.995490678</v>
       </c>
       <c r="Q17" s="11" t="n">
         <f aca="false">SUM(Q5:Q16)</f>
-        <v>61682.6458983051</v>
+        <v>69363.238690678</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3906,27 +3906,27 @@
       </c>
       <c r="C22" s="29" t="n">
         <f aca="false">SUMIF($A$5:$A$16,A22,$P$5:$P$16)</f>
-        <v>41562.7057449153</v>
+        <v>51931.9066728814</v>
       </c>
       <c r="D22" s="29" t="n">
         <f aca="false">SUMIF($A$5:$A$16,A22,$Q$5:$Q$16)</f>
-        <v>44602.7329449152</v>
+        <v>54971.9338728814</v>
       </c>
       <c r="E22" s="29" t="n">
         <f aca="false">SUMIF($A$5:$A$16,A22,$I$5:$I$16)</f>
-        <v>232224.3</v>
+        <v>245041.875</v>
       </c>
       <c r="F22" s="13" t="n">
         <f aca="false">IF(B22=0,0,C22/B22)</f>
-        <v>0.689059745762712</v>
+        <v>0.860968644067797</v>
       </c>
       <c r="G22" s="13" t="n">
         <f aca="false">IF(B22=0,0,D22/B22)</f>
-        <v>0.739459745762712</v>
+        <v>0.911368644067797</v>
       </c>
       <c r="H22" s="13" t="n">
         <f aca="false">IF(B22=0,0,E22/B22)</f>
-        <v>3.85</v>
+        <v>4.0625</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3939,27 +3939,27 @@
       </c>
       <c r="C23" s="29" t="n">
         <f aca="false">SUMIF($A$5:$A$16,A23,$P$5:$P$16)</f>
-        <v>6556.75093220339</v>
+        <v>6784.88415254237</v>
       </c>
       <c r="D23" s="29" t="n">
         <f aca="false">SUMIF($A$5:$A$16,A23,$Q$5:$Q$16)</f>
-        <v>6698.87893220339</v>
+        <v>6927.01215254237</v>
       </c>
       <c r="E23" s="29" t="n">
         <f aca="false">SUMIF($A$5:$A$16,A23,$I$5:$I$16)</f>
-        <v>26790</v>
+        <v>27072</v>
       </c>
       <c r="F23" s="13" t="n">
         <f aca="false">IF(B23=0,0,C23/B23)</f>
-        <v>1.16254449152542</v>
+        <v>1.2029936440678</v>
       </c>
       <c r="G23" s="13" t="n">
         <f aca="false">IF(B23=0,0,D23/B23)</f>
-        <v>1.18774449152542</v>
+        <v>1.2281936440678</v>
       </c>
       <c r="H23" s="13" t="n">
         <f aca="false">IF(B23=0,0,E23/B23)</f>
-        <v>4.75</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4005,27 +4005,27 @@
       </c>
       <c r="C25" s="29" t="n">
         <f aca="false">SUMIF($A$5:$A$16,A25,$P$5:$P$16)</f>
-        <v>4874.74566101695</v>
+        <v>1958.00430508475</v>
       </c>
       <c r="D25" s="29" t="n">
         <f aca="false">SUMIF($A$5:$A$16,A25,$Q$5:$Q$16)</f>
-        <v>5137.83366101695</v>
+        <v>2221.09230508475</v>
       </c>
       <c r="E25" s="29" t="n">
         <f aca="false">SUMIF($A$5:$A$16,A25,$I$5:$I$16)</f>
-        <v>12528</v>
+        <v>9051.48</v>
       </c>
       <c r="F25" s="13" t="n">
         <f aca="false">IF(B25=0,0,C25/B25)</f>
-        <v>1.55643220338983</v>
+        <v>0.625161016949153</v>
       </c>
       <c r="G25" s="13" t="n">
         <f aca="false">IF(B25=0,0,D25/B25)</f>
-        <v>1.64043220338983</v>
+        <v>0.709161016949153</v>
       </c>
       <c r="H25" s="13" t="n">
         <f aca="false">IF(B25=0,0,E25/B25)</f>
-        <v>4</v>
+        <v>2.89</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4038,27 +4038,27 @@
       </c>
       <c r="C26" s="11" t="n">
         <f aca="false">SUM(C22:C25)</f>
-        <v>58237.4026983051</v>
+        <v>65917.995490678</v>
       </c>
       <c r="D26" s="11" t="n">
         <f aca="false">SUM(D22:D25)</f>
-        <v>61682.6458983051</v>
+        <v>69363.238690678</v>
       </c>
       <c r="E26" s="11" t="n">
         <f aca="false">SUM(E22:E25)</f>
-        <v>293277.3</v>
+        <v>302900.355</v>
       </c>
       <c r="F26" s="27" t="n">
         <f aca="false">IF(B26=0,0,C26/B26)</f>
-        <v>0.762918748913409</v>
+        <v>0.863535671588105</v>
       </c>
       <c r="G26" s="27" t="n">
         <f aca="false">IF(B26=0,0,D26/B26)</f>
-        <v>0.808051953865266</v>
+        <v>0.908668876539962</v>
       </c>
       <c r="H26" s="27" t="n">
         <f aca="false">IF(B26=0,0,E26/B26)</f>
-        <v>3.84197681273335</v>
+        <v>3.96804028296325</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4140,15 +4140,15 @@
       </c>
       <c r="D31" s="29" t="n">
         <f aca="false">SUMIF($B$5:$B$16,A31,$I$5:$I$16)</f>
-        <v>161325.3</v>
+        <v>166575.3</v>
       </c>
       <c r="E31" s="29" t="n">
         <f aca="false">SUMIF($B$5:$B$16,A31,$P$5:$P$16)</f>
-        <v>32116.9207728814</v>
+        <v>36259.7861898305</v>
       </c>
       <c r="F31" s="29" t="n">
         <f aca="false">SUMIF($B$5:$B$16,A31,$Q$5:$Q$16)</f>
-        <v>35562.1639728813</v>
+        <v>39705.0293898305</v>
       </c>
       <c r="G31" s="12" t="n">
         <f aca="false">IF($F$17=0,0,B31/$F$17)</f>
@@ -4169,15 +4169,15 @@
       </c>
       <c r="D32" s="29" t="n">
         <f aca="false">SUMIF($B$5:$B$16,A32,$I$5:$I$16)</f>
-        <v>66349.8</v>
+        <v>70722.855</v>
       </c>
       <c r="E32" s="29" t="n">
         <f aca="false">SUMIF($B$5:$B$16,A32,$P$5:$P$16)</f>
-        <v>11061.1966271186</v>
+        <v>14598.9240025424</v>
       </c>
       <c r="F32" s="29" t="n">
         <f aca="false">SUMIF($B$5:$B$16,A32,$Q$5:$Q$16)</f>
-        <v>11061.1966271186</v>
+        <v>14598.9240025424</v>
       </c>
       <c r="G32" s="12" t="n">
         <f aca="false">IF($F$17=0,0,B32/$F$17)</f>
@@ -4896,55 +4896,55 @@
       </c>
       <c r="B19" s="9" t="n">
         <f aca="false">SUMPRODUCT(B$5:B$8,Proyeccion!$H$22:$H$25)</f>
-        <v>10596</v>
+        <v>11079</v>
       </c>
       <c r="C19" s="9" t="n">
         <f aca="false">SUMPRODUCT(C$5:C$8,Proyeccion!$H$22:$H$25)</f>
-        <v>15546</v>
+        <v>16278</v>
       </c>
       <c r="D19" s="9" t="n">
         <f aca="false">SUMPRODUCT(D$5:D$8,Proyeccion!$H$22:$H$25)</f>
-        <v>20292</v>
+        <v>21100.8</v>
       </c>
       <c r="E19" s="9" t="n">
         <f aca="false">SUMPRODUCT(E$5:E$8,Proyeccion!$H$22:$H$25)</f>
-        <v>24096</v>
+        <v>25010.7</v>
       </c>
       <c r="F19" s="9" t="n">
         <f aca="false">SUMPRODUCT(F$5:F$8,Proyeccion!$H$22:$H$25)</f>
-        <v>22420.8</v>
+        <v>23157.6</v>
       </c>
       <c r="G19" s="9" t="n">
         <f aca="false">SUMPRODUCT(G$5:G$8,Proyeccion!$H$22:$H$25)</f>
-        <v>27158.1</v>
+        <v>28003.875</v>
       </c>
       <c r="H19" s="9" t="n">
         <f aca="false">SUMPRODUCT(H$5:H$8,Proyeccion!$H$22:$H$25)</f>
-        <v>33546</v>
+        <v>34643.4</v>
       </c>
       <c r="I19" s="9" t="n">
         <f aca="false">SUMPRODUCT(I$5:I$8,Proyeccion!$H$22:$H$25)</f>
-        <v>35856</v>
+        <v>37080.9</v>
       </c>
       <c r="J19" s="9" t="n">
         <f aca="false">SUMPRODUCT(J$5:J$8,Proyeccion!$H$22:$H$25)</f>
-        <v>39876</v>
+        <v>41167.8</v>
       </c>
       <c r="K19" s="9" t="n">
         <f aca="false">SUMPRODUCT(K$5:K$8,Proyeccion!$H$22:$H$25)</f>
-        <v>30678</v>
+        <v>31430.7</v>
       </c>
       <c r="L19" s="9" t="n">
         <f aca="false">SUMPRODUCT(L$5:L$8,Proyeccion!$H$22:$H$25)</f>
-        <v>14619.6</v>
+        <v>14877.54</v>
       </c>
       <c r="M19" s="9" t="n">
         <f aca="false">SUMPRODUCT(M$5:M$8,Proyeccion!$H$22:$H$25)</f>
-        <v>18592.8</v>
+        <v>19070.04</v>
       </c>
       <c r="N19" s="29" t="n">
         <f aca="false">SUM(B19:M19)</f>
-        <v>293277.3</v>
+        <v>302900.355</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4953,55 +4953,55 @@
       </c>
       <c r="B20" s="29" t="n">
         <f aca="false">B19/(1+Supuestos!$B$26)</f>
-        <v>8979.66101694915</v>
+        <v>9388.98305084746</v>
       </c>
       <c r="C20" s="29" t="n">
         <f aca="false">C19/(1+Supuestos!$B$26)</f>
-        <v>13174.5762711864</v>
+        <v>13794.9152542373</v>
       </c>
       <c r="D20" s="29" t="n">
         <f aca="false">D19/(1+Supuestos!$B$26)</f>
-        <v>17196.6101694915</v>
+        <v>17882.0338983051</v>
       </c>
       <c r="E20" s="29" t="n">
         <f aca="false">E19/(1+Supuestos!$B$26)</f>
-        <v>20420.3389830509</v>
+        <v>21195.5084745763</v>
       </c>
       <c r="F20" s="29" t="n">
         <f aca="false">F19/(1+Supuestos!$B$26)</f>
-        <v>19000.6779661017</v>
+        <v>19625.0847457627</v>
       </c>
       <c r="G20" s="29" t="n">
         <f aca="false">G19/(1+Supuestos!$B$26)</f>
-        <v>23015.3389830509</v>
+        <v>23732.0974576271</v>
       </c>
       <c r="H20" s="29" t="n">
         <f aca="false">H19/(1+Supuestos!$B$26)</f>
-        <v>28428.813559322</v>
+        <v>29358.813559322</v>
       </c>
       <c r="I20" s="29" t="n">
         <f aca="false">I19/(1+Supuestos!$B$26)</f>
-        <v>30386.4406779661</v>
+        <v>31424.4915254237</v>
       </c>
       <c r="J20" s="29" t="n">
         <f aca="false">J19/(1+Supuestos!$B$26)</f>
-        <v>33793.2203389831</v>
+        <v>34887.9661016949</v>
       </c>
       <c r="K20" s="29" t="n">
         <f aca="false">K19/(1+Supuestos!$B$26)</f>
-        <v>25998.3050847458</v>
+        <v>26636.186440678</v>
       </c>
       <c r="L20" s="29" t="n">
         <f aca="false">L19/(1+Supuestos!$B$26)</f>
-        <v>12389.4915254237</v>
+        <v>12608.0847457627</v>
       </c>
       <c r="M20" s="29" t="n">
         <f aca="false">M19/(1+Supuestos!$B$26)</f>
-        <v>15756.6101694915</v>
+        <v>16161.0508474576</v>
       </c>
       <c r="N20" s="29" t="n">
         <f aca="false">SUM(B20:M20)</f>
-        <v>248540.084745763</v>
+        <v>256695.216101695</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5010,55 +5010,55 @@
       </c>
       <c r="B21" s="9" t="n">
         <f aca="false">SUMPRODUCT(B$5:B$8,Proyeccion!$F$22:$F$25)</f>
-        <v>2046.39040677966</v>
+        <v>2437.12922033898</v>
       </c>
       <c r="C21" s="9" t="n">
         <f aca="false">SUMPRODUCT(C$5:C$8,Proyeccion!$F$22:$F$25)</f>
-        <v>2950.86650847458</v>
+        <v>3543.04210169492</v>
       </c>
       <c r="D21" s="9" t="n">
         <f aca="false">SUMPRODUCT(D$5:D$8,Proyeccion!$F$22:$F$25)</f>
-        <v>3938.64106779661</v>
+        <v>4588.95055932204</v>
       </c>
       <c r="E21" s="9" t="n">
         <f aca="false">SUMPRODUCT(E$5:E$8,Proyeccion!$F$22:$F$25)</f>
-        <v>4688.44159322034</v>
+        <v>5422.42438983051</v>
       </c>
       <c r="F21" s="9" t="n">
         <f aca="false">SUMPRODUCT(F$5:F$8,Proyeccion!$F$22:$F$25)</f>
-        <v>4454.12798644068</v>
+        <v>5042.19469830509</v>
       </c>
       <c r="G21" s="9" t="n">
         <f aca="false">SUMPRODUCT(G$5:G$8,Proyeccion!$F$22:$F$25)</f>
-        <v>5443.14319322034</v>
+        <v>6117.37083305085</v>
       </c>
       <c r="H21" s="9" t="n">
         <f aca="false">SUMPRODUCT(H$5:H$8,Proyeccion!$F$22:$F$25)</f>
-        <v>6643.12642372882</v>
+        <v>7518.91642372882</v>
       </c>
       <c r="I21" s="9" t="n">
         <f aca="false">SUMPRODUCT(I$5:I$8,Proyeccion!$F$22:$F$25)</f>
-        <v>7056.56227118644</v>
+        <v>8035.4976101695</v>
       </c>
       <c r="J21" s="9" t="n">
         <f aca="false">SUMPRODUCT(J$5:J$8,Proyeccion!$F$22:$F$25)</f>
-        <v>7919.99913559322</v>
+        <v>8951.05744067797</v>
       </c>
       <c r="K21" s="9" t="n">
         <f aca="false">SUMPRODUCT(K$5:K$8,Proyeccion!$F$22:$F$25)</f>
-        <v>6287.12003389831</v>
+        <v>6880.05757627119</v>
       </c>
       <c r="L21" s="9" t="n">
         <f aca="false">SUMPRODUCT(L$5:L$8,Proyeccion!$F$22:$F$25)</f>
-        <v>3048.93721016949</v>
+        <v>3246.41749830509</v>
       </c>
       <c r="M21" s="9" t="n">
         <f aca="false">SUMPRODUCT(M$5:M$8,Proyeccion!$F$22:$F$25)</f>
-        <v>3760.04686779661</v>
+        <v>4134.93713898305</v>
       </c>
       <c r="N21" s="29" t="n">
         <f aca="false">SUM(B21:M21)</f>
-        <v>58237.4026983051</v>
+        <v>65917.995490678</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5067,55 +5067,55 @@
       </c>
       <c r="B22" s="9" t="n">
         <f aca="false">SUMPRODUCT(B$5:B$8,Proyeccion!$G$22:$G$25)</f>
-        <v>2167.35040677966</v>
+        <v>2558.08922033898</v>
       </c>
       <c r="C22" s="9" t="n">
         <f aca="false">SUMPRODUCT(C$5:C$8,Proyeccion!$G$22:$G$25)</f>
-        <v>3129.28250847458</v>
+        <v>3721.45810169492</v>
       </c>
       <c r="D22" s="9" t="n">
         <f aca="false">SUMPRODUCT(D$5:D$8,Proyeccion!$G$22:$G$25)</f>
-        <v>4178.54506779661</v>
+        <v>4828.85455932204</v>
       </c>
       <c r="E22" s="9" t="n">
         <f aca="false">SUMPRODUCT(E$5:E$8,Proyeccion!$G$22:$G$25)</f>
-        <v>4972.69759322034</v>
+        <v>5706.68038983051</v>
       </c>
       <c r="F22" s="9" t="n">
         <f aca="false">SUMPRODUCT(F$5:F$8,Proyeccion!$G$22:$G$25)</f>
-        <v>4718.62718644068</v>
+        <v>5306.69389830509</v>
       </c>
       <c r="G22" s="9" t="n">
         <f aca="false">SUMPRODUCT(G$5:G$8,Proyeccion!$G$22:$G$25)</f>
-        <v>5755.92559322034</v>
+        <v>6430.15323305085</v>
       </c>
       <c r="H22" s="9" t="n">
         <f aca="false">SUMPRODUCT(H$5:H$8,Proyeccion!$G$22:$G$25)</f>
-        <v>7033.22242372881</v>
+        <v>7909.01242372882</v>
       </c>
       <c r="I22" s="9" t="n">
         <f aca="false">SUMPRODUCT(I$5:I$8,Proyeccion!$G$22:$G$25)</f>
-        <v>7476.89827118644</v>
+        <v>8455.83361016949</v>
       </c>
       <c r="J22" s="9" t="n">
         <f aca="false">SUMPRODUCT(J$5:J$8,Proyeccion!$G$22:$G$25)</f>
-        <v>8378.63913559322</v>
+        <v>9409.69744067797</v>
       </c>
       <c r="K22" s="9" t="n">
         <f aca="false">SUMPRODUCT(K$5:K$8,Proyeccion!$G$22:$G$25)</f>
-        <v>6641.9360338983</v>
+        <v>7234.87357627119</v>
       </c>
       <c r="L22" s="9" t="n">
         <f aca="false">SUMPRODUCT(L$5:L$8,Proyeccion!$G$22:$G$25)</f>
-        <v>3233.19961016949</v>
+        <v>3430.67989830509</v>
       </c>
       <c r="M22" s="9" t="n">
         <f aca="false">SUMPRODUCT(M$5:M$8,Proyeccion!$G$22:$G$25)</f>
-        <v>3996.32206779661</v>
+        <v>4371.21233898305</v>
       </c>
       <c r="N22" s="29" t="n">
         <f aca="false">SUM(B22:M22)</f>
-        <v>61682.6458983051</v>
+        <v>69363.238690678</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5181,55 +5181,55 @@
       </c>
       <c r="B24" s="11" t="n">
         <f aca="false">B21-B23</f>
-        <v>-810.279593220339</v>
+        <v>-419.540779661016</v>
       </c>
       <c r="C24" s="11" t="n">
         <f aca="false">C21-C23</f>
-        <v>94.1965084745771</v>
+        <v>686.372101694917</v>
       </c>
       <c r="D24" s="11" t="n">
         <f aca="false">D21-D23</f>
-        <v>1081.97106779661</v>
+        <v>1732.28055932204</v>
       </c>
       <c r="E24" s="11" t="n">
         <f aca="false">E21-E23</f>
-        <v>1831.77159322034</v>
+        <v>2565.75438983051</v>
       </c>
       <c r="F24" s="11" t="n">
         <f aca="false">F21-F23</f>
-        <v>1597.45798644068</v>
+        <v>2185.52469830509</v>
       </c>
       <c r="G24" s="11" t="n">
         <f aca="false">G21-G23</f>
-        <v>2586.47319322034</v>
+        <v>3260.70083305085</v>
       </c>
       <c r="H24" s="11" t="n">
         <f aca="false">H21-H23</f>
-        <v>3786.45642372882</v>
+        <v>4662.24642372882</v>
       </c>
       <c r="I24" s="11" t="n">
         <f aca="false">I21-I23</f>
-        <v>4199.89227118644</v>
+        <v>5178.8276101695</v>
       </c>
       <c r="J24" s="11" t="n">
         <f aca="false">J21-J23</f>
-        <v>5063.32913559322</v>
+        <v>6094.38744067797</v>
       </c>
       <c r="K24" s="11" t="n">
         <f aca="false">K21-K23</f>
-        <v>3430.45003389831</v>
+        <v>4023.38757627119</v>
       </c>
       <c r="L24" s="11" t="n">
         <f aca="false">L21-L23</f>
-        <v>192.267210169492</v>
+        <v>389.747498305086</v>
       </c>
       <c r="M24" s="11" t="n">
         <f aca="false">M21-M23</f>
-        <v>903.376867796611</v>
+        <v>1278.26713898305</v>
       </c>
       <c r="N24" s="11" t="n">
         <f aca="false">SUM(B24:M24)</f>
-        <v>23957.3626983051</v>
+        <v>31637.955490678</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5238,55 +5238,55 @@
       </c>
       <c r="B25" s="11" t="n">
         <f aca="false">B22-B23</f>
-        <v>-689.319593220339</v>
+        <v>-298.580779661017</v>
       </c>
       <c r="C25" s="11" t="n">
         <f aca="false">C22-C23</f>
-        <v>272.612508474575</v>
+        <v>864.788101694916</v>
       </c>
       <c r="D25" s="11" t="n">
         <f aca="false">D22-D23</f>
-        <v>1321.87506779661</v>
+        <v>1972.18455932204</v>
       </c>
       <c r="E25" s="11" t="n">
         <f aca="false">E22-E23</f>
-        <v>2116.02759322034</v>
+        <v>2850.01038983051</v>
       </c>
       <c r="F25" s="11" t="n">
         <f aca="false">F22-F23</f>
-        <v>1861.95718644068</v>
+        <v>2450.02389830509</v>
       </c>
       <c r="G25" s="11" t="n">
         <f aca="false">G22-G23</f>
-        <v>2899.25559322034</v>
+        <v>3573.48323305085</v>
       </c>
       <c r="H25" s="11" t="n">
         <f aca="false">H22-H23</f>
-        <v>4176.55242372881</v>
+        <v>5052.34242372882</v>
       </c>
       <c r="I25" s="11" t="n">
         <f aca="false">I22-I23</f>
-        <v>4620.22827118644</v>
+        <v>5599.16361016949</v>
       </c>
       <c r="J25" s="11" t="n">
         <f aca="false">J22-J23</f>
-        <v>5521.96913559322</v>
+        <v>6553.02744067797</v>
       </c>
       <c r="K25" s="11" t="n">
         <f aca="false">K22-K23</f>
-        <v>3785.2660338983</v>
+        <v>4378.20357627119</v>
       </c>
       <c r="L25" s="11" t="n">
         <f aca="false">L22-L23</f>
-        <v>376.529610169491</v>
+        <v>574.009898305085</v>
       </c>
       <c r="M25" s="11" t="n">
         <f aca="false">M22-M23</f>
-        <v>1139.65206779661</v>
+        <v>1514.54233898305</v>
       </c>
       <c r="N25" s="11" t="n">
         <f aca="false">SUM(B25:M25)</f>
-        <v>27402.6058983051</v>
+        <v>35083.198690678</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5295,51 +5295,51 @@
       </c>
       <c r="B26" s="29" t="n">
         <f aca="false">B24</f>
-        <v>-810.279593220339</v>
+        <v>-419.540779661016</v>
       </c>
       <c r="C26" s="29" t="n">
         <f aca="false">B26+C24</f>
-        <v>-716.083084745762</v>
+        <v>266.831322033901</v>
       </c>
       <c r="D26" s="29" t="n">
         <f aca="false">C26+D24</f>
-        <v>365.887983050849</v>
+        <v>1999.11188135594</v>
       </c>
       <c r="E26" s="29" t="n">
         <f aca="false">D26+E24</f>
-        <v>2197.65957627119</v>
+        <v>4564.86627118645</v>
       </c>
       <c r="F26" s="29" t="n">
         <f aca="false">E26+F24</f>
-        <v>3795.11756271187</v>
+        <v>6750.39096949154</v>
       </c>
       <c r="G26" s="29" t="n">
         <f aca="false">F26+G24</f>
-        <v>6381.59075593221</v>
+        <v>10011.0918025424</v>
       </c>
       <c r="H26" s="29" t="n">
         <f aca="false">G26+H24</f>
-        <v>10168.047179661</v>
+        <v>14673.3382262712</v>
       </c>
       <c r="I26" s="29" t="n">
         <f aca="false">H26+I24</f>
-        <v>14367.9394508475</v>
+        <v>19852.1658364407</v>
       </c>
       <c r="J26" s="29" t="n">
         <f aca="false">I26+J24</f>
-        <v>19431.2685864407</v>
+        <v>25946.5532771187</v>
       </c>
       <c r="K26" s="29" t="n">
         <f aca="false">J26+K24</f>
-        <v>22861.718620339</v>
+        <v>29969.9408533899</v>
       </c>
       <c r="L26" s="29" t="n">
         <f aca="false">K26+L24</f>
-        <v>23053.9858305085</v>
+        <v>30359.6883516949</v>
       </c>
       <c r="M26" s="29" t="n">
         <f aca="false">L26+M24</f>
-        <v>23957.3626983051</v>
+        <v>31637.955490678</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5348,51 +5348,51 @@
       </c>
       <c r="B27" s="29" t="n">
         <f aca="false">B25</f>
-        <v>-689.319593220339</v>
+        <v>-298.580779661017</v>
       </c>
       <c r="C27" s="29" t="n">
         <f aca="false">B27+C25</f>
-        <v>-416.707084745764</v>
+        <v>566.207322033899</v>
       </c>
       <c r="D27" s="29" t="n">
         <f aca="false">C27+D25</f>
-        <v>905.167983050845</v>
+        <v>2538.39188135593</v>
       </c>
       <c r="E27" s="29" t="n">
         <f aca="false">D27+E25</f>
-        <v>3021.19557627118</v>
+        <v>5388.40227118645</v>
       </c>
       <c r="F27" s="29" t="n">
         <f aca="false">E27+F25</f>
-        <v>4883.15276271186</v>
+        <v>7838.42616949153</v>
       </c>
       <c r="G27" s="29" t="n">
         <f aca="false">F27+G25</f>
-        <v>7782.4083559322</v>
+        <v>11411.9094025424</v>
       </c>
       <c r="H27" s="29" t="n">
         <f aca="false">G27+H25</f>
-        <v>11958.960779661</v>
+        <v>16464.2518262712</v>
       </c>
       <c r="I27" s="29" t="n">
         <f aca="false">H27+I25</f>
-        <v>16579.1890508475</v>
+        <v>22063.4154364407</v>
       </c>
       <c r="J27" s="29" t="n">
         <f aca="false">I27+J25</f>
-        <v>22101.1581864407</v>
+        <v>28616.4428771187</v>
       </c>
       <c r="K27" s="29" t="n">
         <f aca="false">J27+K25</f>
-        <v>25886.424220339</v>
+        <v>32994.6464533899</v>
       </c>
       <c r="L27" s="29" t="n">
         <f aca="false">K27+L25</f>
-        <v>26262.9538305085</v>
+        <v>33568.6563516949</v>
       </c>
       <c r="M27" s="29" t="n">
         <f aca="false">L27+M25</f>
-        <v>27402.6058983051</v>
+        <v>35083.198690678</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
TC5-8 y costeo: se elimina por ahora la suscripción; el pack de 12 se vende por pedido
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Kfbf7cfV7pXUcNjjyaPCzV
</commit_message>
<xml_diff>
--- a/04-reformulacion/Costeo-presentaciones-AndiBite.xlsx
+++ b/04-reformulacion/Costeo-presentaciones-AndiBite.xlsx
@@ -103,7 +103,7 @@
     <t xml:space="preserve">  5. Se resta el costo del canal (delivery, pasarela, comisión) y se suman las contribuciones. Esa suma, menos los costos fijos, es el resultado.</t>
   </si>
   <si>
-    <t xml:space="preserve">  La ventaja: si cambia la mezcla (por ejemplo, más packs de 12 por suscripción), el ingreso y el margen se recalculan solos sin rehacer la proyección.</t>
+    <t xml:space="preserve">  La ventaja: si cambia la mezcla (por ejemplo, más packs de 12), el ingreso y el margen se recalculan solos sin rehacer la proyección.</t>
   </si>
   <si>
     <t xml:space="preserve">Ejemplo para probar: en Supuestos, cambie la maquila (celda B7) de 0.50 a 0.90 y mire cómo sube el punto de equilibrio en Resumen.</t>
@@ -1274,7 +1274,7 @@
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:A25"/>
-  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="110"/>
   </cols>
@@ -1373,7 +1373,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
         <v>17</v>
       </c>
@@ -1408,7 +1408,7 @@
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:E27"/>
-  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="60"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="2" style="0" width="22"/>
@@ -1710,7 +1710,7 @@
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:E65"/>
-  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="62"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
@@ -2120,7 +2120,7 @@
       <c r="D37" s="17"/>
       <c r="E37" s="17"/>
     </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="38" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="5" t="s">
         <v>96</v>
       </c>
@@ -2214,7 +2214,7 @@
       <c r="D44" s="17"/>
       <c r="E44" s="17"/>
     </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="45" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="5" t="s">
         <v>96</v>
       </c>
@@ -2389,7 +2389,7 @@
       <c r="C60" s="17"/>
       <c r="D60" s="17"/>
     </row>
-    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="61" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="5" t="s">
         <v>128</v>
       </c>
@@ -2457,7 +2457,7 @@
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:E25"/>
-  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="62"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="2" style="0" width="24"/>
@@ -2845,7 +2845,7 @@
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:S38"/>
-  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="36"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18"/>
@@ -4271,7 +4271,7 @@
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:N29"/>
-  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="2" style="0" width="11"/>

</xml_diff>

<commit_message>
Costeo v5: personal pagado en stands y coordinador en planilla, sangrecita fresca, maquila S/0.45 y año 1 desde enero de 2027
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Kfbf7cfV7pXUcNjjyaPCzV
</commit_message>
<xml_diff>
--- a/04-reformulacion/Costeo-presentaciones-AndiBite.xlsx
+++ b/04-reformulacion/Costeo-presentaciones-AndiBite.xlsx
@@ -91,7 +91,7 @@
     <t xml:space="preserve">Ejemplos para probar: en Mensual, cambie los brownies por día en cada punto (fila 7); en Supuestos, cambie el alquiler por punto (B57) o la maquila (B7) y mire el resultado en Resumen.</t>
   </si>
   <si>
-    <t xml:space="preserve">AndiBite — Resumen del año 1 (noviembre 2026 a octubre 2027), escenario base con venta física</t>
+    <t xml:space="preserve">AndiBite — Resumen del año 1 (enero a diciembre de 2027), escenario base con venta física</t>
   </si>
   <si>
     <t xml:space="preserve">Todo se calcula desde las hojas Supuestos, Inversion, Costeo, Proyeccion y Mensual. Cambie las celdas azules de Supuestos o Mensual.</t>
@@ -181,22 +181,22 @@
     <t xml:space="preserve">Caja más baja del año, con la cuota del préstamo (opción B)</t>
   </si>
   <si>
-    <t xml:space="preserve">Meses desde noviembre de 2026 para recuperar la inversión (el año 2 al ritmo de agosto a octubre de 2027)</t>
+    <t xml:space="preserve">Meses desde el inicio de ventas (mes 1 = enero de 2027) para recuperar la inversión (el año 2 al ritmo de los meses 10 a 12)</t>
   </si>
   <si>
     <t xml:space="preserve">Notas</t>
   </si>
   <si>
-    <t xml:space="preserve">1. La proyección supone que los documentos (S.A.C., marca, registro sanitario, análisis, etiqueta, carnés y póliza) ya están listos en noviembre de 2026. Su costo está en la hoja Inversion.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2. La venta física (stands, carritos y ferias) es el canal principal; WhatsApp queda para la recompra, sin suscripción. Los socios atienden 2 puntos de venta; el tercero lleva impulsadora.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3. La maquila (S/0.50 por unidad) y el polvo de sangrecita no están cotizados con la planta. Cambiarlos en Supuestos apenas lleguen las cotizaciones.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4. El resultado no incluye sueldos de los socios, intereses del préstamo (hoja Inversion) ni el impuesto a la renta anual.</t>
+    <t xml:space="preserve">1. La proyección supone que los documentos (S.A.C., marca, registro sanitario, análisis, etiqueta, carnés y póliza) ya están listos al inicio de ventas (mes 1, enero de 2027). Su costo está en la hoja Inversion.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2. La venta física (stands, carritos y ferias) es el canal principal; WhatsApp queda para la recompra, sin suscripción. Todos los puntos de venta llevan vendedor(a) pagado(a) y un(a) coordinador(a) en planilla atiende pedidos y despacho.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3. Costo de producción con sangrecita fresca de pollo (S/0.40 de insumos por brownie) y maquila de S/0.45 por brownie.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4. El resultado incluye al personal que opera el negocio (vendedores de stand y coordinador). No incluye intereses del préstamo (hoja Inversion) ni el impuesto a la renta anual.</t>
   </si>
   <si>
     <t xml:space="preserve">Supuestos del costeo — AndiBite (maquila, escenario de 3,000 unidades al mes)</t>
@@ -220,19 +220,19 @@
     <t xml:space="preserve">Fuente o nota</t>
   </si>
   <si>
-    <t xml:space="preserve">Insumos por unidad (promedio de los 3 sabores, sangrecita en polvo)</t>
+    <t xml:space="preserve">Insumos por unidad (promedio de los 3 sabores, con sangrecita fresca de pollo cocida en la planta)</t>
   </si>
   <si>
     <t xml:space="preserve">S/ por unidad</t>
   </si>
   <si>
-    <t xml:space="preserve">Documento 05, tabla 4.2 (precios de Makro, mayoristas, Plaza Vea y Wong sin IGV)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Maquila por unidad (la planta mezcla, hornea, corta, pesa y empaca)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[POR CONFIRMAR] Rango S/0.40-0.60 del documento 03. Cotizar con MAKING y Panificadora Unión</t>
+    <t xml:space="preserve">Recetas del documento 01: 175 g de sangrecita cruda por lote de 24 (Redondos, S/11.29 por kg en Makro), que la planta cuece y licúa con los huevos; resto de insumos según documento 05 (Makro, mayoristas, Plaza Vea y Wong, sin IGV)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Maquila por unidad (la planta cuece la sangrecita, mezcla, hornea, corta, pesa y sella la bolsita)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tarifa de maquila de snacks horneados en Lima: S/20.75 por kg de producto terminado, elaboración y empaque incluidos (Organic Andean Bites, documento 03), actualizada a 2027: S/0.45 por brownie de 20 g</t>
   </si>
   <si>
     <t xml:space="preserve">Descuento de maquila si no se empaca cada unidad (opción C)</t>
@@ -424,22 +424,22 @@
     <t xml:space="preserve">Módulo de 2 x 2 m en malls desde S/500 al mes (Gestión, 15-sep-2023); la entrada de un supermercado de Lima Top cuesta algo más (documento 08)</t>
   </si>
   <si>
-    <t xml:space="preserve">Pago a impulsadora por día de stand</t>
+    <t xml:space="preserve">Pago a vendedor(a) de stand por día</t>
   </si>
   <si>
     <t xml:space="preserve">S/ por día</t>
   </si>
   <si>
-    <t xml:space="preserve">Computrabajo: S/50 a 90 por día de fin de semana (documento 08)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Puntos de venta que atienden los socios (sin pago)</t>
+    <t xml:space="preserve">Pago de impulsadoras en Lima: S/50 a 90 por día de fin de semana (Computrabajo, documento 08)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Puntos de venta que atienden los socios sin pago</t>
   </si>
   <si>
     <t xml:space="preserve">puntos</t>
   </si>
   <si>
-    <t xml:space="preserve">Los 5 socios cubren 2 puntos los fines de semana con turnos rotativos; desde el tercer punto se paga impulsadora</t>
+    <t xml:space="preserve">Todos los puntos de venta llevan un(a) vendedor(a) pagado(a); los socios supervisan</t>
   </si>
   <si>
     <t xml:space="preserve">Stand en feria de emprendimiento (2 a 3 días)</t>
@@ -487,10 +487,10 @@
     <t xml:space="preserve">Documento 05, sección 4.1</t>
   </si>
   <si>
-    <t xml:space="preserve">Asistente de pedidos y despacho</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Los socios atienden WhatsApp y el despacho; las impulsadoras cubren los stands adicionales (Supuestos B58). Versión anterior: S/800</t>
+    <t xml:space="preserve">Coordinador(a) comercial y de operaciones (planilla, medio tiempo de 4 horas)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Media remuneración mínima de 2027 (S/1,300 según el DS 015-2026-TR) más 9 % de EsSalud; microempresa en el REMYPE. Atiende WhatsApp, pedidos y despacho, y lleva el stock a los stands</t>
   </si>
   <si>
     <t xml:space="preserve">Marketing: pauta, degustaciones y material de stand (promedio del año)</t>
@@ -595,7 +595,7 @@
     <t xml:space="preserve">El margen bruto no incluye alquiler del stand, personal, delivery, pasarela, comisiones ni costos fijos: eso se calcula en las hojas Proyeccion y Mensual.</t>
   </si>
   <si>
-    <t xml:space="preserve">Proyección anual por canal y presentación (año 1, noviembre 2026 a octubre 2027)</t>
+    <t xml:space="preserve">Proyección anual por canal y presentación (año 1: enero a diciembre de 2027)</t>
   </si>
   <si>
     <t xml:space="preserve">Paso a paso: unidades del canal (hoja Mensual) × mezcla de presentaciones (Supuestos) = unidades por presentación; ÷ tamaño = envases vendidos; × precio = ingreso; menos costo de producción y costo variable de canal = contribución.</t>
@@ -685,7 +685,7 @@
     <t xml:space="preserve">Inversión inicial: todo lo necesario para vender desde el primer día</t>
   </si>
   <si>
-    <t xml:space="preserve">Los documentos y permisos se pagan aquí, una sola vez. La proyección (hoja Mensual) supone que ya están listos al empezar las ventas en noviembre de 2026.</t>
+    <t xml:space="preserve">Los documentos y permisos se pagan aquí, una sola vez. La proyección (hoja Mensual) supone que ya están listos al empezar las ventas en enero de 2027 (mes 1).</t>
   </si>
   <si>
     <t xml:space="preserve">S/ (sin IGV)</t>
@@ -796,7 +796,7 @@
     <t xml:space="preserve">Empaque inicial (mínimos de compra)</t>
   </si>
   <si>
-    <t xml:space="preserve">Stock inicial para noviembre y diciembre</t>
+    <t xml:space="preserve">Stock inicial para enero y febrero</t>
   </si>
   <si>
     <t xml:space="preserve">Marketing de lanzamiento (degustaciones, influencers, POP)</t>
@@ -871,7 +871,7 @@
     <t xml:space="preserve">Caja que sobra después de financiar la inversión</t>
   </si>
   <si>
-    <t xml:space="preserve">Proyección mensual del año 1 (noviembre 2026 a octubre 2027), escenario base</t>
+    <t xml:space="preserve">Proyección mensual del año 1 (mes 1 = enero de 2027), escenario base</t>
   </si>
   <si>
     <t xml:space="preserve">Supone que los documentos y permisos ya están listos (su costo está en la hoja Inversion). La venta física es el canal principal; WhatsApp queda para la recompra. Cambie los datos azules para probar otro escenario.</t>
@@ -880,40 +880,40 @@
     <t xml:space="preserve">Actividad comercial del mes (datos)</t>
   </si>
   <si>
-    <t xml:space="preserve">Nov-26</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dic-26</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ene-27</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Feb-27</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mar-27</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Abr-27</t>
-  </si>
-  <si>
-    <t xml:space="preserve">May-27</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jun-27</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jul-27</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ago-27</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Set-27</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Oct-27</t>
+    <t xml:space="preserve">M1 Ene-27</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M2 Feb-27</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M3 Mar-27</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M4 Abr-27</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M5 May-27</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M6 Jun-27</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M7 Jul-27</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M8 Ago-27</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M9 Set-27</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M10 Oct-27</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M11 Nov-27</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M12 Dic-27</t>
   </si>
   <si>
     <t xml:space="preserve">Total año</t>
@@ -925,16 +925,16 @@
     <t xml:space="preserve">Días de atención por punto en el mes</t>
   </si>
   <si>
-    <t xml:space="preserve">Brownies vendidos por día en cada punto</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ferias pagadas en el mes (Navidad y campaña escolar)</t>
+    <t xml:space="preserve">Brownies vendidos por día en cada punto (meta: 80 o más)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ferias pagadas en el mes (campaña escolar y Navidad)</t>
   </si>
   <si>
     <t xml:space="preserve">Eventos sin costo (kermeses, cumpleaños, ferias gratuitas)</t>
   </si>
   <si>
-    <t xml:space="preserve">Unidades a colegios (quiosco; año escolar de marzo a diciembre)</t>
+    <t xml:space="preserve">Unidades a colegios (quiosco; año escolar de marzo a mediados de diciembre)</t>
   </si>
   <si>
     <t xml:space="preserve">Unidades a tiendas naturistas</t>
@@ -976,7 +976,7 @@
     <t xml:space="preserve">Alquiler de espacios para stands y carritos</t>
   </si>
   <si>
-    <t xml:space="preserve">Impulsadoras (puntos que no atienden los socios)</t>
+    <t xml:space="preserve">Vendedores de stand (por día de atención)</t>
   </si>
   <si>
     <t xml:space="preserve">Ferias pagadas</t>
@@ -1763,11 +1763,11 @@
       </c>
       <c r="B5" s="6" t="n">
         <f aca="false">Costeo!B15</f>
-        <v>1.69325</v>
+        <v>1.4255</v>
       </c>
       <c r="C5" s="6" t="n">
         <f aca="false">Costeo!B16</f>
-        <v>1.69325</v>
+        <v>1.4255</v>
       </c>
       <c r="D5" s="6" t="n">
         <f aca="false">Costeo!B19</f>
@@ -1775,7 +1775,7 @@
       </c>
       <c r="E5" s="7" t="n">
         <f aca="false">Costeo!B22</f>
-        <v>0.636720909090909</v>
+        <v>0.694165454545455</v>
       </c>
       <c r="F5" s="6" t="n">
         <f aca="false">Costeo!B25</f>
@@ -1783,7 +1783,7 @@
       </c>
       <c r="G5" s="7" t="n">
         <f aca="false">Costeo!B28</f>
-        <v>0.50049125</v>
+        <v>0.5794775</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1792,11 +1792,11 @@
       </c>
       <c r="B6" s="6" t="n">
         <f aca="false">Costeo!C15</f>
-        <v>9.897</v>
+        <v>8.2905</v>
       </c>
       <c r="C6" s="6" t="n">
         <f aca="false">Costeo!C16</f>
-        <v>1.6495</v>
+        <v>1.38175</v>
       </c>
       <c r="D6" s="6" t="n">
         <f aca="false">Costeo!C19</f>
@@ -1804,7 +1804,7 @@
       </c>
       <c r="E6" s="7" t="n">
         <f aca="false">Costeo!C22</f>
-        <v>0.550828461538462</v>
+        <v>0.623738846153846</v>
       </c>
       <c r="F6" s="6" t="n">
         <f aca="false">Costeo!C25</f>
@@ -1812,7 +1812,7 @@
       </c>
       <c r="G6" s="7" t="n">
         <f aca="false">Costeo!C28</f>
-        <v>0.530985542168675</v>
+        <v>0.60711686746988</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1821,11 +1821,11 @@
       </c>
       <c r="B7" s="6" t="n">
         <f aca="false">Costeo!D15</f>
-        <v>9.393</v>
+        <v>7.7865</v>
       </c>
       <c r="C7" s="6" t="n">
         <f aca="false">Costeo!D16</f>
-        <v>1.5655</v>
+        <v>1.29775</v>
       </c>
       <c r="D7" s="6" t="n">
         <f aca="false">Costeo!D19</f>
@@ -1833,7 +1833,7 @@
       </c>
       <c r="E7" s="7" t="n">
         <f aca="false">Costeo!D22</f>
-        <v>0.573702307692308</v>
+        <v>0.646612692307692</v>
       </c>
       <c r="F7" s="6" t="n">
         <f aca="false">Costeo!D25</f>
@@ -1841,7 +1841,7 @@
       </c>
       <c r="G7" s="7" t="n">
         <f aca="false">Costeo!D28</f>
-        <v>0.554869879518072</v>
+        <v>0.631001204819277</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1850,11 +1850,11 @@
       </c>
       <c r="B8" s="6" t="n">
         <f aca="false">Costeo!E15</f>
-        <v>18.66</v>
+        <v>15.447</v>
       </c>
       <c r="C8" s="6" t="n">
         <f aca="false">Costeo!E16</f>
-        <v>1.555</v>
+        <v>1.28725</v>
       </c>
       <c r="D8" s="6" t="n">
         <f aca="false">Costeo!E19</f>
@@ -1862,7 +1862,7 @@
       </c>
       <c r="E8" s="7" t="n">
         <f aca="false">Costeo!E22</f>
-        <v>0.541275</v>
+        <v>0.62026125</v>
       </c>
       <c r="F8" s="6" t="n">
         <f aca="false">Costeo!E25</f>
@@ -1870,7 +1870,7 @@
       </c>
       <c r="G8" s="7" t="n">
         <f aca="false">Costeo!E28</f>
-        <v>0.530515991471215</v>
+        <v>0.611354797441365</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1892,11 +1892,11 @@
       </c>
       <c r="B12" s="8" t="n">
         <f aca="false">Proyeccion!F20</f>
-        <v>47223</v>
+        <v>52786</v>
       </c>
       <c r="C12" s="8" t="n">
         <f aca="false">Proyeccion!F20</f>
-        <v>47223</v>
+        <v>52786</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1905,11 +1905,11 @@
       </c>
       <c r="B13" s="9" t="n">
         <f aca="false">Proyeccion!I20</f>
-        <v>207452.195833333</v>
+        <v>230740.383333333</v>
       </c>
       <c r="C13" s="9" t="n">
         <f aca="false">Proyeccion!I20</f>
-        <v>207452.195833333</v>
+        <v>230740.383333333</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1918,11 +1918,11 @@
       </c>
       <c r="B14" s="9" t="n">
         <f aca="false">Proyeccion!J20</f>
-        <v>175806.945621469</v>
+        <v>195542.697740113</v>
       </c>
       <c r="C14" s="9" t="n">
         <f aca="false">Proyeccion!J20</f>
-        <v>175806.945621469</v>
+        <v>195542.697740113</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1931,11 +1931,11 @@
       </c>
       <c r="B15" s="9" t="n">
         <f aca="false">Proyeccion!P20</f>
-        <v>74368.9355902542</v>
+        <v>96848.2879877119</v>
       </c>
       <c r="C15" s="9" t="n">
         <f aca="false">Proyeccion!Q20</f>
-        <v>75902.9057902542</v>
+        <v>98492.5333877119</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1944,11 +1944,11 @@
       </c>
       <c r="B16" s="9" t="n">
         <f aca="false">Mensual!N33+Mensual!N34+Mensual!N35</f>
-        <v>22830</v>
+        <v>45870</v>
       </c>
       <c r="C16" s="9" t="n">
         <f aca="false">Mensual!N33+Mensual!N34+Mensual!N35</f>
-        <v>22830</v>
+        <v>45870</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1957,11 +1957,11 @@
       </c>
       <c r="B17" s="9" t="n">
         <f aca="false">Supuestos!B72*12</f>
-        <v>20812.6666666667</v>
+        <v>29320.6666666667</v>
       </c>
       <c r="C17" s="9" t="n">
         <f aca="false">Supuestos!B72*12</f>
-        <v>20812.6666666667</v>
+        <v>29320.6666666667</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1970,11 +1970,11 @@
       </c>
       <c r="B18" s="11" t="n">
         <f aca="false">B15-B16-B17</f>
-        <v>30726.2689235876</v>
+        <v>21657.6213210452</v>
       </c>
       <c r="C18" s="11" t="n">
         <f aca="false">C15-C16-C17</f>
-        <v>32260.2391235876</v>
+        <v>23301.8667210452</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1983,11 +1983,11 @@
       </c>
       <c r="B19" s="12" t="n">
         <f aca="false">IF(B14=0,0,B18/B14)</f>
-        <v>0.174772781672372</v>
+        <v>0.1107564821972</v>
       </c>
       <c r="C19" s="12" t="n">
         <f aca="false">IF(C14=0,0,C18/C14)</f>
-        <v>0.183498092237194</v>
+        <v>0.119165108134156</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1996,11 +1996,11 @@
       </c>
       <c r="B20" s="13" t="n">
         <f aca="false">IF(B12=0,0,(B15-B16)/B12)</f>
-        <v>1.09139477776199</v>
+        <v>0.96575394967817</v>
       </c>
       <c r="C20" s="13" t="n">
         <f aca="false">IF(C12=0,0,(C15-C16)/C12)</f>
-        <v>1.12387831756251</v>
+        <v>0.996903220318112</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2009,11 +2009,11 @@
       </c>
       <c r="B21" s="14" t="n">
         <f aca="false">IF(B20&lt;=0,"No alcanza",Supuestos!$B$72/B20)</f>
-        <v>1589.14897178217</v>
+        <v>2530.03250952598</v>
       </c>
       <c r="C21" s="14" t="n">
         <f aca="false">IF(C20&lt;=0,"No alcanza",Supuestos!$B$72/C20)</f>
-        <v>1543.21767916163</v>
+        <v>2450.97903095268</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2022,11 +2022,11 @@
       </c>
       <c r="B22" s="15" t="n">
         <f aca="false">IF(ISNUMBER(B21),B21/6,"No alcanza")</f>
-        <v>264.858161963695</v>
+        <v>421.672084920997</v>
       </c>
       <c r="C22" s="15" t="n">
         <f aca="false">IF(ISNUMBER(C21),C21/6,"No alcanza")</f>
-        <v>257.202946526938</v>
+        <v>408.49650515878</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2048,11 +2048,11 @@
       </c>
       <c r="B24" s="16" t="n">
         <f aca="false">B18-B23</f>
-        <v>-7167.97207641242</v>
+        <v>-16236.6196789548</v>
       </c>
       <c r="C24" s="16" t="n">
         <f aca="false">C18-C23</f>
-        <v>-5634.00187641242</v>
+        <v>-14592.3742789548</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2061,11 +2061,11 @@
       </c>
       <c r="B25" s="9" t="n">
         <f aca="false">MIN(Mensual!B43:M43)</f>
-        <v>7330.53217644292</v>
+        <v>4037.38213254684</v>
       </c>
       <c r="C25" s="9" t="n">
         <f aca="false">MIN(Mensual!B43:M43)</f>
-        <v>7330.53217644292</v>
+        <v>4037.38213254684</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2074,11 +2074,11 @@
       </c>
       <c r="B26" s="17" t="n">
         <f aca="false">IF(B18&gt;=B23,"Dentro del año 1",ROUNDUP(12+(B23-B18)/AVERAGE(Mensual!K37:M37),0))</f>
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C26" s="17" t="n">
         <f aca="false">IF(C18&gt;=C23,"Dentro del año 1",ROUNDUP(12+(C23-C18)/AVERAGE(Mensual!K38:M38),0))</f>
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2169,7 +2169,7 @@
         <v>64</v>
       </c>
       <c r="B6" s="20" t="n">
-        <v>0.605</v>
+        <v>0.4</v>
       </c>
       <c r="C6" s="4" t="s">
         <v>65</v>
@@ -2182,8 +2182,8 @@
       <c r="A7" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="B7" s="21" t="n">
-        <v>0.5</v>
+      <c r="B7" s="20" t="n">
+        <v>0.45</v>
       </c>
       <c r="C7" s="4" t="s">
         <v>65</v>
@@ -2825,7 +2825,7 @@
         <v>135</v>
       </c>
       <c r="B59" s="25" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C59" s="4" t="s">
         <v>136</v>
@@ -2940,7 +2940,7 @@
         <v>153</v>
       </c>
       <c r="B69" s="26" t="n">
-        <v>0</v>
+        <v>709</v>
       </c>
       <c r="D69" s="4" t="s">
         <v>154</v>
@@ -2975,7 +2975,7 @@
       </c>
       <c r="B72" s="30" t="n">
         <f aca="false">SUM(B68:B71)</f>
-        <v>1734.38888888889</v>
+        <v>2443.38888888889</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3109,19 +3109,19 @@
       </c>
       <c r="B6" s="6" t="n">
         <f aca="false">B5*Supuestos!$B$6</f>
-        <v>0.605</v>
+        <v>0.4</v>
       </c>
       <c r="C6" s="6" t="n">
         <f aca="false">C5*Supuestos!$B$6</f>
-        <v>3.63</v>
+        <v>2.4</v>
       </c>
       <c r="D6" s="6" t="n">
         <f aca="false">D5*Supuestos!$B$6</f>
-        <v>3.63</v>
+        <v>2.4</v>
       </c>
       <c r="E6" s="6" t="n">
         <f aca="false">E5*Supuestos!$B$6</f>
-        <v>7.26</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3130,19 +3130,19 @@
       </c>
       <c r="B7" s="6" t="n">
         <f aca="false">B5*Supuestos!$B$7</f>
-        <v>0.5</v>
+        <v>0.45</v>
       </c>
       <c r="C7" s="6" t="n">
         <f aca="false">C5*Supuestos!$B$7</f>
-        <v>3</v>
+        <v>2.7</v>
       </c>
       <c r="D7" s="6" t="n">
         <f aca="false">D5*(Supuestos!$B$7-Supuestos!$B$8)</f>
-        <v>3</v>
+        <v>2.7</v>
       </c>
       <c r="E7" s="6" t="n">
         <f aca="false">E5*Supuestos!$B$7</f>
-        <v>6</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3247,19 +3247,19 @@
       </c>
       <c r="B13" s="13" t="n">
         <f aca="false">Supuestos!$B$15*SUM(B6:B12)</f>
-        <v>0.07225</v>
+        <v>0.0595</v>
       </c>
       <c r="C13" s="13" t="n">
         <f aca="false">Supuestos!$B$15*SUM(C6:C12)</f>
-        <v>0.421</v>
+        <v>0.3445</v>
       </c>
       <c r="D13" s="13" t="n">
         <f aca="false">Supuestos!$B$15*SUM(D6:D12)</f>
-        <v>0.397</v>
+        <v>0.3205</v>
       </c>
       <c r="E13" s="13" t="n">
         <f aca="false">Supuestos!$B$15*SUM(E6:E12)</f>
-        <v>0.788</v>
+        <v>0.635</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3289,19 +3289,19 @@
       </c>
       <c r="B15" s="30" t="n">
         <f aca="false">SUM(B6:B14)</f>
-        <v>1.69325</v>
+        <v>1.4255</v>
       </c>
       <c r="C15" s="30" t="n">
         <f aca="false">SUM(C6:C14)</f>
-        <v>9.897</v>
+        <v>8.2905</v>
       </c>
       <c r="D15" s="30" t="n">
         <f aca="false">SUM(D6:D14)</f>
-        <v>9.393</v>
+        <v>7.7865</v>
       </c>
       <c r="E15" s="30" t="n">
         <f aca="false">SUM(E6:E14)</f>
-        <v>18.66</v>
+        <v>15.447</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3310,19 +3310,19 @@
       </c>
       <c r="B16" s="30" t="n">
         <f aca="false">IF(B5=0,0,B15/B5)</f>
-        <v>1.69325</v>
+        <v>1.4255</v>
       </c>
       <c r="C16" s="30" t="n">
         <f aca="false">IF(C5=0,0,C15/C5)</f>
-        <v>1.6495</v>
+        <v>1.38175</v>
       </c>
       <c r="D16" s="30" t="n">
         <f aca="false">IF(D5=0,0,D15/D5)</f>
-        <v>1.5655</v>
+        <v>1.29775</v>
       </c>
       <c r="E16" s="30" t="n">
         <f aca="false">IF(E5=0,0,E15/E5)</f>
-        <v>1.555</v>
+        <v>1.28725</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3378,19 +3378,19 @@
       </c>
       <c r="B21" s="13" t="n">
         <f aca="false">B20-B15</f>
-        <v>2.96776694915254</v>
+        <v>3.23551694915254</v>
       </c>
       <c r="C21" s="13" t="n">
         <f aca="false">C20-C15</f>
-        <v>12.1368983050847</v>
+        <v>13.7433983050847</v>
       </c>
       <c r="D21" s="13" t="n">
         <f aca="false">D20-D15</f>
-        <v>12.6408983050847</v>
+        <v>14.2473983050847</v>
       </c>
       <c r="E21" s="13" t="n">
         <f aca="false">E20-E15</f>
-        <v>22.0179661016949</v>
+        <v>25.2309661016949</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3399,19 +3399,19 @@
       </c>
       <c r="B22" s="12" t="n">
         <f aca="false">IF(B20=0,0,B21/B20)</f>
-        <v>0.636720909090909</v>
+        <v>0.694165454545455</v>
       </c>
       <c r="C22" s="12" t="n">
         <f aca="false">IF(C20=0,0,C21/C20)</f>
-        <v>0.550828461538462</v>
+        <v>0.623738846153846</v>
       </c>
       <c r="D22" s="12" t="n">
         <f aca="false">IF(D20=0,0,D21/D20)</f>
-        <v>0.573702307692308</v>
+        <v>0.646612692307692</v>
       </c>
       <c r="E22" s="12" t="n">
         <f aca="false">IF(E20=0,0,E21/E20)</f>
-        <v>0.541275</v>
+        <v>0.62026125</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3467,19 +3467,19 @@
       </c>
       <c r="B27" s="13" t="n">
         <f aca="false">B26-B15</f>
-        <v>1.69658050847458</v>
+        <v>1.96433050847458</v>
       </c>
       <c r="C27" s="13" t="n">
         <f aca="false">C26-C15</f>
-        <v>11.2046949152542</v>
+        <v>12.8111949152542</v>
       </c>
       <c r="D27" s="13" t="n">
         <f aca="false">D26-D15</f>
-        <v>11.7086949152542</v>
+        <v>13.3151949152542</v>
       </c>
       <c r="E27" s="13" t="n">
         <f aca="false">E26-E15</f>
-        <v>21.0857627118644</v>
+        <v>24.2987627118644</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3488,19 +3488,19 @@
       </c>
       <c r="B28" s="12" t="n">
         <f aca="false">IF(B26=0,0,B27/B26)</f>
-        <v>0.50049125</v>
+        <v>0.5794775</v>
       </c>
       <c r="C28" s="12" t="n">
         <f aca="false">IF(C26=0,0,C27/C26)</f>
-        <v>0.530985542168675</v>
+        <v>0.60711686746988</v>
       </c>
       <c r="D28" s="12" t="n">
         <f aca="false">IF(D26=0,0,D27/D26)</f>
-        <v>0.554869879518072</v>
+        <v>0.631001204819277</v>
       </c>
       <c r="E28" s="12" t="n">
         <f aca="false">IF(E26=0,0,E27/E26)</f>
-        <v>0.530515991471215</v>
+        <v>0.611354797441365</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3614,7 +3614,7 @@
       </c>
       <c r="D5" s="8" t="n">
         <f aca="false">Mensual!$N$14</f>
-        <v>19565</v>
+        <v>22625</v>
       </c>
       <c r="E5" s="7" t="n">
         <f aca="false">Supuestos!B48</f>
@@ -3622,11 +3622,11 @@
       </c>
       <c r="F5" s="15" t="n">
         <f aca="false">D5*E5</f>
-        <v>11739</v>
+        <v>13575</v>
       </c>
       <c r="G5" s="15" t="n">
         <f aca="false">IF(C5=0,0,F5/C5)</f>
-        <v>11739</v>
+        <v>13575</v>
       </c>
       <c r="H5" s="6" t="n">
         <f aca="false">Supuestos!B40</f>
@@ -3634,19 +3634,19 @@
       </c>
       <c r="I5" s="16" t="n">
         <f aca="false">G5*H5</f>
-        <v>64564.5</v>
+        <v>74662.5</v>
       </c>
       <c r="J5" s="16" t="n">
         <f aca="false">I5/(1+Supuestos!$B$26)</f>
-        <v>54715.6779661017</v>
+        <v>63273.3050847458</v>
       </c>
       <c r="K5" s="6" t="n">
         <f aca="false">Costeo!B15</f>
-        <v>1.69325</v>
+        <v>1.4255</v>
       </c>
       <c r="L5" s="6" t="n">
         <f aca="false">Costeo!B15</f>
-        <v>1.69325</v>
+        <v>1.4255</v>
       </c>
       <c r="M5" s="13" t="n">
         <f aca="false">IF(H5=0,0,C5*Supuestos!$B$32+H5*Supuestos!$B$27*Supuestos!$C$32+H5/(1+Supuestos!$B$26)*Supuestos!$B$28)</f>
@@ -3654,27 +3654,27 @@
       </c>
       <c r="N5" s="13" t="n">
         <f aca="false">IF(H5=0,0,H5/(1+Supuestos!$B$26)-K5-M5)</f>
-        <v>2.48615677966102</v>
+        <v>2.75390677966102</v>
       </c>
       <c r="O5" s="13" t="n">
         <f aca="false">IF(H5=0,0,H5/(1+Supuestos!$B$26)-L5-M5)</f>
-        <v>2.48615677966102</v>
+        <v>2.75390677966102</v>
       </c>
       <c r="P5" s="16" t="n">
         <f aca="false">G5*N5</f>
-        <v>29184.9944364407</v>
+        <v>37384.2845338983</v>
       </c>
       <c r="Q5" s="16" t="n">
         <f aca="false">G5*O5</f>
-        <v>29184.9944364407</v>
+        <v>37384.2845338983</v>
       </c>
       <c r="R5" s="12" t="n">
         <f aca="false">IF(H5=0,0,N5/(H5/(1+Supuestos!$B$26)))</f>
-        <v>0.533393636363636</v>
+        <v>0.590838181818182</v>
       </c>
       <c r="S5" s="12" t="n">
         <f aca="false">IF(H5=0,0,O5/(H5/(1+Supuestos!$B$26)))</f>
-        <v>0.533393636363636</v>
+        <v>0.590838181818182</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3690,7 +3690,7 @@
       </c>
       <c r="D6" s="8" t="n">
         <f aca="false">Mensual!$N$14</f>
-        <v>19565</v>
+        <v>22625</v>
       </c>
       <c r="E6" s="7" t="n">
         <f aca="false">Supuestos!C48</f>
@@ -3698,11 +3698,11 @@
       </c>
       <c r="F6" s="15" t="n">
         <f aca="false">D6*E6</f>
-        <v>6847.75</v>
+        <v>7918.75</v>
       </c>
       <c r="G6" s="15" t="n">
         <f aca="false">IF(C6=0,0,F6/C6)</f>
-        <v>1141.29166666667</v>
+        <v>1319.79166666667</v>
       </c>
       <c r="H6" s="6" t="n">
         <f aca="false">Supuestos!C40</f>
@@ -3710,19 +3710,19 @@
       </c>
       <c r="I6" s="16" t="n">
         <f aca="false">G6*H6</f>
-        <v>29673.5833333333</v>
+        <v>34314.5833333333</v>
       </c>
       <c r="J6" s="16" t="n">
         <f aca="false">I6/(1+Supuestos!$B$26)</f>
-        <v>25147.104519774</v>
+        <v>29080.1553672316</v>
       </c>
       <c r="K6" s="6" t="n">
         <f aca="false">Costeo!C15</f>
-        <v>9.897</v>
+        <v>8.2905</v>
       </c>
       <c r="L6" s="6" t="n">
         <f aca="false">Costeo!D15</f>
-        <v>9.393</v>
+        <v>7.7865</v>
       </c>
       <c r="M6" s="13" t="n">
         <f aca="false">IF(H6=0,0,C6*Supuestos!$B$32+H6*Supuestos!$B$27*Supuestos!$C$32+H6/(1+Supuestos!$B$26)*Supuestos!$B$28)</f>
@@ -3730,27 +3730,27 @@
       </c>
       <c r="N6" s="13" t="n">
         <f aca="false">IF(H6=0,0,H6/(1+Supuestos!$B$26)-K6-M6)</f>
-        <v>9.5165593220339</v>
+        <v>11.1230593220339</v>
       </c>
       <c r="O6" s="13" t="n">
         <f aca="false">IF(H6=0,0,H6/(1+Supuestos!$B$26)-L6-M6)</f>
-        <v>10.0205593220339</v>
+        <v>11.6270593220339</v>
       </c>
       <c r="P6" s="16" t="n">
         <f aca="false">G6*N6</f>
-        <v>10861.1698495763</v>
+        <v>14680.1210010593</v>
       </c>
       <c r="Q6" s="16" t="n">
         <f aca="false">G6*O6</f>
-        <v>11436.3808495763</v>
+        <v>15345.2960010593</v>
       </c>
       <c r="R6" s="12" t="n">
         <f aca="false">IF(H6=0,0,N6/(H6/(1+Supuestos!$B$26)))</f>
-        <v>0.431905384615385</v>
+        <v>0.504815769230769</v>
       </c>
       <c r="S6" s="12" t="n">
         <f aca="false">IF(H6=0,0,O6/(H6/(1+Supuestos!$B$26)))</f>
-        <v>0.454779230769231</v>
+        <v>0.527689615384615</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3766,7 +3766,7 @@
       </c>
       <c r="D7" s="8" t="n">
         <f aca="false">Mensual!$N$14</f>
-        <v>19565</v>
+        <v>22625</v>
       </c>
       <c r="E7" s="7" t="n">
         <f aca="false">Supuestos!D48</f>
@@ -3774,11 +3774,11 @@
       </c>
       <c r="F7" s="15" t="n">
         <f aca="false">D7*E7</f>
-        <v>978.25</v>
+        <v>1131.25</v>
       </c>
       <c r="G7" s="15" t="n">
         <f aca="false">IF(C7=0,0,F7/C7)</f>
-        <v>81.5208333333333</v>
+        <v>94.2708333333333</v>
       </c>
       <c r="H7" s="6" t="n">
         <f aca="false">Supuestos!D40</f>
@@ -3786,19 +3786,19 @@
       </c>
       <c r="I7" s="16" t="n">
         <f aca="false">G7*H7</f>
-        <v>3913</v>
+        <v>4525</v>
       </c>
       <c r="J7" s="16" t="n">
         <f aca="false">I7/(1+Supuestos!$B$26)</f>
-        <v>3316.10169491525</v>
+        <v>3834.74576271186</v>
       </c>
       <c r="K7" s="6" t="n">
         <f aca="false">Costeo!E15</f>
-        <v>18.66</v>
+        <v>15.447</v>
       </c>
       <c r="L7" s="6" t="n">
         <f aca="false">Costeo!E15</f>
-        <v>18.66</v>
+        <v>15.447</v>
       </c>
       <c r="M7" s="13" t="n">
         <f aca="false">IF(H7=0,0,C7*Supuestos!$B$32+H7*Supuestos!$B$27*Supuestos!$C$32+H7/(1+Supuestos!$B$26)*Supuestos!$B$28)</f>
@@ -3806,27 +3806,27 @@
       </c>
       <c r="N7" s="13" t="n">
         <f aca="false">IF(H7=0,0,H7/(1+Supuestos!$B$26)-K7-M7)</f>
-        <v>16.931186440678</v>
+        <v>20.144186440678</v>
       </c>
       <c r="O7" s="13" t="n">
         <f aca="false">IF(H7=0,0,H7/(1+Supuestos!$B$26)-L7-M7)</f>
-        <v>16.931186440678</v>
+        <v>20.144186440678</v>
       </c>
       <c r="P7" s="16" t="n">
         <f aca="false">G7*N7</f>
-        <v>1380.2444279661</v>
+        <v>1899.00924258475</v>
       </c>
       <c r="Q7" s="16" t="n">
         <f aca="false">G7*O7</f>
-        <v>1380.2444279661</v>
+        <v>1899.00924258475</v>
       </c>
       <c r="R7" s="12" t="n">
         <f aca="false">IF(H7=0,0,N7/(H7/(1+Supuestos!$B$26)))</f>
-        <v>0.416225</v>
+        <v>0.49521125</v>
       </c>
       <c r="S7" s="12" t="n">
         <f aca="false">IF(H7=0,0,O7/(H7/(1+Supuestos!$B$26)))</f>
-        <v>0.416225</v>
+        <v>0.49521125</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3870,11 +3870,11 @@
       </c>
       <c r="K8" s="6" t="n">
         <f aca="false">Costeo!B15</f>
-        <v>1.69325</v>
+        <v>1.4255</v>
       </c>
       <c r="L8" s="6" t="n">
         <f aca="false">Costeo!B15</f>
-        <v>1.69325</v>
+        <v>1.4255</v>
       </c>
       <c r="M8" s="13" t="n">
         <f aca="false">IF(H8=0,0,C8*Supuestos!$B$33+H8*Supuestos!$B$27*Supuestos!$C$33+H8/(1+Supuestos!$B$26)*Supuestos!$B$28)</f>
@@ -3882,27 +3882,27 @@
       </c>
       <c r="N8" s="13" t="n">
         <f aca="false">IF(H8=0,0,H8/(1+Supuestos!$B$26)-K8-M8)</f>
-        <v>2.48615677966102</v>
+        <v>2.75390677966102</v>
       </c>
       <c r="O8" s="13" t="n">
         <f aca="false">IF(H8=0,0,H8/(1+Supuestos!$B$26)-L8-M8)</f>
-        <v>2.48615677966102</v>
+        <v>2.75390677966102</v>
       </c>
       <c r="P8" s="16" t="n">
         <f aca="false">G8*N8</f>
-        <v>14096.508940678</v>
+        <v>15614.651440678</v>
       </c>
       <c r="Q8" s="16" t="n">
         <f aca="false">G8*O8</f>
-        <v>14096.508940678</v>
+        <v>15614.651440678</v>
       </c>
       <c r="R8" s="12" t="n">
         <f aca="false">IF(H8=0,0,N8/(H8/(1+Supuestos!$B$26)))</f>
-        <v>0.533393636363636</v>
+        <v>0.590838181818182</v>
       </c>
       <c r="S8" s="12" t="n">
         <f aca="false">IF(H8=0,0,O8/(H8/(1+Supuestos!$B$26)))</f>
-        <v>0.533393636363636</v>
+        <v>0.590838181818182</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3946,11 +3946,11 @@
       </c>
       <c r="K9" s="6" t="n">
         <f aca="false">Costeo!C15</f>
-        <v>9.897</v>
+        <v>8.2905</v>
       </c>
       <c r="L9" s="6" t="n">
         <f aca="false">Costeo!D15</f>
-        <v>9.393</v>
+        <v>7.7865</v>
       </c>
       <c r="M9" s="13" t="n">
         <f aca="false">IF(H9=0,0,C9*Supuestos!$B$33+H9*Supuestos!$B$27*Supuestos!$C$33+H9/(1+Supuestos!$B$26)*Supuestos!$B$28)</f>
@@ -3958,27 +3958,27 @@
       </c>
       <c r="N9" s="13" t="n">
         <f aca="false">IF(H9=0,0,H9/(1+Supuestos!$B$26)-K9-M9)</f>
-        <v>9.5165593220339</v>
+        <v>11.1230593220339</v>
       </c>
       <c r="O9" s="13" t="n">
         <f aca="false">IF(H9=0,0,H9/(1+Supuestos!$B$26)-L9-M9)</f>
-        <v>10.0205593220339</v>
+        <v>11.6270593220339</v>
       </c>
       <c r="P9" s="16" t="n">
         <f aca="false">G9*N9</f>
-        <v>3854.20652542373</v>
+        <v>4504.83902542373</v>
       </c>
       <c r="Q9" s="16" t="n">
         <f aca="false">G9*O9</f>
-        <v>4058.32652542373</v>
+        <v>4708.95902542373</v>
       </c>
       <c r="R9" s="12" t="n">
         <f aca="false">IF(H9=0,0,N9/(H9/(1+Supuestos!$B$26)))</f>
-        <v>0.431905384615385</v>
+        <v>0.504815769230769</v>
       </c>
       <c r="S9" s="12" t="n">
         <f aca="false">IF(H9=0,0,O9/(H9/(1+Supuestos!$B$26)))</f>
-        <v>0.454779230769231</v>
+        <v>0.527689615384615</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4022,11 +4022,11 @@
       </c>
       <c r="K10" s="6" t="n">
         <f aca="false">Costeo!E15</f>
-        <v>18.66</v>
+        <v>15.447</v>
       </c>
       <c r="L10" s="6" t="n">
         <f aca="false">Costeo!E15</f>
-        <v>18.66</v>
+        <v>15.447</v>
       </c>
       <c r="M10" s="13" t="n">
         <f aca="false">IF(H10=0,0,C10*Supuestos!$B$33+H10*Supuestos!$B$27*Supuestos!$C$33+H10/(1+Supuestos!$B$26)*Supuestos!$B$28)</f>
@@ -4034,11 +4034,11 @@
       </c>
       <c r="N10" s="13" t="n">
         <f aca="false">IF(H10=0,0,H10/(1+Supuestos!$B$26)-K10-M10)</f>
-        <v>16.931186440678</v>
+        <v>20.144186440678</v>
       </c>
       <c r="O10" s="13" t="n">
         <f aca="false">IF(H10=0,0,H10/(1+Supuestos!$B$26)-L10-M10)</f>
-        <v>16.931186440678</v>
+        <v>20.144186440678</v>
       </c>
       <c r="P10" s="16" t="n">
         <f aca="false">G10*N10</f>
@@ -4050,11 +4050,11 @@
       </c>
       <c r="R10" s="12" t="n">
         <f aca="false">IF(H10=0,0,N10/(H10/(1+Supuestos!$B$26)))</f>
-        <v>0.416225</v>
+        <v>0.49521125</v>
       </c>
       <c r="S10" s="12" t="n">
         <f aca="false">IF(H10=0,0,O10/(H10/(1+Supuestos!$B$26)))</f>
-        <v>0.416225</v>
+        <v>0.49521125</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4070,7 +4070,7 @@
       </c>
       <c r="D11" s="8" t="n">
         <f aca="false">Mensual!$N$16</f>
-        <v>8773</v>
+        <v>9176</v>
       </c>
       <c r="E11" s="7" t="n">
         <f aca="false">Supuestos!B50</f>
@@ -4078,11 +4078,11 @@
       </c>
       <c r="F11" s="15" t="n">
         <f aca="false">D11*E11</f>
-        <v>877.3</v>
+        <v>917.6</v>
       </c>
       <c r="G11" s="15" t="n">
         <f aca="false">IF(C11=0,0,F11/C11)</f>
-        <v>877.3</v>
+        <v>917.6</v>
       </c>
       <c r="H11" s="6" t="n">
         <f aca="false">Supuestos!B42</f>
@@ -4090,19 +4090,19 @@
       </c>
       <c r="I11" s="16" t="n">
         <f aca="false">G11*H11</f>
-        <v>3509.2</v>
+        <v>3670.4</v>
       </c>
       <c r="J11" s="16" t="n">
         <f aca="false">I11/(1+Supuestos!$B$26)</f>
-        <v>2973.89830508475</v>
+        <v>3110.50847457627</v>
       </c>
       <c r="K11" s="6" t="n">
         <f aca="false">Costeo!B15</f>
-        <v>1.69325</v>
+        <v>1.4255</v>
       </c>
       <c r="L11" s="6" t="n">
         <f aca="false">Costeo!B15</f>
-        <v>1.69325</v>
+        <v>1.4255</v>
       </c>
       <c r="M11" s="13" t="n">
         <f aca="false">IF(H11=0,0,C11*Supuestos!$B$34+H11*Supuestos!$B$27*Supuestos!$C$34+H11/(1+Supuestos!$B$26)*Supuestos!$B$28)</f>
@@ -4110,27 +4110,27 @@
       </c>
       <c r="N11" s="13" t="n">
         <f aca="false">IF(H11=0,0,H11/(1+Supuestos!$B$26)-K11-M11)</f>
-        <v>0.742682203389831</v>
+        <v>1.01043220338983</v>
       </c>
       <c r="O11" s="13" t="n">
         <f aca="false">IF(H11=0,0,H11/(1+Supuestos!$B$26)-L11-M11)</f>
-        <v>0.742682203389831</v>
+        <v>1.01043220338983</v>
       </c>
       <c r="P11" s="16" t="n">
         <f aca="false">G11*N11</f>
-        <v>651.555097033899</v>
+        <v>927.172589830509</v>
       </c>
       <c r="Q11" s="16" t="n">
         <f aca="false">G11*O11</f>
-        <v>651.555097033899</v>
+        <v>927.172589830509</v>
       </c>
       <c r="R11" s="12" t="n">
         <f aca="false">IF(H11=0,0,N11/(H11/(1+Supuestos!$B$26)))</f>
-        <v>0.21909125</v>
+        <v>0.2980775</v>
       </c>
       <c r="S11" s="12" t="n">
         <f aca="false">IF(H11=0,0,O11/(H11/(1+Supuestos!$B$26)))</f>
-        <v>0.21909125</v>
+        <v>0.2980775</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4146,7 +4146,7 @@
       </c>
       <c r="D12" s="8" t="n">
         <f aca="false">Mensual!$N$16</f>
-        <v>8773</v>
+        <v>9176</v>
       </c>
       <c r="E12" s="7" t="n">
         <f aca="false">Supuestos!C50</f>
@@ -4154,11 +4154,11 @@
       </c>
       <c r="F12" s="15" t="n">
         <f aca="false">D12*E12</f>
-        <v>5263.8</v>
+        <v>5505.6</v>
       </c>
       <c r="G12" s="15" t="n">
         <f aca="false">IF(C12=0,0,F12/C12)</f>
-        <v>877.3</v>
+        <v>917.6</v>
       </c>
       <c r="H12" s="6" t="n">
         <f aca="false">Supuestos!C42</f>
@@ -4166,19 +4166,19 @@
       </c>
       <c r="I12" s="16" t="n">
         <f aca="false">G12*H12</f>
-        <v>21844.77</v>
+        <v>22848.24</v>
       </c>
       <c r="J12" s="16" t="n">
         <f aca="false">I12/(1+Supuestos!$B$26)</f>
-        <v>18512.5169491525</v>
+        <v>19362.9152542373</v>
       </c>
       <c r="K12" s="6" t="n">
         <f aca="false">Costeo!C15</f>
-        <v>9.897</v>
+        <v>8.2905</v>
       </c>
       <c r="L12" s="6" t="n">
         <f aca="false">Costeo!D15</f>
-        <v>9.393</v>
+        <v>7.7865</v>
       </c>
       <c r="M12" s="13" t="n">
         <f aca="false">IF(H12=0,0,C12*Supuestos!$B$34+H12*Supuestos!$B$27*Supuestos!$C$34+H12/(1+Supuestos!$B$26)*Supuestos!$B$28)</f>
@@ -4186,27 +4186,27 @@
       </c>
       <c r="N12" s="13" t="n">
         <f aca="false">IF(H12=0,0,H12/(1+Supuestos!$B$26)-K12-M12)</f>
-        <v>5.4466779661017</v>
+        <v>7.05317796610169</v>
       </c>
       <c r="O12" s="13" t="n">
         <f aca="false">IF(H12=0,0,H12/(1+Supuestos!$B$26)-L12-M12)</f>
-        <v>5.9506779661017</v>
+        <v>7.5571779661017</v>
       </c>
       <c r="P12" s="16" t="n">
         <f aca="false">G12*N12</f>
-        <v>4778.37057966102</v>
+        <v>6471.99610169492</v>
       </c>
       <c r="Q12" s="16" t="n">
         <f aca="false">G12*O12</f>
-        <v>5220.52977966102</v>
+        <v>6934.46650169492</v>
       </c>
       <c r="R12" s="12" t="n">
         <f aca="false">IF(H12=0,0,N12/(H12/(1+Supuestos!$B$26)))</f>
-        <v>0.258115662650603</v>
+        <v>0.334246987951807</v>
       </c>
       <c r="S12" s="12" t="n">
         <f aca="false">IF(H12=0,0,O12/(H12/(1+Supuestos!$B$26)))</f>
-        <v>0.282</v>
+        <v>0.358131325301205</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4222,7 +4222,7 @@
       </c>
       <c r="D13" s="8" t="n">
         <f aca="false">Mensual!$N$16</f>
-        <v>8773</v>
+        <v>9176</v>
       </c>
       <c r="E13" s="7" t="n">
         <f aca="false">Supuestos!D50</f>
@@ -4230,11 +4230,11 @@
       </c>
       <c r="F13" s="15" t="n">
         <f aca="false">D13*E13</f>
-        <v>2631.9</v>
+        <v>2752.8</v>
       </c>
       <c r="G13" s="15" t="n">
         <f aca="false">IF(C13=0,0,F13/C13)</f>
-        <v>219.325</v>
+        <v>229.4</v>
       </c>
       <c r="H13" s="6" t="n">
         <f aca="false">Supuestos!D42</f>
@@ -4242,19 +4242,19 @@
       </c>
       <c r="I13" s="16" t="n">
         <f aca="false">G13*H13</f>
-        <v>10286.3425</v>
+        <v>10758.86</v>
       </c>
       <c r="J13" s="16" t="n">
         <f aca="false">I13/(1+Supuestos!$B$26)</f>
-        <v>8717.23940677966</v>
+        <v>9117.67796610169</v>
       </c>
       <c r="K13" s="6" t="n">
         <f aca="false">Costeo!E15</f>
-        <v>18.66</v>
+        <v>15.447</v>
       </c>
       <c r="L13" s="6" t="n">
         <f aca="false">Costeo!E15</f>
-        <v>18.66</v>
+        <v>15.447</v>
       </c>
       <c r="M13" s="13" t="n">
         <f aca="false">IF(H13=0,0,C13*Supuestos!$B$34+H13*Supuestos!$B$27*Supuestos!$C$34+H13/(1+Supuestos!$B$26)*Supuestos!$B$28)</f>
@@ -4262,27 +4262,27 @@
       </c>
       <c r="N13" s="13" t="n">
         <f aca="false">IF(H13=0,0,H13/(1+Supuestos!$B$26)-K13-M13)</f>
-        <v>9.68130508474577</v>
+        <v>12.8943050847458</v>
       </c>
       <c r="O13" s="13" t="n">
         <f aca="false">IF(H13=0,0,H13/(1+Supuestos!$B$26)-L13-M13)</f>
-        <v>9.68130508474577</v>
+        <v>12.8943050847458</v>
       </c>
       <c r="P13" s="16" t="n">
         <f aca="false">G13*N13</f>
-        <v>2123.35223771187</v>
+        <v>2957.95358644068</v>
       </c>
       <c r="Q13" s="16" t="n">
         <f aca="false">G13*O13</f>
-        <v>2123.35223771187</v>
+        <v>2957.95358644068</v>
       </c>
       <c r="R13" s="12" t="n">
         <f aca="false">IF(H13=0,0,N13/(H13/(1+Supuestos!$B$26)))</f>
-        <v>0.243580810234542</v>
+        <v>0.324419616204691</v>
       </c>
       <c r="S13" s="12" t="n">
         <f aca="false">IF(H13=0,0,O13/(H13/(1+Supuestos!$B$26)))</f>
-        <v>0.243580810234542</v>
+        <v>0.324419616204691</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4298,7 +4298,7 @@
       </c>
       <c r="D14" s="8" t="n">
         <f aca="false">Mensual!$N$17</f>
-        <v>7065</v>
+        <v>9165</v>
       </c>
       <c r="E14" s="7" t="n">
         <f aca="false">Supuestos!B51</f>
@@ -4306,11 +4306,11 @@
       </c>
       <c r="F14" s="15" t="n">
         <f aca="false">D14*E14</f>
-        <v>7065</v>
+        <v>9165</v>
       </c>
       <c r="G14" s="15" t="n">
         <f aca="false">IF(C14=0,0,F14/C14)</f>
-        <v>7065</v>
+        <v>9165</v>
       </c>
       <c r="H14" s="6" t="n">
         <f aca="false">Supuestos!B43</f>
@@ -4318,19 +4318,19 @@
       </c>
       <c r="I14" s="16" t="n">
         <f aca="false">G14*H14</f>
-        <v>21195</v>
+        <v>27495</v>
       </c>
       <c r="J14" s="16" t="n">
         <f aca="false">I14/(1+Supuestos!$B$26)</f>
-        <v>17961.8644067797</v>
+        <v>23300.8474576271</v>
       </c>
       <c r="K14" s="6" t="n">
         <f aca="false">Costeo!B15</f>
-        <v>1.69325</v>
+        <v>1.4255</v>
       </c>
       <c r="L14" s="6" t="n">
         <f aca="false">Costeo!B15</f>
-        <v>1.69325</v>
+        <v>1.4255</v>
       </c>
       <c r="M14" s="13" t="n">
         <f aca="false">IF(H14=0,0,C14*Supuestos!$B$35+H14*Supuestos!$B$27*Supuestos!$C$35+H14/(1+Supuestos!$B$26)*Supuestos!$B$28)</f>
@@ -4338,27 +4338,27 @@
       </c>
       <c r="N14" s="13" t="n">
         <f aca="false">IF(H14=0,0,H14/(1+Supuestos!$B$26)-K14-M14)</f>
-        <v>0.723699152542373</v>
+        <v>0.991449152542373</v>
       </c>
       <c r="O14" s="13" t="n">
         <f aca="false">IF(H14=0,0,H14/(1+Supuestos!$B$26)-L14-M14)</f>
-        <v>0.723699152542373</v>
+        <v>0.991449152542373</v>
       </c>
       <c r="P14" s="16" t="n">
         <f aca="false">G14*N14</f>
-        <v>5112.93451271187</v>
+        <v>9086.63148305085</v>
       </c>
       <c r="Q14" s="16" t="n">
         <f aca="false">G14*O14</f>
-        <v>5112.93451271187</v>
+        <v>9086.63148305085</v>
       </c>
       <c r="R14" s="12" t="n">
         <f aca="false">IF(H14=0,0,N14/(H14/(1+Supuestos!$B$26)))</f>
-        <v>0.284655</v>
+        <v>0.38997</v>
       </c>
       <c r="S14" s="12" t="n">
         <f aca="false">IF(H14=0,0,O14/(H14/(1+Supuestos!$B$26)))</f>
-        <v>0.284655</v>
+        <v>0.38997</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4374,7 +4374,7 @@
       </c>
       <c r="D15" s="8" t="n">
         <f aca="false">Mensual!$N$17</f>
-        <v>7065</v>
+        <v>9165</v>
       </c>
       <c r="E15" s="7" t="n">
         <f aca="false">Supuestos!C51</f>
@@ -4402,11 +4402,11 @@
       </c>
       <c r="K15" s="6" t="n">
         <f aca="false">Costeo!C15</f>
-        <v>9.897</v>
+        <v>8.2905</v>
       </c>
       <c r="L15" s="6" t="n">
         <f aca="false">Costeo!D15</f>
-        <v>9.393</v>
+        <v>7.7865</v>
       </c>
       <c r="M15" s="13" t="n">
         <f aca="false">IF(H15=0,0,C15*Supuestos!$B$35+H15*Supuestos!$B$27*Supuestos!$C$35+H15/(1+Supuestos!$B$26)*Supuestos!$B$28)</f>
@@ -4450,7 +4450,7 @@
       </c>
       <c r="D16" s="8" t="n">
         <f aca="false">Mensual!$N$17</f>
-        <v>7065</v>
+        <v>9165</v>
       </c>
       <c r="E16" s="7" t="n">
         <f aca="false">Supuestos!D51</f>
@@ -4478,11 +4478,11 @@
       </c>
       <c r="K16" s="6" t="n">
         <f aca="false">Costeo!E15</f>
-        <v>18.66</v>
+        <v>15.447</v>
       </c>
       <c r="L16" s="6" t="n">
         <f aca="false">Costeo!E15</f>
-        <v>18.66</v>
+        <v>15.447</v>
       </c>
       <c r="M16" s="13" t="n">
         <f aca="false">IF(H16=0,0,C16*Supuestos!$B$35+H16*Supuestos!$B$27*Supuestos!$C$35+H16/(1+Supuestos!$B$26)*Supuestos!$B$28)</f>
@@ -4554,11 +4554,11 @@
       </c>
       <c r="K17" s="6" t="n">
         <f aca="false">Costeo!B15</f>
-        <v>1.69325</v>
+        <v>1.4255</v>
       </c>
       <c r="L17" s="6" t="n">
         <f aca="false">Costeo!B15</f>
-        <v>1.69325</v>
+        <v>1.4255</v>
       </c>
       <c r="M17" s="13" t="n">
         <f aca="false">IF(H17=0,0,C17*Supuestos!$B$36+H17*Supuestos!$B$27*Supuestos!$C$36+H17/(1+Supuestos!$B$26)*Supuestos!$B$28)</f>
@@ -4630,11 +4630,11 @@
       </c>
       <c r="K18" s="6" t="n">
         <f aca="false">Costeo!C15</f>
-        <v>9.897</v>
+        <v>8.2905</v>
       </c>
       <c r="L18" s="6" t="n">
         <f aca="false">Costeo!D15</f>
-        <v>9.393</v>
+        <v>7.7865</v>
       </c>
       <c r="M18" s="13" t="n">
         <f aca="false">IF(H18=0,0,C18*Supuestos!$B$36+H18*Supuestos!$B$27*Supuestos!$C$36+H18/(1+Supuestos!$B$26)*Supuestos!$B$28)</f>
@@ -4642,27 +4642,27 @@
       </c>
       <c r="N18" s="13" t="n">
         <f aca="false">IF(H18=0,0,H18/(1+Supuestos!$B$26)-K18-M18)</f>
-        <v>3.75096610169492</v>
+        <v>5.35746610169491</v>
       </c>
       <c r="O18" s="13" t="n">
         <f aca="false">IF(H18=0,0,H18/(1+Supuestos!$B$26)-L18-M18)</f>
-        <v>4.25496610169492</v>
+        <v>5.86146610169492</v>
       </c>
       <c r="P18" s="16" t="n">
         <f aca="false">G18*N18</f>
-        <v>2325.59898305085</v>
+        <v>3321.62898305085</v>
       </c>
       <c r="Q18" s="16" t="n">
         <f aca="false">G18*O18</f>
-        <v>2638.07898305085</v>
+        <v>3634.10898305085</v>
       </c>
       <c r="R18" s="12" t="n">
         <f aca="false">IF(H18=0,0,N18/(H18/(1+Supuestos!$B$26)))</f>
-        <v>0.255256055363322</v>
+        <v>0.364579584775086</v>
       </c>
       <c r="S18" s="12" t="n">
         <f aca="false">IF(H18=0,0,O18/(H18/(1+Supuestos!$B$26)))</f>
-        <v>0.289553633217993</v>
+        <v>0.398877162629758</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4706,11 +4706,11 @@
       </c>
       <c r="K19" s="6" t="n">
         <f aca="false">Costeo!E15</f>
-        <v>18.66</v>
+        <v>15.447</v>
       </c>
       <c r="L19" s="6" t="n">
         <f aca="false">Costeo!E15</f>
-        <v>18.66</v>
+        <v>15.447</v>
       </c>
       <c r="M19" s="13" t="n">
         <f aca="false">IF(H19=0,0,C19*Supuestos!$B$36+H19*Supuestos!$B$27*Supuestos!$C$36+H19/(1+Supuestos!$B$26)*Supuestos!$B$28)</f>
@@ -4747,23 +4747,23 @@
       </c>
       <c r="F20" s="31" t="n">
         <f aca="false">SUM(F5:F19)</f>
-        <v>47223</v>
+        <v>52786</v>
       </c>
       <c r="I20" s="11" t="n">
         <f aca="false">SUM(I5:I19)</f>
-        <v>207452.195833333</v>
+        <v>230740.383333333</v>
       </c>
       <c r="J20" s="11" t="n">
         <f aca="false">SUM(J5:J19)</f>
-        <v>175806.945621469</v>
+        <v>195542.697740113</v>
       </c>
       <c r="P20" s="11" t="n">
         <f aca="false">SUM(P5:P19)</f>
-        <v>74368.9355902542</v>
+        <v>96848.2879877119</v>
       </c>
       <c r="Q20" s="11" t="n">
         <f aca="false">SUM(Q5:Q19)</f>
-        <v>75902.9057902542</v>
+        <v>98492.5333877119</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4810,27 +4810,27 @@
       </c>
       <c r="B25" s="15" t="n">
         <f aca="false">SUMIF($A$5:$A$19,A25,$F$5:$F$19)</f>
-        <v>19565</v>
+        <v>22625</v>
       </c>
       <c r="C25" s="16" t="n">
         <f aca="false">SUMIF($A$5:$A$19,A25,$P$5:$P$19)</f>
-        <v>41426.4087139831</v>
+        <v>53963.4147775424</v>
       </c>
       <c r="D25" s="16" t="n">
         <f aca="false">SUMIF($A$5:$A$19,A25,$Q$5:$Q$19)</f>
-        <v>42001.6197139831</v>
+        <v>54628.5897775424</v>
       </c>
       <c r="E25" s="16" t="n">
         <f aca="false">SUMIF($A$5:$A$19,A25,$I$5:$I$19)</f>
-        <v>98151.0833333333</v>
+        <v>113502.083333333</v>
       </c>
       <c r="F25" s="13" t="n">
         <f aca="false">IF(B25=0,0,C25/B25)</f>
-        <v>2.11737330508475</v>
+        <v>2.38512330508475</v>
       </c>
       <c r="G25" s="13" t="n">
         <f aca="false">IF(B25=0,0,D25/B25)</f>
-        <v>2.14677330508475</v>
+        <v>2.41452330508475</v>
       </c>
       <c r="H25" s="13" t="n">
         <f aca="false">IF(B25=0,0,E25/B25)</f>
@@ -4847,11 +4847,11 @@
       </c>
       <c r="C26" s="16" t="n">
         <f aca="false">SUMIF($A$5:$A$19,A26,$P$5:$P$19)</f>
-        <v>17950.7154661017</v>
+        <v>20119.4904661017</v>
       </c>
       <c r="D26" s="16" t="n">
         <f aca="false">SUMIF($A$5:$A$19,A26,$Q$5:$Q$19)</f>
-        <v>18154.8354661017</v>
+        <v>20323.6104661017</v>
       </c>
       <c r="E26" s="16" t="n">
         <f aca="false">SUMIF($A$5:$A$19,A26,$I$5:$I$19)</f>
@@ -4859,11 +4859,11 @@
       </c>
       <c r="F26" s="13" t="n">
         <f aca="false">IF(B26=0,0,C26/B26)</f>
-        <v>2.21613771186441</v>
+        <v>2.48388771186441</v>
       </c>
       <c r="G26" s="13" t="n">
         <f aca="false">IF(B26=0,0,D26/B26)</f>
-        <v>2.24133771186441</v>
+        <v>2.50908771186441</v>
       </c>
       <c r="H26" s="13" t="n">
         <f aca="false">IF(B26=0,0,E26/B26)</f>
@@ -4876,27 +4876,27 @@
       </c>
       <c r="B27" s="15" t="n">
         <f aca="false">SUMIF($A$5:$A$19,A27,$F$5:$F$19)</f>
-        <v>8773</v>
+        <v>9176</v>
       </c>
       <c r="C27" s="16" t="n">
         <f aca="false">SUMIF($A$5:$A$19,A27,$P$5:$P$19)</f>
-        <v>7553.27791440678</v>
+        <v>10357.1222779661</v>
       </c>
       <c r="D27" s="16" t="n">
         <f aca="false">SUMIF($A$5:$A$19,A27,$Q$5:$Q$19)</f>
-        <v>7995.43711440678</v>
+        <v>10819.5926779661</v>
       </c>
       <c r="E27" s="16" t="n">
         <f aca="false">SUMIF($A$5:$A$19,A27,$I$5:$I$19)</f>
-        <v>35640.3125</v>
+        <v>37277.5</v>
       </c>
       <c r="F27" s="13" t="n">
         <f aca="false">IF(B27=0,0,C27/B27)</f>
-        <v>0.860968644067797</v>
+        <v>1.1287186440678</v>
       </c>
       <c r="G27" s="13" t="n">
         <f aca="false">IF(B27=0,0,D27/B27)</f>
-        <v>0.911368644067797</v>
+        <v>1.1791186440678</v>
       </c>
       <c r="H27" s="13" t="n">
         <f aca="false">IF(B27=0,0,E27/B27)</f>
@@ -4909,27 +4909,27 @@
       </c>
       <c r="B28" s="15" t="n">
         <f aca="false">SUMIF($A$5:$A$19,A28,$F$5:$F$19)</f>
-        <v>7065</v>
+        <v>9165</v>
       </c>
       <c r="C28" s="16" t="n">
         <f aca="false">SUMIF($A$5:$A$19,A28,$P$5:$P$19)</f>
-        <v>5112.93451271187</v>
+        <v>9086.63148305085</v>
       </c>
       <c r="D28" s="16" t="n">
         <f aca="false">SUMIF($A$5:$A$19,A28,$Q$5:$Q$19)</f>
-        <v>5112.93451271187</v>
+        <v>9086.63148305085</v>
       </c>
       <c r="E28" s="16" t="n">
         <f aca="false">SUMIF($A$5:$A$19,A28,$I$5:$I$19)</f>
-        <v>21195</v>
+        <v>27495</v>
       </c>
       <c r="F28" s="13" t="n">
         <f aca="false">IF(B28=0,0,C28/B28)</f>
-        <v>0.723699152542373</v>
+        <v>0.991449152542373</v>
       </c>
       <c r="G28" s="13" t="n">
         <f aca="false">IF(B28=0,0,D28/B28)</f>
-        <v>0.723699152542373</v>
+        <v>0.991449152542373</v>
       </c>
       <c r="H28" s="13" t="n">
         <f aca="false">IF(B28=0,0,E28/B28)</f>
@@ -4946,11 +4946,11 @@
       </c>
       <c r="C29" s="16" t="n">
         <f aca="false">SUMIF($A$5:$A$19,A29,$P$5:$P$19)</f>
-        <v>2325.59898305085</v>
+        <v>3321.62898305085</v>
       </c>
       <c r="D29" s="16" t="n">
         <f aca="false">SUMIF($A$5:$A$19,A29,$Q$5:$Q$19)</f>
-        <v>2638.07898305085</v>
+        <v>3634.10898305085</v>
       </c>
       <c r="E29" s="16" t="n">
         <f aca="false">SUMIF($A$5:$A$19,A29,$I$5:$I$19)</f>
@@ -4958,11 +4958,11 @@
       </c>
       <c r="F29" s="13" t="n">
         <f aca="false">IF(B29=0,0,C29/B29)</f>
-        <v>0.625161016949153</v>
+        <v>0.892911016949152</v>
       </c>
       <c r="G29" s="13" t="n">
         <f aca="false">IF(B29=0,0,D29/B29)</f>
-        <v>0.709161016949153</v>
+        <v>0.976911016949153</v>
       </c>
       <c r="H29" s="13" t="n">
         <f aca="false">IF(B29=0,0,E29/B29)</f>
@@ -4975,31 +4975,31 @@
       </c>
       <c r="B30" s="31" t="n">
         <f aca="false">SUM(B25:B29)</f>
-        <v>47223</v>
+        <v>52786</v>
       </c>
       <c r="C30" s="11" t="n">
         <f aca="false">SUM(C25:C29)</f>
-        <v>74368.9355902542</v>
+        <v>96848.2879877119</v>
       </c>
       <c r="D30" s="11" t="n">
         <f aca="false">SUM(D25:D29)</f>
-        <v>75902.9057902542</v>
+        <v>98492.5333877119</v>
       </c>
       <c r="E30" s="11" t="n">
         <f aca="false">SUM(E25:E29)</f>
-        <v>207452.195833333</v>
+        <v>230740.383333333</v>
       </c>
       <c r="F30" s="30" t="n">
         <f aca="false">IF(B30=0,0,C30/B30)</f>
-        <v>1.57484563857134</v>
+        <v>1.83473436115091</v>
       </c>
       <c r="G30" s="30" t="n">
         <f aca="false">IF(B30=0,0,D30/B30)</f>
-        <v>1.60732917837186</v>
+        <v>1.86588363179085</v>
       </c>
       <c r="H30" s="30" t="n">
         <f aca="false">IF(B30=0,0,E30/B30)</f>
-        <v>4.3930329676923</v>
+        <v>4.37124205913184</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5044,27 +5044,27 @@
       </c>
       <c r="B34" s="15" t="n">
         <f aca="false">SUMIF($B$5:$B$19,A34,$F$5:$F$19)</f>
-        <v>25351.3</v>
+        <v>29327.6</v>
       </c>
       <c r="C34" s="15" t="n">
         <f aca="false">SUMIF($B$5:$B$19,A34,$G$5:$G$19)</f>
-        <v>25351.3</v>
+        <v>29327.6</v>
       </c>
       <c r="D34" s="16" t="n">
         <f aca="false">SUMIF($B$5:$B$19,A34,$I$5:$I$19)</f>
-        <v>120453.7</v>
+        <v>137012.9</v>
       </c>
       <c r="E34" s="16" t="n">
         <f aca="false">SUMIF($B$5:$B$19,A34,$P$5:$P$19)</f>
-        <v>49045.9929868644</v>
+        <v>63012.7400474576</v>
       </c>
       <c r="F34" s="16" t="n">
         <f aca="false">SUMIF($B$5:$B$19,A34,$Q$5:$Q$19)</f>
-        <v>49045.9929868644</v>
+        <v>63012.7400474576</v>
       </c>
       <c r="G34" s="12" t="n">
         <f aca="false">IF($F$20=0,0,B34/$F$20)</f>
-        <v>0.536842216716431</v>
+        <v>0.555594286363809</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5073,27 +5073,27 @@
       </c>
       <c r="B35" s="15" t="n">
         <f aca="false">SUMIF($B$5:$B$19,A35,$F$5:$F$19)</f>
-        <v>18261.55</v>
+        <v>19574.35</v>
       </c>
       <c r="C35" s="15" t="n">
         <f aca="false">SUMIF($B$5:$B$19,A35,$G$5:$G$19)</f>
-        <v>3043.59166666667</v>
+        <v>3262.39166666667</v>
       </c>
       <c r="D35" s="16" t="n">
         <f aca="false">SUMIF($B$5:$B$19,A35,$I$5:$I$19)</f>
-        <v>72799.1533333333</v>
+        <v>78443.6233333333</v>
       </c>
       <c r="E35" s="16" t="n">
         <f aca="false">SUMIF($B$5:$B$19,A35,$P$5:$P$19)</f>
-        <v>21819.3459377119</v>
+        <v>28978.5851112288</v>
       </c>
       <c r="F35" s="16" t="n">
         <f aca="false">SUMIF($B$5:$B$19,A35,$Q$5:$Q$19)</f>
-        <v>23353.3161377119</v>
+        <v>30622.8305112288</v>
       </c>
       <c r="G35" s="12" t="n">
         <f aca="false">IF($F$20=0,0,B35/$F$20)</f>
-        <v>0.386708807149059</v>
+        <v>0.370824650475505</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5102,27 +5102,27 @@
       </c>
       <c r="B36" s="15" t="n">
         <f aca="false">SUMIF($B$5:$B$19,A36,$F$5:$F$19)</f>
-        <v>3610.15</v>
+        <v>3884.05</v>
       </c>
       <c r="C36" s="15" t="n">
         <f aca="false">SUMIF($B$5:$B$19,A36,$G$5:$G$19)</f>
-        <v>300.845833333333</v>
+        <v>323.670833333333</v>
       </c>
       <c r="D36" s="16" t="n">
         <f aca="false">SUMIF($B$5:$B$19,A36,$I$5:$I$19)</f>
-        <v>14199.3425</v>
+        <v>15283.86</v>
       </c>
       <c r="E36" s="16" t="n">
         <f aca="false">SUMIF($B$5:$B$19,A36,$P$5:$P$19)</f>
-        <v>3503.59666567797</v>
+        <v>4856.96282902542</v>
       </c>
       <c r="F36" s="16" t="n">
         <f aca="false">SUMIF($B$5:$B$19,A36,$Q$5:$Q$19)</f>
-        <v>3503.59666567797</v>
+        <v>4856.96282902542</v>
       </c>
       <c r="G36" s="12" t="n">
         <f aca="false">IF($F$20=0,0,B36/$F$20)</f>
-        <v>0.0764489761345107</v>
+        <v>0.0735810631606865</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5164,7 +5164,7 @@
       </c>
       <c r="C40" s="15" t="n">
         <f aca="false">$F$20*B40</f>
-        <v>18889.2</v>
+        <v>21114.4</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5178,7 +5178,7 @@
       </c>
       <c r="C41" s="15" t="n">
         <f aca="false">$F$20*B41</f>
-        <v>16528.05</v>
+        <v>18475.1</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5192,7 +5192,7 @@
       </c>
       <c r="C42" s="15" t="n">
         <f aca="false">$F$20*B42</f>
-        <v>11805.75</v>
+        <v>13196.5</v>
       </c>
     </row>
   </sheetData>
@@ -5723,7 +5723,7 @@
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="58"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="2" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="2" style="0" width="12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="13"/>
   </cols>
   <sheetData>
@@ -5792,7 +5792,7 @@
         <v>2</v>
       </c>
       <c r="D5" s="25" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E5" s="25" t="n">
         <v>2</v>
@@ -5807,10 +5807,10 @@
         <v>2</v>
       </c>
       <c r="I5" s="25" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J5" s="25" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K5" s="25" t="n">
         <v>3</v>
@@ -5823,7 +5823,7 @@
       </c>
       <c r="N5" s="15" t="n">
         <f aca="false">SUM(B5:M5)</f>
-        <v>25</v>
+        <v>28</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5834,7 +5834,7 @@
         <v>9</v>
       </c>
       <c r="C6" s="25" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D6" s="25" t="n">
         <v>9</v>
@@ -5849,13 +5849,13 @@
         <v>9</v>
       </c>
       <c r="H6" s="25" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="I6" s="25" t="n">
         <v>9</v>
       </c>
       <c r="J6" s="25" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="K6" s="25" t="n">
         <v>9</v>
@@ -5864,7 +5864,7 @@
         <v>9</v>
       </c>
       <c r="M6" s="25" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="N6" s="15" t="n">
         <f aca="false">SUM(B6:M6)</f>
@@ -5879,16 +5879,16 @@
         <v>50</v>
       </c>
       <c r="C7" s="25" t="n">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="D7" s="25" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="E7" s="25" t="n">
         <v>80</v>
       </c>
       <c r="F7" s="25" t="n">
-        <v>100</v>
+        <v>85</v>
       </c>
       <c r="G7" s="25" t="n">
         <v>80</v>
@@ -5897,13 +5897,13 @@
         <v>85</v>
       </c>
       <c r="I7" s="25" t="n">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="J7" s="25" t="n">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="K7" s="25" t="n">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="L7" s="25" t="n">
         <v>90</v>
@@ -5913,7 +5913,7 @@
       </c>
       <c r="N7" s="15" t="n">
         <f aca="false">SUM(B7:M7)</f>
-        <v>965</v>
+        <v>1005</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5924,37 +5924,37 @@
         <v>0</v>
       </c>
       <c r="C8" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="M8" s="25" t="n">
         <v>2</v>
-      </c>
-      <c r="D8" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="E8" s="25" t="n">
-        <v>1</v>
-      </c>
-      <c r="F8" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="G8" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="H8" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="I8" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="J8" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="K8" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="L8" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="M8" s="25" t="n">
-        <v>0</v>
       </c>
       <c r="N8" s="15" t="n">
         <f aca="false">SUM(B8:M8)</f>
@@ -5966,40 +5966,40 @@
         <v>301</v>
       </c>
       <c r="B9" s="25" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C9" s="25" t="n">
         <v>2</v>
       </c>
       <c r="D9" s="25" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E9" s="25" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F9" s="25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G9" s="25" t="n">
         <v>4</v>
       </c>
       <c r="H9" s="25" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="I9" s="25" t="n">
         <v>4</v>
       </c>
       <c r="J9" s="25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K9" s="25" t="n">
         <v>4</v>
       </c>
       <c r="L9" s="25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M9" s="25" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N9" s="15" t="n">
         <f aca="false">SUM(B9:M9)</f>
@@ -6017,38 +6017,38 @@
         <v>0</v>
       </c>
       <c r="D10" s="29" t="n">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="E10" s="29" t="n">
-        <v>0</v>
+        <v>600</v>
       </c>
       <c r="F10" s="29" t="n">
-        <v>300</v>
+        <v>765</v>
       </c>
       <c r="G10" s="29" t="n">
+        <v>900</v>
+      </c>
+      <c r="H10" s="29" t="n">
         <v>600</v>
       </c>
-      <c r="H10" s="29" t="n">
-        <v>765</v>
-      </c>
       <c r="I10" s="29" t="n">
-        <v>900</v>
+        <v>1200</v>
       </c>
       <c r="J10" s="29" t="n">
+        <v>1200</v>
+      </c>
+      <c r="K10" s="29" t="n">
+        <v>1500</v>
+      </c>
+      <c r="L10" s="29" t="n">
+        <v>1500</v>
+      </c>
+      <c r="M10" s="29" t="n">
         <v>600</v>
-      </c>
-      <c r="K10" s="29" t="n">
-        <v>1200</v>
-      </c>
-      <c r="L10" s="29" t="n">
-        <v>1200</v>
-      </c>
-      <c r="M10" s="29" t="n">
-        <v>1500</v>
       </c>
       <c r="N10" s="15" t="n">
         <f aca="false">SUM(B10:M10)</f>
-        <v>7065</v>
+        <v>9165</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6150,11 +6150,11 @@
       </c>
       <c r="C14" s="15" t="n">
         <f aca="false">C5*C6*C7</f>
-        <v>2160</v>
+        <v>1440</v>
       </c>
       <c r="D14" s="15" t="n">
         <f aca="false">D5*D6*D7</f>
-        <v>450</v>
+        <v>1800</v>
       </c>
       <c r="E14" s="15" t="n">
         <f aca="false">E5*E6*E7</f>
@@ -6162,7 +6162,7 @@
       </c>
       <c r="F14" s="15" t="n">
         <f aca="false">F5*F6*F7</f>
-        <v>1800</v>
+        <v>1530</v>
       </c>
       <c r="G14" s="15" t="n">
         <f aca="false">G5*G6*G7</f>
@@ -6170,19 +6170,19 @@
       </c>
       <c r="H14" s="15" t="n">
         <f aca="false">H5*H6*H7</f>
-        <v>1530</v>
+        <v>1700</v>
       </c>
       <c r="I14" s="15" t="n">
         <f aca="false">I5*I6*I7</f>
-        <v>1440</v>
+        <v>2295</v>
       </c>
       <c r="J14" s="15" t="n">
         <f aca="false">J5*J6*J7</f>
-        <v>1700</v>
+        <v>2430</v>
       </c>
       <c r="K14" s="15" t="n">
         <f aca="false">K5*K6*K7</f>
-        <v>2295</v>
+        <v>2430</v>
       </c>
       <c r="L14" s="15" t="n">
         <f aca="false">L5*L6*L7</f>
@@ -6190,11 +6190,11 @@
       </c>
       <c r="M14" s="15" t="n">
         <f aca="false">M5*M6*M7</f>
-        <v>2430</v>
+        <v>3240</v>
       </c>
       <c r="N14" s="15" t="n">
         <f aca="false">SUM(B14:M14)</f>
-        <v>19565</v>
+        <v>22625</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6203,23 +6203,23 @@
       </c>
       <c r="B15" s="15" t="n">
         <f aca="false">B8*Supuestos!$B$61+B9*Supuestos!$B$62</f>
-        <v>450</v>
+        <v>150</v>
       </c>
       <c r="C15" s="15" t="n">
         <f aca="false">C8*Supuestos!$B$61+C9*Supuestos!$B$62</f>
-        <v>1700</v>
+        <v>1000</v>
       </c>
       <c r="D15" s="15" t="n">
         <f aca="false">D8*Supuestos!$B$61+D9*Supuestos!$B$62</f>
-        <v>150</v>
+        <v>600</v>
       </c>
       <c r="E15" s="15" t="n">
         <f aca="false">E8*Supuestos!$B$61+E9*Supuestos!$B$62</f>
-        <v>1000</v>
+        <v>600</v>
       </c>
       <c r="F15" s="15" t="n">
         <f aca="false">F8*Supuestos!$B$61+F9*Supuestos!$B$62</f>
-        <v>600</v>
+        <v>750</v>
       </c>
       <c r="G15" s="15" t="n">
         <f aca="false">G8*Supuestos!$B$61+G9*Supuestos!$B$62</f>
@@ -6227,7 +6227,7 @@
       </c>
       <c r="H15" s="15" t="n">
         <f aca="false">H8*Supuestos!$B$61+H9*Supuestos!$B$62</f>
-        <v>750</v>
+        <v>450</v>
       </c>
       <c r="I15" s="15" t="n">
         <f aca="false">I8*Supuestos!$B$61+I9*Supuestos!$B$62</f>
@@ -6235,7 +6235,7 @@
       </c>
       <c r="J15" s="15" t="n">
         <f aca="false">J8*Supuestos!$B$61+J9*Supuestos!$B$62</f>
-        <v>450</v>
+        <v>600</v>
       </c>
       <c r="K15" s="15" t="n">
         <f aca="false">K8*Supuestos!$B$61+K9*Supuestos!$B$62</f>
@@ -6243,11 +6243,11 @@
       </c>
       <c r="L15" s="15" t="n">
         <f aca="false">L8*Supuestos!$B$61+L9*Supuestos!$B$62</f>
-        <v>600</v>
+        <v>450</v>
       </c>
       <c r="M15" s="15" t="n">
         <f aca="false">M8*Supuestos!$B$61+M9*Supuestos!$B$62</f>
-        <v>600</v>
+        <v>1700</v>
       </c>
       <c r="N15" s="15" t="n">
         <f aca="false">SUM(B15:M15)</f>
@@ -6264,23 +6264,23 @@
       </c>
       <c r="C16" s="8" t="n">
         <f aca="false">ROUND(Supuestos!$B$63*(B14+B15),0)</f>
-        <v>315</v>
+        <v>210</v>
       </c>
       <c r="D16" s="8" t="n">
         <f aca="false">ROUND(Supuestos!$B$63*(C14+C15),0)</f>
-        <v>1351</v>
+        <v>854</v>
       </c>
       <c r="E16" s="8" t="n">
         <f aca="false">ROUND(Supuestos!$B$63*(D14+D15),0)</f>
-        <v>210</v>
+        <v>840</v>
       </c>
       <c r="F16" s="8" t="n">
         <f aca="false">ROUND(Supuestos!$B$63*(E14+E15),0)</f>
-        <v>854</v>
+        <v>714</v>
       </c>
       <c r="G16" s="8" t="n">
         <f aca="false">ROUND(Supuestos!$B$63*(F14+F15),0)</f>
-        <v>840</v>
+        <v>798</v>
       </c>
       <c r="H16" s="8" t="n">
         <f aca="false">ROUND(Supuestos!$B$63*(G14+G15),0)</f>
@@ -6288,27 +6288,27 @@
       </c>
       <c r="I16" s="8" t="n">
         <f aca="false">ROUND(Supuestos!$B$63*(H14+H15),0)</f>
-        <v>798</v>
+        <v>753</v>
       </c>
       <c r="J16" s="8" t="n">
         <f aca="false">ROUND(Supuestos!$B$63*(I14+I15),0)</f>
-        <v>714</v>
+        <v>1013</v>
       </c>
       <c r="K16" s="8" t="n">
         <f aca="false">ROUND(Supuestos!$B$63*(J14+J15),0)</f>
-        <v>753</v>
+        <v>1061</v>
       </c>
       <c r="L16" s="8" t="n">
         <f aca="false">ROUND(Supuestos!$B$63*(K14+K15),0)</f>
-        <v>1013</v>
+        <v>1061</v>
       </c>
       <c r="M16" s="8" t="n">
         <f aca="false">ROUND(Supuestos!$B$63*(L14+L15),0)</f>
-        <v>1061</v>
+        <v>1008</v>
       </c>
       <c r="N16" s="15" t="n">
         <f aca="false">SUM(B16:M16)</f>
-        <v>8773</v>
+        <v>9176</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6325,47 +6325,47 @@
       </c>
       <c r="D17" s="15" t="n">
         <f aca="false">D10</f>
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="E17" s="15" t="n">
         <f aca="false">E10</f>
-        <v>0</v>
+        <v>600</v>
       </c>
       <c r="F17" s="15" t="n">
         <f aca="false">F10</f>
-        <v>300</v>
+        <v>765</v>
       </c>
       <c r="G17" s="15" t="n">
         <f aca="false">G10</f>
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="H17" s="15" t="n">
         <f aca="false">H10</f>
-        <v>765</v>
+        <v>600</v>
       </c>
       <c r="I17" s="15" t="n">
         <f aca="false">I10</f>
-        <v>900</v>
+        <v>1200</v>
       </c>
       <c r="J17" s="15" t="n">
         <f aca="false">J10</f>
-        <v>600</v>
+        <v>1200</v>
       </c>
       <c r="K17" s="15" t="n">
         <f aca="false">K10</f>
-        <v>1200</v>
+        <v>1500</v>
       </c>
       <c r="L17" s="15" t="n">
         <f aca="false">L10</f>
-        <v>1200</v>
+        <v>1500</v>
       </c>
       <c r="M17" s="15" t="n">
         <f aca="false">M10</f>
-        <v>1500</v>
+        <v>600</v>
       </c>
       <c r="N17" s="15" t="n">
         <f aca="false">SUM(B17:M17)</f>
-        <v>7065</v>
+        <v>9165</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6431,55 +6431,55 @@
       </c>
       <c r="B19" s="31" t="n">
         <f aca="false">SUM(B14:B18)</f>
-        <v>1170</v>
+        <v>870</v>
       </c>
       <c r="C19" s="31" t="n">
         <f aca="false">SUM(C14:C18)</f>
-        <v>4355</v>
+        <v>2830</v>
       </c>
       <c r="D19" s="31" t="n">
         <f aca="false">SUM(D14:D18)</f>
-        <v>2131</v>
+        <v>3734</v>
       </c>
       <c r="E19" s="31" t="n">
         <f aca="false">SUM(E14:E18)</f>
-        <v>2890</v>
+        <v>3720</v>
       </c>
       <c r="F19" s="31" t="n">
         <f aca="false">SUM(F14:F18)</f>
-        <v>3854</v>
+        <v>4059</v>
       </c>
       <c r="G19" s="31" t="n">
         <f aca="false">SUM(G14:G18)</f>
-        <v>3780</v>
+        <v>4038</v>
       </c>
       <c r="H19" s="31" t="n">
         <f aca="false">SUM(H14:H18)</f>
-        <v>4119</v>
+        <v>3824</v>
       </c>
       <c r="I19" s="31" t="n">
         <f aca="false">SUM(I14:I18)</f>
-        <v>4098</v>
+        <v>5208</v>
       </c>
       <c r="J19" s="31" t="n">
         <f aca="false">SUM(J14:J18)</f>
-        <v>3824</v>
+        <v>5603</v>
       </c>
       <c r="K19" s="31" t="n">
         <f aca="false">SUM(K14:K18)</f>
-        <v>5268</v>
+        <v>6011</v>
       </c>
       <c r="L19" s="31" t="n">
         <f aca="false">SUM(L14:L18)</f>
-        <v>5663</v>
+        <v>5861</v>
       </c>
       <c r="M19" s="31" t="n">
         <f aca="false">SUM(M14:M18)</f>
-        <v>6071</v>
+        <v>7028</v>
       </c>
       <c r="N19" s="31" t="n">
         <f aca="false">SUM(N14:N18)</f>
-        <v>47223</v>
+        <v>52786</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6506,55 +6506,55 @@
       </c>
       <c r="B22" s="8" t="n">
         <f aca="false">SUMPRODUCT(B$14:B$18,Supuestos!$B$48:$B$52)</f>
-        <v>600</v>
+        <v>390</v>
       </c>
       <c r="C22" s="8" t="n">
         <f aca="false">SUMPRODUCT(C$14:C$18,Supuestos!$B$48:$B$52)</f>
-        <v>2517.5</v>
+        <v>1585</v>
       </c>
       <c r="D22" s="8" t="n">
         <f aca="false">SUMPRODUCT(D$14:D$18,Supuestos!$B$48:$B$52)</f>
-        <v>510.1</v>
+        <v>1885.4</v>
       </c>
       <c r="E22" s="8" t="n">
         <f aca="false">SUMPRODUCT(E$14:E$18,Supuestos!$B$48:$B$52)</f>
-        <v>1585</v>
+        <v>1968</v>
       </c>
       <c r="F22" s="8" t="n">
         <f aca="false">SUMPRODUCT(F$14:F$18,Supuestos!$B$48:$B$52)</f>
-        <v>1885.4</v>
+        <v>2279.4</v>
       </c>
       <c r="G22" s="8" t="n">
         <f aca="false">SUMPRODUCT(G$14:G$18,Supuestos!$B$48:$B$52)</f>
-        <v>1968</v>
+        <v>2263.8</v>
       </c>
       <c r="H22" s="8" t="n">
         <f aca="false">SUMPRODUCT(H$14:H$18,Supuestos!$B$48:$B$52)</f>
-        <v>2279.4</v>
+        <v>2006.4</v>
       </c>
       <c r="I22" s="8" t="n">
         <f aca="false">SUMPRODUCT(I$14:I$18,Supuestos!$B$48:$B$52)</f>
-        <v>2263.8</v>
+        <v>3072.3</v>
       </c>
       <c r="J22" s="8" t="n">
         <f aca="false">SUMPRODUCT(J$14:J$18,Supuestos!$B$48:$B$52)</f>
-        <v>2006.4</v>
+        <v>3179.3</v>
       </c>
       <c r="K22" s="8" t="n">
         <f aca="false">SUMPRODUCT(K$14:K$18,Supuestos!$B$48:$B$52)</f>
-        <v>3072.3</v>
+        <v>3484.1</v>
       </c>
       <c r="L22" s="8" t="n">
         <f aca="false">SUMPRODUCT(L$14:L$18,Supuestos!$B$48:$B$52)</f>
-        <v>3179.3</v>
+        <v>3379.1</v>
       </c>
       <c r="M22" s="8" t="n">
         <f aca="false">SUMPRODUCT(M$14:M$18,Supuestos!$B$48:$B$52)</f>
-        <v>3484.1</v>
+        <v>3834.8</v>
       </c>
       <c r="N22" s="15" t="n">
         <f aca="false">SUM(B22:M22)</f>
-        <v>25351.3</v>
+        <v>29327.6</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6563,55 +6563,55 @@
       </c>
       <c r="B23" s="8" t="n">
         <f aca="false">SUMPRODUCT(B$14:B$18,Supuestos!$C$48:$C$52)</f>
-        <v>502.5</v>
+        <v>412.5</v>
       </c>
       <c r="C23" s="8" t="n">
         <f aca="false">SUMPRODUCT(C$14:C$18,Supuestos!$C$48:$C$52)</f>
-        <v>1635</v>
+        <v>1110</v>
       </c>
       <c r="D23" s="8" t="n">
         <f aca="false">SUMPRODUCT(D$14:D$18,Supuestos!$C$48:$C$52)</f>
-        <v>1193.1</v>
+        <v>1502.4</v>
       </c>
       <c r="E23" s="8" t="n">
         <f aca="false">SUMPRODUCT(E$14:E$18,Supuestos!$C$48:$C$52)</f>
-        <v>1170</v>
+        <v>1428</v>
       </c>
       <c r="F23" s="8" t="n">
         <f aca="false">SUMPRODUCT(F$14:F$18,Supuestos!$C$48:$C$52)</f>
-        <v>1622.4</v>
+        <v>1488.9</v>
       </c>
       <c r="G23" s="8" t="n">
         <f aca="false">SUMPRODUCT(G$14:G$18,Supuestos!$C$48:$C$52)</f>
-        <v>1488</v>
+        <v>1462.8</v>
       </c>
       <c r="H23" s="8" t="n">
         <f aca="false">SUMPRODUCT(H$14:H$18,Supuestos!$C$48:$C$52)</f>
-        <v>1548.9</v>
+        <v>1518.4</v>
       </c>
       <c r="I23" s="8" t="n">
         <f aca="false">SUMPRODUCT(I$14:I$18,Supuestos!$C$48:$C$52)</f>
-        <v>1522.8</v>
+        <v>1795.05</v>
       </c>
       <c r="J23" s="8" t="n">
         <f aca="false">SUMPRODUCT(J$14:J$18,Supuestos!$C$48:$C$52)</f>
-        <v>1518.4</v>
+        <v>1998.3</v>
       </c>
       <c r="K23" s="8" t="n">
         <f aca="false">SUMPRODUCT(K$14:K$18,Supuestos!$C$48:$C$52)</f>
-        <v>1855.05</v>
+        <v>2087.1</v>
       </c>
       <c r="L23" s="8" t="n">
         <f aca="false">SUMPRODUCT(L$14:L$18,Supuestos!$C$48:$C$52)</f>
-        <v>2058.3</v>
+        <v>2042.1</v>
       </c>
       <c r="M23" s="8" t="n">
         <f aca="false">SUMPRODUCT(M$14:M$18,Supuestos!$C$48:$C$52)</f>
-        <v>2147.1</v>
+        <v>2728.8</v>
       </c>
       <c r="N23" s="15" t="n">
         <f aca="false">SUM(B23:M23)</f>
-        <v>18261.55</v>
+        <v>19574.35</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6624,51 +6624,51 @@
       </c>
       <c r="C24" s="8" t="n">
         <f aca="false">SUMPRODUCT(C$14:C$18,Supuestos!$D$48:$D$52)</f>
-        <v>202.5</v>
+        <v>135</v>
       </c>
       <c r="D24" s="8" t="n">
         <f aca="false">SUMPRODUCT(D$14:D$18,Supuestos!$D$48:$D$52)</f>
-        <v>427.8</v>
+        <v>346.2</v>
       </c>
       <c r="E24" s="8" t="n">
         <f aca="false">SUMPRODUCT(E$14:E$18,Supuestos!$D$48:$D$52)</f>
-        <v>135</v>
+        <v>324</v>
       </c>
       <c r="F24" s="8" t="n">
         <f aca="false">SUMPRODUCT(F$14:F$18,Supuestos!$D$48:$D$52)</f>
-        <v>346.2</v>
+        <v>290.7</v>
       </c>
       <c r="G24" s="8" t="n">
         <f aca="false">SUMPRODUCT(G$14:G$18,Supuestos!$D$48:$D$52)</f>
-        <v>324</v>
+        <v>311.4</v>
       </c>
       <c r="H24" s="8" t="n">
         <f aca="false">SUMPRODUCT(H$14:H$18,Supuestos!$D$48:$D$52)</f>
-        <v>290.7</v>
+        <v>299.2</v>
       </c>
       <c r="I24" s="8" t="n">
         <f aca="false">SUMPRODUCT(I$14:I$18,Supuestos!$D$48:$D$52)</f>
-        <v>311.4</v>
+        <v>340.65</v>
       </c>
       <c r="J24" s="8" t="n">
         <f aca="false">SUMPRODUCT(J$14:J$18,Supuestos!$D$48:$D$52)</f>
-        <v>299.2</v>
+        <v>425.4</v>
       </c>
       <c r="K24" s="8" t="n">
         <f aca="false">SUMPRODUCT(K$14:K$18,Supuestos!$D$48:$D$52)</f>
-        <v>340.65</v>
+        <v>439.8</v>
       </c>
       <c r="L24" s="8" t="n">
         <f aca="false">SUMPRODUCT(L$14:L$18,Supuestos!$D$48:$D$52)</f>
-        <v>425.4</v>
+        <v>439.8</v>
       </c>
       <c r="M24" s="8" t="n">
         <f aca="false">SUMPRODUCT(M$14:M$18,Supuestos!$D$48:$D$52)</f>
-        <v>439.8</v>
+        <v>464.4</v>
       </c>
       <c r="N24" s="15" t="n">
         <f aca="false">SUM(B24:M24)</f>
-        <v>3610.15</v>
+        <v>3884.05</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6677,55 +6677,55 @@
       </c>
       <c r="B25" s="15" t="n">
         <f aca="false">B23/Costeo!$C$5</f>
-        <v>83.75</v>
+        <v>68.75</v>
       </c>
       <c r="C25" s="15" t="n">
         <f aca="false">C23/Costeo!$C$5</f>
-        <v>272.5</v>
+        <v>185</v>
       </c>
       <c r="D25" s="15" t="n">
         <f aca="false">D23/Costeo!$C$5</f>
-        <v>198.85</v>
+        <v>250.4</v>
       </c>
       <c r="E25" s="15" t="n">
         <f aca="false">E23/Costeo!$C$5</f>
-        <v>195</v>
+        <v>238</v>
       </c>
       <c r="F25" s="15" t="n">
         <f aca="false">F23/Costeo!$C$5</f>
-        <v>270.4</v>
+        <v>248.15</v>
       </c>
       <c r="G25" s="15" t="n">
         <f aca="false">G23/Costeo!$C$5</f>
-        <v>248</v>
+        <v>243.8</v>
       </c>
       <c r="H25" s="15" t="n">
         <f aca="false">H23/Costeo!$C$5</f>
-        <v>258.15</v>
+        <v>253.066666666667</v>
       </c>
       <c r="I25" s="15" t="n">
         <f aca="false">I23/Costeo!$C$5</f>
-        <v>253.8</v>
+        <v>299.175</v>
       </c>
       <c r="J25" s="15" t="n">
         <f aca="false">J23/Costeo!$C$5</f>
-        <v>253.066666666667</v>
+        <v>333.05</v>
       </c>
       <c r="K25" s="15" t="n">
         <f aca="false">K23/Costeo!$C$5</f>
-        <v>309.175</v>
+        <v>347.85</v>
       </c>
       <c r="L25" s="15" t="n">
         <f aca="false">L23/Costeo!$C$5</f>
-        <v>343.05</v>
+        <v>340.35</v>
       </c>
       <c r="M25" s="15" t="n">
         <f aca="false">M23/Costeo!$C$5</f>
-        <v>357.85</v>
+        <v>454.8</v>
       </c>
       <c r="N25" s="15" t="n">
         <f aca="false">SUM(B25:M25)</f>
-        <v>3043.59166666667</v>
+        <v>3262.39166666667</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6738,51 +6738,51 @@
       </c>
       <c r="C26" s="15" t="n">
         <f aca="false">C24/Costeo!$E$5</f>
-        <v>16.875</v>
+        <v>11.25</v>
       </c>
       <c r="D26" s="15" t="n">
         <f aca="false">D24/Costeo!$E$5</f>
-        <v>35.65</v>
+        <v>28.85</v>
       </c>
       <c r="E26" s="15" t="n">
         <f aca="false">E24/Costeo!$E$5</f>
-        <v>11.25</v>
+        <v>27</v>
       </c>
       <c r="F26" s="15" t="n">
         <f aca="false">F24/Costeo!$E$5</f>
-        <v>28.85</v>
+        <v>24.225</v>
       </c>
       <c r="G26" s="15" t="n">
         <f aca="false">G24/Costeo!$E$5</f>
-        <v>27</v>
+        <v>25.95</v>
       </c>
       <c r="H26" s="15" t="n">
         <f aca="false">H24/Costeo!$E$5</f>
-        <v>24.225</v>
+        <v>24.9333333333333</v>
       </c>
       <c r="I26" s="15" t="n">
         <f aca="false">I24/Costeo!$E$5</f>
-        <v>25.95</v>
+        <v>28.3875</v>
       </c>
       <c r="J26" s="15" t="n">
         <f aca="false">J24/Costeo!$E$5</f>
-        <v>24.9333333333333</v>
+        <v>35.45</v>
       </c>
       <c r="K26" s="15" t="n">
         <f aca="false">K24/Costeo!$E$5</f>
-        <v>28.3875</v>
+        <v>36.65</v>
       </c>
       <c r="L26" s="15" t="n">
         <f aca="false">L24/Costeo!$E$5</f>
-        <v>35.45</v>
+        <v>36.65</v>
       </c>
       <c r="M26" s="15" t="n">
         <f aca="false">M24/Costeo!$E$5</f>
-        <v>36.65</v>
+        <v>38.7</v>
       </c>
       <c r="N26" s="15" t="n">
         <f aca="false">SUM(B26:M26)</f>
-        <v>300.845833333333</v>
+        <v>323.670833333333</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6809,55 +6809,55 @@
       </c>
       <c r="B29" s="9" t="n">
         <f aca="false">SUMPRODUCT(B$14:B$18,Proyeccion!$H$25:$H$29)</f>
-        <v>5531.175</v>
+        <v>3986.175</v>
       </c>
       <c r="C29" s="9" t="n">
         <f aca="false">SUMPRODUCT(C$14:C$18,Proyeccion!$H$25:$H$29)</f>
-        <v>21390.8875</v>
+        <v>13747.325</v>
       </c>
       <c r="D29" s="9" t="n">
         <f aca="false">SUMPRODUCT(D$14:D$18,Proyeccion!$H$25:$H$29)</f>
-        <v>9038.6375</v>
+        <v>17009.575</v>
       </c>
       <c r="E29" s="9" t="n">
         <f aca="false">SUMPRODUCT(E$14:E$18,Proyeccion!$H$25:$H$29)</f>
-        <v>13920.725</v>
+        <v>16220.1</v>
       </c>
       <c r="F29" s="9" t="n">
         <f aca="false">SUMPRODUCT(F$14:F$18,Proyeccion!$H$25:$H$29)</f>
-        <v>17356.375</v>
+        <v>17600.625</v>
       </c>
       <c r="G29" s="9" t="n">
         <f aca="false">SUMPRODUCT(G$14:G$18,Proyeccion!$H$25:$H$29)</f>
-        <v>16393.5</v>
+        <v>17122.875</v>
       </c>
       <c r="H29" s="9" t="n">
         <f aca="false">SUMPRODUCT(H$14:H$18,Proyeccion!$H$25:$H$29)</f>
-        <v>17774.025</v>
+        <v>16586.8583333333</v>
       </c>
       <c r="I29" s="9" t="n">
         <f aca="false">SUMPRODUCT(I$14:I$18,Proyeccion!$H$25:$H$29)</f>
-        <v>17296.275</v>
+        <v>22302.7125</v>
       </c>
       <c r="J29" s="9" t="n">
         <f aca="false">SUMPRODUCT(J$14:J$18,Proyeccion!$H$25:$H$29)</f>
-        <v>16586.8583333333</v>
+        <v>24036.2125</v>
       </c>
       <c r="K29" s="9" t="n">
         <f aca="false">SUMPRODUCT(K$14:K$18,Proyeccion!$H$25:$H$29)</f>
-        <v>22476.1125</v>
+        <v>25304.6125</v>
       </c>
       <c r="L29" s="9" t="n">
         <f aca="false">SUMPRODUCT(L$14:L$18,Proyeccion!$H$25:$H$29)</f>
-        <v>24209.6125</v>
+        <v>24532.1125</v>
       </c>
       <c r="M29" s="9" t="n">
         <f aca="false">SUMPRODUCT(M$14:M$18,Proyeccion!$H$25:$H$29)</f>
-        <v>25478.0125</v>
+        <v>32291.2</v>
       </c>
       <c r="N29" s="16" t="n">
         <f aca="false">SUM(B29:M29)</f>
-        <v>207452.195833333</v>
+        <v>230740.383333333</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6866,55 +6866,55 @@
       </c>
       <c r="B30" s="16" t="n">
         <f aca="false">B29/(1+Supuestos!$B$26)</f>
-        <v>4687.43644067797</v>
+        <v>3378.11440677966</v>
       </c>
       <c r="C30" s="16" t="n">
         <f aca="false">C29/(1+Supuestos!$B$26)</f>
-        <v>18127.8707627119</v>
+        <v>11650.2754237288</v>
       </c>
       <c r="D30" s="16" t="n">
         <f aca="false">D29/(1+Supuestos!$B$26)</f>
-        <v>7659.86228813559</v>
+        <v>14414.8940677966</v>
       </c>
       <c r="E30" s="16" t="n">
         <f aca="false">E29/(1+Supuestos!$B$26)</f>
-        <v>11797.2245762712</v>
+        <v>13745.8474576271</v>
       </c>
       <c r="F30" s="16" t="n">
         <f aca="false">F29/(1+Supuestos!$B$26)</f>
-        <v>14708.7923728814</v>
+        <v>14915.7838983051</v>
       </c>
       <c r="G30" s="16" t="n">
         <f aca="false">G29/(1+Supuestos!$B$26)</f>
-        <v>13892.7966101695</v>
+        <v>14510.9110169492</v>
       </c>
       <c r="H30" s="16" t="n">
         <f aca="false">H29/(1+Supuestos!$B$26)</f>
-        <v>15062.7330508475</v>
+        <v>14056.6596045198</v>
       </c>
       <c r="I30" s="16" t="n">
         <f aca="false">I29/(1+Supuestos!$B$26)</f>
-        <v>14657.8601694915</v>
+        <v>18900.6038135593</v>
       </c>
       <c r="J30" s="16" t="n">
         <f aca="false">J29/(1+Supuestos!$B$26)</f>
-        <v>14056.6596045198</v>
+        <v>20369.6716101695</v>
       </c>
       <c r="K30" s="16" t="n">
         <f aca="false">K29/(1+Supuestos!$B$26)</f>
-        <v>19047.5529661017</v>
+        <v>21444.5868644068</v>
       </c>
       <c r="L30" s="16" t="n">
         <f aca="false">L29/(1+Supuestos!$B$26)</f>
-        <v>20516.6207627119</v>
+        <v>20789.9258474576</v>
       </c>
       <c r="M30" s="16" t="n">
         <f aca="false">M29/(1+Supuestos!$B$26)</f>
-        <v>21591.5360169492</v>
+        <v>27365.4237288136</v>
       </c>
       <c r="N30" s="16" t="n">
         <f aca="false">SUM(B30:M30)</f>
-        <v>175806.945621469</v>
+        <v>195542.697740113</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6923,55 +6923,55 @@
       </c>
       <c r="B31" s="9" t="n">
         <f aca="false">SUMPRODUCT(B$14:B$18,Proyeccion!$F$25:$F$29)</f>
-        <v>2154.24457627119</v>
+        <v>1722.34576271186</v>
       </c>
       <c r="C31" s="9" t="n">
         <f aca="false">SUMPRODUCT(C$14:C$18,Proyeccion!$F$25:$F$29)</f>
-        <v>8724.69455508475</v>
+        <v>6316.22016949153</v>
       </c>
       <c r="D31" s="9" t="n">
         <f aca="false">SUMPRODUCT(D$14:D$18,Proyeccion!$F$25:$F$29)</f>
-        <v>2560.93626525424</v>
+        <v>7205.63902711864</v>
       </c>
       <c r="E31" s="9" t="n">
         <f aca="false">SUMPRODUCT(E$14:E$18,Proyeccion!$F$25:$F$29)</f>
-        <v>5595.99733050848</v>
+        <v>6682.20198305085</v>
       </c>
       <c r="F31" s="9" t="n">
         <f aca="false">SUMPRODUCT(F$14:F$18,Proyeccion!$F$25:$F$29)</f>
-        <v>6280.87984915254</v>
+        <v>7344.39145932203</v>
       </c>
       <c r="G31" s="9" t="n">
         <f aca="false">SUMPRODUCT(G$14:G$18,Proyeccion!$F$25:$F$29)</f>
-        <v>5723.6816440678</v>
+        <v>6985.80520677966</v>
       </c>
       <c r="H31" s="9" t="n">
         <f aca="false">SUMPRODUCT(H$14:H$18,Proyeccion!$F$25:$F$29)</f>
-        <v>6295.10387033898</v>
+        <v>6894.68165847458</v>
       </c>
       <c r="I31" s="9" t="n">
         <f aca="false">SUMPRODUCT(I$14:I$18,Proyeccion!$F$25:$F$29)</f>
-        <v>5942.14036779661</v>
+        <v>9325.30270042373</v>
       </c>
       <c r="J31" s="9" t="n">
         <f aca="false">SUMPRODUCT(J$14:J$18,Proyeccion!$F$25:$F$29)</f>
-        <v>5870.80565847458</v>
+        <v>9940.7611940678</v>
       </c>
       <c r="K31" s="9" t="n">
         <f aca="false">SUMPRODUCT(K$14:K$18,Proyeccion!$F$25:$F$29)</f>
-        <v>7968.37036144068</v>
+        <v>10345.9490957627</v>
       </c>
       <c r="L31" s="9" t="n">
         <f aca="false">SUMPRODUCT(L$14:L$18,Proyeccion!$F$25:$F$29)</f>
-        <v>8478.06760508475</v>
+        <v>9973.36593898305</v>
       </c>
       <c r="M31" s="9" t="n">
         <f aca="false">SUMPRODUCT(M$14:M$18,Proyeccion!$F$25:$F$29)</f>
-        <v>8774.01350677966</v>
+        <v>14111.6237915254</v>
       </c>
       <c r="N31" s="16" t="n">
         <f aca="false">SUM(B31:M31)</f>
-        <v>74368.9355902542</v>
+        <v>96848.2879877119</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6980,55 +6980,55 @@
       </c>
       <c r="B32" s="9" t="n">
         <f aca="false">SUMPRODUCT(B$14:B$18,Proyeccion!$G$25:$G$29)</f>
-        <v>2196.45457627119</v>
+        <v>1756.99576271186</v>
       </c>
       <c r="C32" s="9" t="n">
         <f aca="false">SUMPRODUCT(C$14:C$18,Proyeccion!$G$25:$G$29)</f>
-        <v>8862.03455508475</v>
+        <v>6409.46016949153</v>
       </c>
       <c r="D32" s="9" t="n">
         <f aca="false">SUMPRODUCT(D$14:D$18,Proyeccion!$G$25:$G$29)</f>
-        <v>2661.15666525424</v>
+        <v>7331.84062711865</v>
       </c>
       <c r="E32" s="9" t="n">
         <f aca="false">SUMPRODUCT(E$14:E$18,Proyeccion!$G$25:$G$29)</f>
-        <v>5694.27733050848</v>
+        <v>6802.15398305085</v>
       </c>
       <c r="F32" s="9" t="n">
         <f aca="false">SUMPRODUCT(F$14:F$18,Proyeccion!$G$25:$G$29)</f>
-        <v>6417.16144915254</v>
+        <v>7469.45905932204</v>
       </c>
       <c r="G32" s="9" t="n">
         <f aca="false">SUMPRODUCT(G$14:G$18,Proyeccion!$G$25:$G$29)</f>
-        <v>5848.6736440678</v>
+        <v>7108.68040677966</v>
       </c>
       <c r="H32" s="9" t="n">
         <f aca="false">SUMPRODUCT(H$14:H$18,Proyeccion!$G$25:$G$29)</f>
-        <v>6425.21147033898</v>
+        <v>7022.22725847458</v>
       </c>
       <c r="I32" s="9" t="n">
         <f aca="false">SUMPRODUCT(I$14:I$18,Proyeccion!$G$25:$G$29)</f>
-        <v>6070.05556779661</v>
+        <v>9476.08690042373</v>
       </c>
       <c r="J32" s="9" t="n">
         <f aca="false">SUMPRODUCT(J$14:J$18,Proyeccion!$G$25:$G$29)</f>
-        <v>5998.35125847458</v>
+        <v>10108.6183940678</v>
       </c>
       <c r="K32" s="9" t="n">
         <f aca="false">SUMPRODUCT(K$14:K$18,Proyeccion!$G$25:$G$29)</f>
-        <v>8124.19456144068</v>
+        <v>10521.2654957627</v>
       </c>
       <c r="L32" s="9" t="n">
         <f aca="false">SUMPRODUCT(L$14:L$18,Proyeccion!$G$25:$G$29)</f>
-        <v>8650.96480508475</v>
+        <v>10144.9023389831</v>
       </c>
       <c r="M32" s="9" t="n">
         <f aca="false">SUMPRODUCT(M$14:M$18,Proyeccion!$G$25:$G$29)</f>
-        <v>8954.36990677966</v>
+        <v>14340.8429915254</v>
       </c>
       <c r="N32" s="16" t="n">
         <f aca="false">SUM(B32:M32)</f>
-        <v>75902.9057902542</v>
+        <v>98492.5333877119</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7045,7 +7045,7 @@
       </c>
       <c r="D33" s="9" t="n">
         <f aca="false">D5*Supuestos!$B$57</f>
-        <v>600</v>
+        <v>1200</v>
       </c>
       <c r="E33" s="9" t="n">
         <f aca="false">E5*Supuestos!$B$57</f>
@@ -7065,11 +7065,11 @@
       </c>
       <c r="I33" s="9" t="n">
         <f aca="false">I5*Supuestos!$B$57</f>
-        <v>1200</v>
+        <v>1800</v>
       </c>
       <c r="J33" s="9" t="n">
         <f aca="false">J5*Supuestos!$B$57</f>
-        <v>1200</v>
+        <v>1800</v>
       </c>
       <c r="K33" s="9" t="n">
         <f aca="false">K5*Supuestos!$B$57</f>
@@ -7085,7 +7085,7 @@
       </c>
       <c r="N33" s="16" t="n">
         <f aca="false">SUM(B33:M33)</f>
-        <v>15000</v>
+        <v>16800</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7094,55 +7094,55 @@
       </c>
       <c r="B34" s="9" t="n">
         <f aca="false">MAX(0,B5-Supuestos!$B$59)*B6*Supuestos!$B$58</f>
-        <v>0</v>
+        <v>810</v>
       </c>
       <c r="C34" s="9" t="n">
         <f aca="false">MAX(0,C5-Supuestos!$B$59)*C6*Supuestos!$B$58</f>
-        <v>0</v>
+        <v>1620</v>
       </c>
       <c r="D34" s="9" t="n">
         <f aca="false">MAX(0,D5-Supuestos!$B$59)*D6*Supuestos!$B$58</f>
-        <v>0</v>
+        <v>1620</v>
       </c>
       <c r="E34" s="9" t="n">
         <f aca="false">MAX(0,E5-Supuestos!$B$59)*E6*Supuestos!$B$58</f>
-        <v>0</v>
+        <v>1620</v>
       </c>
       <c r="F34" s="9" t="n">
         <f aca="false">MAX(0,F5-Supuestos!$B$59)*F6*Supuestos!$B$58</f>
-        <v>0</v>
+        <v>1620</v>
       </c>
       <c r="G34" s="9" t="n">
         <f aca="false">MAX(0,G5-Supuestos!$B$59)*G6*Supuestos!$B$58</f>
-        <v>0</v>
+        <v>1620</v>
       </c>
       <c r="H34" s="9" t="n">
         <f aca="false">MAX(0,H5-Supuestos!$B$59)*H6*Supuestos!$B$58</f>
-        <v>0</v>
+        <v>1800</v>
       </c>
       <c r="I34" s="9" t="n">
         <f aca="false">MAX(0,I5-Supuestos!$B$59)*I6*Supuestos!$B$58</f>
-        <v>0</v>
+        <v>2430</v>
       </c>
       <c r="J34" s="9" t="n">
         <f aca="false">MAX(0,J5-Supuestos!$B$59)*J6*Supuestos!$B$58</f>
-        <v>0</v>
+        <v>2430</v>
       </c>
       <c r="K34" s="9" t="n">
         <f aca="false">MAX(0,K5-Supuestos!$B$59)*K6*Supuestos!$B$58</f>
-        <v>810</v>
+        <v>2430</v>
       </c>
       <c r="L34" s="9" t="n">
         <f aca="false">MAX(0,L5-Supuestos!$B$59)*L6*Supuestos!$B$58</f>
-        <v>810</v>
+        <v>2430</v>
       </c>
       <c r="M34" s="9" t="n">
         <f aca="false">MAX(0,M5-Supuestos!$B$59)*M6*Supuestos!$B$58</f>
-        <v>810</v>
+        <v>3240</v>
       </c>
       <c r="N34" s="16" t="n">
         <f aca="false">SUM(B34:M34)</f>
-        <v>2430</v>
+        <v>23670</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7155,7 +7155,7 @@
       </c>
       <c r="C35" s="9" t="n">
         <f aca="false">C8*Supuestos!$B$60</f>
-        <v>3600</v>
+        <v>1800</v>
       </c>
       <c r="D35" s="9" t="n">
         <f aca="false">D8*Supuestos!$B$60</f>
@@ -7163,7 +7163,7 @@
       </c>
       <c r="E35" s="9" t="n">
         <f aca="false">E8*Supuestos!$B$60</f>
-        <v>1800</v>
+        <v>0</v>
       </c>
       <c r="F35" s="9" t="n">
         <f aca="false">F8*Supuestos!$B$60</f>
@@ -7195,7 +7195,7 @@
       </c>
       <c r="M35" s="9" t="n">
         <f aca="false">M8*Supuestos!$B$60</f>
-        <v>0</v>
+        <v>3600</v>
       </c>
       <c r="N35" s="16" t="n">
         <f aca="false">SUM(B35:M35)</f>
@@ -7208,55 +7208,55 @@
       </c>
       <c r="B36" s="9" t="n">
         <f aca="false">Supuestos!$B$72</f>
-        <v>1734.38888888889</v>
+        <v>2443.38888888889</v>
       </c>
       <c r="C36" s="9" t="n">
         <f aca="false">Supuestos!$B$72</f>
-        <v>1734.38888888889</v>
+        <v>2443.38888888889</v>
       </c>
       <c r="D36" s="9" t="n">
         <f aca="false">Supuestos!$B$72</f>
-        <v>1734.38888888889</v>
+        <v>2443.38888888889</v>
       </c>
       <c r="E36" s="9" t="n">
         <f aca="false">Supuestos!$B$72</f>
-        <v>1734.38888888889</v>
+        <v>2443.38888888889</v>
       </c>
       <c r="F36" s="9" t="n">
         <f aca="false">Supuestos!$B$72</f>
-        <v>1734.38888888889</v>
+        <v>2443.38888888889</v>
       </c>
       <c r="G36" s="9" t="n">
         <f aca="false">Supuestos!$B$72</f>
-        <v>1734.38888888889</v>
+        <v>2443.38888888889</v>
       </c>
       <c r="H36" s="9" t="n">
         <f aca="false">Supuestos!$B$72</f>
-        <v>1734.38888888889</v>
+        <v>2443.38888888889</v>
       </c>
       <c r="I36" s="9" t="n">
         <f aca="false">Supuestos!$B$72</f>
-        <v>1734.38888888889</v>
+        <v>2443.38888888889</v>
       </c>
       <c r="J36" s="9" t="n">
         <f aca="false">Supuestos!$B$72</f>
-        <v>1734.38888888889</v>
+        <v>2443.38888888889</v>
       </c>
       <c r="K36" s="9" t="n">
         <f aca="false">Supuestos!$B$72</f>
-        <v>1734.38888888889</v>
+        <v>2443.38888888889</v>
       </c>
       <c r="L36" s="9" t="n">
         <f aca="false">Supuestos!$B$72</f>
-        <v>1734.38888888889</v>
+        <v>2443.38888888889</v>
       </c>
       <c r="M36" s="9" t="n">
         <f aca="false">Supuestos!$B$72</f>
-        <v>1734.38888888889</v>
+        <v>2443.38888888889</v>
       </c>
       <c r="N36" s="16" t="n">
         <f aca="false">SUM(B36:M36)</f>
-        <v>20812.6666666667</v>
+        <v>29320.6666666667</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7265,55 +7265,55 @@
       </c>
       <c r="B37" s="11" t="n">
         <f aca="false">B31-B33-B34-B35-B36</f>
-        <v>-180.144312617702</v>
+        <v>-2131.04312617702</v>
       </c>
       <c r="C37" s="11" t="n">
         <f aca="false">C31-C33-C34-C35-C36</f>
-        <v>2190.30566619586</v>
+        <v>-747.168719397363</v>
       </c>
       <c r="D37" s="11" t="n">
         <f aca="false">D31-D33-D34-D35-D36</f>
-        <v>226.547376365349</v>
+        <v>1942.25013822976</v>
       </c>
       <c r="E37" s="11" t="n">
         <f aca="false">E31-E33-E34-E35-E36</f>
-        <v>861.608441619586</v>
+        <v>1418.81309416196</v>
       </c>
       <c r="F37" s="11" t="n">
         <f aca="false">F31-F33-F34-F35-F36</f>
-        <v>3346.49096026365</v>
+        <v>2081.00257043314</v>
       </c>
       <c r="G37" s="11" t="n">
         <f aca="false">G31-G33-G34-G35-G36</f>
-        <v>2789.29275517891</v>
+        <v>1722.41631789077</v>
       </c>
       <c r="H37" s="11" t="n">
         <f aca="false">H31-H33-H34-H35-H36</f>
-        <v>3360.7149814501</v>
+        <v>1451.29276958569</v>
       </c>
       <c r="I37" s="11" t="n">
         <f aca="false">I31-I33-I34-I35-I36</f>
-        <v>3007.75147890772</v>
+        <v>2651.91381153484</v>
       </c>
       <c r="J37" s="11" t="n">
         <f aca="false">J31-J33-J34-J35-J36</f>
-        <v>2936.41676958569</v>
+        <v>3267.37230517891</v>
       </c>
       <c r="K37" s="11" t="n">
         <f aca="false">K31-K33-K34-K35-K36</f>
-        <v>3623.98147255179</v>
+        <v>3672.56020687382</v>
       </c>
       <c r="L37" s="11" t="n">
         <f aca="false">L31-L33-L34-L35-L36</f>
-        <v>4133.67871619586</v>
+        <v>3299.97705009416</v>
       </c>
       <c r="M37" s="11" t="n">
         <f aca="false">M31-M33-M34-M35-M36</f>
-        <v>4429.62461789077</v>
+        <v>3028.23490263653</v>
       </c>
       <c r="N37" s="11" t="n">
         <f aca="false">SUM(B37:M37)</f>
-        <v>30726.2689235876</v>
+        <v>21657.6213210452</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7322,55 +7322,55 @@
       </c>
       <c r="B38" s="11" t="n">
         <f aca="false">B32-B33-B34-B35-B36</f>
-        <v>-137.934312617702</v>
+        <v>-2096.39312617702</v>
       </c>
       <c r="C38" s="11" t="n">
         <f aca="false">C32-C33-C34-C35-C36</f>
-        <v>2327.64566619586</v>
+        <v>-653.928719397363</v>
       </c>
       <c r="D38" s="11" t="n">
         <f aca="false">D32-D33-D34-D35-D36</f>
-        <v>326.767776365349</v>
+        <v>2068.45173822976</v>
       </c>
       <c r="E38" s="11" t="n">
         <f aca="false">E32-E33-E34-E35-E36</f>
-        <v>959.888441619586</v>
+        <v>1538.76509416196</v>
       </c>
       <c r="F38" s="11" t="n">
         <f aca="false">F32-F33-F34-F35-F36</f>
-        <v>3482.77256026365</v>
+        <v>2206.07017043315</v>
       </c>
       <c r="G38" s="11" t="n">
         <f aca="false">G32-G33-G34-G35-G36</f>
-        <v>2914.28475517891</v>
+        <v>1845.29151789077</v>
       </c>
       <c r="H38" s="11" t="n">
         <f aca="false">H32-H33-H34-H35-H36</f>
-        <v>3490.8225814501</v>
+        <v>1578.83836958569</v>
       </c>
       <c r="I38" s="11" t="n">
         <f aca="false">I32-I33-I34-I35-I36</f>
-        <v>3135.66667890772</v>
+        <v>2802.69801153484</v>
       </c>
       <c r="J38" s="11" t="n">
         <f aca="false">J32-J33-J34-J35-J36</f>
-        <v>3063.96236958569</v>
+        <v>3435.22950517891</v>
       </c>
       <c r="K38" s="11" t="n">
         <f aca="false">K32-K33-K34-K35-K36</f>
-        <v>3779.80567255179</v>
+        <v>3847.87660687382</v>
       </c>
       <c r="L38" s="11" t="n">
         <f aca="false">L32-L33-L34-L35-L36</f>
-        <v>4306.57591619586</v>
+        <v>3471.51345009416</v>
       </c>
       <c r="M38" s="11" t="n">
         <f aca="false">M32-M33-M34-M35-M36</f>
-        <v>4609.98101789077</v>
+        <v>3257.45410263654</v>
       </c>
       <c r="N38" s="11" t="n">
         <f aca="false">SUM(B38:M38)</f>
-        <v>32260.2391235876</v>
+        <v>23301.8667210452</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7379,51 +7379,51 @@
       </c>
       <c r="B39" s="16" t="n">
         <f aca="false">B37</f>
-        <v>-180.144312617702</v>
+        <v>-2131.04312617702</v>
       </c>
       <c r="C39" s="16" t="n">
         <f aca="false">B39+C37</f>
-        <v>2010.16135357816</v>
+        <v>-2878.21184557439</v>
       </c>
       <c r="D39" s="16" t="n">
         <f aca="false">C39+D37</f>
-        <v>2236.7087299435</v>
+        <v>-935.961707344633</v>
       </c>
       <c r="E39" s="16" t="n">
         <f aca="false">D39+E37</f>
-        <v>3098.31717156309</v>
+        <v>482.851386817326</v>
       </c>
       <c r="F39" s="16" t="n">
         <f aca="false">E39+F37</f>
-        <v>6444.80813182675</v>
+        <v>2563.85395725047</v>
       </c>
       <c r="G39" s="16" t="n">
         <f aca="false">F39+G37</f>
-        <v>9234.10088700565</v>
+        <v>4286.27027514124</v>
       </c>
       <c r="H39" s="16" t="n">
         <f aca="false">G39+H37</f>
-        <v>12594.8158684558</v>
+        <v>5737.56304472693</v>
       </c>
       <c r="I39" s="16" t="n">
         <f aca="false">H39+I37</f>
-        <v>15602.5673473635</v>
+        <v>8389.47685626177</v>
       </c>
       <c r="J39" s="16" t="n">
         <f aca="false">I39+J37</f>
-        <v>18538.9841169492</v>
+        <v>11656.8491614407</v>
       </c>
       <c r="K39" s="16" t="n">
         <f aca="false">J39+K37</f>
-        <v>22162.965589501</v>
+        <v>15329.4093683145</v>
       </c>
       <c r="L39" s="16" t="n">
         <f aca="false">K39+L37</f>
-        <v>26296.6443056968</v>
+        <v>18629.3864184087</v>
       </c>
       <c r="M39" s="16" t="n">
         <f aca="false">L39+M37</f>
-        <v>30726.2689235876</v>
+        <v>21657.6213210452</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7432,51 +7432,51 @@
       </c>
       <c r="B40" s="16" t="n">
         <f aca="false">B38</f>
-        <v>-137.934312617702</v>
+        <v>-2096.39312617702</v>
       </c>
       <c r="C40" s="16" t="n">
         <f aca="false">B40+C38</f>
-        <v>2189.71135357816</v>
+        <v>-2750.32184557439</v>
       </c>
       <c r="D40" s="16" t="n">
         <f aca="false">C40+D38</f>
-        <v>2516.4791299435</v>
+        <v>-681.870107344631</v>
       </c>
       <c r="E40" s="16" t="n">
         <f aca="false">D40+E38</f>
-        <v>3476.36757156309</v>
+        <v>856.894986817329</v>
       </c>
       <c r="F40" s="16" t="n">
         <f aca="false">E40+F38</f>
-        <v>6959.14013182675</v>
+        <v>3062.96515725047</v>
       </c>
       <c r="G40" s="16" t="n">
         <f aca="false">F40+G38</f>
-        <v>9873.42488700565</v>
+        <v>4908.25667514125</v>
       </c>
       <c r="H40" s="16" t="n">
         <f aca="false">G40+H38</f>
-        <v>13364.2474684558</v>
+        <v>6487.09504472694</v>
       </c>
       <c r="I40" s="16" t="n">
         <f aca="false">H40+I38</f>
-        <v>16499.9141473635</v>
+        <v>9289.79305626178</v>
       </c>
       <c r="J40" s="16" t="n">
         <f aca="false">I40+J38</f>
-        <v>19563.8765169492</v>
+        <v>12725.0225614407</v>
       </c>
       <c r="K40" s="16" t="n">
         <f aca="false">J40+K38</f>
-        <v>23343.682189501</v>
+        <v>16572.8991683145</v>
       </c>
       <c r="L40" s="16" t="n">
         <f aca="false">K40+L38</f>
-        <v>27650.2581056968</v>
+        <v>20044.4126184087</v>
       </c>
       <c r="M40" s="16" t="n">
         <f aca="false">L40+M38</f>
-        <v>32260.2391235876</v>
+        <v>23301.8667210452</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7599,51 +7599,51 @@
       </c>
       <c r="B43" s="11" t="n">
         <f aca="false">Inversion!$B$34+Inversion!$B$52+B37+B42-B41</f>
-        <v>7330.53217644292</v>
+        <v>5379.63336288359</v>
       </c>
       <c r="C43" s="11" t="n">
         <f aca="false">B43+C37+C42-C41</f>
-        <v>8925.75533169939</v>
+        <v>4037.38213254684</v>
       </c>
       <c r="D43" s="11" t="n">
         <f aca="false">C43+D37+D42-D41</f>
-        <v>8557.22019712535</v>
+        <v>5384.54975983721</v>
       </c>
       <c r="E43" s="11" t="n">
         <f aca="false">D43+E37+E42-E41</f>
-        <v>8823.74612780555</v>
+        <v>6208.28034305978</v>
       </c>
       <c r="F43" s="11" t="n">
         <f aca="false">E43+F37+F42-F41</f>
-        <v>11575.1545771298</v>
+        <v>7694.20040255354</v>
       </c>
       <c r="G43" s="11" t="n">
         <f aca="false">F43+G37+G42-G41</f>
-        <v>13769.3648213693</v>
+        <v>8821.53420950493</v>
       </c>
       <c r="H43" s="11" t="n">
         <f aca="false">G43+H37+H42-H41</f>
-        <v>16534.9972918801</v>
+        <v>9677.74446815123</v>
       </c>
       <c r="I43" s="11" t="n">
         <f aca="false">H43+I37+I42-I41</f>
-        <v>18947.6662598484</v>
+        <v>11734.5757687467</v>
       </c>
       <c r="J43" s="11" t="n">
         <f aca="false">I43+J37+J42-J41</f>
-        <v>21289.0005184947</v>
+        <v>14406.8655629862</v>
       </c>
       <c r="K43" s="11" t="n">
         <f aca="false">J43+K37+K42-K41</f>
-        <v>24317.8994801071</v>
+        <v>17484.3432589206</v>
       </c>
       <c r="L43" s="11" t="n">
         <f aca="false">K43+L37+L42-L41</f>
-        <v>27856.4956853636</v>
+        <v>20189.2377980754</v>
       </c>
       <c r="M43" s="11" t="n">
         <f aca="false">L43+M37+M42-M41</f>
-        <v>31691.037792315</v>
+        <v>22622.3901897726</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Costeo v5: utilidad neta (intereses y renta RMT), carnés y uniformes del personal en administración
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Kfbf7cfV7pXUcNjjyaPCzV
</commit_message>
<xml_diff>
--- a/04-reformulacion/Costeo-presentaciones-AndiBite.xlsx
+++ b/04-reformulacion/Costeo-presentaciones-AndiBite.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="479" uniqueCount="327">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="486" uniqueCount="334">
   <si>
     <t xml:space="preserve">Cómo usar este archivo</t>
   </si>
@@ -151,7 +151,7 @@
     <t xml:space="preserve">Contribución (ventas sin IGV menos producción y costos variables de canal)</t>
   </si>
   <si>
-    <t xml:space="preserve">Stands, carritos y ferias del año (alquiler, impulsadoras y ferias pagadas)</t>
+    <t xml:space="preserve">Stands, carritos y ferias del año (espacio, vendedores de stand y ferias pagadas)</t>
   </si>
   <si>
     <t xml:space="preserve">Costos fijos del año</t>
@@ -184,6 +184,27 @@
     <t xml:space="preserve">Meses desde el inicio de ventas (mes 1 = enero de 2027) para recuperar la inversión (el año 2 al ritmo de los meses 10 a 12)</t>
   </si>
   <si>
+    <t xml:space="preserve">De resultado operativo a utilidad neta (año 1, opción B)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Resultado operativo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Más: pagos a cuenta de renta ya restados en el costo de canal (1 % de las ventas sin IGV)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Menos: intereses del préstamo en el año 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Utilidad antes de impuestos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Impuesto a la renta del Régimen MYPE Tributario (10 % hasta 15 UIT de utilidad)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Utilidad neta del año 1</t>
+  </si>
+  <si>
     <t xml:space="preserve">Notas</t>
   </si>
   <si>
@@ -196,7 +217,7 @@
     <t xml:space="preserve">3. Costo de producción con sangrecita fresca de pollo (S/0.40 de insumos por brownie) y maquila de S/0.45 por brownie.</t>
   </si>
   <si>
-    <t xml:space="preserve">4. El resultado incluye al personal que opera el negocio (vendedores de stand y coordinador). No incluye intereses del préstamo (hoja Inversion) ni el impuesto a la renta anual.</t>
+    <t xml:space="preserve">4. El resultado operativo ya incluye al personal que opera el negocio (vendedores de stand y coordinador en planilla). La utilidad neta descuenta además los intereses del préstamo y el impuesto a la renta (filas 29 a 34).</t>
   </si>
   <si>
     <t xml:space="preserve">Supuestos del costeo — AndiBite (maquila, escenario de 3,000 unidades al mes)</t>
@@ -481,10 +502,10 @@
     <t xml:space="preserve">8. Costos fijos mensuales (S/ sin IGV)</t>
   </si>
   <si>
-    <t xml:space="preserve">Administración: contador, software, web, teléfono, movilidad, banco</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Documento 05, sección 4.1</t>
+    <t xml:space="preserve">Administración: contador, software de facturación, web, teléfono, movilidad, GS1, banco, carnés de sanidad y uniformes del personal de stand</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Documento 05, sección 4.1 (S/700) más S/60 al mes de carnés de sanidad (S/9 a 20 por persona cada 6 meses), uniformes y reposición del material de stand</t>
   </si>
   <si>
     <t xml:space="preserve">Coordinador(a) comercial y de operaciones (planilla, medio tiempo de 4 horas)</t>
@@ -973,7 +994,7 @@
     <t xml:space="preserve">Contribución con pack de 6 opción C</t>
   </si>
   <si>
-    <t xml:space="preserve">Alquiler de espacios para stands y carritos</t>
+    <t xml:space="preserve">Espacio para stands y carrito</t>
   </si>
   <si>
     <t xml:space="preserve">Vendedores de stand (por día de atención)</t>
@@ -1717,7 +1738,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:G32"/>
+  <dimension ref="A1:G40"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="70"/>
@@ -1957,11 +1978,11 @@
       </c>
       <c r="B17" s="9" t="n">
         <f aca="false">Supuestos!B72*12</f>
-        <v>29320.6666666667</v>
+        <v>30040.6666666667</v>
       </c>
       <c r="C17" s="9" t="n">
         <f aca="false">Supuestos!B72*12</f>
-        <v>29320.6666666667</v>
+        <v>30040.6666666667</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1970,11 +1991,11 @@
       </c>
       <c r="B18" s="11" t="n">
         <f aca="false">B15-B16-B17</f>
-        <v>21657.6213210452</v>
+        <v>20937.6213210452</v>
       </c>
       <c r="C18" s="11" t="n">
         <f aca="false">C15-C16-C17</f>
-        <v>23301.8667210452</v>
+        <v>22581.8667210452</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1983,11 +2004,11 @@
       </c>
       <c r="B19" s="12" t="n">
         <f aca="false">IF(B14=0,0,B18/B14)</f>
-        <v>0.1107564821972</v>
+        <v>0.107074421919209</v>
       </c>
       <c r="C19" s="12" t="n">
         <f aca="false">IF(C14=0,0,C18/C14)</f>
-        <v>0.119165108134156</v>
+        <v>0.115483047856166</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2009,11 +2030,11 @@
       </c>
       <c r="B21" s="14" t="n">
         <f aca="false">IF(B20&lt;=0,"No alcanza",Supuestos!$B$72/B20)</f>
-        <v>2530.03250952598</v>
+        <v>2592.16013532549</v>
       </c>
       <c r="C21" s="14" t="n">
         <f aca="false">IF(C20&lt;=0,"No alcanza",Supuestos!$B$72/C20)</f>
-        <v>2450.97903095268</v>
+        <v>2511.16541492368</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2022,11 +2043,11 @@
       </c>
       <c r="B22" s="15" t="n">
         <f aca="false">IF(ISNUMBER(B21),B21/6,"No alcanza")</f>
-        <v>421.672084920997</v>
+        <v>432.026689220915</v>
       </c>
       <c r="C22" s="15" t="n">
         <f aca="false">IF(ISNUMBER(C21),C21/6,"No alcanza")</f>
-        <v>408.49650515878</v>
+        <v>418.527569153947</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2048,11 +2069,11 @@
       </c>
       <c r="B24" s="16" t="n">
         <f aca="false">B18-B23</f>
-        <v>-16236.6196789548</v>
+        <v>-16956.6196789548</v>
       </c>
       <c r="C24" s="16" t="n">
         <f aca="false">C18-C23</f>
-        <v>-14592.3742789548</v>
+        <v>-15312.3742789548</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2061,11 +2082,11 @@
       </c>
       <c r="B25" s="9" t="n">
         <f aca="false">MIN(Mensual!B43:M43)</f>
-        <v>4037.38213254684</v>
+        <v>3917.38213254684</v>
       </c>
       <c r="C25" s="9" t="n">
         <f aca="false">MIN(Mensual!B43:M43)</f>
-        <v>4037.38213254684</v>
+        <v>3917.38213254684</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2074,7 +2095,7 @@
       </c>
       <c r="B26" s="17" t="n">
         <f aca="false">IF(B18&gt;=B23,"Dentro del año 1",ROUNDUP(12+(B23-B18)/AVERAGE(Mensual!K37:M37),0))</f>
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C26" s="17" t="n">
         <f aca="false">IF(C18&gt;=C23,"Dentro del año 1",ROUNDUP(12+(C23-C18)/AVERAGE(Mensual!K38:M38),0))</f>
@@ -2090,20 +2111,79 @@
       <c r="A29" s="4" t="s">
         <v>53</v>
       </c>
+      <c r="B29" s="16" t="n">
+        <f aca="false">B18</f>
+        <v>20937.6213210452</v>
+      </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="4" t="s">
         <v>54</v>
       </c>
+      <c r="B30" s="9" t="n">
+        <f aca="false">Supuestos!B28*B14</f>
+        <v>1955.42697740113</v>
+      </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="4" t="s">
         <v>55</v>
       </c>
+      <c r="B31" s="9" t="n">
+        <f aca="false">-CUMIPMT((1+Inversion!B48)^(1/12)-1,Inversion!B49,Inversion!B47,1,12,0)</f>
+        <v>3221.74190432229</v>
+      </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="4" t="s">
         <v>56</v>
+      </c>
+      <c r="B32" s="16" t="n">
+        <f aca="false">B29+B30-B31</f>
+        <v>19671.306394124</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="B33" s="16" t="n">
+        <f aca="false">MAX(0,0.1*B32)</f>
+        <v>1967.13063941241</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="10" t="s">
+        <v>58</v>
+      </c>
+      <c r="B34" s="11" t="n">
+        <f aca="false">B32-B33</f>
+        <v>17704.1757547116</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="10" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="4" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="4" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="4" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="4" t="s">
+        <v>63</v>
       </c>
     </row>
   </sheetData>
@@ -2134,17 +2214,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
-        <v>58</v>
+        <v>65</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="18" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="B4" s="19"/>
       <c r="C4" s="19"/>
@@ -2152,161 +2232,161 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>61</v>
+        <v>68</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>62</v>
+        <v>69</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>63</v>
+        <v>70</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>64</v>
+        <v>71</v>
       </c>
       <c r="B6" s="20" t="n">
         <v>0.4</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>65</v>
+        <v>72</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>66</v>
+        <v>73</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>67</v>
+        <v>74</v>
       </c>
       <c r="B7" s="20" t="n">
         <v>0.45</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>65</v>
+        <v>72</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>68</v>
+        <v>75</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="B8" s="21" t="n">
         <v>0</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>65</v>
+        <v>72</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>70</v>
+        <v>77</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="B9" s="20" t="n">
         <v>0.09</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>65</v>
+        <v>72</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>72</v>
+        <v>79</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="B10" s="20" t="n">
         <v>0.25</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>65</v>
+        <v>72</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>74</v>
+        <v>81</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="B11" s="20" t="n">
         <v>0.01</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>65</v>
+        <v>72</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>76</v>
+        <v>83</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="B12" s="20" t="n">
         <v>0.083</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>65</v>
+        <v>72</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>78</v>
+        <v>85</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="B13" s="20" t="n">
         <v>0.053</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>65</v>
+        <v>72</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>80</v>
+        <v>87</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>81</v>
+        <v>88</v>
       </c>
       <c r="B14" s="20" t="n">
         <v>0.04</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>65</v>
+        <v>72</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="B15" s="22" t="n">
         <v>0.05</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>85</v>
+        <v>92</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="18" t="s">
-        <v>86</v>
+        <v>93</v>
       </c>
       <c r="B17" s="19"/>
       <c r="C17" s="19"/>
@@ -2314,77 +2394,77 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>61</v>
+        <v>68</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>62</v>
+        <v>69</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>63</v>
+        <v>70</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>87</v>
+        <v>94</v>
       </c>
       <c r="B19" s="23" t="n">
         <v>0.53</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>89</v>
+        <v>96</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>90</v>
+        <v>97</v>
       </c>
       <c r="B20" s="23" t="n">
         <v>0.72</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>91</v>
+        <v>98</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
-        <v>92</v>
+        <v>99</v>
       </c>
       <c r="B21" s="24" t="n">
         <v>0.7</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>93</v>
+        <v>100</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
-        <v>94</v>
+        <v>101</v>
       </c>
       <c r="B22" s="23" t="n">
         <v>0.72</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>95</v>
+        <v>102</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="18" t="s">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="B24" s="19"/>
       <c r="C24" s="19"/>
@@ -2392,63 +2472,63 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="5" t="s">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>61</v>
+        <v>68</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>62</v>
+        <v>69</v>
       </c>
       <c r="D25" s="5" t="s">
-        <v>63</v>
+        <v>70</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="s">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="B26" s="22" t="n">
         <v>0.18</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>98</v>
+        <v>105</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
-        <v>99</v>
+        <v>106</v>
       </c>
       <c r="B27" s="22" t="n">
         <v>0.03</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>100</v>
+        <v>107</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
-        <v>101</v>
+        <v>108</v>
       </c>
       <c r="B28" s="22" t="n">
         <v>0.01</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>102</v>
+        <v>109</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="18" t="s">
-        <v>103</v>
+        <v>110</v>
       </c>
       <c r="B30" s="19"/>
       <c r="C30" s="19"/>
@@ -2456,21 +2536,21 @@
     </row>
     <row r="31" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="5" t="s">
-        <v>104</v>
+        <v>111</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>105</v>
+        <v>112</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>106</v>
+        <v>113</v>
       </c>
       <c r="D31" s="5" t="s">
-        <v>107</v>
+        <v>114</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="4" t="s">
-        <v>108</v>
+        <v>115</v>
       </c>
       <c r="B32" s="23" t="n">
         <v>0.27</v>
@@ -2479,12 +2559,12 @@
         <v>1</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>109</v>
+        <v>116</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="4" t="s">
-        <v>110</v>
+        <v>117</v>
       </c>
       <c r="B33" s="23" t="n">
         <v>0.27</v>
@@ -2493,12 +2573,12 @@
         <v>1</v>
       </c>
       <c r="D33" s="4" t="s">
-        <v>111</v>
+        <v>118</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="4" t="s">
-        <v>112</v>
+        <v>119</v>
       </c>
       <c r="B34" s="23" t="n">
         <v>0.8</v>
@@ -2507,12 +2587,12 @@
         <v>1</v>
       </c>
       <c r="D34" s="4" t="s">
-        <v>113</v>
+        <v>120</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="4" t="s">
-        <v>114</v>
+        <v>121</v>
       </c>
       <c r="B35" s="23" t="n">
         <v>0.1</v>
@@ -2521,12 +2601,12 @@
         <v>0</v>
       </c>
       <c r="D35" s="4" t="s">
-        <v>115</v>
+        <v>122</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="4" t="s">
-        <v>116</v>
+        <v>123</v>
       </c>
       <c r="B36" s="23" t="n">
         <v>0.15</v>
@@ -2535,12 +2615,12 @@
         <v>0</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>117</v>
+        <v>124</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="18" t="s">
-        <v>118</v>
+        <v>125</v>
       </c>
       <c r="B38" s="19"/>
       <c r="C38" s="19"/>
@@ -2549,24 +2629,24 @@
     </row>
     <row r="39" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="5" t="s">
-        <v>104</v>
+        <v>111</v>
       </c>
       <c r="B39" s="5" t="s">
         <v>30</v>
       </c>
       <c r="C39" s="5" t="s">
-        <v>119</v>
+        <v>126</v>
       </c>
       <c r="D39" s="5" t="s">
         <v>33</v>
       </c>
       <c r="E39" s="5" t="s">
-        <v>107</v>
+        <v>114</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="4" t="s">
-        <v>108</v>
+        <v>115</v>
       </c>
       <c r="B40" s="26" t="n">
         <v>5.5</v>
@@ -2578,12 +2658,12 @@
         <v>48</v>
       </c>
       <c r="E40" s="4" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="4" t="s">
-        <v>110</v>
+        <v>117</v>
       </c>
       <c r="B41" s="26" t="n">
         <v>5.5</v>
@@ -2595,12 +2675,12 @@
         <v>48</v>
       </c>
       <c r="E41" s="4" t="s">
-        <v>121</v>
+        <v>128</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="4" t="s">
-        <v>112</v>
+        <v>119</v>
       </c>
       <c r="B42" s="26" t="n">
         <v>4</v>
@@ -2612,12 +2692,12 @@
         <v>46.9</v>
       </c>
       <c r="E42" s="4" t="s">
-        <v>122</v>
+        <v>129</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="4" t="s">
-        <v>114</v>
+        <v>121</v>
       </c>
       <c r="B43" s="26" t="n">
         <v>3</v>
@@ -2629,12 +2709,12 @@
         <v>0</v>
       </c>
       <c r="E43" s="4" t="s">
-        <v>123</v>
+        <v>130</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="4" t="s">
-        <v>116</v>
+        <v>123</v>
       </c>
       <c r="B44" s="26" t="n">
         <v>0</v>
@@ -2646,12 +2726,12 @@
         <v>0</v>
       </c>
       <c r="E44" s="4" t="s">
-        <v>124</v>
+        <v>131</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="18" t="s">
-        <v>125</v>
+        <v>132</v>
       </c>
       <c r="B46" s="19"/>
       <c r="C46" s="19"/>
@@ -2660,24 +2740,24 @@
     </row>
     <row r="47" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="5" t="s">
-        <v>104</v>
+        <v>111</v>
       </c>
       <c r="B47" s="5" t="s">
         <v>30</v>
       </c>
       <c r="C47" s="5" t="s">
-        <v>119</v>
+        <v>126</v>
       </c>
       <c r="D47" s="5" t="s">
         <v>33</v>
       </c>
       <c r="E47" s="5" t="s">
-        <v>126</v>
+        <v>133</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="4" t="s">
-        <v>108</v>
+        <v>115</v>
       </c>
       <c r="B48" s="27" t="n">
         <v>0.6</v>
@@ -2695,7 +2775,7 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="4" t="s">
-        <v>110</v>
+        <v>117</v>
       </c>
       <c r="B49" s="27" t="n">
         <v>0.7</v>
@@ -2713,7 +2793,7 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="4" t="s">
-        <v>112</v>
+        <v>119</v>
       </c>
       <c r="B50" s="27" t="n">
         <v>0.1</v>
@@ -2731,7 +2811,7 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="4" t="s">
-        <v>114</v>
+        <v>121</v>
       </c>
       <c r="B51" s="27" t="n">
         <v>1</v>
@@ -2749,7 +2829,7 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="4" t="s">
-        <v>116</v>
+        <v>123</v>
       </c>
       <c r="B52" s="27" t="n">
         <v>0</v>
@@ -2767,12 +2847,12 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="4" t="s">
-        <v>127</v>
+        <v>134</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="18" t="s">
-        <v>128</v>
+        <v>135</v>
       </c>
       <c r="B55" s="19"/>
       <c r="C55" s="19"/>
@@ -2780,133 +2860,133 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="5" t="s">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="B56" s="5" t="s">
-        <v>61</v>
+        <v>68</v>
       </c>
       <c r="C56" s="5" t="s">
-        <v>62</v>
+        <v>69</v>
       </c>
       <c r="D56" s="5" t="s">
-        <v>63</v>
+        <v>70</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="4" t="s">
-        <v>129</v>
+        <v>136</v>
       </c>
       <c r="B57" s="26" t="n">
         <v>600</v>
       </c>
       <c r="C57" s="4" t="s">
-        <v>130</v>
+        <v>137</v>
       </c>
       <c r="D57" s="4" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="4" t="s">
-        <v>132</v>
+        <v>139</v>
       </c>
       <c r="B58" s="26" t="n">
         <v>90</v>
       </c>
       <c r="C58" s="4" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="D58" s="4" t="s">
-        <v>134</v>
+        <v>141</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="4" t="s">
-        <v>135</v>
+        <v>142</v>
       </c>
       <c r="B59" s="25" t="n">
         <v>0</v>
       </c>
       <c r="C59" s="4" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="D59" s="4" t="s">
-        <v>137</v>
+        <v>144</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="4" t="s">
-        <v>138</v>
+        <v>145</v>
       </c>
       <c r="B60" s="26" t="n">
         <v>1800</v>
       </c>
       <c r="C60" s="4" t="s">
-        <v>139</v>
+        <v>146</v>
       </c>
       <c r="D60" s="4" t="s">
-        <v>140</v>
+        <v>147</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="4" t="s">
-        <v>141</v>
+        <v>148</v>
       </c>
       <c r="B61" s="28" t="n">
         <v>700</v>
       </c>
       <c r="C61" s="4" t="s">
-        <v>142</v>
+        <v>149</v>
       </c>
       <c r="D61" s="4" t="s">
-        <v>143</v>
+        <v>150</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="4" t="s">
-        <v>144</v>
+        <v>151</v>
       </c>
       <c r="B62" s="28" t="n">
         <v>150</v>
       </c>
       <c r="C62" s="4" t="s">
-        <v>142</v>
+        <v>149</v>
       </c>
       <c r="D62" s="4" t="s">
-        <v>145</v>
+        <v>152</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="4" t="s">
-        <v>146</v>
+        <v>153</v>
       </c>
       <c r="B63" s="27" t="n">
         <v>0.35</v>
       </c>
       <c r="C63" s="4" t="s">
-        <v>147</v>
+        <v>154</v>
       </c>
       <c r="D63" s="4" t="s">
-        <v>148</v>
+        <v>155</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="4" t="s">
-        <v>149</v>
+        <v>156</v>
       </c>
       <c r="B64" s="29" t="n">
         <v>150</v>
       </c>
       <c r="C64" s="4" t="s">
-        <v>142</v>
+        <v>149</v>
       </c>
       <c r="D64" s="4" t="s">
-        <v>145</v>
+        <v>152</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="18" t="s">
-        <v>150</v>
+        <v>157</v>
       </c>
       <c r="B66" s="19"/>
       <c r="C66" s="19"/>
@@ -2914,73 +2994,73 @@
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="5" t="s">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="B67" s="5" t="s">
-        <v>130</v>
+        <v>137</v>
       </c>
       <c r="C67" s="5"/>
       <c r="D67" s="5" t="s">
-        <v>63</v>
+        <v>70</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="4" t="s">
-        <v>151</v>
+        <v>158</v>
       </c>
       <c r="B68" s="26" t="n">
-        <v>700</v>
+        <v>760</v>
       </c>
       <c r="D68" s="4" t="s">
-        <v>152</v>
+        <v>159</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="4" t="s">
-        <v>153</v>
+        <v>160</v>
       </c>
       <c r="B69" s="26" t="n">
         <v>709</v>
       </c>
       <c r="D69" s="4" t="s">
-        <v>154</v>
+        <v>161</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="4" t="s">
-        <v>155</v>
+        <v>162</v>
       </c>
       <c r="B70" s="26" t="n">
         <v>900</v>
       </c>
       <c r="D70" s="4" t="s">
-        <v>156</v>
+        <v>163</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="4" t="s">
-        <v>157</v>
+        <v>164</v>
       </c>
       <c r="B71" s="6" t="n">
         <f aca="false">Inversion!B37/36</f>
         <v>134.388888888889</v>
       </c>
       <c r="D71" s="4" t="s">
-        <v>158</v>
+        <v>165</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="10" t="s">
-        <v>159</v>
+        <v>166</v>
       </c>
       <c r="B72" s="30" t="n">
         <f aca="false">SUM(B68:B71)</f>
-        <v>2443.38888888889</v>
+        <v>2503.38888888889</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="18" t="s">
-        <v>160</v>
+        <v>167</v>
       </c>
       <c r="B74" s="19"/>
       <c r="C74" s="19"/>
@@ -2988,30 +3068,30 @@
     </row>
     <row r="75" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="5" t="s">
-        <v>161</v>
+        <v>168</v>
       </c>
       <c r="B75" s="5" t="s">
-        <v>147</v>
+        <v>154</v>
       </c>
       <c r="C75" s="5"/>
       <c r="D75" s="5" t="s">
-        <v>107</v>
+        <v>114</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="4" t="s">
-        <v>162</v>
+        <v>169</v>
       </c>
       <c r="B76" s="22" t="n">
         <v>0.4</v>
       </c>
       <c r="D76" s="4" t="s">
-        <v>163</v>
+        <v>170</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="4" t="s">
-        <v>164</v>
+        <v>171</v>
       </c>
       <c r="B77" s="22" t="n">
         <v>0.35</v>
@@ -3020,7 +3100,7 @@
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="4" t="s">
-        <v>165</v>
+        <v>172</v>
       </c>
       <c r="B78" s="22" t="n">
         <v>0.25</v>
@@ -3029,7 +3109,7 @@
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="10" t="s">
-        <v>166</v>
+        <v>173</v>
       </c>
       <c r="B79" s="12" t="n">
         <f aca="false">SUM(B76:B78)</f>
@@ -3061,17 +3141,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>167</v>
+        <v>174</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
-        <v>168</v>
+        <v>175</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="B4" s="5" t="s">
         <v>30</v>
@@ -3083,12 +3163,12 @@
         <v>32</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>169</v>
+        <v>176</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>170</v>
+        <v>177</v>
       </c>
       <c r="B5" s="25" t="n">
         <v>1</v>
@@ -3105,7 +3185,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>171</v>
+        <v>178</v>
       </c>
       <c r="B6" s="6" t="n">
         <f aca="false">B5*Supuestos!$B$6</f>
@@ -3126,7 +3206,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>172</v>
+        <v>179</v>
       </c>
       <c r="B7" s="6" t="n">
         <f aca="false">B5*Supuestos!$B$7</f>
@@ -3147,7 +3227,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>173</v>
+        <v>180</v>
       </c>
       <c r="B8" s="6" t="n">
         <f aca="false">B5*Supuestos!$B$9</f>
@@ -3167,7 +3247,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>174</v>
+        <v>181</v>
       </c>
       <c r="B9" s="6" t="n">
         <f aca="false">Supuestos!$B$10</f>
@@ -3185,7 +3265,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>175</v>
+        <v>182</v>
       </c>
       <c r="B10" s="13" t="n">
         <v>0</v>
@@ -3203,7 +3283,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>176</v>
+        <v>183</v>
       </c>
       <c r="B11" s="13" t="n">
         <v>0</v>
@@ -3223,7 +3303,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>177</v>
+        <v>184</v>
       </c>
       <c r="B12" s="13" t="n">
         <v>0</v>
@@ -3243,7 +3323,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>178</v>
+        <v>185</v>
       </c>
       <c r="B13" s="13" t="n">
         <f aca="false">Supuestos!$B$15*SUM(B6:B12)</f>
@@ -3264,7 +3344,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>179</v>
+        <v>186</v>
       </c>
       <c r="B14" s="13" t="n">
         <f aca="false">B5*(Supuestos!$B$12+Supuestos!$B$13+Supuestos!$B$14)</f>
@@ -3285,7 +3365,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="10" t="s">
-        <v>180</v>
+        <v>187</v>
       </c>
       <c r="B15" s="30" t="n">
         <f aca="false">SUM(B6:B14)</f>
@@ -3306,7 +3386,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="10" t="s">
-        <v>181</v>
+        <v>188</v>
       </c>
       <c r="B16" s="30" t="n">
         <f aca="false">IF(B5=0,0,B15/B5)</f>
@@ -3327,12 +3407,12 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="10" t="s">
-        <v>182</v>
+        <v>189</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>183</v>
+        <v>190</v>
       </c>
       <c r="B19" s="6" t="n">
         <f aca="false">Supuestos!B40</f>
@@ -3353,7 +3433,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>184</v>
+        <v>191</v>
       </c>
       <c r="B20" s="13" t="n">
         <f aca="false">B19/(1+Supuestos!$B$26)</f>
@@ -3374,7 +3454,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
-        <v>185</v>
+        <v>192</v>
       </c>
       <c r="B21" s="13" t="n">
         <f aca="false">B20-B15</f>
@@ -3395,7 +3475,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
-        <v>186</v>
+        <v>193</v>
       </c>
       <c r="B22" s="12" t="n">
         <f aca="false">IF(B20=0,0,B21/B20)</f>
@@ -3416,12 +3496,12 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="10" t="s">
-        <v>187</v>
+        <v>194</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
-        <v>183</v>
+        <v>190</v>
       </c>
       <c r="B25" s="6" t="n">
         <f aca="false">Supuestos!B42</f>
@@ -3442,7 +3522,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="s">
-        <v>184</v>
+        <v>191</v>
       </c>
       <c r="B26" s="13" t="n">
         <f aca="false">B25/(1+Supuestos!$B$26)</f>
@@ -3463,7 +3543,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
-        <v>185</v>
+        <v>192</v>
       </c>
       <c r="B27" s="13" t="n">
         <f aca="false">B26-B15</f>
@@ -3484,7 +3564,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
-        <v>186</v>
+        <v>193</v>
       </c>
       <c r="B28" s="12" t="n">
         <f aca="false">IF(B26=0,0,B27/B26)</f>
@@ -3505,7 +3585,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="4" t="s">
-        <v>188</v>
+        <v>195</v>
       </c>
     </row>
   </sheetData>
@@ -3534,76 +3614,76 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>189</v>
+        <v>196</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
-        <v>190</v>
+        <v>197</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>104</v>
+        <v>111</v>
       </c>
       <c r="B4" s="5" t="s">
         <v>23</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>191</v>
+        <v>198</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>192</v>
+        <v>199</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>193</v>
+        <v>200</v>
       </c>
       <c r="F4" s="5" t="s">
         <v>37</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>194</v>
+        <v>201</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>195</v>
+        <v>202</v>
       </c>
       <c r="I4" s="5" t="s">
-        <v>196</v>
+        <v>203</v>
       </c>
       <c r="J4" s="5" t="s">
-        <v>197</v>
+        <v>204</v>
       </c>
       <c r="K4" s="5" t="s">
-        <v>198</v>
+        <v>205</v>
       </c>
       <c r="L4" s="5" t="s">
-        <v>199</v>
+        <v>206</v>
       </c>
       <c r="M4" s="5" t="s">
-        <v>200</v>
+        <v>207</v>
       </c>
       <c r="N4" s="5" t="s">
-        <v>201</v>
+        <v>208</v>
       </c>
       <c r="O4" s="5" t="s">
-        <v>202</v>
+        <v>209</v>
       </c>
       <c r="P4" s="5" t="s">
-        <v>203</v>
+        <v>210</v>
       </c>
       <c r="Q4" s="5" t="s">
-        <v>204</v>
+        <v>211</v>
       </c>
       <c r="R4" s="5" t="s">
-        <v>205</v>
+        <v>212</v>
       </c>
       <c r="S4" s="5" t="s">
-        <v>206</v>
+        <v>213</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>108</v>
+        <v>115</v>
       </c>
       <c r="B5" s="4" t="s">
         <v>30</v>
@@ -3679,10 +3759,10 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>108</v>
+        <v>115</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>119</v>
+        <v>126</v>
       </c>
       <c r="C6" s="17" t="n">
         <f aca="false">Costeo!C5</f>
@@ -3755,7 +3835,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>108</v>
+        <v>115</v>
       </c>
       <c r="B7" s="4" t="s">
         <v>33</v>
@@ -3831,7 +3911,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>110</v>
+        <v>117</v>
       </c>
       <c r="B8" s="4" t="s">
         <v>30</v>
@@ -3907,10 +3987,10 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>110</v>
+        <v>117</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>119</v>
+        <v>126</v>
       </c>
       <c r="C9" s="17" t="n">
         <f aca="false">Costeo!C5</f>
@@ -3983,7 +4063,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>110</v>
+        <v>117</v>
       </c>
       <c r="B10" s="4" t="s">
         <v>33</v>
@@ -4059,7 +4139,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>112</v>
+        <v>119</v>
       </c>
       <c r="B11" s="4" t="s">
         <v>30</v>
@@ -4135,10 +4215,10 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>112</v>
+        <v>119</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>119</v>
+        <v>126</v>
       </c>
       <c r="C12" s="17" t="n">
         <f aca="false">Costeo!C5</f>
@@ -4211,7 +4291,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>112</v>
+        <v>119</v>
       </c>
       <c r="B13" s="4" t="s">
         <v>33</v>
@@ -4287,7 +4367,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>114</v>
+        <v>121</v>
       </c>
       <c r="B14" s="4" t="s">
         <v>30</v>
@@ -4363,10 +4443,10 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>114</v>
+        <v>121</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>119</v>
+        <v>126</v>
       </c>
       <c r="C15" s="17" t="n">
         <f aca="false">Costeo!C5</f>
@@ -4439,7 +4519,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>114</v>
+        <v>121</v>
       </c>
       <c r="B16" s="4" t="s">
         <v>33</v>
@@ -4515,7 +4595,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>116</v>
+        <v>123</v>
       </c>
       <c r="B17" s="4" t="s">
         <v>30</v>
@@ -4591,10 +4671,10 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>116</v>
+        <v>123</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>119</v>
+        <v>126</v>
       </c>
       <c r="C18" s="17" t="n">
         <f aca="false">Costeo!C5</f>
@@ -4667,7 +4747,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>116</v>
+        <v>123</v>
       </c>
       <c r="B19" s="4" t="s">
         <v>33</v>
@@ -4743,7 +4823,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="10" t="s">
-        <v>207</v>
+        <v>214</v>
       </c>
       <c r="F20" s="31" t="n">
         <f aca="false">SUM(F5:F19)</f>
@@ -4768,7 +4848,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="18" t="s">
-        <v>208</v>
+        <v>215</v>
       </c>
       <c r="B23" s="19"/>
       <c r="C23" s="19"/>
@@ -4780,33 +4860,33 @@
     </row>
     <row r="24" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="5" t="s">
-        <v>104</v>
+        <v>111</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>209</v>
+        <v>216</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>210</v>
+        <v>217</v>
       </c>
       <c r="D24" s="5" t="s">
-        <v>211</v>
+        <v>218</v>
       </c>
       <c r="E24" s="5" t="s">
-        <v>196</v>
+        <v>203</v>
       </c>
       <c r="F24" s="5" t="s">
-        <v>212</v>
+        <v>219</v>
       </c>
       <c r="G24" s="5" t="s">
-        <v>213</v>
+        <v>220</v>
       </c>
       <c r="H24" s="5" t="s">
-        <v>214</v>
+        <v>221</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
-        <v>108</v>
+        <v>115</v>
       </c>
       <c r="B25" s="15" t="n">
         <f aca="false">SUMIF($A$5:$A$19,A25,$F$5:$F$19)</f>
@@ -4839,7 +4919,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="s">
-        <v>110</v>
+        <v>117</v>
       </c>
       <c r="B26" s="15" t="n">
         <f aca="false">SUMIF($A$5:$A$19,A26,$F$5:$F$19)</f>
@@ -4872,7 +4952,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
-        <v>112</v>
+        <v>119</v>
       </c>
       <c r="B27" s="15" t="n">
         <f aca="false">SUMIF($A$5:$A$19,A27,$F$5:$F$19)</f>
@@ -4905,7 +4985,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
-        <v>114</v>
+        <v>121</v>
       </c>
       <c r="B28" s="15" t="n">
         <f aca="false">SUMIF($A$5:$A$19,A28,$F$5:$F$19)</f>
@@ -4938,7 +5018,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="s">
-        <v>116</v>
+        <v>123</v>
       </c>
       <c r="B29" s="15" t="n">
         <f aca="false">SUMIF($A$5:$A$19,A29,$F$5:$F$19)</f>
@@ -4971,7 +5051,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="10" t="s">
-        <v>207</v>
+        <v>214</v>
       </c>
       <c r="B30" s="31" t="n">
         <f aca="false">SUM(B25:B29)</f>
@@ -5004,7 +5084,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="18" t="s">
-        <v>215</v>
+        <v>222</v>
       </c>
       <c r="B32" s="19"/>
       <c r="C32" s="19"/>
@@ -5019,22 +5099,22 @@
         <v>23</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>209</v>
+        <v>216</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>194</v>
+        <v>201</v>
       </c>
       <c r="D33" s="5" t="s">
-        <v>196</v>
+        <v>203</v>
       </c>
       <c r="E33" s="5" t="s">
-        <v>210</v>
+        <v>217</v>
       </c>
       <c r="F33" s="5" t="s">
-        <v>211</v>
+        <v>218</v>
       </c>
       <c r="G33" s="5" t="s">
-        <v>147</v>
+        <v>154</v>
       </c>
       <c r="H33" s="5"/>
     </row>
@@ -5069,7 +5149,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="4" t="s">
-        <v>119</v>
+        <v>126</v>
       </c>
       <c r="B35" s="15" t="n">
         <f aca="false">SUMIF($B$5:$B$19,A35,$F$5:$F$19)</f>
@@ -5127,7 +5207,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="18" t="s">
-        <v>216</v>
+        <v>223</v>
       </c>
       <c r="B38" s="19"/>
       <c r="C38" s="19"/>
@@ -5139,13 +5219,13 @@
     </row>
     <row r="39" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="5" t="s">
-        <v>161</v>
+        <v>168</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>147</v>
+        <v>154</v>
       </c>
       <c r="C39" s="5" t="s">
-        <v>217</v>
+        <v>224</v>
       </c>
       <c r="D39" s="5"/>
       <c r="E39" s="5"/>
@@ -5221,156 +5301,156 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>218</v>
+        <v>225</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
-        <v>219</v>
+        <v>226</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>220</v>
+        <v>227</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>63</v>
+        <v>70</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="18" t="s">
-        <v>221</v>
+        <v>228</v>
       </c>
       <c r="B5" s="19"/>
       <c r="C5" s="19"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>222</v>
+        <v>229</v>
       </c>
       <c r="B6" s="26" t="n">
         <v>150</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>223</v>
+        <v>230</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>224</v>
+        <v>231</v>
       </c>
       <c r="B7" s="26" t="n">
         <v>0</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>225</v>
+        <v>232</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>226</v>
+        <v>233</v>
       </c>
       <c r="B8" s="26" t="n">
         <v>401.2</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>227</v>
+        <v>234</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>228</v>
+        <v>235</v>
       </c>
       <c r="B9" s="26" t="n">
         <v>400</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>223</v>
+        <v>230</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>229</v>
+        <v>236</v>
       </c>
       <c r="B10" s="26" t="n">
         <v>1800</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>223</v>
+        <v>230</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>230</v>
+        <v>237</v>
       </c>
       <c r="B11" s="26" t="n">
         <v>1125</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>223</v>
+        <v>230</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>231</v>
+        <v>238</v>
       </c>
       <c r="B12" s="26" t="n">
         <v>1050</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>223</v>
+        <v>230</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>232</v>
+        <v>239</v>
       </c>
       <c r="B13" s="26" t="n">
         <v>650</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>223</v>
+        <v>230</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>233</v>
+        <v>240</v>
       </c>
       <c r="B14" s="26" t="n">
         <v>0</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>234</v>
+        <v>241</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>235</v>
+        <v>242</v>
       </c>
       <c r="B15" s="26" t="n">
         <v>75</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>236</v>
+        <v>243</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>237</v>
+        <v>244</v>
       </c>
       <c r="B16" s="33" t="n">
         <v>600</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>238</v>
+        <v>245</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="10" t="s">
-        <v>239</v>
+        <v>246</v>
       </c>
       <c r="B17" s="30" t="n">
         <f aca="false">SUM(B6:B16)</f>
@@ -5379,69 +5459,69 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="18" t="s">
-        <v>240</v>
+        <v>247</v>
       </c>
       <c r="B18" s="19"/>
       <c r="C18" s="19"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>241</v>
+        <v>248</v>
       </c>
       <c r="B19" s="26" t="n">
         <v>942.81</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>242</v>
+        <v>249</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>243</v>
+        <v>250</v>
       </c>
       <c r="B20" s="26" t="n">
         <v>148</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>223</v>
+        <v>230</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
-        <v>244</v>
+        <v>251</v>
       </c>
       <c r="B21" s="26" t="n">
         <v>750</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>223</v>
+        <v>230</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
-        <v>245</v>
+        <v>252</v>
       </c>
       <c r="B22" s="26" t="n">
         <v>150</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>223</v>
+        <v>230</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="4" t="s">
-        <v>246</v>
+        <v>253</v>
       </c>
       <c r="B23" s="33" t="n">
         <v>1750</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>247</v>
+        <v>254</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="10" t="s">
-        <v>248</v>
+        <v>255</v>
       </c>
       <c r="B24" s="30" t="n">
         <f aca="false">SUM(B19:B23)</f>
@@ -5450,47 +5530,47 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="18" t="s">
-        <v>249</v>
+        <v>256</v>
       </c>
       <c r="B25" s="19"/>
       <c r="C25" s="19"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="s">
-        <v>250</v>
+        <v>257</v>
       </c>
       <c r="B26" s="26" t="n">
         <v>800</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>223</v>
+        <v>230</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
-        <v>251</v>
+        <v>258</v>
       </c>
       <c r="B27" s="26" t="n">
         <v>300</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>223</v>
+        <v>230</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
-        <v>252</v>
+        <v>259</v>
       </c>
       <c r="B28" s="26" t="n">
         <v>150</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>223</v>
+        <v>230</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="10" t="s">
-        <v>253</v>
+        <v>260</v>
       </c>
       <c r="B29" s="30" t="n">
         <f aca="false">SUM(B26:B28)</f>
@@ -5499,58 +5579,58 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="18" t="s">
-        <v>254</v>
+        <v>261</v>
       </c>
       <c r="B30" s="19"/>
       <c r="C30" s="19"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="4" t="s">
-        <v>255</v>
+        <v>262</v>
       </c>
       <c r="B31" s="26" t="n">
         <v>3030</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>223</v>
+        <v>230</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="4" t="s">
-        <v>256</v>
+        <v>263</v>
       </c>
       <c r="B32" s="26" t="n">
         <v>4135.3</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>223</v>
+        <v>230</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="4" t="s">
-        <v>257</v>
+        <v>264</v>
       </c>
       <c r="B33" s="26" t="n">
         <v>3204</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>223</v>
+        <v>230</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="4" t="s">
-        <v>258</v>
+        <v>265</v>
       </c>
       <c r="B34" s="26" t="n">
         <v>8000</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>223</v>
+        <v>230</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="10" t="s">
-        <v>259</v>
+        <v>266</v>
       </c>
       <c r="B35" s="30" t="n">
         <f aca="false">SUM(B31:B34)</f>
@@ -5559,14 +5639,14 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="18" t="s">
-        <v>260</v>
+        <v>267</v>
       </c>
       <c r="B36" s="19"/>
       <c r="C36" s="19"/>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="10" t="s">
-        <v>261</v>
+        <v>268</v>
       </c>
       <c r="B37" s="30" t="n">
         <f aca="false">B38+B39</f>
@@ -5575,29 +5655,29 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="4" t="s">
-        <v>262</v>
+        <v>269</v>
       </c>
       <c r="B38" s="26" t="n">
         <v>2338</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>223</v>
+        <v>230</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="4" t="s">
-        <v>263</v>
+        <v>270</v>
       </c>
       <c r="B39" s="26" t="n">
         <v>2500</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>264</v>
+        <v>271</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="4" t="s">
-        <v>265</v>
+        <v>272</v>
       </c>
       <c r="B41" s="13" t="n">
         <f aca="false">0.1*(B17+B24+B29+B35+B37)</f>
@@ -5606,7 +5686,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="10" t="s">
-        <v>266</v>
+        <v>273</v>
       </c>
       <c r="B42" s="30" t="n">
         <f aca="false">B17+B24+B29+B35+B37+B41</f>
@@ -5615,70 +5695,70 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="18" t="s">
-        <v>267</v>
+        <v>274</v>
       </c>
       <c r="B44" s="19"/>
       <c r="C44" s="19"/>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="5" t="s">
-        <v>268</v>
+        <v>275</v>
       </c>
       <c r="B45" s="5" t="s">
-        <v>269</v>
+        <v>276</v>
       </c>
       <c r="C45" s="5" t="s">
-        <v>107</v>
+        <v>114</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="4" t="s">
-        <v>270</v>
+        <v>277</v>
       </c>
       <c r="B46" s="26" t="n">
         <v>25000</v>
       </c>
       <c r="C46" s="4" t="s">
-        <v>271</v>
+        <v>278</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="4" t="s">
-        <v>272</v>
+        <v>279</v>
       </c>
       <c r="B47" s="13" t="n">
         <f aca="false">MAX(0,CEILING(B42-B46,500))</f>
         <v>13000</v>
       </c>
       <c r="C47" s="4" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="4" t="s">
-        <v>274</v>
+        <v>281</v>
       </c>
       <c r="B48" s="27" t="n">
         <v>0.35</v>
       </c>
       <c r="C48" s="4" t="s">
-        <v>275</v>
+        <v>282</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="4" t="s">
-        <v>276</v>
+        <v>283</v>
       </c>
       <c r="B49" s="25" t="n">
         <v>24</v>
       </c>
       <c r="C49" s="4" t="s">
-        <v>277</v>
+        <v>284</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="4" t="s">
-        <v>278</v>
+        <v>285</v>
       </c>
       <c r="B50" s="13" t="n">
         <f aca="false">PMT((1+B48)^(1/12)-1,B49,-B47)</f>
@@ -5687,7 +5767,7 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="4" t="s">
-        <v>279</v>
+        <v>286</v>
       </c>
       <c r="B51" s="13" t="n">
         <f aca="false">B50*B49-B47</f>
@@ -5696,7 +5776,7 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="4" t="s">
-        <v>280</v>
+        <v>287</v>
       </c>
       <c r="B52" s="13" t="n">
         <f aca="false">B46+B47-B42</f>
@@ -5729,61 +5809,61 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>281</v>
+        <v>288</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
-        <v>282</v>
+        <v>289</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>283</v>
+        <v>290</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>284</v>
+        <v>291</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>285</v>
+        <v>292</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>286</v>
+        <v>293</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>287</v>
+        <v>294</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>288</v>
+        <v>295</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>289</v>
+        <v>296</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>290</v>
+        <v>297</v>
       </c>
       <c r="I4" s="5" t="s">
-        <v>291</v>
+        <v>298</v>
       </c>
       <c r="J4" s="5" t="s">
-        <v>292</v>
+        <v>299</v>
       </c>
       <c r="K4" s="5" t="s">
-        <v>293</v>
+        <v>300</v>
       </c>
       <c r="L4" s="5" t="s">
-        <v>294</v>
+        <v>301</v>
       </c>
       <c r="M4" s="5" t="s">
-        <v>295</v>
+        <v>302</v>
       </c>
       <c r="N4" s="5" t="s">
-        <v>296</v>
+        <v>303</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>297</v>
+        <v>304</v>
       </c>
       <c r="B5" s="25" t="n">
         <v>1</v>
@@ -5828,7 +5908,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>298</v>
+        <v>305</v>
       </c>
       <c r="B6" s="25" t="n">
         <v>9</v>
@@ -5873,7 +5953,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>299</v>
+        <v>306</v>
       </c>
       <c r="B7" s="25" t="n">
         <v>50</v>
@@ -5918,7 +5998,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>300</v>
+        <v>307</v>
       </c>
       <c r="B8" s="25" t="n">
         <v>0</v>
@@ -5963,7 +6043,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>301</v>
+        <v>308</v>
       </c>
       <c r="B9" s="25" t="n">
         <v>1</v>
@@ -6008,7 +6088,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>302</v>
+        <v>309</v>
       </c>
       <c r="B10" s="29" t="n">
         <v>0</v>
@@ -6053,7 +6133,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>303</v>
+        <v>310</v>
       </c>
       <c r="B11" s="29" t="n">
         <v>120</v>
@@ -6098,51 +6178,51 @@
     </row>
     <row r="13" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>304</v>
+        <v>311</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>284</v>
+        <v>291</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>285</v>
+        <v>292</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>286</v>
+        <v>293</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>287</v>
+        <v>294</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>288</v>
+        <v>295</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>289</v>
+        <v>296</v>
       </c>
       <c r="H13" s="5" t="s">
-        <v>290</v>
+        <v>297</v>
       </c>
       <c r="I13" s="5" t="s">
-        <v>291</v>
+        <v>298</v>
       </c>
       <c r="J13" s="5" t="s">
-        <v>292</v>
+        <v>299</v>
       </c>
       <c r="K13" s="5" t="s">
-        <v>293</v>
+        <v>300</v>
       </c>
       <c r="L13" s="5" t="s">
-        <v>294</v>
+        <v>301</v>
       </c>
       <c r="M13" s="5" t="s">
-        <v>295</v>
+        <v>302</v>
       </c>
       <c r="N13" s="5" t="s">
-        <v>296</v>
+        <v>303</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>108</v>
+        <v>115</v>
       </c>
       <c r="B14" s="15" t="n">
         <f aca="false">B5*B6*B7</f>
@@ -6199,7 +6279,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>110</v>
+        <v>117</v>
       </c>
       <c r="B15" s="15" t="n">
         <f aca="false">B8*Supuestos!$B$61+B9*Supuestos!$B$62</f>
@@ -6256,7 +6336,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>112</v>
+        <v>119</v>
       </c>
       <c r="B16" s="8" t="n">
         <f aca="false">Supuestos!$B$64</f>
@@ -6313,7 +6393,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>114</v>
+        <v>121</v>
       </c>
       <c r="B17" s="15" t="n">
         <f aca="false">B10</f>
@@ -6370,7 +6450,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>116</v>
+        <v>123</v>
       </c>
       <c r="B18" s="15" t="n">
         <f aca="false">B11</f>
@@ -6427,7 +6507,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="10" t="s">
-        <v>305</v>
+        <v>312</v>
       </c>
       <c r="B19" s="31" t="n">
         <f aca="false">SUM(B14:B18)</f>
@@ -6484,7 +6564,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="18" t="s">
-        <v>306</v>
+        <v>313</v>
       </c>
       <c r="B21" s="19"/>
       <c r="C21" s="19"/>
@@ -6502,7 +6582,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
-        <v>307</v>
+        <v>314</v>
       </c>
       <c r="B22" s="8" t="n">
         <f aca="false">SUMPRODUCT(B$14:B$18,Supuestos!$B$48:$B$52)</f>
@@ -6559,7 +6639,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="4" t="s">
-        <v>308</v>
+        <v>315</v>
       </c>
       <c r="B23" s="8" t="n">
         <f aca="false">SUMPRODUCT(B$14:B$18,Supuestos!$C$48:$C$52)</f>
@@ -6616,7 +6696,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="4" t="s">
-        <v>309</v>
+        <v>316</v>
       </c>
       <c r="B24" s="8" t="n">
         <f aca="false">SUMPRODUCT(B$14:B$18,Supuestos!$D$48:$D$52)</f>
@@ -6673,7 +6753,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
-        <v>310</v>
+        <v>317</v>
       </c>
       <c r="B25" s="15" t="n">
         <f aca="false">B23/Costeo!$C$5</f>
@@ -6730,7 +6810,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="s">
-        <v>311</v>
+        <v>318</v>
       </c>
       <c r="B26" s="15" t="n">
         <f aca="false">B24/Costeo!$E$5</f>
@@ -6787,7 +6867,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="18" t="s">
-        <v>312</v>
+        <v>319</v>
       </c>
       <c r="B28" s="19"/>
       <c r="C28" s="19"/>
@@ -6919,7 +6999,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="4" t="s">
-        <v>313</v>
+        <v>320</v>
       </c>
       <c r="B31" s="9" t="n">
         <f aca="false">SUMPRODUCT(B$14:B$18,Proyeccion!$F$25:$F$29)</f>
@@ -6976,7 +7056,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="4" t="s">
-        <v>314</v>
+        <v>321</v>
       </c>
       <c r="B32" s="9" t="n">
         <f aca="false">SUMPRODUCT(B$14:B$18,Proyeccion!$G$25:$G$29)</f>
@@ -7033,7 +7113,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="4" t="s">
-        <v>315</v>
+        <v>322</v>
       </c>
       <c r="B33" s="9" t="n">
         <f aca="false">B5*Supuestos!$B$57</f>
@@ -7090,7 +7170,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="4" t="s">
-        <v>316</v>
+        <v>323</v>
       </c>
       <c r="B34" s="9" t="n">
         <f aca="false">MAX(0,B5-Supuestos!$B$59)*B6*Supuestos!$B$58</f>
@@ -7147,7 +7227,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="4" t="s">
-        <v>317</v>
+        <v>324</v>
       </c>
       <c r="B35" s="9" t="n">
         <f aca="false">B8*Supuestos!$B$60</f>
@@ -7204,284 +7284,284 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="4" t="s">
-        <v>318</v>
+        <v>325</v>
       </c>
       <c r="B36" s="9" t="n">
         <f aca="false">Supuestos!$B$72</f>
-        <v>2443.38888888889</v>
+        <v>2503.38888888889</v>
       </c>
       <c r="C36" s="9" t="n">
         <f aca="false">Supuestos!$B$72</f>
-        <v>2443.38888888889</v>
+        <v>2503.38888888889</v>
       </c>
       <c r="D36" s="9" t="n">
         <f aca="false">Supuestos!$B$72</f>
-        <v>2443.38888888889</v>
+        <v>2503.38888888889</v>
       </c>
       <c r="E36" s="9" t="n">
         <f aca="false">Supuestos!$B$72</f>
-        <v>2443.38888888889</v>
+        <v>2503.38888888889</v>
       </c>
       <c r="F36" s="9" t="n">
         <f aca="false">Supuestos!$B$72</f>
-        <v>2443.38888888889</v>
+        <v>2503.38888888889</v>
       </c>
       <c r="G36" s="9" t="n">
         <f aca="false">Supuestos!$B$72</f>
-        <v>2443.38888888889</v>
+        <v>2503.38888888889</v>
       </c>
       <c r="H36" s="9" t="n">
         <f aca="false">Supuestos!$B$72</f>
-        <v>2443.38888888889</v>
+        <v>2503.38888888889</v>
       </c>
       <c r="I36" s="9" t="n">
         <f aca="false">Supuestos!$B$72</f>
-        <v>2443.38888888889</v>
+        <v>2503.38888888889</v>
       </c>
       <c r="J36" s="9" t="n">
         <f aca="false">Supuestos!$B$72</f>
-        <v>2443.38888888889</v>
+        <v>2503.38888888889</v>
       </c>
       <c r="K36" s="9" t="n">
         <f aca="false">Supuestos!$B$72</f>
-        <v>2443.38888888889</v>
+        <v>2503.38888888889</v>
       </c>
       <c r="L36" s="9" t="n">
         <f aca="false">Supuestos!$B$72</f>
-        <v>2443.38888888889</v>
+        <v>2503.38888888889</v>
       </c>
       <c r="M36" s="9" t="n">
         <f aca="false">Supuestos!$B$72</f>
-        <v>2443.38888888889</v>
+        <v>2503.38888888889</v>
       </c>
       <c r="N36" s="16" t="n">
         <f aca="false">SUM(B36:M36)</f>
-        <v>29320.6666666667</v>
+        <v>30040.6666666667</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="10" t="s">
-        <v>319</v>
+        <v>326</v>
       </c>
       <c r="B37" s="11" t="n">
         <f aca="false">B31-B33-B34-B35-B36</f>
-        <v>-2131.04312617702</v>
+        <v>-2191.04312617702</v>
       </c>
       <c r="C37" s="11" t="n">
         <f aca="false">C31-C33-C34-C35-C36</f>
-        <v>-747.168719397363</v>
+        <v>-807.168719397363</v>
       </c>
       <c r="D37" s="11" t="n">
         <f aca="false">D31-D33-D34-D35-D36</f>
-        <v>1942.25013822976</v>
+        <v>1882.25013822976</v>
       </c>
       <c r="E37" s="11" t="n">
         <f aca="false">E31-E33-E34-E35-E36</f>
-        <v>1418.81309416196</v>
+        <v>1358.81309416196</v>
       </c>
       <c r="F37" s="11" t="n">
         <f aca="false">F31-F33-F34-F35-F36</f>
-        <v>2081.00257043314</v>
+        <v>2021.00257043314</v>
       </c>
       <c r="G37" s="11" t="n">
         <f aca="false">G31-G33-G34-G35-G36</f>
-        <v>1722.41631789077</v>
+        <v>1662.41631789077</v>
       </c>
       <c r="H37" s="11" t="n">
         <f aca="false">H31-H33-H34-H35-H36</f>
-        <v>1451.29276958569</v>
+        <v>1391.29276958569</v>
       </c>
       <c r="I37" s="11" t="n">
         <f aca="false">I31-I33-I34-I35-I36</f>
-        <v>2651.91381153484</v>
+        <v>2591.91381153484</v>
       </c>
       <c r="J37" s="11" t="n">
         <f aca="false">J31-J33-J34-J35-J36</f>
-        <v>3267.37230517891</v>
+        <v>3207.37230517891</v>
       </c>
       <c r="K37" s="11" t="n">
         <f aca="false">K31-K33-K34-K35-K36</f>
-        <v>3672.56020687382</v>
+        <v>3612.56020687382</v>
       </c>
       <c r="L37" s="11" t="n">
         <f aca="false">L31-L33-L34-L35-L36</f>
-        <v>3299.97705009416</v>
+        <v>3239.97705009416</v>
       </c>
       <c r="M37" s="11" t="n">
         <f aca="false">M31-M33-M34-M35-M36</f>
-        <v>3028.23490263653</v>
+        <v>2968.23490263653</v>
       </c>
       <c r="N37" s="11" t="n">
         <f aca="false">SUM(B37:M37)</f>
-        <v>21657.6213210452</v>
+        <v>20937.6213210452</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="10" t="s">
-        <v>320</v>
+        <v>327</v>
       </c>
       <c r="B38" s="11" t="n">
         <f aca="false">B32-B33-B34-B35-B36</f>
-        <v>-2096.39312617702</v>
+        <v>-2156.39312617702</v>
       </c>
       <c r="C38" s="11" t="n">
         <f aca="false">C32-C33-C34-C35-C36</f>
-        <v>-653.928719397363</v>
+        <v>-713.928719397363</v>
       </c>
       <c r="D38" s="11" t="n">
         <f aca="false">D32-D33-D34-D35-D36</f>
-        <v>2068.45173822976</v>
+        <v>2008.45173822976</v>
       </c>
       <c r="E38" s="11" t="n">
         <f aca="false">E32-E33-E34-E35-E36</f>
-        <v>1538.76509416196</v>
+        <v>1478.76509416196</v>
       </c>
       <c r="F38" s="11" t="n">
         <f aca="false">F32-F33-F34-F35-F36</f>
-        <v>2206.07017043315</v>
+        <v>2146.07017043315</v>
       </c>
       <c r="G38" s="11" t="n">
         <f aca="false">G32-G33-G34-G35-G36</f>
-        <v>1845.29151789077</v>
+        <v>1785.29151789077</v>
       </c>
       <c r="H38" s="11" t="n">
         <f aca="false">H32-H33-H34-H35-H36</f>
-        <v>1578.83836958569</v>
+        <v>1518.83836958569</v>
       </c>
       <c r="I38" s="11" t="n">
         <f aca="false">I32-I33-I34-I35-I36</f>
-        <v>2802.69801153484</v>
+        <v>2742.69801153484</v>
       </c>
       <c r="J38" s="11" t="n">
         <f aca="false">J32-J33-J34-J35-J36</f>
-        <v>3435.22950517891</v>
+        <v>3375.22950517891</v>
       </c>
       <c r="K38" s="11" t="n">
         <f aca="false">K32-K33-K34-K35-K36</f>
-        <v>3847.87660687382</v>
+        <v>3787.87660687382</v>
       </c>
       <c r="L38" s="11" t="n">
         <f aca="false">L32-L33-L34-L35-L36</f>
-        <v>3471.51345009416</v>
+        <v>3411.51345009416</v>
       </c>
       <c r="M38" s="11" t="n">
         <f aca="false">M32-M33-M34-M35-M36</f>
-        <v>3257.45410263654</v>
+        <v>3197.45410263654</v>
       </c>
       <c r="N38" s="11" t="n">
         <f aca="false">SUM(B38:M38)</f>
-        <v>23301.8667210452</v>
+        <v>22581.8667210452</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="4" t="s">
-        <v>321</v>
+        <v>328</v>
       </c>
       <c r="B39" s="16" t="n">
         <f aca="false">B37</f>
-        <v>-2131.04312617702</v>
+        <v>-2191.04312617702</v>
       </c>
       <c r="C39" s="16" t="n">
         <f aca="false">B39+C37</f>
-        <v>-2878.21184557439</v>
+        <v>-2998.21184557439</v>
       </c>
       <c r="D39" s="16" t="n">
         <f aca="false">C39+D37</f>
-        <v>-935.961707344633</v>
+        <v>-1115.96170734463</v>
       </c>
       <c r="E39" s="16" t="n">
         <f aca="false">D39+E37</f>
-        <v>482.851386817326</v>
+        <v>242.851386817326</v>
       </c>
       <c r="F39" s="16" t="n">
         <f aca="false">E39+F37</f>
-        <v>2563.85395725047</v>
+        <v>2263.85395725047</v>
       </c>
       <c r="G39" s="16" t="n">
         <f aca="false">F39+G37</f>
-        <v>4286.27027514124</v>
+        <v>3926.27027514124</v>
       </c>
       <c r="H39" s="16" t="n">
         <f aca="false">G39+H37</f>
-        <v>5737.56304472693</v>
+        <v>5317.56304472693</v>
       </c>
       <c r="I39" s="16" t="n">
         <f aca="false">H39+I37</f>
-        <v>8389.47685626177</v>
+        <v>7909.47685626177</v>
       </c>
       <c r="J39" s="16" t="n">
         <f aca="false">I39+J37</f>
-        <v>11656.8491614407</v>
+        <v>11116.8491614407</v>
       </c>
       <c r="K39" s="16" t="n">
         <f aca="false">J39+K37</f>
-        <v>15329.4093683145</v>
+        <v>14729.4093683145</v>
       </c>
       <c r="L39" s="16" t="n">
         <f aca="false">K39+L37</f>
-        <v>18629.3864184087</v>
+        <v>17969.3864184087</v>
       </c>
       <c r="M39" s="16" t="n">
         <f aca="false">L39+M37</f>
-        <v>21657.6213210452</v>
+        <v>20937.6213210452</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="4" t="s">
-        <v>322</v>
+        <v>329</v>
       </c>
       <c r="B40" s="16" t="n">
         <f aca="false">B38</f>
-        <v>-2096.39312617702</v>
+        <v>-2156.39312617702</v>
       </c>
       <c r="C40" s="16" t="n">
         <f aca="false">B40+C38</f>
-        <v>-2750.32184557439</v>
+        <v>-2870.32184557439</v>
       </c>
       <c r="D40" s="16" t="n">
         <f aca="false">C40+D38</f>
-        <v>-681.870107344631</v>
+        <v>-861.870107344631</v>
       </c>
       <c r="E40" s="16" t="n">
         <f aca="false">D40+E38</f>
-        <v>856.894986817329</v>
+        <v>616.894986817329</v>
       </c>
       <c r="F40" s="16" t="n">
         <f aca="false">E40+F38</f>
-        <v>3062.96515725047</v>
+        <v>2762.96515725047</v>
       </c>
       <c r="G40" s="16" t="n">
         <f aca="false">F40+G38</f>
-        <v>4908.25667514125</v>
+        <v>4548.25667514125</v>
       </c>
       <c r="H40" s="16" t="n">
         <f aca="false">G40+H38</f>
-        <v>6487.09504472694</v>
+        <v>6067.09504472694</v>
       </c>
       <c r="I40" s="16" t="n">
         <f aca="false">H40+I38</f>
-        <v>9289.79305626178</v>
+        <v>8809.79305626178</v>
       </c>
       <c r="J40" s="16" t="n">
         <f aca="false">I40+J38</f>
-        <v>12725.0225614407</v>
+        <v>12185.0225614407</v>
       </c>
       <c r="K40" s="16" t="n">
         <f aca="false">J40+K38</f>
-        <v>16572.8991683145</v>
+        <v>15972.8991683145</v>
       </c>
       <c r="L40" s="16" t="n">
         <f aca="false">K40+L38</f>
-        <v>20044.4126184087</v>
+        <v>19384.4126184087</v>
       </c>
       <c r="M40" s="16" t="n">
         <f aca="false">L40+M38</f>
-        <v>23301.8667210452</v>
+        <v>22581.8667210452</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="4" t="s">
-        <v>323</v>
+        <v>330</v>
       </c>
       <c r="B41" s="9" t="n">
         <f aca="false">IF(1&lt;=Inversion!$B$49,Inversion!$B$50,0)</f>
@@ -7538,7 +7618,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="4" t="s">
-        <v>324</v>
+        <v>331</v>
       </c>
       <c r="B42" s="9" t="n">
         <f aca="false">Supuestos!$B$71</f>
@@ -7595,60 +7675,60 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="10" t="s">
-        <v>325</v>
+        <v>332</v>
       </c>
       <c r="B43" s="11" t="n">
         <f aca="false">Inversion!$B$34+Inversion!$B$52+B37+B42-B41</f>
-        <v>5379.63336288359</v>
+        <v>5319.63336288359</v>
       </c>
       <c r="C43" s="11" t="n">
         <f aca="false">B43+C37+C42-C41</f>
-        <v>4037.38213254684</v>
+        <v>3917.38213254684</v>
       </c>
       <c r="D43" s="11" t="n">
         <f aca="false">C43+D37+D42-D41</f>
-        <v>5384.54975983721</v>
+        <v>5204.54975983721</v>
       </c>
       <c r="E43" s="11" t="n">
         <f aca="false">D43+E37+E42-E41</f>
-        <v>6208.28034305978</v>
+        <v>5968.28034305978</v>
       </c>
       <c r="F43" s="11" t="n">
         <f aca="false">E43+F37+F42-F41</f>
-        <v>7694.20040255354</v>
+        <v>7394.20040255354</v>
       </c>
       <c r="G43" s="11" t="n">
         <f aca="false">F43+G37+G42-G41</f>
-        <v>8821.53420950493</v>
+        <v>8461.53420950493</v>
       </c>
       <c r="H43" s="11" t="n">
         <f aca="false">G43+H37+H42-H41</f>
-        <v>9677.74446815123</v>
+        <v>9257.74446815123</v>
       </c>
       <c r="I43" s="11" t="n">
         <f aca="false">H43+I37+I42-I41</f>
-        <v>11734.5757687467</v>
+        <v>11254.5757687467</v>
       </c>
       <c r="J43" s="11" t="n">
         <f aca="false">I43+J37+J42-J41</f>
-        <v>14406.8655629862</v>
+        <v>13866.8655629862</v>
       </c>
       <c r="K43" s="11" t="n">
         <f aca="false">J43+K37+K42-K41</f>
-        <v>17484.3432589206</v>
+        <v>16884.3432589206</v>
       </c>
       <c r="L43" s="11" t="n">
         <f aca="false">K43+L37+L42-L41</f>
-        <v>20189.2377980754</v>
+        <v>19529.2377980754</v>
       </c>
       <c r="M43" s="11" t="n">
         <f aca="false">L43+M37+M42-M41</f>
-        <v>22622.3901897726</v>
+        <v>21902.3901897726</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="4" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Costeo v6: sangrecita de res en polvo, precios nuevos y app Andi, Misión Hierro
Insumos S/0.605 por brownie con polvo liofilizado a granel; unidad S/6.00 y packs S/27.90 / S/51.90 (WhatsApp S/26.90 / S/49.90); app S/6,000 de inversión y S/250 al mes; código único por envase S/0.04; hierro medido por lote en control de calidad.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Kfbf7cfV7pXUcNjjyaPCzV
</commit_message>
<xml_diff>
--- a/04-reformulacion/Costeo-presentaciones-AndiBite.xlsx
+++ b/04-reformulacion/Costeo-presentaciones-AndiBite.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="486" uniqueCount="334">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="486" uniqueCount="337">
   <si>
     <t xml:space="preserve">Cómo usar este archivo</t>
   </si>
@@ -214,7 +214,7 @@
     <t xml:space="preserve">2. La venta física (stands, carritos y ferias) es el canal principal; WhatsApp queda para la recompra, sin suscripción. Todos los puntos de venta llevan vendedor(a) pagado(a) y un(a) coordinador(a) en planilla atiende pedidos y despacho.</t>
   </si>
   <si>
-    <t xml:space="preserve">3. Costo de producción con sangrecita fresca de pollo (S/0.40 de insumos por brownie) y maquila de S/0.45 por brownie.</t>
+    <t xml:space="preserve">3. Costo de producción con sangrecita de res en polvo liofilizada (S/0.605 de insumos por brownie, polvo a S/300 por kg a granel) y maquila de S/0.45 por brownie. Cada envase trae un código único de la app Andi, Misión Hierro.</t>
   </si>
   <si>
     <t xml:space="preserve">4. El resultado operativo ya incluye al personal que opera el negocio (vendedores de stand y coordinador en planilla). La utilidad neta descuenta además los intereses del préstamo y el impuesto a la renta (filas 29 a 34).</t>
@@ -241,16 +241,16 @@
     <t xml:space="preserve">Fuente o nota</t>
   </si>
   <si>
-    <t xml:space="preserve">Insumos por unidad (promedio de los 3 sabores, con sangrecita fresca de pollo cocida en la planta)</t>
+    <t xml:space="preserve">Insumos por unidad (promedio de los 3 sabores, con sangrecita de res en polvo liofilizada)</t>
   </si>
   <si>
     <t xml:space="preserve">S/ por unidad</t>
   </si>
   <si>
-    <t xml:space="preserve">Recetas del documento 01: 175 g de sangrecita cruda por lote de 24 (Redondos, S/11.29 por kg en Makro), que la planta cuece y licúa con los huevos; resto de insumos según documento 05 (Makro, mayoristas, Plaza Vea y Wong, sin IGV)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Maquila por unidad (la planta cuece la sangrecita, mezcla, hornea, corta, pesa y sella la bolsita)</t>
+    <t xml:space="preserve">Receta 5 del documento 01: 22 g de sangrecita en polvo + 98 g de agua por lote de 24 (0.92 g de polvo por brownie). Polvo de res liofilizado con registro sanitario, comprado a granel en bolsas de 1 a 5 kg a S/300 por kg (en sobre de tienda cuesta S/417 a 667 por kg: Malli, Allpa Manta). Resto de insumos según documento 05 (Makro, mayoristas, Plaza Vea y Wong, sin IGV)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Maquila por unidad (la planta hidrata la sangrecita en polvo, mezcla, hornea, corta, pesa y sella la bolsita)</t>
   </si>
   <si>
     <t xml:space="preserve">Tarifa de maquila de snacks horneados en Lima: S/20.75 por kg de producto terminado, elaboración y empaque incluidos (Organic Andean Bites, documento 03), actualizada a 2027: S/0.45 por brownie de 20 g</t>
@@ -268,10 +268,10 @@
     <t xml:space="preserve">Documento 05, tabla 4.2</t>
   </si>
   <si>
-    <t xml:space="preserve">Etiqueta individual con rotulado completo (solo unidad que se vende suelta)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Imprenta Peruana, 1,000 unidades sin IGV (documento 02)</t>
+    <t xml:space="preserve">Etiqueta individual con rotulado completo y código único de la app (solo unidad que se vende suelta)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Imprenta Peruana, 1,000 unidades sin IGV (documento 02): S/0.25, más S/0.04 por el código único impreso con dato variable (QR de la app Andi, Misión Hierro)</t>
   </si>
   <si>
     <t xml:space="preserve">Papel manteca separador entre brownies (opción C)</t>
@@ -280,10 +280,10 @@
     <t xml:space="preserve">[HIPÓTESIS] Rollo de supermercado prorrateado</t>
   </si>
   <si>
-    <t xml:space="preserve">Control de calidad por lote, prorrateado por unidad</t>
-  </si>
-  <si>
-    <t xml:space="preserve">S/250 por análisis microbiológico al mes / 3,000 unidades (documento 05)</t>
+    <t xml:space="preserve">Control de calidad por lote (microbiológico y hierro medido), prorrateado por unidad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cada lote mensual: análisis microbiológico S/250 (documento 05) + hierro por lote S/375 (el resultado se publica en la app) = S/625 / 4,400 unidades al mes en promedio del año 1</t>
   </si>
   <si>
     <t xml:space="preserve">Transporte planta-almacén por unidad</t>
@@ -319,10 +319,10 @@
     <t xml:space="preserve">S/0.625 con IGV por 1,000 unidades (documento 02)</t>
   </si>
   <si>
-    <t xml:space="preserve">Etiquetas del doypack de 6 (frente y reverso)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2 x S/0.36, 1,000 unidades (documento 02)</t>
+    <t xml:space="preserve">Etiquetas del doypack de 6 (frente y reverso, con código único de la app)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2 x S/0.36, 1,000 unidades (documento 02), más S/0.04 del código único de la app</t>
   </si>
   <si>
     <t xml:space="preserve">Doypack kraft para 12 unidades</t>
@@ -331,7 +331,7 @@
     <t xml:space="preserve">[HIPÓTESIS] Talla mayor; cotizar</t>
   </si>
   <si>
-    <t xml:space="preserve">Etiquetas del doypack de 12 (frente y reverso)</t>
+    <t xml:space="preserve">Etiquetas del doypack de 12 (frente y reverso, con código único de la app)</t>
   </si>
   <si>
     <t xml:space="preserve">Mismo sticker que el pack de 6</t>
@@ -409,13 +409,13 @@
     <t xml:space="preserve">Pack de 6</t>
   </si>
   <si>
-    <t xml:space="preserve">Precio de lista en físico. La unidad suelta (S/5.50) es la compra de prueba y deja más margen; el pack de 6 (S/4.33 por brownie) queda como la compra conveniente</t>
+    <t xml:space="preserve">Precio de lista en físico. La unidad suelta (S/6.00) es la compra de prueba y deja más margen; el pack de 6 (S/4.65 por brownie) es la compra conveniente. Incluye hierro medido por lote y la app Andi, Misión Hierro</t>
   </si>
   <si>
     <t xml:space="preserve">Mismo precio que en el stand</t>
   </si>
   <si>
-    <t xml:space="preserve">S/4.15 por brownie en el pack de 6, a la par de Fika (S/4.00) y Mamalama (S/4.10) por 20 g. Unidad = caja degustación de 3 (S/12.00)</t>
+    <t xml:space="preserve">S/4.48 por brownie en el pack de 6 (Fika S/4.00 y Mamalama S/4.10 por 20 g no miden su hierro ni traen app). Unidad = caja degustación de 3 (S/12.00)</t>
   </si>
   <si>
     <t xml:space="preserve">El alumno paga S/4.00; el concesionario se queda 25 %</t>
@@ -502,10 +502,10 @@
     <t xml:space="preserve">8. Costos fijos mensuales (S/ sin IGV)</t>
   </si>
   <si>
-    <t xml:space="preserve">Administración: contador, software de facturación, web, teléfono, movilidad, GS1, banco, carnés de sanidad y uniformes del personal de stand</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Documento 05, sección 4.1 (S/700) más S/60 al mes de carnés de sanidad (S/9 a 20 por persona cada 6 meses), uniformes y reposición del material de stand</t>
+    <t xml:space="preserve">Administración: contador, software de facturación, web, teléfono, movilidad, GS1, banco, carnés de sanidad, uniformes del personal de stand y app (servidor, base de datos y mantenimiento)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Documento 05, sección 4.1 (S/700) más S/60 al mes de carnés de sanidad (S/9 a 20 por persona cada 6 meses), uniformes y reposición del material de stand, más S/250 al mes de la app (Cloud Run y Firestore de Google, envío de recordatorios y mantenimiento de un desarrollador)</t>
   </si>
   <si>
     <t xml:space="preserve">Coordinador(a) comercial y de operaciones (planilla, medio tiempo de 4 horas)</t>
@@ -796,7 +796,7 @@
     <t xml:space="preserve">Subtotal desarrollo</t>
   </si>
   <si>
-    <t xml:space="preserve">3. Marca y puntos de venta</t>
+    <t xml:space="preserve">3. Marca, app y puntos de venta</t>
   </si>
   <si>
     <t xml:space="preserve">Identidad de marca</t>
@@ -805,7 +805,10 @@
     <t xml:space="preserve">Fotos de producto</t>
   </si>
   <si>
-    <t xml:space="preserve">Web y dominio</t>
+    <t xml:space="preserve">Web, dominio y app Andi, Misión Hierro (diseño, desarrollo, pruebas y publicación)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Web y dominio S/150 (documento 05) más S/6,000 de la app web instalable (PWA) para padres y niños, con desarrollador freelance (documento 09)</t>
   </si>
   <si>
     <t xml:space="preserve">Subtotal marca</t>
@@ -817,7 +820,13 @@
     <t xml:space="preserve">Empaque inicial (mínimos de compra)</t>
   </si>
   <si>
+    <t xml:space="preserve">Documento 05, más S/120 de los códigos únicos de la app en las primeras 3,000 etiquetas</t>
+  </si>
+  <si>
     <t xml:space="preserve">Stock inicial para enero y febrero</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Documento 05, actualizado al costo con sangrecita en polvo (pack de 6 de S/8.29 a S/9.62)</t>
   </si>
   <si>
     <t xml:space="preserve">Marketing de lanzamiento (degustaciones, influencers, POP)</t>
@@ -1784,19 +1793,19 @@
       </c>
       <c r="B5" s="6" t="n">
         <f aca="false">Costeo!B15</f>
-        <v>1.4255</v>
+        <v>1.74175</v>
       </c>
       <c r="C5" s="6" t="n">
         <f aca="false">Costeo!B16</f>
-        <v>1.4255</v>
+        <v>1.74175</v>
       </c>
       <c r="D5" s="6" t="n">
         <f aca="false">Costeo!B19</f>
-        <v>5.5</v>
+        <v>6</v>
       </c>
       <c r="E5" s="7" t="n">
         <f aca="false">Costeo!B22</f>
-        <v>0.694165454545455</v>
+        <v>0.657455833333333</v>
       </c>
       <c r="F5" s="6" t="n">
         <f aca="false">Costeo!B25</f>
@@ -1804,7 +1813,7 @@
       </c>
       <c r="G5" s="7" t="n">
         <f aca="false">Costeo!B28</f>
-        <v>0.5794775</v>
+        <v>0.48618375</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1813,27 +1822,27 @@
       </c>
       <c r="B6" s="6" t="n">
         <f aca="false">Costeo!C15</f>
-        <v>8.2905</v>
+        <v>9.978</v>
       </c>
       <c r="C6" s="6" t="n">
         <f aca="false">Costeo!C16</f>
-        <v>1.38175</v>
+        <v>1.663</v>
       </c>
       <c r="D6" s="6" t="n">
         <f aca="false">Costeo!C19</f>
-        <v>26</v>
+        <v>27.9</v>
       </c>
       <c r="E6" s="7" t="n">
         <f aca="false">Costeo!C22</f>
-        <v>0.623738846153846</v>
+        <v>0.577991397849462</v>
       </c>
       <c r="F6" s="6" t="n">
         <f aca="false">Costeo!C25</f>
-        <v>24.9</v>
+        <v>26.9</v>
       </c>
       <c r="G6" s="7" t="n">
         <f aca="false">Costeo!C28</f>
-        <v>0.60711686746988</v>
+        <v>0.562303345724907</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1842,27 +1851,27 @@
       </c>
       <c r="B7" s="6" t="n">
         <f aca="false">Costeo!D15</f>
-        <v>7.7865</v>
+        <v>9.474</v>
       </c>
       <c r="C7" s="6" t="n">
         <f aca="false">Costeo!D16</f>
-        <v>1.29775</v>
+        <v>1.579</v>
       </c>
       <c r="D7" s="6" t="n">
         <f aca="false">Costeo!D19</f>
-        <v>26</v>
+        <v>27.9</v>
       </c>
       <c r="E7" s="7" t="n">
         <f aca="false">Costeo!D22</f>
-        <v>0.646612692307692</v>
+        <v>0.59930752688172</v>
       </c>
       <c r="F7" s="6" t="n">
         <f aca="false">Costeo!D25</f>
-        <v>24.9</v>
+        <v>26.9</v>
       </c>
       <c r="G7" s="7" t="n">
         <f aca="false">Costeo!D28</f>
-        <v>0.631001204819277</v>
+        <v>0.584411895910781</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1871,27 +1880,27 @@
       </c>
       <c r="B8" s="6" t="n">
         <f aca="false">Costeo!E15</f>
-        <v>15.447</v>
+        <v>18.78</v>
       </c>
       <c r="C8" s="6" t="n">
         <f aca="false">Costeo!E16</f>
-        <v>1.28725</v>
+        <v>1.565</v>
       </c>
       <c r="D8" s="6" t="n">
         <f aca="false">Costeo!E19</f>
-        <v>48</v>
+        <v>51.9</v>
       </c>
       <c r="E8" s="7" t="n">
         <f aca="false">Costeo!E22</f>
-        <v>0.62026125</v>
+        <v>0.573017341040462</v>
       </c>
       <c r="F8" s="6" t="n">
         <f aca="false">Costeo!E25</f>
-        <v>46.9</v>
+        <v>49.9</v>
       </c>
       <c r="G8" s="7" t="n">
         <f aca="false">Costeo!E28</f>
-        <v>0.611354797441365</v>
+        <v>0.55590380761523</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1926,11 +1935,11 @@
       </c>
       <c r="B13" s="9" t="n">
         <f aca="false">Proyeccion!I20</f>
-        <v>230740.383333333</v>
+        <v>246531.04375</v>
       </c>
       <c r="C13" s="9" t="n">
         <f aca="false">Proyeccion!I20</f>
-        <v>230740.383333333</v>
+        <v>246531.04375</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1939,11 +1948,11 @@
       </c>
       <c r="B14" s="9" t="n">
         <f aca="false">Proyeccion!J20</f>
-        <v>195542.697740113</v>
+        <v>208924.613347458</v>
       </c>
       <c r="C14" s="9" t="n">
         <f aca="false">Proyeccion!J20</f>
-        <v>195542.697740113</v>
+        <v>208924.613347458</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1952,11 +1961,11 @@
       </c>
       <c r="B15" s="9" t="n">
         <f aca="false">Proyeccion!P20</f>
-        <v>96848.2879877119</v>
+        <v>93763.7303014831</v>
       </c>
       <c r="C15" s="9" t="n">
         <f aca="false">Proyeccion!Q20</f>
-        <v>98492.5333877119</v>
+        <v>95407.9757014831</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1978,11 +1987,11 @@
       </c>
       <c r="B17" s="9" t="n">
         <f aca="false">Supuestos!B72*12</f>
-        <v>30040.6666666667</v>
+        <v>33040.6666666667</v>
       </c>
       <c r="C17" s="9" t="n">
         <f aca="false">Supuestos!B72*12</f>
-        <v>30040.6666666667</v>
+        <v>33040.6666666667</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1991,11 +2000,11 @@
       </c>
       <c r="B18" s="11" t="n">
         <f aca="false">B15-B16-B17</f>
-        <v>20937.6213210452</v>
+        <v>14853.0636348164</v>
       </c>
       <c r="C18" s="11" t="n">
         <f aca="false">C15-C16-C17</f>
-        <v>22581.8667210452</v>
+        <v>16497.3090348164</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2004,11 +2013,11 @@
       </c>
       <c r="B19" s="12" t="n">
         <f aca="false">IF(B14=0,0,B18/B14)</f>
-        <v>0.107074421919209</v>
+        <v>0.0710929334597576</v>
       </c>
       <c r="C19" s="12" t="n">
         <f aca="false">IF(C14=0,0,C18/C14)</f>
-        <v>0.115483047856166</v>
+        <v>0.0789629750678543</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2017,11 +2026,11 @@
       </c>
       <c r="B20" s="13" t="n">
         <f aca="false">IF(B12=0,0,(B15-B16)/B12)</f>
-        <v>0.96575394967817</v>
+        <v>0.907318802362048</v>
       </c>
       <c r="C20" s="13" t="n">
         <f aca="false">IF(C12=0,0,(C15-C16)/C12)</f>
-        <v>0.996903220318112</v>
+        <v>0.93846807300199</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2030,11 +2039,11 @@
       </c>
       <c r="B21" s="14" t="n">
         <f aca="false">IF(B20&lt;=0,"No alcanza",Supuestos!$B$72/B20)</f>
-        <v>2592.16013532549</v>
+        <v>3034.64326069394</v>
       </c>
       <c r="C21" s="14" t="n">
         <f aca="false">IF(C20&lt;=0,"No alcanza",Supuestos!$B$72/C20)</f>
-        <v>2511.16541492368</v>
+        <v>2933.91855098628</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2043,11 +2052,11 @@
       </c>
       <c r="B22" s="15" t="n">
         <f aca="false">IF(ISNUMBER(B21),B21/6,"No alcanza")</f>
-        <v>432.026689220915</v>
+        <v>505.773876782324</v>
       </c>
       <c r="C22" s="15" t="n">
         <f aca="false">IF(ISNUMBER(C21),C21/6,"No alcanza")</f>
-        <v>418.527569153947</v>
+        <v>488.986425164381</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2056,11 +2065,11 @@
       </c>
       <c r="B23" s="9" t="n">
         <f aca="false">Inversion!B42</f>
-        <v>37894.241</v>
+        <v>45358.181</v>
       </c>
       <c r="C23" s="9" t="n">
         <f aca="false">Inversion!B42</f>
-        <v>37894.241</v>
+        <v>45358.181</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2069,11 +2078,11 @@
       </c>
       <c r="B24" s="16" t="n">
         <f aca="false">B18-B23</f>
-        <v>-16956.6196789548</v>
+        <v>-30505.1173651836</v>
       </c>
       <c r="C24" s="16" t="n">
         <f aca="false">C18-C23</f>
-        <v>-15312.3742789548</v>
+        <v>-28860.8719651836</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2082,11 +2091,11 @@
       </c>
       <c r="B25" s="9" t="n">
         <f aca="false">MIN(Mensual!B43:M43)</f>
-        <v>3917.38213254684</v>
+        <v>2649.79051817523</v>
       </c>
       <c r="C25" s="9" t="n">
         <f aca="false">MIN(Mensual!B43:M43)</f>
-        <v>3917.38213254684</v>
+        <v>2649.79051817523</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2095,11 +2104,11 @@
       </c>
       <c r="B26" s="17" t="n">
         <f aca="false">IF(B18&gt;=B23,"Dentro del año 1",ROUNDUP(12+(B23-B18)/AVERAGE(Mensual!K37:M37),0))</f>
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="C26" s="17" t="n">
         <f aca="false">IF(C18&gt;=C23,"Dentro del año 1",ROUNDUP(12+(C23-C18)/AVERAGE(Mensual!K38:M38),0))</f>
-        <v>17</v>
+        <v>23</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2113,7 +2122,7 @@
       </c>
       <c r="B29" s="16" t="n">
         <f aca="false">B18</f>
-        <v>20937.6213210452</v>
+        <v>14853.0636348164</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2122,7 +2131,7 @@
       </c>
       <c r="B30" s="9" t="n">
         <f aca="false">Supuestos!B28*B14</f>
-        <v>1955.42697740113</v>
+        <v>2089.24613347458</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2131,7 +2140,7 @@
       </c>
       <c r="B31" s="9" t="n">
         <f aca="false">-CUMIPMT((1+Inversion!B48)^(1/12)-1,Inversion!B49,Inversion!B47,1,12,0)</f>
-        <v>3221.74190432229</v>
+        <v>5080.43915681592</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2140,7 +2149,7 @@
       </c>
       <c r="B32" s="16" t="n">
         <f aca="false">B29+B30-B31</f>
-        <v>19671.306394124</v>
+        <v>11861.8706114751</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2149,7 +2158,7 @@
       </c>
       <c r="B33" s="16" t="n">
         <f aca="false">MAX(0,0.1*B32)</f>
-        <v>1967.13063941241</v>
+        <v>1186.18706114751</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2158,7 +2167,7 @@
       </c>
       <c r="B34" s="11" t="n">
         <f aca="false">B32-B33</f>
-        <v>17704.1757547116</v>
+        <v>10675.6835503275</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2249,7 +2258,7 @@
         <v>71</v>
       </c>
       <c r="B6" s="20" t="n">
-        <v>0.4</v>
+        <v>0.605</v>
       </c>
       <c r="C6" s="4" t="s">
         <v>72</v>
@@ -2305,7 +2314,7 @@
         <v>80</v>
       </c>
       <c r="B10" s="20" t="n">
-        <v>0.25</v>
+        <v>0.29</v>
       </c>
       <c r="C10" s="4" t="s">
         <v>72</v>
@@ -2333,7 +2342,7 @@
         <v>84</v>
       </c>
       <c r="B12" s="20" t="n">
-        <v>0.083</v>
+        <v>0.142</v>
       </c>
       <c r="C12" s="4" t="s">
         <v>72</v>
@@ -2425,7 +2434,7 @@
         <v>97</v>
       </c>
       <c r="B20" s="23" t="n">
-        <v>0.72</v>
+        <v>0.76</v>
       </c>
       <c r="C20" s="4" t="s">
         <v>95</v>
@@ -2453,7 +2462,7 @@
         <v>101</v>
       </c>
       <c r="B22" s="23" t="n">
-        <v>0.72</v>
+        <v>0.76</v>
       </c>
       <c r="C22" s="4" t="s">
         <v>95</v>
@@ -2649,13 +2658,13 @@
         <v>115</v>
       </c>
       <c r="B40" s="26" t="n">
-        <v>5.5</v>
+        <v>6</v>
       </c>
       <c r="C40" s="26" t="n">
-        <v>26</v>
+        <v>27.9</v>
       </c>
       <c r="D40" s="26" t="n">
-        <v>48</v>
+        <v>51.9</v>
       </c>
       <c r="E40" s="4" t="s">
         <v>127</v>
@@ -2666,13 +2675,13 @@
         <v>117</v>
       </c>
       <c r="B41" s="26" t="n">
-        <v>5.5</v>
+        <v>6</v>
       </c>
       <c r="C41" s="26" t="n">
-        <v>26</v>
+        <v>27.9</v>
       </c>
       <c r="D41" s="26" t="n">
-        <v>48</v>
+        <v>51.9</v>
       </c>
       <c r="E41" s="4" t="s">
         <v>128</v>
@@ -2686,10 +2695,10 @@
         <v>4</v>
       </c>
       <c r="C42" s="26" t="n">
-        <v>24.9</v>
+        <v>26.9</v>
       </c>
       <c r="D42" s="26" t="n">
-        <v>46.9</v>
+        <v>49.9</v>
       </c>
       <c r="E42" s="4" t="s">
         <v>129</v>
@@ -3009,7 +3018,7 @@
         <v>158</v>
       </c>
       <c r="B68" s="26" t="n">
-        <v>760</v>
+        <v>1010</v>
       </c>
       <c r="D68" s="4" t="s">
         <v>159</v>
@@ -3055,7 +3064,7 @@
       </c>
       <c r="B72" s="30" t="n">
         <f aca="false">SUM(B68:B71)</f>
-        <v>2503.38888888889</v>
+        <v>2753.38888888889</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3189,19 +3198,19 @@
       </c>
       <c r="B6" s="6" t="n">
         <f aca="false">B5*Supuestos!$B$6</f>
-        <v>0.4</v>
+        <v>0.605</v>
       </c>
       <c r="C6" s="6" t="n">
         <f aca="false">C5*Supuestos!$B$6</f>
-        <v>2.4</v>
+        <v>3.63</v>
       </c>
       <c r="D6" s="6" t="n">
         <f aca="false">D5*Supuestos!$B$6</f>
-        <v>2.4</v>
+        <v>3.63</v>
       </c>
       <c r="E6" s="6" t="n">
         <f aca="false">E5*Supuestos!$B$6</f>
-        <v>4.8</v>
+        <v>7.26</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3251,7 +3260,7 @@
       </c>
       <c r="B9" s="6" t="n">
         <f aca="false">Supuestos!$B$10</f>
-        <v>0.25</v>
+        <v>0.29</v>
       </c>
       <c r="C9" s="13" t="n">
         <v>0</v>
@@ -3310,15 +3319,15 @@
       </c>
       <c r="C12" s="6" t="n">
         <f aca="false">Supuestos!$B$20</f>
-        <v>0.72</v>
+        <v>0.76</v>
       </c>
       <c r="D12" s="6" t="n">
         <f aca="false">Supuestos!$B$20</f>
-        <v>0.72</v>
+        <v>0.76</v>
       </c>
       <c r="E12" s="6" t="n">
         <f aca="false">Supuestos!$B$22</f>
-        <v>0.72</v>
+        <v>0.76</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3327,19 +3336,19 @@
       </c>
       <c r="B13" s="13" t="n">
         <f aca="false">Supuestos!$B$15*SUM(B6:B12)</f>
-        <v>0.0595</v>
+        <v>0.07175</v>
       </c>
       <c r="C13" s="13" t="n">
         <f aca="false">Supuestos!$B$15*SUM(C6:C12)</f>
-        <v>0.3445</v>
+        <v>0.408</v>
       </c>
       <c r="D13" s="13" t="n">
         <f aca="false">Supuestos!$B$15*SUM(D6:D12)</f>
-        <v>0.3205</v>
+        <v>0.384</v>
       </c>
       <c r="E13" s="13" t="n">
         <f aca="false">Supuestos!$B$15*SUM(E6:E12)</f>
-        <v>0.635</v>
+        <v>0.76</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3348,19 +3357,19 @@
       </c>
       <c r="B14" s="13" t="n">
         <f aca="false">B5*(Supuestos!$B$12+Supuestos!$B$13+Supuestos!$B$14)</f>
-        <v>0.176</v>
+        <v>0.235</v>
       </c>
       <c r="C14" s="13" t="n">
         <f aca="false">C5*(Supuestos!$B$12+Supuestos!$B$13+Supuestos!$B$14)</f>
-        <v>1.056</v>
+        <v>1.41</v>
       </c>
       <c r="D14" s="13" t="n">
         <f aca="false">D5*(Supuestos!$B$12+Supuestos!$B$13+Supuestos!$B$14)</f>
-        <v>1.056</v>
+        <v>1.41</v>
       </c>
       <c r="E14" s="13" t="n">
         <f aca="false">E5*(Supuestos!$B$12+Supuestos!$B$13+Supuestos!$B$14)</f>
-        <v>2.112</v>
+        <v>2.82</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3369,19 +3378,19 @@
       </c>
       <c r="B15" s="30" t="n">
         <f aca="false">SUM(B6:B14)</f>
-        <v>1.4255</v>
+        <v>1.74175</v>
       </c>
       <c r="C15" s="30" t="n">
         <f aca="false">SUM(C6:C14)</f>
-        <v>8.2905</v>
+        <v>9.978</v>
       </c>
       <c r="D15" s="30" t="n">
         <f aca="false">SUM(D6:D14)</f>
-        <v>7.7865</v>
+        <v>9.474</v>
       </c>
       <c r="E15" s="30" t="n">
         <f aca="false">SUM(E6:E14)</f>
-        <v>15.447</v>
+        <v>18.78</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3390,19 +3399,19 @@
       </c>
       <c r="B16" s="30" t="n">
         <f aca="false">IF(B5=0,0,B15/B5)</f>
-        <v>1.4255</v>
+        <v>1.74175</v>
       </c>
       <c r="C16" s="30" t="n">
         <f aca="false">IF(C5=0,0,C15/C5)</f>
-        <v>1.38175</v>
+        <v>1.663</v>
       </c>
       <c r="D16" s="30" t="n">
         <f aca="false">IF(D5=0,0,D15/D5)</f>
-        <v>1.29775</v>
+        <v>1.579</v>
       </c>
       <c r="E16" s="30" t="n">
         <f aca="false">IF(E5=0,0,E15/E5)</f>
-        <v>1.28725</v>
+        <v>1.565</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3416,19 +3425,19 @@
       </c>
       <c r="B19" s="6" t="n">
         <f aca="false">Supuestos!B40</f>
-        <v>5.5</v>
+        <v>6</v>
       </c>
       <c r="C19" s="6" t="n">
         <f aca="false">Supuestos!C40</f>
-        <v>26</v>
+        <v>27.9</v>
       </c>
       <c r="D19" s="6" t="n">
         <f aca="false">Supuestos!C40</f>
-        <v>26</v>
+        <v>27.9</v>
       </c>
       <c r="E19" s="6" t="n">
         <f aca="false">Supuestos!D40</f>
-        <v>48</v>
+        <v>51.9</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3437,19 +3446,19 @@
       </c>
       <c r="B20" s="13" t="n">
         <f aca="false">B19/(1+Supuestos!$B$26)</f>
-        <v>4.66101694915254</v>
+        <v>5.08474576271187</v>
       </c>
       <c r="C20" s="13" t="n">
         <f aca="false">C19/(1+Supuestos!$B$26)</f>
-        <v>22.0338983050847</v>
+        <v>23.6440677966102</v>
       </c>
       <c r="D20" s="13" t="n">
         <f aca="false">D19/(1+Supuestos!$B$26)</f>
-        <v>22.0338983050847</v>
+        <v>23.6440677966102</v>
       </c>
       <c r="E20" s="13" t="n">
         <f aca="false">E19/(1+Supuestos!$B$26)</f>
-        <v>40.6779661016949</v>
+        <v>43.9830508474576</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3458,19 +3467,19 @@
       </c>
       <c r="B21" s="13" t="n">
         <f aca="false">B20-B15</f>
-        <v>3.23551694915254</v>
+        <v>3.34299576271187</v>
       </c>
       <c r="C21" s="13" t="n">
         <f aca="false">C20-C15</f>
-        <v>13.7433983050847</v>
+        <v>13.6660677966102</v>
       </c>
       <c r="D21" s="13" t="n">
         <f aca="false">D20-D15</f>
-        <v>14.2473983050847</v>
+        <v>14.1700677966102</v>
       </c>
       <c r="E21" s="13" t="n">
         <f aca="false">E20-E15</f>
-        <v>25.2309661016949</v>
+        <v>25.2030508474576</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3479,19 +3488,19 @@
       </c>
       <c r="B22" s="12" t="n">
         <f aca="false">IF(B20=0,0,B21/B20)</f>
-        <v>0.694165454545455</v>
+        <v>0.657455833333333</v>
       </c>
       <c r="C22" s="12" t="n">
         <f aca="false">IF(C20=0,0,C21/C20)</f>
-        <v>0.623738846153846</v>
+        <v>0.577991397849462</v>
       </c>
       <c r="D22" s="12" t="n">
         <f aca="false">IF(D20=0,0,D21/D20)</f>
-        <v>0.646612692307692</v>
+        <v>0.59930752688172</v>
       </c>
       <c r="E22" s="12" t="n">
         <f aca="false">IF(E20=0,0,E21/E20)</f>
-        <v>0.62026125</v>
+        <v>0.573017341040462</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3509,15 +3518,15 @@
       </c>
       <c r="C25" s="6" t="n">
         <f aca="false">Supuestos!C42</f>
-        <v>24.9</v>
+        <v>26.9</v>
       </c>
       <c r="D25" s="6" t="n">
         <f aca="false">Supuestos!C42</f>
-        <v>24.9</v>
+        <v>26.9</v>
       </c>
       <c r="E25" s="6" t="n">
         <f aca="false">Supuestos!D42</f>
-        <v>46.9</v>
+        <v>49.9</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3530,15 +3539,15 @@
       </c>
       <c r="C26" s="13" t="n">
         <f aca="false">C25/(1+Supuestos!$B$26)</f>
-        <v>21.1016949152542</v>
+        <v>22.7966101694915</v>
       </c>
       <c r="D26" s="13" t="n">
         <f aca="false">D25/(1+Supuestos!$B$26)</f>
-        <v>21.1016949152542</v>
+        <v>22.7966101694915</v>
       </c>
       <c r="E26" s="13" t="n">
         <f aca="false">E25/(1+Supuestos!$B$26)</f>
-        <v>39.7457627118644</v>
+        <v>42.2881355932203</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3547,19 +3556,19 @@
       </c>
       <c r="B27" s="13" t="n">
         <f aca="false">B26-B15</f>
-        <v>1.96433050847458</v>
+        <v>1.64808050847458</v>
       </c>
       <c r="C27" s="13" t="n">
         <f aca="false">C26-C15</f>
-        <v>12.8111949152542</v>
+        <v>12.8186101694915</v>
       </c>
       <c r="D27" s="13" t="n">
         <f aca="false">D26-D15</f>
-        <v>13.3151949152542</v>
+        <v>13.3226101694915</v>
       </c>
       <c r="E27" s="13" t="n">
         <f aca="false">E26-E15</f>
-        <v>24.2987627118644</v>
+        <v>23.5081355932203</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3568,19 +3577,19 @@
       </c>
       <c r="B28" s="12" t="n">
         <f aca="false">IF(B26=0,0,B27/B26)</f>
-        <v>0.5794775</v>
+        <v>0.48618375</v>
       </c>
       <c r="C28" s="12" t="n">
         <f aca="false">IF(C26=0,0,C27/C26)</f>
-        <v>0.60711686746988</v>
+        <v>0.562303345724907</v>
       </c>
       <c r="D28" s="12" t="n">
         <f aca="false">IF(D26=0,0,D27/D26)</f>
-        <v>0.631001204819277</v>
+        <v>0.584411895910781</v>
       </c>
       <c r="E28" s="12" t="n">
         <f aca="false">IF(E26=0,0,E27/E26)</f>
-        <v>0.611354797441365</v>
+        <v>0.55590380761523</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3710,51 +3719,51 @@
       </c>
       <c r="H5" s="6" t="n">
         <f aca="false">Supuestos!B40</f>
-        <v>5.5</v>
+        <v>6</v>
       </c>
       <c r="I5" s="16" t="n">
         <f aca="false">G5*H5</f>
-        <v>74662.5</v>
+        <v>81450</v>
       </c>
       <c r="J5" s="16" t="n">
         <f aca="false">I5/(1+Supuestos!$B$26)</f>
-        <v>63273.3050847458</v>
+        <v>69025.4237288136</v>
       </c>
       <c r="K5" s="6" t="n">
         <f aca="false">Costeo!B15</f>
-        <v>1.4255</v>
+        <v>1.74175</v>
       </c>
       <c r="L5" s="6" t="n">
         <f aca="false">Costeo!B15</f>
-        <v>1.4255</v>
+        <v>1.74175</v>
       </c>
       <c r="M5" s="13" t="n">
         <f aca="false">IF(H5=0,0,C5*Supuestos!$B$32+H5*Supuestos!$B$27*Supuestos!$C$32+H5/(1+Supuestos!$B$26)*Supuestos!$B$28)</f>
-        <v>0.481610169491525</v>
+        <v>0.500847457627119</v>
       </c>
       <c r="N5" s="13" t="n">
         <f aca="false">IF(H5=0,0,H5/(1+Supuestos!$B$26)-K5-M5)</f>
-        <v>2.75390677966102</v>
+        <v>2.84214830508475</v>
       </c>
       <c r="O5" s="13" t="n">
         <f aca="false">IF(H5=0,0,H5/(1+Supuestos!$B$26)-L5-M5)</f>
-        <v>2.75390677966102</v>
+        <v>2.84214830508475</v>
       </c>
       <c r="P5" s="16" t="n">
         <f aca="false">G5*N5</f>
-        <v>37384.2845338983</v>
+        <v>38582.1632415254</v>
       </c>
       <c r="Q5" s="16" t="n">
         <f aca="false">G5*O5</f>
-        <v>37384.2845338983</v>
+        <v>38582.1632415254</v>
       </c>
       <c r="R5" s="12" t="n">
         <f aca="false">IF(H5=0,0,N5/(H5/(1+Supuestos!$B$26)))</f>
-        <v>0.590838181818182</v>
+        <v>0.558955833333333</v>
       </c>
       <c r="S5" s="12" t="n">
         <f aca="false">IF(H5=0,0,O5/(H5/(1+Supuestos!$B$26)))</f>
-        <v>0.590838181818182</v>
+        <v>0.558955833333333</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3786,51 +3795,51 @@
       </c>
       <c r="H6" s="6" t="n">
         <f aca="false">Supuestos!C40</f>
-        <v>26</v>
+        <v>27.9</v>
       </c>
       <c r="I6" s="16" t="n">
         <f aca="false">G6*H6</f>
-        <v>34314.5833333333</v>
+        <v>36822.1875</v>
       </c>
       <c r="J6" s="16" t="n">
         <f aca="false">I6/(1+Supuestos!$B$26)</f>
-        <v>29080.1553672316</v>
+        <v>31205.2436440678</v>
       </c>
       <c r="K6" s="6" t="n">
         <f aca="false">Costeo!C15</f>
-        <v>8.2905</v>
+        <v>9.978</v>
       </c>
       <c r="L6" s="6" t="n">
         <f aca="false">Costeo!D15</f>
-        <v>7.7865</v>
+        <v>9.474</v>
       </c>
       <c r="M6" s="13" t="n">
         <f aca="false">IF(H6=0,0,C6*Supuestos!$B$32+H6*Supuestos!$B$27*Supuestos!$C$32+H6/(1+Supuestos!$B$26)*Supuestos!$B$28)</f>
-        <v>2.62033898305085</v>
+        <v>2.6934406779661</v>
       </c>
       <c r="N6" s="13" t="n">
         <f aca="false">IF(H6=0,0,H6/(1+Supuestos!$B$26)-K6-M6)</f>
-        <v>11.1230593220339</v>
+        <v>10.9726271186441</v>
       </c>
       <c r="O6" s="13" t="n">
         <f aca="false">IF(H6=0,0,H6/(1+Supuestos!$B$26)-L6-M6)</f>
-        <v>11.6270593220339</v>
+        <v>11.4766271186441</v>
       </c>
       <c r="P6" s="16" t="n">
         <f aca="false">G6*N6</f>
-        <v>14680.1210010593</v>
+        <v>14481.5818326271</v>
       </c>
       <c r="Q6" s="16" t="n">
         <f aca="false">G6*O6</f>
-        <v>15345.2960010593</v>
+        <v>15146.7568326271</v>
       </c>
       <c r="R6" s="12" t="n">
         <f aca="false">IF(H6=0,0,N6/(H6/(1+Supuestos!$B$26)))</f>
-        <v>0.504815769230769</v>
+        <v>0.464075268817204</v>
       </c>
       <c r="S6" s="12" t="n">
         <f aca="false">IF(H6=0,0,O6/(H6/(1+Supuestos!$B$26)))</f>
-        <v>0.527689615384615</v>
+        <v>0.485391397849462</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3862,51 +3871,51 @@
       </c>
       <c r="H7" s="6" t="n">
         <f aca="false">Supuestos!D40</f>
-        <v>48</v>
+        <v>51.9</v>
       </c>
       <c r="I7" s="16" t="n">
         <f aca="false">G7*H7</f>
-        <v>4525</v>
+        <v>4892.65625</v>
       </c>
       <c r="J7" s="16" t="n">
         <f aca="false">I7/(1+Supuestos!$B$26)</f>
-        <v>3834.74576271186</v>
+        <v>4146.3188559322</v>
       </c>
       <c r="K7" s="6" t="n">
         <f aca="false">Costeo!E15</f>
-        <v>15.447</v>
+        <v>18.78</v>
       </c>
       <c r="L7" s="6" t="n">
         <f aca="false">Costeo!E15</f>
-        <v>15.447</v>
+        <v>18.78</v>
       </c>
       <c r="M7" s="13" t="n">
         <f aca="false">IF(H7=0,0,C7*Supuestos!$B$32+H7*Supuestos!$B$27*Supuestos!$C$32+H7/(1+Supuestos!$B$26)*Supuestos!$B$28)</f>
-        <v>5.08677966101695</v>
+        <v>5.23683050847458</v>
       </c>
       <c r="N7" s="13" t="n">
         <f aca="false">IF(H7=0,0,H7/(1+Supuestos!$B$26)-K7-M7)</f>
-        <v>20.144186440678</v>
+        <v>19.9662203389831</v>
       </c>
       <c r="O7" s="13" t="n">
         <f aca="false">IF(H7=0,0,H7/(1+Supuestos!$B$26)-L7-M7)</f>
-        <v>20.144186440678</v>
+        <v>19.9662203389831</v>
       </c>
       <c r="P7" s="16" t="n">
         <f aca="false">G7*N7</f>
-        <v>1899.00924258475</v>
+        <v>1882.23222987288</v>
       </c>
       <c r="Q7" s="16" t="n">
         <f aca="false">G7*O7</f>
-        <v>1899.00924258475</v>
+        <v>1882.23222987288</v>
       </c>
       <c r="R7" s="12" t="n">
         <f aca="false">IF(H7=0,0,N7/(H7/(1+Supuestos!$B$26)))</f>
-        <v>0.49521125</v>
+        <v>0.453952601156069</v>
       </c>
       <c r="S7" s="12" t="n">
         <f aca="false">IF(H7=0,0,O7/(H7/(1+Supuestos!$B$26)))</f>
-        <v>0.49521125</v>
+        <v>0.453952601156069</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3938,51 +3947,51 @@
       </c>
       <c r="H8" s="6" t="n">
         <f aca="false">Supuestos!B41</f>
-        <v>5.5</v>
+        <v>6</v>
       </c>
       <c r="I8" s="16" t="n">
         <f aca="false">G8*H8</f>
-        <v>31185</v>
+        <v>34020</v>
       </c>
       <c r="J8" s="16" t="n">
         <f aca="false">I8/(1+Supuestos!$B$26)</f>
-        <v>26427.9661016949</v>
+        <v>28830.5084745763</v>
       </c>
       <c r="K8" s="6" t="n">
         <f aca="false">Costeo!B15</f>
-        <v>1.4255</v>
+        <v>1.74175</v>
       </c>
       <c r="L8" s="6" t="n">
         <f aca="false">Costeo!B15</f>
-        <v>1.4255</v>
+        <v>1.74175</v>
       </c>
       <c r="M8" s="13" t="n">
         <f aca="false">IF(H8=0,0,C8*Supuestos!$B$33+H8*Supuestos!$B$27*Supuestos!$C$33+H8/(1+Supuestos!$B$26)*Supuestos!$B$28)</f>
-        <v>0.481610169491525</v>
+        <v>0.500847457627119</v>
       </c>
       <c r="N8" s="13" t="n">
         <f aca="false">IF(H8=0,0,H8/(1+Supuestos!$B$26)-K8-M8)</f>
-        <v>2.75390677966102</v>
+        <v>2.84214830508475</v>
       </c>
       <c r="O8" s="13" t="n">
         <f aca="false">IF(H8=0,0,H8/(1+Supuestos!$B$26)-L8-M8)</f>
-        <v>2.75390677966102</v>
+        <v>2.84214830508475</v>
       </c>
       <c r="P8" s="16" t="n">
         <f aca="false">G8*N8</f>
-        <v>15614.651440678</v>
+        <v>16114.9808898305</v>
       </c>
       <c r="Q8" s="16" t="n">
         <f aca="false">G8*O8</f>
-        <v>15614.651440678</v>
+        <v>16114.9808898305</v>
       </c>
       <c r="R8" s="12" t="n">
         <f aca="false">IF(H8=0,0,N8/(H8/(1+Supuestos!$B$26)))</f>
-        <v>0.590838181818182</v>
+        <v>0.558955833333333</v>
       </c>
       <c r="S8" s="12" t="n">
         <f aca="false">IF(H8=0,0,O8/(H8/(1+Supuestos!$B$26)))</f>
-        <v>0.590838181818182</v>
+        <v>0.558955833333333</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4014,51 +4023,51 @@
       </c>
       <c r="H9" s="6" t="n">
         <f aca="false">Supuestos!C41</f>
-        <v>26</v>
+        <v>27.9</v>
       </c>
       <c r="I9" s="16" t="n">
         <f aca="false">G9*H9</f>
-        <v>10530</v>
+        <v>11299.5</v>
       </c>
       <c r="J9" s="16" t="n">
         <f aca="false">I9/(1+Supuestos!$B$26)</f>
-        <v>8923.72881355932</v>
+        <v>9575.84745762712</v>
       </c>
       <c r="K9" s="6" t="n">
         <f aca="false">Costeo!C15</f>
-        <v>8.2905</v>
+        <v>9.978</v>
       </c>
       <c r="L9" s="6" t="n">
         <f aca="false">Costeo!D15</f>
-        <v>7.7865</v>
+        <v>9.474</v>
       </c>
       <c r="M9" s="13" t="n">
         <f aca="false">IF(H9=0,0,C9*Supuestos!$B$33+H9*Supuestos!$B$27*Supuestos!$C$33+H9/(1+Supuestos!$B$26)*Supuestos!$B$28)</f>
-        <v>2.62033898305085</v>
+        <v>2.6934406779661</v>
       </c>
       <c r="N9" s="13" t="n">
         <f aca="false">IF(H9=0,0,H9/(1+Supuestos!$B$26)-K9-M9)</f>
-        <v>11.1230593220339</v>
+        <v>10.9726271186441</v>
       </c>
       <c r="O9" s="13" t="n">
         <f aca="false">IF(H9=0,0,H9/(1+Supuestos!$B$26)-L9-M9)</f>
-        <v>11.6270593220339</v>
+        <v>11.4766271186441</v>
       </c>
       <c r="P9" s="16" t="n">
         <f aca="false">G9*N9</f>
-        <v>4504.83902542373</v>
+        <v>4443.91398305085</v>
       </c>
       <c r="Q9" s="16" t="n">
         <f aca="false">G9*O9</f>
-        <v>4708.95902542373</v>
+        <v>4648.03398305085</v>
       </c>
       <c r="R9" s="12" t="n">
         <f aca="false">IF(H9=0,0,N9/(H9/(1+Supuestos!$B$26)))</f>
-        <v>0.504815769230769</v>
+        <v>0.464075268817204</v>
       </c>
       <c r="S9" s="12" t="n">
         <f aca="false">IF(H9=0,0,O9/(H9/(1+Supuestos!$B$26)))</f>
-        <v>0.527689615384615</v>
+        <v>0.485391397849462</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4090,7 +4099,7 @@
       </c>
       <c r="H10" s="6" t="n">
         <f aca="false">Supuestos!D41</f>
-        <v>48</v>
+        <v>51.9</v>
       </c>
       <c r="I10" s="16" t="n">
         <f aca="false">G10*H10</f>
@@ -4102,23 +4111,23 @@
       </c>
       <c r="K10" s="6" t="n">
         <f aca="false">Costeo!E15</f>
-        <v>15.447</v>
+        <v>18.78</v>
       </c>
       <c r="L10" s="6" t="n">
         <f aca="false">Costeo!E15</f>
-        <v>15.447</v>
+        <v>18.78</v>
       </c>
       <c r="M10" s="13" t="n">
         <f aca="false">IF(H10=0,0,C10*Supuestos!$B$33+H10*Supuestos!$B$27*Supuestos!$C$33+H10/(1+Supuestos!$B$26)*Supuestos!$B$28)</f>
-        <v>5.08677966101695</v>
+        <v>5.23683050847458</v>
       </c>
       <c r="N10" s="13" t="n">
         <f aca="false">IF(H10=0,0,H10/(1+Supuestos!$B$26)-K10-M10)</f>
-        <v>20.144186440678</v>
+        <v>19.9662203389831</v>
       </c>
       <c r="O10" s="13" t="n">
         <f aca="false">IF(H10=0,0,H10/(1+Supuestos!$B$26)-L10-M10)</f>
-        <v>20.144186440678</v>
+        <v>19.9662203389831</v>
       </c>
       <c r="P10" s="16" t="n">
         <f aca="false">G10*N10</f>
@@ -4130,11 +4139,11 @@
       </c>
       <c r="R10" s="12" t="n">
         <f aca="false">IF(H10=0,0,N10/(H10/(1+Supuestos!$B$26)))</f>
-        <v>0.49521125</v>
+        <v>0.453952601156069</v>
       </c>
       <c r="S10" s="12" t="n">
         <f aca="false">IF(H10=0,0,O10/(H10/(1+Supuestos!$B$26)))</f>
-        <v>0.49521125</v>
+        <v>0.453952601156069</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4178,11 +4187,11 @@
       </c>
       <c r="K11" s="6" t="n">
         <f aca="false">Costeo!B15</f>
-        <v>1.4255</v>
+        <v>1.74175</v>
       </c>
       <c r="L11" s="6" t="n">
         <f aca="false">Costeo!B15</f>
-        <v>1.4255</v>
+        <v>1.74175</v>
       </c>
       <c r="M11" s="13" t="n">
         <f aca="false">IF(H11=0,0,C11*Supuestos!$B$34+H11*Supuestos!$B$27*Supuestos!$C$34+H11/(1+Supuestos!$B$26)*Supuestos!$B$28)</f>
@@ -4190,27 +4199,27 @@
       </c>
       <c r="N11" s="13" t="n">
         <f aca="false">IF(H11=0,0,H11/(1+Supuestos!$B$26)-K11-M11)</f>
-        <v>1.01043220338983</v>
+        <v>0.694182203389831</v>
       </c>
       <c r="O11" s="13" t="n">
         <f aca="false">IF(H11=0,0,H11/(1+Supuestos!$B$26)-L11-M11)</f>
-        <v>1.01043220338983</v>
+        <v>0.694182203389831</v>
       </c>
       <c r="P11" s="16" t="n">
         <f aca="false">G11*N11</f>
-        <v>927.172589830509</v>
+        <v>636.981589830509</v>
       </c>
       <c r="Q11" s="16" t="n">
         <f aca="false">G11*O11</f>
-        <v>927.172589830509</v>
+        <v>636.981589830509</v>
       </c>
       <c r="R11" s="12" t="n">
         <f aca="false">IF(H11=0,0,N11/(H11/(1+Supuestos!$B$26)))</f>
-        <v>0.2980775</v>
+        <v>0.20478375</v>
       </c>
       <c r="S11" s="12" t="n">
         <f aca="false">IF(H11=0,0,O11/(H11/(1+Supuestos!$B$26)))</f>
-        <v>0.2980775</v>
+        <v>0.20478375</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4242,51 +4251,51 @@
       </c>
       <c r="H12" s="6" t="n">
         <f aca="false">Supuestos!C42</f>
-        <v>24.9</v>
+        <v>26.9</v>
       </c>
       <c r="I12" s="16" t="n">
         <f aca="false">G12*H12</f>
-        <v>22848.24</v>
+        <v>24683.44</v>
       </c>
       <c r="J12" s="16" t="n">
         <f aca="false">I12/(1+Supuestos!$B$26)</f>
-        <v>19362.9152542373</v>
+        <v>20918.1694915254</v>
       </c>
       <c r="K12" s="6" t="n">
         <f aca="false">Costeo!C15</f>
-        <v>8.2905</v>
+        <v>9.978</v>
       </c>
       <c r="L12" s="6" t="n">
         <f aca="false">Costeo!D15</f>
-        <v>7.7865</v>
+        <v>9.474</v>
       </c>
       <c r="M12" s="13" t="n">
         <f aca="false">IF(H12=0,0,C12*Supuestos!$B$34+H12*Supuestos!$B$27*Supuestos!$C$34+H12/(1+Supuestos!$B$26)*Supuestos!$B$28)</f>
-        <v>5.75801694915254</v>
+        <v>5.83496610169492</v>
       </c>
       <c r="N12" s="13" t="n">
         <f aca="false">IF(H12=0,0,H12/(1+Supuestos!$B$26)-K12-M12)</f>
-        <v>7.05317796610169</v>
+        <v>6.98364406779661</v>
       </c>
       <c r="O12" s="13" t="n">
         <f aca="false">IF(H12=0,0,H12/(1+Supuestos!$B$26)-L12-M12)</f>
-        <v>7.5571779661017</v>
+        <v>7.48764406779661</v>
       </c>
       <c r="P12" s="16" t="n">
         <f aca="false">G12*N12</f>
-        <v>6471.99610169492</v>
+        <v>6408.19179661017</v>
       </c>
       <c r="Q12" s="16" t="n">
         <f aca="false">G12*O12</f>
-        <v>6934.46650169492</v>
+        <v>6870.66219661017</v>
       </c>
       <c r="R12" s="12" t="n">
         <f aca="false">IF(H12=0,0,N12/(H12/(1+Supuestos!$B$26)))</f>
-        <v>0.334246987951807</v>
+        <v>0.306345724907063</v>
       </c>
       <c r="S12" s="12" t="n">
         <f aca="false">IF(H12=0,0,O12/(H12/(1+Supuestos!$B$26)))</f>
-        <v>0.358131325301205</v>
+        <v>0.328454275092937</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4318,51 +4327,51 @@
       </c>
       <c r="H13" s="6" t="n">
         <f aca="false">Supuestos!D42</f>
-        <v>46.9</v>
+        <v>49.9</v>
       </c>
       <c r="I13" s="16" t="n">
         <f aca="false">G13*H13</f>
-        <v>10758.86</v>
+        <v>11447.06</v>
       </c>
       <c r="J13" s="16" t="n">
         <f aca="false">I13/(1+Supuestos!$B$26)</f>
-        <v>9117.67796610169</v>
+        <v>9700.89830508474</v>
       </c>
       <c r="K13" s="6" t="n">
         <f aca="false">Costeo!E15</f>
-        <v>15.447</v>
+        <v>18.78</v>
       </c>
       <c r="L13" s="6" t="n">
         <f aca="false">Costeo!E15</f>
-        <v>15.447</v>
+        <v>18.78</v>
       </c>
       <c r="M13" s="13" t="n">
         <f aca="false">IF(H13=0,0,C13*Supuestos!$B$34+H13*Supuestos!$B$27*Supuestos!$C$34+H13/(1+Supuestos!$B$26)*Supuestos!$B$28)</f>
-        <v>11.4044576271186</v>
+        <v>11.5198813559322</v>
       </c>
       <c r="N13" s="13" t="n">
         <f aca="false">IF(H13=0,0,H13/(1+Supuestos!$B$26)-K13-M13)</f>
-        <v>12.8943050847458</v>
+        <v>11.9882542372881</v>
       </c>
       <c r="O13" s="13" t="n">
         <f aca="false">IF(H13=0,0,H13/(1+Supuestos!$B$26)-L13-M13)</f>
-        <v>12.8943050847458</v>
+        <v>11.9882542372881</v>
       </c>
       <c r="P13" s="16" t="n">
         <f aca="false">G13*N13</f>
-        <v>2957.95358644068</v>
+        <v>2750.1055220339</v>
       </c>
       <c r="Q13" s="16" t="n">
         <f aca="false">G13*O13</f>
-        <v>2957.95358644068</v>
+        <v>2750.1055220339</v>
       </c>
       <c r="R13" s="12" t="n">
         <f aca="false">IF(H13=0,0,N13/(H13/(1+Supuestos!$B$26)))</f>
-        <v>0.324419616204691</v>
+        <v>0.283489779559118</v>
       </c>
       <c r="S13" s="12" t="n">
         <f aca="false">IF(H13=0,0,O13/(H13/(1+Supuestos!$B$26)))</f>
-        <v>0.324419616204691</v>
+        <v>0.283489779559118</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4406,11 +4415,11 @@
       </c>
       <c r="K14" s="6" t="n">
         <f aca="false">Costeo!B15</f>
-        <v>1.4255</v>
+        <v>1.74175</v>
       </c>
       <c r="L14" s="6" t="n">
         <f aca="false">Costeo!B15</f>
-        <v>1.4255</v>
+        <v>1.74175</v>
       </c>
       <c r="M14" s="13" t="n">
         <f aca="false">IF(H14=0,0,C14*Supuestos!$B$35+H14*Supuestos!$B$27*Supuestos!$C$35+H14/(1+Supuestos!$B$26)*Supuestos!$B$28)</f>
@@ -4418,27 +4427,27 @@
       </c>
       <c r="N14" s="13" t="n">
         <f aca="false">IF(H14=0,0,H14/(1+Supuestos!$B$26)-K14-M14)</f>
-        <v>0.991449152542373</v>
+        <v>0.675199152542373</v>
       </c>
       <c r="O14" s="13" t="n">
         <f aca="false">IF(H14=0,0,H14/(1+Supuestos!$B$26)-L14-M14)</f>
-        <v>0.991449152542373</v>
+        <v>0.675199152542373</v>
       </c>
       <c r="P14" s="16" t="n">
         <f aca="false">G14*N14</f>
-        <v>9086.63148305085</v>
+        <v>6188.20023305085</v>
       </c>
       <c r="Q14" s="16" t="n">
         <f aca="false">G14*O14</f>
-        <v>9086.63148305085</v>
+        <v>6188.20023305085</v>
       </c>
       <c r="R14" s="12" t="n">
         <f aca="false">IF(H14=0,0,N14/(H14/(1+Supuestos!$B$26)))</f>
-        <v>0.38997</v>
+        <v>0.265578333333333</v>
       </c>
       <c r="S14" s="12" t="n">
         <f aca="false">IF(H14=0,0,O14/(H14/(1+Supuestos!$B$26)))</f>
-        <v>0.38997</v>
+        <v>0.265578333333333</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4482,11 +4491,11 @@
       </c>
       <c r="K15" s="6" t="n">
         <f aca="false">Costeo!C15</f>
-        <v>8.2905</v>
+        <v>9.978</v>
       </c>
       <c r="L15" s="6" t="n">
         <f aca="false">Costeo!D15</f>
-        <v>7.7865</v>
+        <v>9.474</v>
       </c>
       <c r="M15" s="13" t="n">
         <f aca="false">IF(H15=0,0,C15*Supuestos!$B$35+H15*Supuestos!$B$27*Supuestos!$C$35+H15/(1+Supuestos!$B$26)*Supuestos!$B$28)</f>
@@ -4558,11 +4567,11 @@
       </c>
       <c r="K16" s="6" t="n">
         <f aca="false">Costeo!E15</f>
-        <v>15.447</v>
+        <v>18.78</v>
       </c>
       <c r="L16" s="6" t="n">
         <f aca="false">Costeo!E15</f>
-        <v>15.447</v>
+        <v>18.78</v>
       </c>
       <c r="M16" s="13" t="n">
         <f aca="false">IF(H16=0,0,C16*Supuestos!$B$35+H16*Supuestos!$B$27*Supuestos!$C$35+H16/(1+Supuestos!$B$26)*Supuestos!$B$28)</f>
@@ -4634,11 +4643,11 @@
       </c>
       <c r="K17" s="6" t="n">
         <f aca="false">Costeo!B15</f>
-        <v>1.4255</v>
+        <v>1.74175</v>
       </c>
       <c r="L17" s="6" t="n">
         <f aca="false">Costeo!B15</f>
-        <v>1.4255</v>
+        <v>1.74175</v>
       </c>
       <c r="M17" s="13" t="n">
         <f aca="false">IF(H17=0,0,C17*Supuestos!$B$36+H17*Supuestos!$B$27*Supuestos!$C$36+H17/(1+Supuestos!$B$26)*Supuestos!$B$28)</f>
@@ -4710,11 +4719,11 @@
       </c>
       <c r="K18" s="6" t="n">
         <f aca="false">Costeo!C15</f>
-        <v>8.2905</v>
+        <v>9.978</v>
       </c>
       <c r="L18" s="6" t="n">
         <f aca="false">Costeo!D15</f>
-        <v>7.7865</v>
+        <v>9.474</v>
       </c>
       <c r="M18" s="13" t="n">
         <f aca="false">IF(H18=0,0,C18*Supuestos!$B$36+H18*Supuestos!$B$27*Supuestos!$C$36+H18/(1+Supuestos!$B$26)*Supuestos!$B$28)</f>
@@ -4722,27 +4731,27 @@
       </c>
       <c r="N18" s="13" t="n">
         <f aca="false">IF(H18=0,0,H18/(1+Supuestos!$B$26)-K18-M18)</f>
-        <v>5.35746610169491</v>
+        <v>3.66996610169492</v>
       </c>
       <c r="O18" s="13" t="n">
         <f aca="false">IF(H18=0,0,H18/(1+Supuestos!$B$26)-L18-M18)</f>
-        <v>5.86146610169492</v>
+        <v>4.17396610169492</v>
       </c>
       <c r="P18" s="16" t="n">
         <f aca="false">G18*N18</f>
-        <v>3321.62898305085</v>
+        <v>2275.37898305085</v>
       </c>
       <c r="Q18" s="16" t="n">
         <f aca="false">G18*O18</f>
-        <v>3634.10898305085</v>
+        <v>2587.85898305085</v>
       </c>
       <c r="R18" s="12" t="n">
         <f aca="false">IF(H18=0,0,N18/(H18/(1+Supuestos!$B$26)))</f>
-        <v>0.364579584775086</v>
+        <v>0.249743944636678</v>
       </c>
       <c r="S18" s="12" t="n">
         <f aca="false">IF(H18=0,0,O18/(H18/(1+Supuestos!$B$26)))</f>
-        <v>0.398877162629758</v>
+        <v>0.28404152249135</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4786,11 +4795,11 @@
       </c>
       <c r="K19" s="6" t="n">
         <f aca="false">Costeo!E15</f>
-        <v>15.447</v>
+        <v>18.78</v>
       </c>
       <c r="L19" s="6" t="n">
         <f aca="false">Costeo!E15</f>
-        <v>15.447</v>
+        <v>18.78</v>
       </c>
       <c r="M19" s="13" t="n">
         <f aca="false">IF(H19=0,0,C19*Supuestos!$B$36+H19*Supuestos!$B$27*Supuestos!$C$36+H19/(1+Supuestos!$B$26)*Supuestos!$B$28)</f>
@@ -4831,19 +4840,19 @@
       </c>
       <c r="I20" s="11" t="n">
         <f aca="false">SUM(I5:I19)</f>
-        <v>230740.383333333</v>
+        <v>246531.04375</v>
       </c>
       <c r="J20" s="11" t="n">
         <f aca="false">SUM(J5:J19)</f>
-        <v>195542.697740113</v>
+        <v>208924.613347458</v>
       </c>
       <c r="P20" s="11" t="n">
         <f aca="false">SUM(P5:P19)</f>
-        <v>96848.2879877119</v>
+        <v>93763.7303014831</v>
       </c>
       <c r="Q20" s="11" t="n">
         <f aca="false">SUM(Q5:Q19)</f>
-        <v>98492.5333877119</v>
+        <v>95407.9757014831</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4894,27 +4903,27 @@
       </c>
       <c r="C25" s="16" t="n">
         <f aca="false">SUMIF($A$5:$A$19,A25,$P$5:$P$19)</f>
-        <v>53963.4147775424</v>
+        <v>54945.9773040254</v>
       </c>
       <c r="D25" s="16" t="n">
         <f aca="false">SUMIF($A$5:$A$19,A25,$Q$5:$Q$19)</f>
-        <v>54628.5897775424</v>
+        <v>55611.1523040254</v>
       </c>
       <c r="E25" s="16" t="n">
         <f aca="false">SUMIF($A$5:$A$19,A25,$I$5:$I$19)</f>
-        <v>113502.083333333</v>
+        <v>123164.84375</v>
       </c>
       <c r="F25" s="13" t="n">
         <f aca="false">IF(B25=0,0,C25/B25)</f>
-        <v>2.38512330508475</v>
+        <v>2.42855148305085</v>
       </c>
       <c r="G25" s="13" t="n">
         <f aca="false">IF(B25=0,0,D25/B25)</f>
-        <v>2.41452330508475</v>
+        <v>2.45795148305085</v>
       </c>
       <c r="H25" s="13" t="n">
         <f aca="false">IF(B25=0,0,E25/B25)</f>
-        <v>5.01666666666667</v>
+        <v>5.44375</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4927,27 +4936,27 @@
       </c>
       <c r="C26" s="16" t="n">
         <f aca="false">SUMIF($A$5:$A$19,A26,$P$5:$P$19)</f>
-        <v>20119.4904661017</v>
+        <v>20558.8948728814</v>
       </c>
       <c r="D26" s="16" t="n">
         <f aca="false">SUMIF($A$5:$A$19,A26,$Q$5:$Q$19)</f>
-        <v>20323.6104661017</v>
+        <v>20763.0148728814</v>
       </c>
       <c r="E26" s="16" t="n">
         <f aca="false">SUMIF($A$5:$A$19,A26,$I$5:$I$19)</f>
-        <v>41715</v>
+        <v>45319.5</v>
       </c>
       <c r="F26" s="13" t="n">
         <f aca="false">IF(B26=0,0,C26/B26)</f>
-        <v>2.48388771186441</v>
+        <v>2.53813516949153</v>
       </c>
       <c r="G26" s="13" t="n">
         <f aca="false">IF(B26=0,0,D26/B26)</f>
-        <v>2.50908771186441</v>
+        <v>2.56333516949153</v>
       </c>
       <c r="H26" s="13" t="n">
         <f aca="false">IF(B26=0,0,E26/B26)</f>
-        <v>5.15</v>
+        <v>5.595</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4960,27 +4969,27 @@
       </c>
       <c r="C27" s="16" t="n">
         <f aca="false">SUMIF($A$5:$A$19,A27,$P$5:$P$19)</f>
-        <v>10357.1222779661</v>
+        <v>9795.27890847458</v>
       </c>
       <c r="D27" s="16" t="n">
         <f aca="false">SUMIF($A$5:$A$19,A27,$Q$5:$Q$19)</f>
-        <v>10819.5926779661</v>
+        <v>10257.7493084746</v>
       </c>
       <c r="E27" s="16" t="n">
         <f aca="false">SUMIF($A$5:$A$19,A27,$I$5:$I$19)</f>
-        <v>37277.5</v>
+        <v>39800.9</v>
       </c>
       <c r="F27" s="13" t="n">
         <f aca="false">IF(B27=0,0,C27/B27)</f>
-        <v>1.1287186440678</v>
+        <v>1.06748898305085</v>
       </c>
       <c r="G27" s="13" t="n">
         <f aca="false">IF(B27=0,0,D27/B27)</f>
-        <v>1.1791186440678</v>
+        <v>1.11788898305085</v>
       </c>
       <c r="H27" s="13" t="n">
         <f aca="false">IF(B27=0,0,E27/B27)</f>
-        <v>4.0625</v>
+        <v>4.3375</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4993,11 +5002,11 @@
       </c>
       <c r="C28" s="16" t="n">
         <f aca="false">SUMIF($A$5:$A$19,A28,$P$5:$P$19)</f>
-        <v>9086.63148305085</v>
+        <v>6188.20023305085</v>
       </c>
       <c r="D28" s="16" t="n">
         <f aca="false">SUMIF($A$5:$A$19,A28,$Q$5:$Q$19)</f>
-        <v>9086.63148305085</v>
+        <v>6188.20023305085</v>
       </c>
       <c r="E28" s="16" t="n">
         <f aca="false">SUMIF($A$5:$A$19,A28,$I$5:$I$19)</f>
@@ -5005,11 +5014,11 @@
       </c>
       <c r="F28" s="13" t="n">
         <f aca="false">IF(B28=0,0,C28/B28)</f>
-        <v>0.991449152542373</v>
+        <v>0.675199152542373</v>
       </c>
       <c r="G28" s="13" t="n">
         <f aca="false">IF(B28=0,0,D28/B28)</f>
-        <v>0.991449152542373</v>
+        <v>0.675199152542373</v>
       </c>
       <c r="H28" s="13" t="n">
         <f aca="false">IF(B28=0,0,E28/B28)</f>
@@ -5026,11 +5035,11 @@
       </c>
       <c r="C29" s="16" t="n">
         <f aca="false">SUMIF($A$5:$A$19,A29,$P$5:$P$19)</f>
-        <v>3321.62898305085</v>
+        <v>2275.37898305085</v>
       </c>
       <c r="D29" s="16" t="n">
         <f aca="false">SUMIF($A$5:$A$19,A29,$Q$5:$Q$19)</f>
-        <v>3634.10898305085</v>
+        <v>2587.85898305085</v>
       </c>
       <c r="E29" s="16" t="n">
         <f aca="false">SUMIF($A$5:$A$19,A29,$I$5:$I$19)</f>
@@ -5038,11 +5047,11 @@
       </c>
       <c r="F29" s="13" t="n">
         <f aca="false">IF(B29=0,0,C29/B29)</f>
-        <v>0.892911016949152</v>
+        <v>0.611661016949153</v>
       </c>
       <c r="G29" s="13" t="n">
         <f aca="false">IF(B29=0,0,D29/B29)</f>
-        <v>0.976911016949153</v>
+        <v>0.695661016949153</v>
       </c>
       <c r="H29" s="13" t="n">
         <f aca="false">IF(B29=0,0,E29/B29)</f>
@@ -5059,27 +5068,27 @@
       </c>
       <c r="C30" s="11" t="n">
         <f aca="false">SUM(C25:C29)</f>
-        <v>96848.2879877119</v>
+        <v>93763.7303014831</v>
       </c>
       <c r="D30" s="11" t="n">
         <f aca="false">SUM(D25:D29)</f>
-        <v>98492.5333877119</v>
+        <v>95407.9757014831</v>
       </c>
       <c r="E30" s="11" t="n">
         <f aca="false">SUM(E25:E29)</f>
-        <v>230740.383333333</v>
+        <v>246531.04375</v>
       </c>
       <c r="F30" s="30" t="n">
         <f aca="false">IF(B30=0,0,C30/B30)</f>
-        <v>1.83473436115091</v>
+        <v>1.77629921383479</v>
       </c>
       <c r="G30" s="30" t="n">
         <f aca="false">IF(B30=0,0,D30/B30)</f>
-        <v>1.86588363179085</v>
+        <v>1.80744848447473</v>
       </c>
       <c r="H30" s="30" t="n">
         <f aca="false">IF(B30=0,0,E30/B30)</f>
-        <v>4.37124205913184</v>
+        <v>4.67038691603834</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5132,15 +5141,15 @@
       </c>
       <c r="D34" s="16" t="n">
         <f aca="false">SUMIF($B$5:$B$19,A34,$I$5:$I$19)</f>
-        <v>137012.9</v>
+        <v>146635.4</v>
       </c>
       <c r="E34" s="16" t="n">
         <f aca="false">SUMIF($B$5:$B$19,A34,$P$5:$P$19)</f>
-        <v>63012.7400474576</v>
+        <v>61522.3259542373</v>
       </c>
       <c r="F34" s="16" t="n">
         <f aca="false">SUMIF($B$5:$B$19,A34,$Q$5:$Q$19)</f>
-        <v>63012.7400474576</v>
+        <v>61522.3259542373</v>
       </c>
       <c r="G34" s="12" t="n">
         <f aca="false">IF($F$20=0,0,B34/$F$20)</f>
@@ -5161,15 +5170,15 @@
       </c>
       <c r="D35" s="16" t="n">
         <f aca="false">SUMIF($B$5:$B$19,A35,$I$5:$I$19)</f>
-        <v>78443.6233333333</v>
+        <v>83555.9275</v>
       </c>
       <c r="E35" s="16" t="n">
         <f aca="false">SUMIF($B$5:$B$19,A35,$P$5:$P$19)</f>
-        <v>28978.5851112288</v>
+        <v>27609.066595339</v>
       </c>
       <c r="F35" s="16" t="n">
         <f aca="false">SUMIF($B$5:$B$19,A35,$Q$5:$Q$19)</f>
-        <v>30622.8305112288</v>
+        <v>29253.311995339</v>
       </c>
       <c r="G35" s="12" t="n">
         <f aca="false">IF($F$20=0,0,B35/$F$20)</f>
@@ -5190,15 +5199,15 @@
       </c>
       <c r="D36" s="16" t="n">
         <f aca="false">SUMIF($B$5:$B$19,A36,$I$5:$I$19)</f>
-        <v>15283.86</v>
+        <v>16339.71625</v>
       </c>
       <c r="E36" s="16" t="n">
         <f aca="false">SUMIF($B$5:$B$19,A36,$P$5:$P$19)</f>
-        <v>4856.96282902542</v>
+        <v>4632.33775190678</v>
       </c>
       <c r="F36" s="16" t="n">
         <f aca="false">SUMIF($B$5:$B$19,A36,$Q$5:$Q$19)</f>
-        <v>4856.96282902542</v>
+        <v>4632.33775190678</v>
       </c>
       <c r="G36" s="12" t="n">
         <f aca="false">IF($F$20=0,0,B36/$F$20)</f>
@@ -5562,53 +5571,53 @@
         <v>259</v>
       </c>
       <c r="B28" s="26" t="n">
-        <v>150</v>
+        <v>6150</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>230</v>
+        <v>260</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="10" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="B29" s="30" t="n">
         <f aca="false">SUM(B26:B28)</f>
-        <v>1250</v>
+        <v>7250</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="18" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="B30" s="19"/>
       <c r="C30" s="19"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="4" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="B31" s="26" t="n">
-        <v>3030</v>
+        <v>3150</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>230</v>
+        <v>264</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="4" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="B32" s="26" t="n">
-        <v>4135.3</v>
+        <v>4800.7</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>230</v>
+        <v>266</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="4" t="s">
-        <v>264</v>
+        <v>267</v>
       </c>
       <c r="B33" s="26" t="n">
         <v>3204</v>
@@ -5619,7 +5628,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="4" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
       <c r="B34" s="26" t="n">
         <v>8000</v>
@@ -5630,23 +5639,23 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="10" t="s">
-        <v>266</v>
+        <v>269</v>
       </c>
       <c r="B35" s="30" t="n">
         <f aca="false">SUM(B31:B34)</f>
-        <v>18369.3</v>
+        <v>19154.7</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="18" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="B36" s="19"/>
       <c r="C36" s="19"/>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="10" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
       <c r="B37" s="30" t="n">
         <f aca="false">B38+B39</f>
@@ -5655,7 +5664,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="4" t="s">
-        <v>269</v>
+        <v>272</v>
       </c>
       <c r="B38" s="26" t="n">
         <v>2338</v>
@@ -5666,46 +5675,46 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="4" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="B39" s="26" t="n">
         <v>2500</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="4" t="s">
-        <v>272</v>
+        <v>275</v>
       </c>
       <c r="B41" s="13" t="n">
         <f aca="false">0.1*(B17+B24+B29+B35+B37)</f>
-        <v>3444.931</v>
+        <v>4123.471</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="10" t="s">
-        <v>273</v>
+        <v>276</v>
       </c>
       <c r="B42" s="30" t="n">
         <f aca="false">B17+B24+B29+B35+B37+B41</f>
-        <v>37894.241</v>
+        <v>45358.181</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="18" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="B44" s="19"/>
       <c r="C44" s="19"/>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="5" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
       <c r="B45" s="5" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="C45" s="5" t="s">
         <v>114</v>
@@ -5713,74 +5722,74 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="4" t="s">
-        <v>277</v>
+        <v>280</v>
       </c>
       <c r="B46" s="26" t="n">
         <v>25000</v>
       </c>
       <c r="C46" s="4" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="4" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="B47" s="13" t="n">
         <f aca="false">MAX(0,CEILING(B42-B46,500))</f>
-        <v>13000</v>
+        <v>20500</v>
       </c>
       <c r="C47" s="4" t="s">
-        <v>280</v>
+        <v>283</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="4" t="s">
-        <v>281</v>
+        <v>284</v>
       </c>
       <c r="B48" s="27" t="n">
         <v>0.35</v>
       </c>
       <c r="C48" s="4" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="4" t="s">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="B49" s="25" t="n">
         <v>24</v>
       </c>
       <c r="C49" s="4" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="4" t="s">
-        <v>285</v>
+        <v>288</v>
       </c>
       <c r="B50" s="13" t="n">
         <f aca="false">PMT((1+B48)^(1/12)-1,B49,-B47)</f>
-        <v>729.471399828276</v>
+        <v>1150.32028434459</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="4" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
       <c r="B51" s="13" t="n">
         <f aca="false">B50*B49-B47</f>
-        <v>4507.31359587862</v>
+        <v>7107.68682427012</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="4" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="B52" s="13" t="n">
         <f aca="false">B46+B47-B42</f>
-        <v>105.759000000005</v>
+        <v>141.818999999996</v>
       </c>
     </row>
   </sheetData>
@@ -5809,61 +5818,61 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>291</v>
+        <v>294</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>292</v>
+        <v>295</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>294</v>
+        <v>297</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>296</v>
+        <v>299</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="I4" s="5" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="J4" s="5" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
       <c r="K4" s="5" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
       <c r="L4" s="5" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
       <c r="M4" s="5" t="s">
-        <v>302</v>
+        <v>305</v>
       </c>
       <c r="N4" s="5" t="s">
-        <v>303</v>
+        <v>306</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>304</v>
+        <v>307</v>
       </c>
       <c r="B5" s="25" t="n">
         <v>1</v>
@@ -5908,7 +5917,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>305</v>
+        <v>308</v>
       </c>
       <c r="B6" s="25" t="n">
         <v>9</v>
@@ -5953,7 +5962,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>306</v>
+        <v>309</v>
       </c>
       <c r="B7" s="25" t="n">
         <v>50</v>
@@ -5998,7 +6007,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
       <c r="B8" s="25" t="n">
         <v>0</v>
@@ -6043,7 +6052,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="B9" s="25" t="n">
         <v>1</v>
@@ -6088,7 +6097,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="B10" s="29" t="n">
         <v>0</v>
@@ -6133,7 +6142,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
       <c r="B11" s="29" t="n">
         <v>120</v>
@@ -6178,46 +6187,46 @@
     </row>
     <row r="13" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>291</v>
+        <v>294</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>292</v>
+        <v>295</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>294</v>
+        <v>297</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>296</v>
+        <v>299</v>
       </c>
       <c r="H13" s="5" t="s">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="I13" s="5" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="J13" s="5" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
       <c r="K13" s="5" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
       <c r="L13" s="5" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
       <c r="M13" s="5" t="s">
-        <v>302</v>
+        <v>305</v>
       </c>
       <c r="N13" s="5" t="s">
-        <v>303</v>
+        <v>306</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6507,7 +6516,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="10" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="B19" s="31" t="n">
         <f aca="false">SUM(B14:B18)</f>
@@ -6564,7 +6573,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="18" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="B21" s="19"/>
       <c r="C21" s="19"/>
@@ -6582,7 +6591,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
       <c r="B22" s="8" t="n">
         <f aca="false">SUMPRODUCT(B$14:B$18,Supuestos!$B$48:$B$52)</f>
@@ -6639,7 +6648,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="4" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="B23" s="8" t="n">
         <f aca="false">SUMPRODUCT(B$14:B$18,Supuestos!$C$48:$C$52)</f>
@@ -6696,7 +6705,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="4" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="B24" s="8" t="n">
         <f aca="false">SUMPRODUCT(B$14:B$18,Supuestos!$D$48:$D$52)</f>
@@ -6753,7 +6762,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="B25" s="15" t="n">
         <f aca="false">B23/Costeo!$C$5</f>
@@ -6810,7 +6819,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="B26" s="15" t="n">
         <f aca="false">B24/Costeo!$E$5</f>
@@ -6867,7 +6876,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="18" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="B28" s="19"/>
       <c r="C28" s="19"/>
@@ -6889,55 +6898,55 @@
       </c>
       <c r="B29" s="9" t="n">
         <f aca="false">SUMPRODUCT(B$14:B$18,Proyeccion!$H$25:$H$29)</f>
-        <v>3986.175</v>
+        <v>4286.3625</v>
       </c>
       <c r="C29" s="9" t="n">
         <f aca="false">SUMPRODUCT(C$14:C$18,Proyeccion!$H$25:$H$29)</f>
-        <v>13747.325</v>
+        <v>14865.075</v>
       </c>
       <c r="D29" s="9" t="n">
         <f aca="false">SUMPRODUCT(D$14:D$18,Proyeccion!$H$25:$H$29)</f>
-        <v>17009.575</v>
+        <v>18280.175</v>
       </c>
       <c r="E29" s="9" t="n">
         <f aca="false">SUMPRODUCT(E$14:E$18,Proyeccion!$H$25:$H$29)</f>
-        <v>16220.1</v>
+        <v>17333.1</v>
       </c>
       <c r="F29" s="9" t="n">
         <f aca="false">SUMPRODUCT(F$14:F$18,Proyeccion!$H$25:$H$29)</f>
-        <v>17600.625</v>
+        <v>18784.1625</v>
       </c>
       <c r="G29" s="9" t="n">
         <f aca="false">SUMPRODUCT(G$14:G$18,Proyeccion!$H$25:$H$29)</f>
-        <v>17122.875</v>
+        <v>18224.325</v>
       </c>
       <c r="H29" s="9" t="n">
         <f aca="false">SUMPRODUCT(H$14:H$18,Proyeccion!$H$25:$H$29)</f>
-        <v>16586.8583333333</v>
+        <v>17709.5</v>
       </c>
       <c r="I29" s="9" t="n">
         <f aca="false">SUMPRODUCT(I$14:I$18,Proyeccion!$H$25:$H$29)</f>
-        <v>22302.7125</v>
+        <v>23756.94375</v>
       </c>
       <c r="J29" s="9" t="n">
         <f aca="false">SUMPRODUCT(J$14:J$18,Proyeccion!$H$25:$H$29)</f>
-        <v>24036.2125</v>
+        <v>25619.6</v>
       </c>
       <c r="K29" s="9" t="n">
         <f aca="false">SUMPRODUCT(K$14:K$18,Proyeccion!$H$25:$H$29)</f>
-        <v>25304.6125</v>
+        <v>26901.2</v>
       </c>
       <c r="L29" s="9" t="n">
         <f aca="false">SUMPRODUCT(L$14:L$18,Proyeccion!$H$25:$H$29)</f>
-        <v>24532.1125</v>
+        <v>26061.95</v>
       </c>
       <c r="M29" s="9" t="n">
         <f aca="false">SUMPRODUCT(M$14:M$18,Proyeccion!$H$25:$H$29)</f>
-        <v>32291.2</v>
+        <v>34708.65</v>
       </c>
       <c r="N29" s="16" t="n">
         <f aca="false">SUM(B29:M29)</f>
-        <v>230740.383333333</v>
+        <v>246531.04375</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6946,174 +6955,174 @@
       </c>
       <c r="B30" s="16" t="n">
         <f aca="false">B29/(1+Supuestos!$B$26)</f>
-        <v>3378.11440677966</v>
+        <v>3632.51059322034</v>
       </c>
       <c r="C30" s="16" t="n">
         <f aca="false">C29/(1+Supuestos!$B$26)</f>
-        <v>11650.2754237288</v>
+        <v>12597.5211864407</v>
       </c>
       <c r="D30" s="16" t="n">
         <f aca="false">D29/(1+Supuestos!$B$26)</f>
-        <v>14414.8940677966</v>
+        <v>15491.6737288136</v>
       </c>
       <c r="E30" s="16" t="n">
         <f aca="false">E29/(1+Supuestos!$B$26)</f>
-        <v>13745.8474576271</v>
+        <v>14689.0677966102</v>
       </c>
       <c r="F30" s="16" t="n">
         <f aca="false">F29/(1+Supuestos!$B$26)</f>
-        <v>14915.7838983051</v>
+        <v>15918.781779661</v>
       </c>
       <c r="G30" s="16" t="n">
         <f aca="false">G29/(1+Supuestos!$B$26)</f>
-        <v>14510.9110169492</v>
+        <v>15444.343220339</v>
       </c>
       <c r="H30" s="16" t="n">
         <f aca="false">H29/(1+Supuestos!$B$26)</f>
-        <v>14056.6596045198</v>
+        <v>15008.0508474576</v>
       </c>
       <c r="I30" s="16" t="n">
         <f aca="false">I29/(1+Supuestos!$B$26)</f>
-        <v>18900.6038135593</v>
+        <v>20133.0031779661</v>
       </c>
       <c r="J30" s="16" t="n">
         <f aca="false">J29/(1+Supuestos!$B$26)</f>
-        <v>20369.6716101695</v>
+        <v>21711.5254237288</v>
       </c>
       <c r="K30" s="16" t="n">
         <f aca="false">K29/(1+Supuestos!$B$26)</f>
-        <v>21444.5868644068</v>
+        <v>22797.6271186441</v>
       </c>
       <c r="L30" s="16" t="n">
         <f aca="false">L29/(1+Supuestos!$B$26)</f>
-        <v>20789.9258474576</v>
+        <v>22086.3983050848</v>
       </c>
       <c r="M30" s="16" t="n">
         <f aca="false">M29/(1+Supuestos!$B$26)</f>
-        <v>27365.4237288136</v>
+        <v>29414.1101694915</v>
       </c>
       <c r="N30" s="16" t="n">
         <f aca="false">SUM(B30:M30)</f>
-        <v>195542.697740113</v>
+        <v>208924.613347458</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="4" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
       <c r="B31" s="9" t="n">
         <f aca="false">SUMPRODUCT(B$14:B$18,Proyeccion!$F$25:$F$29)</f>
-        <v>1722.34576271186</v>
+        <v>1707.09111228814</v>
       </c>
       <c r="C31" s="9" t="n">
         <f aca="false">SUMPRODUCT(C$14:C$18,Proyeccion!$F$25:$F$29)</f>
-        <v>6316.22016949153</v>
+        <v>6369.52097457627</v>
       </c>
       <c r="D31" s="9" t="n">
         <f aca="false">SUMPRODUCT(D$14:D$18,Proyeccion!$F$25:$F$29)</f>
-        <v>7205.63902711864</v>
+        <v>7118.56809152542</v>
       </c>
       <c r="E31" s="9" t="n">
         <f aca="false">SUMPRODUCT(E$14:E$18,Proyeccion!$F$25:$F$29)</f>
-        <v>6682.20198305085</v>
+        <v>6468.60411864407</v>
       </c>
       <c r="F31" s="9" t="n">
         <f aca="false">SUMPRODUCT(F$14:F$18,Proyeccion!$F$25:$F$29)</f>
-        <v>7344.39145932203</v>
+        <v>7081.49793686441</v>
       </c>
       <c r="G31" s="9" t="n">
         <f aca="false">SUMPRODUCT(G$14:G$18,Proyeccion!$F$25:$F$29)</f>
-        <v>6985.80520677966</v>
+        <v>6663.02898813559</v>
       </c>
       <c r="H31" s="9" t="n">
         <f aca="false">SUMPRODUCT(H$14:H$18,Proyeccion!$F$25:$F$29)</f>
-        <v>6894.68165847458</v>
+        <v>6658.20293898305</v>
       </c>
       <c r="I31" s="9" t="n">
         <f aca="false">SUMPRODUCT(I$14:I$18,Proyeccion!$F$25:$F$29)</f>
-        <v>9325.30270042373</v>
+        <v>8930.66290868644</v>
       </c>
       <c r="J31" s="9" t="n">
         <f aca="false">SUMPRODUCT(J$14:J$18,Proyeccion!$F$25:$F$29)</f>
-        <v>9940.7611940678</v>
+        <v>9536.06449449153</v>
       </c>
       <c r="K31" s="9" t="n">
         <f aca="false">SUMPRODUCT(K$14:K$18,Proyeccion!$F$25:$F$29)</f>
-        <v>10345.9490957627</v>
+        <v>9826.56337245763</v>
       </c>
       <c r="L31" s="9" t="n">
         <f aca="false">SUMPRODUCT(L$14:L$18,Proyeccion!$F$25:$F$29)</f>
-        <v>9973.36593898305</v>
+        <v>9445.8430970339</v>
       </c>
       <c r="M31" s="9" t="n">
         <f aca="false">SUMPRODUCT(M$14:M$18,Proyeccion!$F$25:$F$29)</f>
-        <v>14111.6237915254</v>
+        <v>13958.0822677966</v>
       </c>
       <c r="N31" s="16" t="n">
         <f aca="false">SUM(B31:M31)</f>
-        <v>96848.2879877119</v>
+        <v>93763.7303014831</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="4" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
       <c r="B32" s="9" t="n">
         <f aca="false">SUMPRODUCT(B$14:B$18,Proyeccion!$G$25:$G$29)</f>
-        <v>1756.99576271186</v>
+        <v>1741.74111228814</v>
       </c>
       <c r="C32" s="9" t="n">
         <f aca="false">SUMPRODUCT(C$14:C$18,Proyeccion!$G$25:$G$29)</f>
-        <v>6409.46016949153</v>
+        <v>6462.76097457627</v>
       </c>
       <c r="D32" s="9" t="n">
         <f aca="false">SUMPRODUCT(D$14:D$18,Proyeccion!$G$25:$G$29)</f>
-        <v>7331.84062711865</v>
+        <v>7244.76969152542</v>
       </c>
       <c r="E32" s="9" t="n">
         <f aca="false">SUMPRODUCT(E$14:E$18,Proyeccion!$G$25:$G$29)</f>
-        <v>6802.15398305085</v>
+        <v>6588.55611864407</v>
       </c>
       <c r="F32" s="9" t="n">
         <f aca="false">SUMPRODUCT(F$14:F$18,Proyeccion!$G$25:$G$29)</f>
-        <v>7469.45905932204</v>
+        <v>7206.56553686441</v>
       </c>
       <c r="G32" s="9" t="n">
         <f aca="false">SUMPRODUCT(G$14:G$18,Proyeccion!$G$25:$G$29)</f>
-        <v>7108.68040677966</v>
+        <v>6785.90418813559</v>
       </c>
       <c r="H32" s="9" t="n">
         <f aca="false">SUMPRODUCT(H$14:H$18,Proyeccion!$G$25:$G$29)</f>
-        <v>7022.22725847458</v>
+        <v>6785.74853898305</v>
       </c>
       <c r="I32" s="9" t="n">
         <f aca="false">SUMPRODUCT(I$14:I$18,Proyeccion!$G$25:$G$29)</f>
-        <v>9476.08690042373</v>
+        <v>9081.44710868644</v>
       </c>
       <c r="J32" s="9" t="n">
         <f aca="false">SUMPRODUCT(J$14:J$18,Proyeccion!$G$25:$G$29)</f>
-        <v>10108.6183940678</v>
+        <v>9703.92169449153</v>
       </c>
       <c r="K32" s="9" t="n">
         <f aca="false">SUMPRODUCT(K$14:K$18,Proyeccion!$G$25:$G$29)</f>
-        <v>10521.2654957627</v>
+        <v>10001.8797724576</v>
       </c>
       <c r="L32" s="9" t="n">
         <f aca="false">SUMPRODUCT(L$14:L$18,Proyeccion!$G$25:$G$29)</f>
-        <v>10144.9023389831</v>
+        <v>9617.3794970339</v>
       </c>
       <c r="M32" s="9" t="n">
         <f aca="false">SUMPRODUCT(M$14:M$18,Proyeccion!$G$25:$G$29)</f>
-        <v>14340.8429915254</v>
+        <v>14187.3014677966</v>
       </c>
       <c r="N32" s="16" t="n">
         <f aca="false">SUM(B32:M32)</f>
-        <v>98492.5333877119</v>
+        <v>95407.9757014831</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="4" t="s">
-        <v>322</v>
+        <v>325</v>
       </c>
       <c r="B33" s="9" t="n">
         <f aca="false">B5*Supuestos!$B$57</f>
@@ -7170,7 +7179,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="4" t="s">
-        <v>323</v>
+        <v>326</v>
       </c>
       <c r="B34" s="9" t="n">
         <f aca="false">MAX(0,B5-Supuestos!$B$59)*B6*Supuestos!$B$58</f>
@@ -7227,7 +7236,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="4" t="s">
-        <v>324</v>
+        <v>327</v>
       </c>
       <c r="B35" s="9" t="n">
         <f aca="false">B8*Supuestos!$B$60</f>
@@ -7284,341 +7293,341 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="4" t="s">
-        <v>325</v>
+        <v>328</v>
       </c>
       <c r="B36" s="9" t="n">
         <f aca="false">Supuestos!$B$72</f>
-        <v>2503.38888888889</v>
+        <v>2753.38888888889</v>
       </c>
       <c r="C36" s="9" t="n">
         <f aca="false">Supuestos!$B$72</f>
-        <v>2503.38888888889</v>
+        <v>2753.38888888889</v>
       </c>
       <c r="D36" s="9" t="n">
         <f aca="false">Supuestos!$B$72</f>
-        <v>2503.38888888889</v>
+        <v>2753.38888888889</v>
       </c>
       <c r="E36" s="9" t="n">
         <f aca="false">Supuestos!$B$72</f>
-        <v>2503.38888888889</v>
+        <v>2753.38888888889</v>
       </c>
       <c r="F36" s="9" t="n">
         <f aca="false">Supuestos!$B$72</f>
-        <v>2503.38888888889</v>
+        <v>2753.38888888889</v>
       </c>
       <c r="G36" s="9" t="n">
         <f aca="false">Supuestos!$B$72</f>
-        <v>2503.38888888889</v>
+        <v>2753.38888888889</v>
       </c>
       <c r="H36" s="9" t="n">
         <f aca="false">Supuestos!$B$72</f>
-        <v>2503.38888888889</v>
+        <v>2753.38888888889</v>
       </c>
       <c r="I36" s="9" t="n">
         <f aca="false">Supuestos!$B$72</f>
-        <v>2503.38888888889</v>
+        <v>2753.38888888889</v>
       </c>
       <c r="J36" s="9" t="n">
         <f aca="false">Supuestos!$B$72</f>
-        <v>2503.38888888889</v>
+        <v>2753.38888888889</v>
       </c>
       <c r="K36" s="9" t="n">
         <f aca="false">Supuestos!$B$72</f>
-        <v>2503.38888888889</v>
+        <v>2753.38888888889</v>
       </c>
       <c r="L36" s="9" t="n">
         <f aca="false">Supuestos!$B$72</f>
-        <v>2503.38888888889</v>
+        <v>2753.38888888889</v>
       </c>
       <c r="M36" s="9" t="n">
         <f aca="false">Supuestos!$B$72</f>
-        <v>2503.38888888889</v>
+        <v>2753.38888888889</v>
       </c>
       <c r="N36" s="16" t="n">
         <f aca="false">SUM(B36:M36)</f>
-        <v>30040.6666666667</v>
+        <v>33040.6666666667</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="10" t="s">
-        <v>326</v>
+        <v>329</v>
       </c>
       <c r="B37" s="11" t="n">
         <f aca="false">B31-B33-B34-B35-B36</f>
-        <v>-2191.04312617702</v>
+        <v>-2456.29777660075</v>
       </c>
       <c r="C37" s="11" t="n">
         <f aca="false">C31-C33-C34-C35-C36</f>
-        <v>-807.168719397363</v>
+        <v>-1003.86791431262</v>
       </c>
       <c r="D37" s="11" t="n">
         <f aca="false">D31-D33-D34-D35-D36</f>
-        <v>1882.25013822976</v>
+        <v>1545.17920263653</v>
       </c>
       <c r="E37" s="11" t="n">
         <f aca="false">E31-E33-E34-E35-E36</f>
-        <v>1358.81309416196</v>
+        <v>895.215229755179</v>
       </c>
       <c r="F37" s="11" t="n">
         <f aca="false">F31-F33-F34-F35-F36</f>
-        <v>2021.00257043314</v>
+        <v>1508.10904797552</v>
       </c>
       <c r="G37" s="11" t="n">
         <f aca="false">G31-G33-G34-G35-G36</f>
-        <v>1662.41631789077</v>
+        <v>1089.64009924671</v>
       </c>
       <c r="H37" s="11" t="n">
         <f aca="false">H31-H33-H34-H35-H36</f>
-        <v>1391.29276958569</v>
+        <v>904.814050094162</v>
       </c>
       <c r="I37" s="11" t="n">
         <f aca="false">I31-I33-I34-I35-I36</f>
-        <v>2591.91381153484</v>
+        <v>1947.27401979755</v>
       </c>
       <c r="J37" s="11" t="n">
         <f aca="false">J31-J33-J34-J35-J36</f>
-        <v>3207.37230517891</v>
+        <v>2552.67560560264</v>
       </c>
       <c r="K37" s="11" t="n">
         <f aca="false">K31-K33-K34-K35-K36</f>
-        <v>3612.56020687382</v>
+        <v>2843.17448356874</v>
       </c>
       <c r="L37" s="11" t="n">
         <f aca="false">L31-L33-L34-L35-L36</f>
-        <v>3239.97705009416</v>
+        <v>2462.45420814501</v>
       </c>
       <c r="M37" s="11" t="n">
         <f aca="false">M31-M33-M34-M35-M36</f>
-        <v>2968.23490263653</v>
+        <v>2564.69337890772</v>
       </c>
       <c r="N37" s="11" t="n">
         <f aca="false">SUM(B37:M37)</f>
-        <v>20937.6213210452</v>
+        <v>14853.0636348164</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="10" t="s">
-        <v>327</v>
+        <v>330</v>
       </c>
       <c r="B38" s="11" t="n">
         <f aca="false">B32-B33-B34-B35-B36</f>
-        <v>-2156.39312617702</v>
+        <v>-2421.64777660075</v>
       </c>
       <c r="C38" s="11" t="n">
         <f aca="false">C32-C33-C34-C35-C36</f>
-        <v>-713.928719397363</v>
+        <v>-910.627914312618</v>
       </c>
       <c r="D38" s="11" t="n">
         <f aca="false">D32-D33-D34-D35-D36</f>
-        <v>2008.45173822976</v>
+        <v>1671.38080263654</v>
       </c>
       <c r="E38" s="11" t="n">
         <f aca="false">E32-E33-E34-E35-E36</f>
-        <v>1478.76509416196</v>
+        <v>1015.16722975518</v>
       </c>
       <c r="F38" s="11" t="n">
         <f aca="false">F32-F33-F34-F35-F36</f>
-        <v>2146.07017043315</v>
+        <v>1633.17664797552</v>
       </c>
       <c r="G38" s="11" t="n">
         <f aca="false">G32-G33-G34-G35-G36</f>
-        <v>1785.29151789077</v>
+        <v>1212.5152992467</v>
       </c>
       <c r="H38" s="11" t="n">
         <f aca="false">H32-H33-H34-H35-H36</f>
-        <v>1518.83836958569</v>
+        <v>1032.35965009416</v>
       </c>
       <c r="I38" s="11" t="n">
         <f aca="false">I32-I33-I34-I35-I36</f>
-        <v>2742.69801153484</v>
+        <v>2098.05821979755</v>
       </c>
       <c r="J38" s="11" t="n">
         <f aca="false">J32-J33-J34-J35-J36</f>
-        <v>3375.22950517891</v>
+        <v>2720.53280560264</v>
       </c>
       <c r="K38" s="11" t="n">
         <f aca="false">K32-K33-K34-K35-K36</f>
-        <v>3787.87660687382</v>
+        <v>3018.49088356874</v>
       </c>
       <c r="L38" s="11" t="n">
         <f aca="false">L32-L33-L34-L35-L36</f>
-        <v>3411.51345009416</v>
+        <v>2633.99060814501</v>
       </c>
       <c r="M38" s="11" t="n">
         <f aca="false">M32-M33-M34-M35-M36</f>
-        <v>3197.45410263654</v>
+        <v>2793.91257890772</v>
       </c>
       <c r="N38" s="11" t="n">
         <f aca="false">SUM(B38:M38)</f>
-        <v>22581.8667210452</v>
+        <v>16497.3090348164</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="4" t="s">
-        <v>328</v>
+        <v>331</v>
       </c>
       <c r="B39" s="16" t="n">
         <f aca="false">B37</f>
-        <v>-2191.04312617702</v>
+        <v>-2456.29777660075</v>
       </c>
       <c r="C39" s="16" t="n">
         <f aca="false">B39+C37</f>
-        <v>-2998.21184557439</v>
+        <v>-3460.16569091337</v>
       </c>
       <c r="D39" s="16" t="n">
         <f aca="false">C39+D37</f>
-        <v>-1115.96170734463</v>
+        <v>-1914.98648827684</v>
       </c>
       <c r="E39" s="16" t="n">
         <f aca="false">D39+E37</f>
-        <v>242.851386817326</v>
+        <v>-1019.77125852166</v>
       </c>
       <c r="F39" s="16" t="n">
         <f aca="false">E39+F37</f>
-        <v>2263.85395725047</v>
+        <v>488.337789453862</v>
       </c>
       <c r="G39" s="16" t="n">
         <f aca="false">F39+G37</f>
-        <v>3926.27027514124</v>
+        <v>1577.97788870057</v>
       </c>
       <c r="H39" s="16" t="n">
         <f aca="false">G39+H37</f>
-        <v>5317.56304472693</v>
+        <v>2482.79193879473</v>
       </c>
       <c r="I39" s="16" t="n">
         <f aca="false">H39+I37</f>
-        <v>7909.47685626177</v>
+        <v>4430.06595859228</v>
       </c>
       <c r="J39" s="16" t="n">
         <f aca="false">I39+J37</f>
-        <v>11116.8491614407</v>
+        <v>6982.74156419492</v>
       </c>
       <c r="K39" s="16" t="n">
         <f aca="false">J39+K37</f>
-        <v>14729.4093683145</v>
+        <v>9825.91604776366</v>
       </c>
       <c r="L39" s="16" t="n">
         <f aca="false">K39+L37</f>
-        <v>17969.3864184087</v>
+        <v>12288.3702559087</v>
       </c>
       <c r="M39" s="16" t="n">
         <f aca="false">L39+M37</f>
-        <v>20937.6213210452</v>
+        <v>14853.0636348164</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="4" t="s">
-        <v>329</v>
+        <v>332</v>
       </c>
       <c r="B40" s="16" t="n">
         <f aca="false">B38</f>
-        <v>-2156.39312617702</v>
+        <v>-2421.64777660075</v>
       </c>
       <c r="C40" s="16" t="n">
         <f aca="false">B40+C38</f>
-        <v>-2870.32184557439</v>
+        <v>-3332.27569091337</v>
       </c>
       <c r="D40" s="16" t="n">
         <f aca="false">C40+D38</f>
-        <v>-861.870107344631</v>
+        <v>-1660.89488827684</v>
       </c>
       <c r="E40" s="16" t="n">
         <f aca="false">D40+E38</f>
-        <v>616.894986817329</v>
+        <v>-645.727658521656</v>
       </c>
       <c r="F40" s="16" t="n">
         <f aca="false">E40+F38</f>
-        <v>2762.96515725047</v>
+        <v>987.448989453862</v>
       </c>
       <c r="G40" s="16" t="n">
         <f aca="false">F40+G38</f>
-        <v>4548.25667514125</v>
+        <v>2199.96428870057</v>
       </c>
       <c r="H40" s="16" t="n">
         <f aca="false">G40+H38</f>
-        <v>6067.09504472694</v>
+        <v>3232.32393879473</v>
       </c>
       <c r="I40" s="16" t="n">
         <f aca="false">H40+I38</f>
-        <v>8809.79305626178</v>
+        <v>5330.38215859228</v>
       </c>
       <c r="J40" s="16" t="n">
         <f aca="false">I40+J38</f>
-        <v>12185.0225614407</v>
+        <v>8050.91496419492</v>
       </c>
       <c r="K40" s="16" t="n">
         <f aca="false">J40+K38</f>
-        <v>15972.8991683145</v>
+        <v>11069.4058477637</v>
       </c>
       <c r="L40" s="16" t="n">
         <f aca="false">K40+L38</f>
-        <v>19384.4126184087</v>
+        <v>13703.3964559087</v>
       </c>
       <c r="M40" s="16" t="n">
         <f aca="false">L40+M38</f>
-        <v>22581.8667210452</v>
+        <v>16497.3090348164</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="4" t="s">
-        <v>330</v>
+        <v>333</v>
       </c>
       <c r="B41" s="9" t="n">
         <f aca="false">IF(1&lt;=Inversion!$B$49,Inversion!$B$50,0)</f>
-        <v>729.471399828276</v>
+        <v>1150.32028434459</v>
       </c>
       <c r="C41" s="9" t="n">
         <f aca="false">IF(2&lt;=Inversion!$B$49,Inversion!$B$50,0)</f>
-        <v>729.471399828276</v>
+        <v>1150.32028434459</v>
       </c>
       <c r="D41" s="9" t="n">
         <f aca="false">IF(3&lt;=Inversion!$B$49,Inversion!$B$50,0)</f>
-        <v>729.471399828276</v>
+        <v>1150.32028434459</v>
       </c>
       <c r="E41" s="9" t="n">
         <f aca="false">IF(4&lt;=Inversion!$B$49,Inversion!$B$50,0)</f>
-        <v>729.471399828276</v>
+        <v>1150.32028434459</v>
       </c>
       <c r="F41" s="9" t="n">
         <f aca="false">IF(5&lt;=Inversion!$B$49,Inversion!$B$50,0)</f>
-        <v>729.471399828276</v>
+        <v>1150.32028434459</v>
       </c>
       <c r="G41" s="9" t="n">
         <f aca="false">IF(6&lt;=Inversion!$B$49,Inversion!$B$50,0)</f>
-        <v>729.471399828276</v>
+        <v>1150.32028434459</v>
       </c>
       <c r="H41" s="9" t="n">
         <f aca="false">IF(7&lt;=Inversion!$B$49,Inversion!$B$50,0)</f>
-        <v>729.471399828276</v>
+        <v>1150.32028434459</v>
       </c>
       <c r="I41" s="9" t="n">
         <f aca="false">IF(8&lt;=Inversion!$B$49,Inversion!$B$50,0)</f>
-        <v>729.471399828276</v>
+        <v>1150.32028434459</v>
       </c>
       <c r="J41" s="9" t="n">
         <f aca="false">IF(9&lt;=Inversion!$B$49,Inversion!$B$50,0)</f>
-        <v>729.471399828276</v>
+        <v>1150.32028434459</v>
       </c>
       <c r="K41" s="9" t="n">
         <f aca="false">IF(10&lt;=Inversion!$B$49,Inversion!$B$50,0)</f>
-        <v>729.471399828276</v>
+        <v>1150.32028434459</v>
       </c>
       <c r="L41" s="9" t="n">
         <f aca="false">IF(11&lt;=Inversion!$B$49,Inversion!$B$50,0)</f>
-        <v>729.471399828276</v>
+        <v>1150.32028434459</v>
       </c>
       <c r="M41" s="9" t="n">
         <f aca="false">IF(12&lt;=Inversion!$B$49,Inversion!$B$50,0)</f>
-        <v>729.471399828276</v>
+        <v>1150.32028434459</v>
       </c>
       <c r="N41" s="16" t="n">
         <f aca="false">SUM(B41:M41)</f>
-        <v>8753.65679793931</v>
+        <v>13803.8434121351</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="4" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
       <c r="B42" s="9" t="n">
         <f aca="false">Supuestos!$B$71</f>
@@ -7675,60 +7684,60 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="10" t="s">
-        <v>332</v>
+        <v>335</v>
       </c>
       <c r="B43" s="11" t="n">
         <f aca="false">Inversion!$B$34+Inversion!$B$52+B37+B42-B41</f>
-        <v>5319.63336288359</v>
+        <v>4669.58982794354</v>
       </c>
       <c r="C43" s="11" t="n">
         <f aca="false">B43+C37+C42-C41</f>
-        <v>3917.38213254684</v>
+        <v>2649.79051817523</v>
       </c>
       <c r="D43" s="11" t="n">
         <f aca="false">C43+D37+D42-D41</f>
-        <v>5204.54975983721</v>
+        <v>3179.03832535606</v>
       </c>
       <c r="E43" s="11" t="n">
         <f aca="false">D43+E37+E42-E41</f>
-        <v>5968.28034305978</v>
+        <v>3058.32215965554</v>
       </c>
       <c r="F43" s="11" t="n">
         <f aca="false">E43+F37+F42-F41</f>
-        <v>7394.20040255354</v>
+        <v>3550.49981217536</v>
       </c>
       <c r="G43" s="11" t="n">
         <f aca="false">F43+G37+G42-G41</f>
-        <v>8461.53420950493</v>
+        <v>3624.20851596636</v>
       </c>
       <c r="H43" s="11" t="n">
         <f aca="false">G43+H37+H42-H41</f>
-        <v>9257.74446815123</v>
+        <v>3513.09117060482</v>
       </c>
       <c r="I43" s="11" t="n">
         <f aca="false">H43+I37+I42-I41</f>
-        <v>11254.5757687467</v>
+        <v>4444.43379494668</v>
       </c>
       <c r="J43" s="11" t="n">
         <f aca="false">I43+J37+J42-J41</f>
-        <v>13866.8655629862</v>
+        <v>5981.17800509361</v>
       </c>
       <c r="K43" s="11" t="n">
         <f aca="false">J43+K37+K42-K41</f>
-        <v>16884.3432589206</v>
+        <v>7808.42109320665</v>
       </c>
       <c r="L43" s="11" t="n">
         <f aca="false">K43+L37+L42-L41</f>
-        <v>19529.2377980754</v>
+        <v>9254.94390589596</v>
       </c>
       <c r="M43" s="11" t="n">
         <f aca="false">L43+M37+M42-M41</f>
-        <v>21902.3901897726</v>
+        <v>10803.705889348</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="4" t="s">
-        <v>333</v>
+        <v>336</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Excel de costeo: bloque de costo total por unidad en Resumen y nota de pauta Meta/YouTube
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Kfbf7cfV7pXUcNjjyaPCzV
</commit_message>
<xml_diff>
--- a/04-reformulacion/Costeo-presentaciones-AndiBite.xlsx
+++ b/04-reformulacion/Costeo-presentaciones-AndiBite.xlsx
@@ -181,7 +181,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="77">
+  <cellXfs count="78">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -409,6 +409,9 @@
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
     <xf numFmtId="164" fontId="11" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
   </cellXfs>
@@ -866,7 +869,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G51"/>
+  <dimension ref="A1:G61"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="70" customWidth="1" style="38" min="1" max="1"/>
@@ -1531,6 +1534,135 @@
       <c r="A51" s="43" t="inlineStr">
         <is>
           <t>5. Respaldo: línea de crédito de S/3,000 (hoja Inversion) por si las ventas por punto bajan; con 20 % menos, la caja más baja del año 1 llegaría a unos −S/2,200 y la línea la cubre.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="44" t="inlineStr">
+        <is>
+          <t>Costo total por unidad, año 1 (promedio de las 52,331 unidades)</t>
+        </is>
+      </c>
+      <c r="B53" s="44" t="inlineStr">
+        <is>
+          <t>Opción B (bolsitas)</t>
+        </is>
+      </c>
+      <c r="C53" s="44" t="inlineStr">
+        <is>
+          <t>Opción C (sueltos)</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="43" t="inlineStr">
+        <is>
+          <t>Costo de producción por unidad (insumos, maquila, empaque, merma y control de calidad)</t>
+        </is>
+      </c>
+      <c r="B54" s="52">
+        <f>IF(B12=0,0,SUMPRODUCT(Proyeccion!K5:K24,Proyeccion!G5:G24)/B12)</f>
+        <v/>
+      </c>
+      <c r="C54" s="52">
+        <f>IF(C12=0,0,SUMPRODUCT(Proyeccion!L5:L24,Proyeccion!G5:G24)/C12)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="43" t="inlineStr">
+        <is>
+          <t>Costo variable de canal por unidad (delivery, pasarela, degustación y comisiones)</t>
+        </is>
+      </c>
+      <c r="B55" s="52">
+        <f>IF(B12=0,0,SUMPRODUCT(Proyeccion!M5:M24,Proyeccion!G5:G24)/B12)</f>
+        <v/>
+      </c>
+      <c r="C55" s="52">
+        <f>IF(C12=0,0,SUMPRODUCT(Proyeccion!M5:M24,Proyeccion!G5:G24)/C12)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="43" t="inlineStr">
+        <is>
+          <t>Stands, vendedores, ferias y eventos por unidad</t>
+        </is>
+      </c>
+      <c r="B56" s="52">
+        <f>IF(B12=0,0,B16/B12)</f>
+        <v/>
+      </c>
+      <c r="C56" s="52">
+        <f>IF(C12=0,0,C16/C12)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="43" t="inlineStr">
+        <is>
+          <t>Costos fijos por unidad (administración, coordinadora, marketing y depreciación)</t>
+        </is>
+      </c>
+      <c r="B57" s="52">
+        <f>IF(B12=0,0,B17/B12)</f>
+        <v/>
+      </c>
+      <c r="C57" s="52">
+        <f>IF(C12=0,0,C17/C12)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="49" t="inlineStr">
+        <is>
+          <t>Costo total por unidad</t>
+        </is>
+      </c>
+      <c r="B58" s="77">
+        <f>SUM(B54:B57)</f>
+        <v/>
+      </c>
+      <c r="C58" s="77">
+        <f>SUM(C54:C57)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="43" t="inlineStr">
+        <is>
+          <t>Venta promedio por unidad sin IGV</t>
+        </is>
+      </c>
+      <c r="B59" s="52">
+        <f>IF(B12=0,0,B14/B12)</f>
+        <v/>
+      </c>
+      <c r="C59" s="52">
+        <f>IF(C12=0,0,C14/C12)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="43" t="inlineStr">
+        <is>
+          <t>Resultado operativo por unidad (venta menos costo total)</t>
+        </is>
+      </c>
+      <c r="B60" s="52">
+        <f>B59-B58</f>
+        <v/>
+      </c>
+      <c r="C60" s="52">
+        <f>C59-C58</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="43" t="inlineStr">
+        <is>
+          <t>El costo total por unidad suma lo que cuesta producir, vender y sostener el negocio, repartido entre todas las unidades del año. Es informativo: el punto de equilibrio de la fila 21 se calcula con la contribución por unidad (fila 20) y los costos fijos.</t>
         </is>
       </c>
     </row>
@@ -2782,7 +2914,7 @@
       </c>
       <c r="D72" s="43" t="inlineStr">
         <is>
-          <t>La captación se hace en el stand; la pauta apoya las fechas clave (plan de marketing mes a mes en el documento 05)</t>
+          <t>S/700 al mes = S/8,400 en el año. Desde el 19-oct-2026: pauta S/5,050 (S/4,050 en Instagram y Facebook y S/1,000 en YouTube), degustaciones extra S/1,750 y material S/1,600. El detalle mes a mes está en Presupuesto-marketing-AndiBite.xlsx</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Excel de costeo: sale la opción C; todas las presentaciones con bolsita individual (cifras sin cambio)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Kfbf7cfV7pXUcNjjyaPCzV
</commit_message>
<xml_diff>
--- a/04-reformulacion/Costeo-presentaciones-AndiBite.xlsx
+++ b/04-reformulacion/Costeo-presentaciones-AndiBite.xlsx
@@ -683,7 +683,7 @@
     <row r="3" ht="35.05" customHeight="1" s="39">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>Qué es: el costeo de AndiBite con cuatro presentaciones (unidad individual, pack de 6, pack de 12 y caja de 3 sabores) y dos formas de armar el pack de 6 (opción B con bolsitas y opción C con brownies sueltos). La planta de maquila hornea y empaca; no hay planta propia.</t>
+          <t>Qué es: el costeo de AndiBite con cuatro presentaciones (unidad individual, pack de 6, pack de 12 y caja de 3 sabores), todas con cada brownie en bolsita individual. La planta de maquila hornea y empaca; no hay planta propia.</t>
         </is>
       </c>
     </row>
@@ -852,7 +852,7 @@
     <row r="30">
       <c r="A30" s="41" t="inlineStr">
         <is>
-          <t>Actualizado el 20-oct-2026: campaña «Lo que nadie ve» con concurso #LoQueNadieVe; pauta 2027 S/4,050 en Meta y S/1,000 en YouTube; embajadores papás y mamás. Ninguna cifra cambió; el detalle está en Presupuesto-marketing-AndiBite.xlsx.</t>
+          <t>Actualizado el 20-oct-2026: campaña «Lo que nadie ve» con concurso #LoQueNadieVe; pauta 2027 S/4,050 en Meta y S/1,000 en YouTube; embajadores papás y mamás. Ninguna cifra cambió; el detalle está en Presupuesto-marketing-AndiBite.xlsx. 27-oct-2026: se retira la opción C (brownies sueltos); todas las presentaciones llevan bolsita individual. Cifras sin cambio.</t>
         </is>
       </c>
     </row>
@@ -961,7 +961,7 @@
     <row r="6" ht="15" customHeight="1" s="39">
       <c r="A6" s="43" t="inlineStr">
         <is>
-          <t>Pack de 6 — opción B (con bolsitas)</t>
+          <t>Pack de 6</t>
         </is>
       </c>
       <c r="B6" s="45">
@@ -990,35 +990,13 @@
       </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="39">
-      <c r="A7" s="43" t="inlineStr">
-        <is>
-          <t>Pack de 6 — opción C (sueltos)</t>
-        </is>
-      </c>
-      <c r="B7" s="45">
-        <f>Costeo!D15</f>
-        <v/>
-      </c>
-      <c r="C7" s="45">
-        <f>Costeo!D16</f>
-        <v/>
-      </c>
-      <c r="D7" s="45">
-        <f>Costeo!D19</f>
-        <v/>
-      </c>
-      <c r="E7" s="46">
-        <f>Costeo!D22</f>
-        <v/>
-      </c>
-      <c r="F7" s="45">
-        <f>Costeo!D25</f>
-        <v/>
-      </c>
-      <c r="G7" s="46">
-        <f>Costeo!D28</f>
-        <v/>
-      </c>
+      <c r="A7" s="43" t="n"/>
+      <c r="B7" s="45" t="n"/>
+      <c r="C7" s="45" t="n"/>
+      <c r="D7" s="45" t="n"/>
+      <c r="E7" s="46" t="n"/>
+      <c r="F7" s="45" t="n"/>
+      <c r="G7" s="46" t="n"/>
     </row>
     <row r="8" ht="15" customHeight="1" s="39">
       <c r="A8" s="43" t="inlineStr">
@@ -1090,14 +1068,10 @@
       </c>
       <c r="B11" s="44" t="inlineStr">
         <is>
-          <t>Opción B (bolsitas)</t>
-        </is>
-      </c>
-      <c r="C11" s="44" t="inlineStr">
-        <is>
-          <t>Opción C (sueltos)</t>
-        </is>
-      </c>
+          <t>Año 1</t>
+        </is>
+      </c>
+      <c r="C11" s="44" t="n"/>
       <c r="D11" s="44" t="n"/>
       <c r="E11" s="44" t="n"/>
     </row>
@@ -1111,10 +1085,7 @@
         <f>Proyeccion!F25</f>
         <v/>
       </c>
-      <c r="C12" s="47">
-        <f>Proyeccion!F25</f>
-        <v/>
-      </c>
+      <c r="C12" s="47" t="n"/>
     </row>
     <row r="13" ht="15" customHeight="1" s="39">
       <c r="A13" s="43" t="inlineStr">
@@ -1126,10 +1097,7 @@
         <f>Proyeccion!I25</f>
         <v/>
       </c>
-      <c r="C13" s="48">
-        <f>Proyeccion!I25</f>
-        <v/>
-      </c>
+      <c r="C13" s="48" t="n"/>
     </row>
     <row r="14" ht="15" customHeight="1" s="39">
       <c r="A14" s="43" t="inlineStr">
@@ -1141,10 +1109,7 @@
         <f>Proyeccion!J25</f>
         <v/>
       </c>
-      <c r="C14" s="48">
-        <f>Proyeccion!J25</f>
-        <v/>
-      </c>
+      <c r="C14" s="48" t="n"/>
     </row>
     <row r="15" ht="15" customHeight="1" s="39">
       <c r="A15" s="43" t="inlineStr">
@@ -1156,10 +1121,7 @@
         <f>Proyeccion!P25</f>
         <v/>
       </c>
-      <c r="C15" s="48">
-        <f>Proyeccion!Q25</f>
-        <v/>
-      </c>
+      <c r="C15" s="48" t="n"/>
     </row>
     <row r="16" ht="15" customHeight="1" s="39">
       <c r="A16" s="43" t="inlineStr">
@@ -1171,10 +1133,7 @@
         <f>SUM(Mensual!N33:N36)</f>
         <v/>
       </c>
-      <c r="C16" s="48">
-        <f>SUM(Mensual!N33:N36)</f>
-        <v/>
-      </c>
+      <c r="C16" s="48" t="n"/>
     </row>
     <row r="17" ht="15" customHeight="1" s="39">
       <c r="A17" s="43" t="inlineStr">
@@ -1186,10 +1145,7 @@
         <f>Supuestos!B75*12</f>
         <v/>
       </c>
-      <c r="C17" s="48">
-        <f>Supuestos!B75*12</f>
-        <v/>
-      </c>
+      <c r="C17" s="48" t="n"/>
     </row>
     <row r="18" ht="15" customHeight="1" s="39">
       <c r="A18" s="49" t="inlineStr">
@@ -1201,10 +1157,7 @@
         <f>B15-B16-B17</f>
         <v/>
       </c>
-      <c r="C18" s="50">
-        <f>C15-C16-C17</f>
-        <v/>
-      </c>
+      <c r="C18" s="50" t="n"/>
     </row>
     <row r="19" ht="15" customHeight="1" s="39">
       <c r="A19" s="43" t="inlineStr">
@@ -1216,10 +1169,7 @@
         <f>IF(B14=0,0,B18/B14)</f>
         <v/>
       </c>
-      <c r="C19" s="51">
-        <f>IF(C14=0,0,C18/C14)</f>
-        <v/>
-      </c>
+      <c r="C19" s="51" t="n"/>
     </row>
     <row r="20" ht="15" customHeight="1" s="39">
       <c r="A20" s="43" t="inlineStr">
@@ -1231,10 +1181,7 @@
         <f>IF(B12=0,0,(B15-B16)/B12)</f>
         <v/>
       </c>
-      <c r="C20" s="52">
-        <f>IF(C12=0,0,(C15-C16)/C12)</f>
-        <v/>
-      </c>
+      <c r="C20" s="52" t="n"/>
     </row>
     <row r="21" ht="15" customHeight="1" s="39">
       <c r="A21" s="49" t="inlineStr">
@@ -1246,10 +1193,7 @@
         <f>IF(B20&lt;=0,"No alcanza",Supuestos!$B$75/B20)</f>
         <v/>
       </c>
-      <c r="C21" s="53">
-        <f>IF(C20&lt;=0,"No alcanza",Supuestos!$B$75/C20)</f>
-        <v/>
-      </c>
+      <c r="C21" s="53" t="n"/>
     </row>
     <row r="22" ht="15" customHeight="1" s="39">
       <c r="A22" s="43" t="inlineStr">
@@ -1261,10 +1205,7 @@
         <f>IF(ISNUMBER(B21),B21/6,"No alcanza")</f>
         <v/>
       </c>
-      <c r="C22" s="54">
-        <f>IF(ISNUMBER(C21),C21/6,"No alcanza")</f>
-        <v/>
-      </c>
+      <c r="C22" s="54" t="n"/>
     </row>
     <row r="23" ht="15" customHeight="1" s="39">
       <c r="A23" s="43" t="inlineStr">
@@ -1276,10 +1217,7 @@
         <f>Inversion!B42</f>
         <v/>
       </c>
-      <c r="C23" s="48">
-        <f>Inversion!B42</f>
-        <v/>
-      </c>
+      <c r="C23" s="48" t="n"/>
     </row>
     <row r="24" ht="15" customHeight="1" s="39">
       <c r="A24" s="43" t="inlineStr">
@@ -1291,25 +1229,19 @@
         <f>B18-B23</f>
         <v/>
       </c>
-      <c r="C24" s="55">
-        <f>C18-C23</f>
-        <v/>
-      </c>
+      <c r="C24" s="55" t="n"/>
     </row>
     <row r="25" ht="15" customHeight="1" s="39">
       <c r="A25" s="43" t="inlineStr">
         <is>
-          <t>Caja más baja del año, con la cuota del préstamo (opción B)</t>
+          <t>Caja más baja del año, con la cuota del préstamo</t>
         </is>
       </c>
       <c r="B25" s="48">
         <f>MIN(Mensual!B44:M44)</f>
         <v/>
       </c>
-      <c r="C25" s="48">
-        <f>MIN(Mensual!B44:M44)</f>
-        <v/>
-      </c>
+      <c r="C25" s="48" t="n"/>
     </row>
     <row r="26" ht="15" customHeight="1" s="39">
       <c r="A26" s="49" t="inlineStr">
@@ -1321,16 +1253,12 @@
         <f>IF(B18&gt;=B23,"Dentro del año 1",IF(Anio2!M31&gt;=B23,12+COUNTIF(Anio2!B31:M31,"&lt;"&amp;B23)+1,ROUNDUP(24+(B23-Anio2!M31)/AVERAGE(Anio2!B30:M30),0)))</f>
         <v/>
       </c>
-      <c r="C26" s="57" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="C26" s="57" t="n"/>
     </row>
     <row r="28" ht="15" customHeight="1" s="39">
       <c r="A28" s="49" t="inlineStr">
         <is>
-          <t>De resultado operativo a utilidad neta (año 1, opción B)</t>
+          <t>De resultado operativo a utilidad neta (año 1)</t>
         </is>
       </c>
     </row>
@@ -1545,14 +1473,10 @@
       </c>
       <c r="B53" s="44" t="inlineStr">
         <is>
-          <t>Opción B (bolsitas)</t>
-        </is>
-      </c>
-      <c r="C53" s="44" t="inlineStr">
-        <is>
-          <t>Opción C (sueltos)</t>
-        </is>
-      </c>
+          <t>Año 1</t>
+        </is>
+      </c>
+      <c r="C53" s="44" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="43" t="inlineStr">
@@ -1564,10 +1488,7 @@
         <f>IF(B12=0,0,SUMPRODUCT(Proyeccion!K5:K24,Proyeccion!G5:G24)/B12)</f>
         <v/>
       </c>
-      <c r="C54" s="52">
-        <f>IF(C12=0,0,SUMPRODUCT(Proyeccion!L5:L24,Proyeccion!G5:G24)/C12)</f>
-        <v/>
-      </c>
+      <c r="C54" s="52" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="43" t="inlineStr">
@@ -1579,10 +1500,7 @@
         <f>IF(B12=0,0,SUMPRODUCT(Proyeccion!M5:M24,Proyeccion!G5:G24)/B12)</f>
         <v/>
       </c>
-      <c r="C55" s="52">
-        <f>IF(C12=0,0,SUMPRODUCT(Proyeccion!M5:M24,Proyeccion!G5:G24)/C12)</f>
-        <v/>
-      </c>
+      <c r="C55" s="52" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="43" t="inlineStr">
@@ -1594,10 +1512,7 @@
         <f>IF(B12=0,0,B16/B12)</f>
         <v/>
       </c>
-      <c r="C56" s="52">
-        <f>IF(C12=0,0,C16/C12)</f>
-        <v/>
-      </c>
+      <c r="C56" s="52" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="43" t="inlineStr">
@@ -1609,10 +1524,7 @@
         <f>IF(B12=0,0,B17/B12)</f>
         <v/>
       </c>
-      <c r="C57" s="52">
-        <f>IF(C12=0,0,C17/C12)</f>
-        <v/>
-      </c>
+      <c r="C57" s="52" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="49" t="inlineStr">
@@ -1624,10 +1536,7 @@
         <f>SUM(B54:B57)</f>
         <v/>
       </c>
-      <c r="C58" s="77">
-        <f>SUM(C54:C57)</f>
-        <v/>
-      </c>
+      <c r="C58" s="77" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="43" t="inlineStr">
@@ -1639,10 +1548,7 @@
         <f>IF(B12=0,0,B14/B12)</f>
         <v/>
       </c>
-      <c r="C59" s="52">
-        <f>IF(C12=0,0,C14/C12)</f>
-        <v/>
-      </c>
+      <c r="C59" s="52" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="43" t="inlineStr">
@@ -1654,10 +1560,7 @@
         <f>B59-B58</f>
         <v/>
       </c>
-      <c r="C60" s="52">
-        <f>C59-C58</f>
-        <v/>
-      </c>
+      <c r="C60" s="52" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="43" t="inlineStr">
@@ -1777,24 +1680,10 @@
       </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="39">
-      <c r="A8" s="43" t="inlineStr">
-        <is>
-          <t>Descuento de maquila si no se empaca cada unidad (opción C)</t>
-        </is>
-      </c>
-      <c r="B8" s="62" t="n">
-        <v>0</v>
-      </c>
-      <c r="C8" s="43" t="inlineStr">
-        <is>
-          <t>S/ por unidad</t>
-        </is>
-      </c>
-      <c r="D8" s="43" t="inlineStr">
-        <is>
-          <t>[HIPÓTESIS] Dejar en 0 hasta que la planta lo confirme</t>
-        </is>
-      </c>
+      <c r="A8" s="43" t="n"/>
+      <c r="B8" s="62" t="n"/>
+      <c r="C8" s="43" t="n"/>
+      <c r="D8" s="43" t="n"/>
     </row>
     <row r="9" ht="15" customHeight="1" s="39">
       <c r="A9" s="43" t="inlineStr">
@@ -1837,24 +1726,10 @@
       </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="39">
-      <c r="A11" s="43" t="inlineStr">
-        <is>
-          <t>Papel manteca separador entre brownies (opción C)</t>
-        </is>
-      </c>
-      <c r="B11" s="61" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="C11" s="43" t="inlineStr">
-        <is>
-          <t>S/ por unidad</t>
-        </is>
-      </c>
-      <c r="D11" s="43" t="inlineStr">
-        <is>
-          <t>[HIPÓTESIS] Rollo de supermercado prorrateado</t>
-        </is>
-      </c>
+      <c r="A11" s="43" t="n"/>
+      <c r="B11" s="61" t="n"/>
+      <c r="C11" s="43" t="n"/>
+      <c r="D11" s="43" t="n"/>
     </row>
     <row r="12" ht="15" customHeight="1" s="39">
       <c r="A12" s="43" t="inlineStr">
@@ -3066,7 +2941,7 @@
     <row r="2" ht="15" customHeight="1" s="39">
       <c r="A2" s="43" t="inlineStr">
         <is>
-          <t>Opción B: cada brownie en bolsita sin etiqueta, dentro del doypack con etiqueta. Opción C: brownies sueltos con papel manteca dentro del doypack. Unidad individual: bolsita con etiqueta completa. Caja de 3 sabores: 3 bolsitas en una caja kraft con una etiqueta.</t>
+          <t>Todas las presentaciones llevan cada brownie en una bolsita individual: sin etiqueta dentro del doypack (pack de 6 y de 12) o de la caja kraft (3 sabores), que llevan la etiqueta; la unidad individual lleva bolsita con etiqueta completa.</t>
         </is>
       </c>
     </row>
@@ -3083,14 +2958,10 @@
       </c>
       <c r="C4" s="44" t="inlineStr">
         <is>
-          <t>Pack de 6 — opción B (con bolsitas)</t>
-        </is>
-      </c>
-      <c r="D4" s="44" t="inlineStr">
-        <is>
-          <t>Pack de 6 — opción C (sueltos)</t>
-        </is>
-      </c>
+          <t>Pack de 6 (con bolsitas)</t>
+        </is>
+      </c>
+      <c r="D4" s="44" t="n"/>
       <c r="E4" s="44" t="inlineStr">
         <is>
           <t>Pack de 12 (con bolsitas)</t>
@@ -3114,9 +2985,7 @@
       <c r="C5" s="67" t="n">
         <v>6</v>
       </c>
-      <c r="D5" s="67" t="n">
-        <v>6</v>
-      </c>
+      <c r="D5" s="67" t="n"/>
       <c r="E5" s="67" t="n">
         <v>12</v>
       </c>
@@ -3138,10 +3007,7 @@
         <f>C5*Supuestos!$B$6</f>
         <v/>
       </c>
-      <c r="D6" s="45">
-        <f>D5*Supuestos!$B$6</f>
-        <v/>
-      </c>
+      <c r="D6" s="45" t="n"/>
       <c r="E6" s="45">
         <f>E5*Supuestos!$B$6</f>
         <v/>
@@ -3165,10 +3031,7 @@
         <f>C5*Supuestos!$B$7</f>
         <v/>
       </c>
-      <c r="D7" s="45">
-        <f>D5*(Supuestos!$B$7-Supuestos!$B$8)</f>
-        <v/>
-      </c>
+      <c r="D7" s="45" t="n"/>
       <c r="E7" s="45">
         <f>E5*Supuestos!$B$7</f>
         <v/>
@@ -3192,9 +3055,7 @@
         <f>C5*Supuestos!$B$9</f>
         <v/>
       </c>
-      <c r="D8" s="52" t="n">
-        <v>0</v>
-      </c>
+      <c r="D8" s="52" t="n"/>
       <c r="E8" s="45">
         <f>E5*Supuestos!$B$9</f>
         <v/>
@@ -3217,9 +3078,7 @@
       <c r="C9" s="52" t="n">
         <v>0</v>
       </c>
-      <c r="D9" s="52" t="n">
-        <v>0</v>
-      </c>
+      <c r="D9" s="52" t="n"/>
       <c r="E9" s="52" t="n">
         <v>0</v>
       </c>
@@ -3229,27 +3088,12 @@
       </c>
     </row>
     <row r="10" ht="15" customHeight="1" s="39">
-      <c r="A10" s="43" t="inlineStr">
-        <is>
-          <t>Papel manteca separador</t>
-        </is>
-      </c>
-      <c r="B10" s="52" t="n">
-        <v>0</v>
-      </c>
-      <c r="C10" s="52" t="n">
-        <v>0</v>
-      </c>
-      <c r="D10" s="45">
-        <f>D5*Supuestos!$B$11</f>
-        <v/>
-      </c>
-      <c r="E10" s="52" t="n">
-        <v>0</v>
-      </c>
-      <c r="F10" s="52" t="n">
-        <v>0</v>
-      </c>
+      <c r="A10" s="43" t="n"/>
+      <c r="B10" s="52" t="n"/>
+      <c r="C10" s="52" t="n"/>
+      <c r="D10" s="45" t="n"/>
+      <c r="E10" s="52" t="n"/>
+      <c r="F10" s="52" t="n"/>
     </row>
     <row r="11" ht="15" customHeight="1" s="39">
       <c r="A11" s="43" t="inlineStr">
@@ -3264,10 +3108,7 @@
         <f>Supuestos!$B$19</f>
         <v/>
       </c>
-      <c r="D11" s="45">
-        <f>Supuestos!$B$19</f>
-        <v/>
-      </c>
+      <c r="D11" s="45" t="n"/>
       <c r="E11" s="45">
         <f>Supuestos!$B$21</f>
         <v/>
@@ -3290,10 +3131,7 @@
         <f>Supuestos!$B$20</f>
         <v/>
       </c>
-      <c r="D12" s="45">
-        <f>Supuestos!$B$20</f>
-        <v/>
-      </c>
+      <c r="D12" s="45" t="n"/>
       <c r="E12" s="45">
         <f>Supuestos!$B$22</f>
         <v/>
@@ -3316,10 +3154,7 @@
         <f>Supuestos!$B$15*SUM(C6:C12)</f>
         <v/>
       </c>
-      <c r="D13" s="52">
-        <f>Supuestos!$B$15*SUM(D6:D12)</f>
-        <v/>
-      </c>
+      <c r="D13" s="52" t="n"/>
       <c r="E13" s="52">
         <f>Supuestos!$B$15*SUM(E6:E12)</f>
         <v/>
@@ -3343,10 +3178,7 @@
         <f>C5*(Supuestos!$B$12+Supuestos!$B$13+Supuestos!$B$14)</f>
         <v/>
       </c>
-      <c r="D14" s="52">
-        <f>D5*(Supuestos!$B$12+Supuestos!$B$13+Supuestos!$B$14)</f>
-        <v/>
-      </c>
+      <c r="D14" s="52" t="n"/>
       <c r="E14" s="52">
         <f>E5*(Supuestos!$B$12+Supuestos!$B$13+Supuestos!$B$14)</f>
         <v/>
@@ -3370,10 +3202,7 @@
         <f>SUM(C6:C14)</f>
         <v/>
       </c>
-      <c r="D15" s="72">
-        <f>SUM(D6:D14)</f>
-        <v/>
-      </c>
+      <c r="D15" s="72" t="n"/>
       <c r="E15" s="72">
         <f>SUM(E6:E14)</f>
         <v/>
@@ -3397,10 +3226,7 @@
         <f>IF(C5=0,0,C15/C5)</f>
         <v/>
       </c>
-      <c r="D16" s="72">
-        <f>IF(D5=0,0,D15/D5)</f>
-        <v/>
-      </c>
+      <c r="D16" s="72" t="n"/>
       <c r="E16" s="72">
         <f>IF(E5=0,0,E15/E5)</f>
         <v/>
@@ -3410,6 +3236,7 @@
         <v/>
       </c>
     </row>
+    <row r="17"/>
     <row r="18" ht="15" customHeight="1" s="39">
       <c r="A18" s="49" t="inlineStr">
         <is>
@@ -3431,10 +3258,7 @@
         <f>Supuestos!C40</f>
         <v/>
       </c>
-      <c r="D19" s="45">
-        <f>Supuestos!C40</f>
-        <v/>
-      </c>
+      <c r="D19" s="45" t="n"/>
       <c r="E19" s="45">
         <f>Supuestos!D40</f>
         <v/>
@@ -3458,10 +3282,7 @@
         <f>C19/(1+Supuestos!$B$26)</f>
         <v/>
       </c>
-      <c r="D20" s="52">
-        <f>D19/(1+Supuestos!$B$26)</f>
-        <v/>
-      </c>
+      <c r="D20" s="52" t="n"/>
       <c r="E20" s="52">
         <f>E19/(1+Supuestos!$B$26)</f>
         <v/>
@@ -3485,10 +3306,7 @@
         <f>C20-C15</f>
         <v/>
       </c>
-      <c r="D21" s="52">
-        <f>D20-D15</f>
-        <v/>
-      </c>
+      <c r="D21" s="52" t="n"/>
       <c r="E21" s="52">
         <f>E20-E15</f>
         <v/>
@@ -3512,10 +3330,7 @@
         <f>IF(C20=0,0,C21/C20)</f>
         <v/>
       </c>
-      <c r="D22" s="51">
-        <f>IF(D20=0,0,D21/D20)</f>
-        <v/>
-      </c>
+      <c r="D22" s="51" t="n"/>
       <c r="E22" s="51">
         <f>IF(E20=0,0,E21/E20)</f>
         <v/>
@@ -3525,6 +3340,7 @@
         <v/>
       </c>
     </row>
+    <row r="23"/>
     <row r="24" ht="15" customHeight="1" s="39">
       <c r="A24" s="49" t="inlineStr">
         <is>
@@ -3546,10 +3362,7 @@
         <f>Supuestos!C42</f>
         <v/>
       </c>
-      <c r="D25" s="45">
-        <f>Supuestos!C42</f>
-        <v/>
-      </c>
+      <c r="D25" s="45" t="n"/>
       <c r="E25" s="45">
         <f>Supuestos!D42</f>
         <v/>
@@ -3573,10 +3386,7 @@
         <f>C25/(1+Supuestos!$B$26)</f>
         <v/>
       </c>
-      <c r="D26" s="52">
-        <f>D25/(1+Supuestos!$B$26)</f>
-        <v/>
-      </c>
+      <c r="D26" s="52" t="n"/>
       <c r="E26" s="52">
         <f>E25/(1+Supuestos!$B$26)</f>
         <v/>
@@ -3600,10 +3410,7 @@
         <f>C26-C15</f>
         <v/>
       </c>
-      <c r="D27" s="52">
-        <f>D26-D15</f>
-        <v/>
-      </c>
+      <c r="D27" s="52" t="n"/>
       <c r="E27" s="52">
         <f>E26-E15</f>
         <v/>
@@ -3627,10 +3434,7 @@
         <f>IF(C26=0,0,C27/C26)</f>
         <v/>
       </c>
-      <c r="D28" s="51">
-        <f>IF(D26=0,0,D27/D26)</f>
-        <v/>
-      </c>
+      <c r="D28" s="51" t="n"/>
       <c r="E28" s="51">
         <f>IF(E26=0,0,E27/E26)</f>
         <v/>
@@ -3735,14 +3539,10 @@
       </c>
       <c r="K4" s="44" t="inlineStr">
         <is>
-          <t>Costo de producción por envase — opción B</t>
-        </is>
-      </c>
-      <c r="L4" s="44" t="inlineStr">
-        <is>
-          <t>Costo de producción por envase — opción C</t>
-        </is>
-      </c>
+          <t>Costo de producción por envase</t>
+        </is>
+      </c>
+      <c r="L4" s="44" t="n"/>
       <c r="M4" s="44" t="inlineStr">
         <is>
           <t>Costo variable de canal por envase</t>
@@ -3750,24 +3550,16 @@
       </c>
       <c r="N4" s="44" t="inlineStr">
         <is>
-          <t>Contribución por envase — opción B</t>
-        </is>
-      </c>
-      <c r="O4" s="44" t="inlineStr">
-        <is>
-          <t>Contribución por envase — opción C</t>
-        </is>
-      </c>
+          <t>Contribución por envase</t>
+        </is>
+      </c>
+      <c r="O4" s="44" t="n"/>
       <c r="P4" s="44" t="inlineStr">
         <is>
-          <t>Contribución total — opción B</t>
-        </is>
-      </c>
-      <c r="Q4" s="44" t="inlineStr">
-        <is>
-          <t>Contribución total — opción C</t>
-        </is>
-      </c>
+          <t>Contribución total</t>
+        </is>
+      </c>
+      <c r="Q4" s="44" t="n"/>
       <c r="R4" s="44" t="inlineStr">
         <is>
           <t>Margen de contribución % — B</t>
@@ -3826,10 +3618,7 @@
         <f>Costeo!B15</f>
         <v/>
       </c>
-      <c r="L5" s="45">
-        <f>Costeo!B15</f>
-        <v/>
-      </c>
+      <c r="L5" s="45" t="n"/>
       <c r="M5" s="52">
         <f>IF(H5=0,0,C5*Supuestos!$B$32+H5*Supuestos!$B$27*Supuestos!$C$32+H5/(1+Supuestos!$B$26)*Supuestos!$B$28)</f>
         <v/>
@@ -3838,18 +3627,12 @@
         <f>IF(H5=0,0,H5/(1+Supuestos!$B$26)-K5-M5)</f>
         <v/>
       </c>
-      <c r="O5" s="52">
-        <f>IF(H5=0,0,H5/(1+Supuestos!$B$26)-L5-M5)</f>
-        <v/>
-      </c>
+      <c r="O5" s="52" t="n"/>
       <c r="P5" s="55">
         <f>G5*N5</f>
         <v/>
       </c>
-      <c r="Q5" s="55">
-        <f>G5*O5</f>
-        <v/>
-      </c>
+      <c r="Q5" s="55" t="n"/>
       <c r="R5" s="51">
         <f>IF(H5=0,0,N5/(H5/(1+Supuestos!$B$26)))</f>
         <v/>
@@ -3906,10 +3689,7 @@
         <f>Costeo!C15</f>
         <v/>
       </c>
-      <c r="L6" s="45">
-        <f>Costeo!D15</f>
-        <v/>
-      </c>
+      <c r="L6" s="45" t="n"/>
       <c r="M6" s="52">
         <f>IF(H6=0,0,C6*Supuestos!$B$32+H6*Supuestos!$B$27*Supuestos!$C$32+H6/(1+Supuestos!$B$26)*Supuestos!$B$28)</f>
         <v/>
@@ -3918,18 +3698,12 @@
         <f>IF(H6=0,0,H6/(1+Supuestos!$B$26)-K6-M6)</f>
         <v/>
       </c>
-      <c r="O6" s="52">
-        <f>IF(H6=0,0,H6/(1+Supuestos!$B$26)-L6-M6)</f>
-        <v/>
-      </c>
+      <c r="O6" s="52" t="n"/>
       <c r="P6" s="55">
         <f>G6*N6</f>
         <v/>
       </c>
-      <c r="Q6" s="55">
-        <f>G6*O6</f>
-        <v/>
-      </c>
+      <c r="Q6" s="55" t="n"/>
       <c r="R6" s="51">
         <f>IF(H6=0,0,N6/(H6/(1+Supuestos!$B$26)))</f>
         <v/>
@@ -3986,10 +3760,7 @@
         <f>Costeo!E15</f>
         <v/>
       </c>
-      <c r="L7" s="45">
-        <f>Costeo!E15</f>
-        <v/>
-      </c>
+      <c r="L7" s="45" t="n"/>
       <c r="M7" s="52">
         <f>IF(H7=0,0,C7*Supuestos!$B$32+H7*Supuestos!$B$27*Supuestos!$C$32+H7/(1+Supuestos!$B$26)*Supuestos!$B$28)</f>
         <v/>
@@ -3998,18 +3769,12 @@
         <f>IF(H7=0,0,H7/(1+Supuestos!$B$26)-K7-M7)</f>
         <v/>
       </c>
-      <c r="O7" s="52">
-        <f>IF(H7=0,0,H7/(1+Supuestos!$B$26)-L7-M7)</f>
-        <v/>
-      </c>
+      <c r="O7" s="52" t="n"/>
       <c r="P7" s="55">
         <f>G7*N7</f>
         <v/>
       </c>
-      <c r="Q7" s="55">
-        <f>G7*O7</f>
-        <v/>
-      </c>
+      <c r="Q7" s="55" t="n"/>
       <c r="R7" s="51">
         <f>IF(H7=0,0,N7/(H7/(1+Supuestos!$B$26)))</f>
         <v/>
@@ -4066,10 +3831,7 @@
         <f>Costeo!F15</f>
         <v/>
       </c>
-      <c r="L8" s="45">
-        <f>Costeo!F15</f>
-        <v/>
-      </c>
+      <c r="L8" s="45" t="n"/>
       <c r="M8" s="52">
         <f>IF(H8=0,0,C8*Supuestos!$B$32+H8*Supuestos!$B$27*Supuestos!$C$32+H8/(1+Supuestos!$B$26)*Supuestos!$B$28)</f>
         <v/>
@@ -4078,18 +3840,12 @@
         <f>IF(H8=0,0,H8/(1+Supuestos!$B$26)-K8-M8)</f>
         <v/>
       </c>
-      <c r="O8" s="52">
-        <f>IF(H8=0,0,H8/(1+Supuestos!$B$26)-L8-M8)</f>
-        <v/>
-      </c>
+      <c r="O8" s="52" t="n"/>
       <c r="P8" s="55">
         <f>G8*N8</f>
         <v/>
       </c>
-      <c r="Q8" s="55">
-        <f>G8*O8</f>
-        <v/>
-      </c>
+      <c r="Q8" s="55" t="n"/>
       <c r="R8" s="51">
         <f>IF(H8=0,0,N8/(H8/(1+Supuestos!$B$26)))</f>
         <v/>
@@ -4146,10 +3902,7 @@
         <f>Costeo!B15</f>
         <v/>
       </c>
-      <c r="L9" s="45">
-        <f>Costeo!B15</f>
-        <v/>
-      </c>
+      <c r="L9" s="45" t="n"/>
       <c r="M9" s="52">
         <f>IF(H9=0,0,C9*Supuestos!$B$33+H9*Supuestos!$B$27*Supuestos!$C$33+H9/(1+Supuestos!$B$26)*Supuestos!$B$28)</f>
         <v/>
@@ -4158,18 +3911,12 @@
         <f>IF(H9=0,0,H9/(1+Supuestos!$B$26)-K9-M9)</f>
         <v/>
       </c>
-      <c r="O9" s="52">
-        <f>IF(H9=0,0,H9/(1+Supuestos!$B$26)-L9-M9)</f>
-        <v/>
-      </c>
+      <c r="O9" s="52" t="n"/>
       <c r="P9" s="55">
         <f>G9*N9</f>
         <v/>
       </c>
-      <c r="Q9" s="55">
-        <f>G9*O9</f>
-        <v/>
-      </c>
+      <c r="Q9" s="55" t="n"/>
       <c r="R9" s="51">
         <f>IF(H9=0,0,N9/(H9/(1+Supuestos!$B$26)))</f>
         <v/>
@@ -4226,10 +3973,7 @@
         <f>Costeo!C15</f>
         <v/>
       </c>
-      <c r="L10" s="45">
-        <f>Costeo!D15</f>
-        <v/>
-      </c>
+      <c r="L10" s="45" t="n"/>
       <c r="M10" s="52">
         <f>IF(H10=0,0,C10*Supuestos!$B$33+H10*Supuestos!$B$27*Supuestos!$C$33+H10/(1+Supuestos!$B$26)*Supuestos!$B$28)</f>
         <v/>
@@ -4238,18 +3982,12 @@
         <f>IF(H10=0,0,H10/(1+Supuestos!$B$26)-K10-M10)</f>
         <v/>
       </c>
-      <c r="O10" s="52">
-        <f>IF(H10=0,0,H10/(1+Supuestos!$B$26)-L10-M10)</f>
-        <v/>
-      </c>
+      <c r="O10" s="52" t="n"/>
       <c r="P10" s="55">
         <f>G10*N10</f>
         <v/>
       </c>
-      <c r="Q10" s="55">
-        <f>G10*O10</f>
-        <v/>
-      </c>
+      <c r="Q10" s="55" t="n"/>
       <c r="R10" s="51">
         <f>IF(H10=0,0,N10/(H10/(1+Supuestos!$B$26)))</f>
         <v/>
@@ -4306,10 +4044,7 @@
         <f>Costeo!E15</f>
         <v/>
       </c>
-      <c r="L11" s="45">
-        <f>Costeo!E15</f>
-        <v/>
-      </c>
+      <c r="L11" s="45" t="n"/>
       <c r="M11" s="52">
         <f>IF(H11=0,0,C11*Supuestos!$B$33+H11*Supuestos!$B$27*Supuestos!$C$33+H11/(1+Supuestos!$B$26)*Supuestos!$B$28)</f>
         <v/>
@@ -4318,18 +4053,12 @@
         <f>IF(H11=0,0,H11/(1+Supuestos!$B$26)-K11-M11)</f>
         <v/>
       </c>
-      <c r="O11" s="52">
-        <f>IF(H11=0,0,H11/(1+Supuestos!$B$26)-L11-M11)</f>
-        <v/>
-      </c>
+      <c r="O11" s="52" t="n"/>
       <c r="P11" s="55">
         <f>G11*N11</f>
         <v/>
       </c>
-      <c r="Q11" s="55">
-        <f>G11*O11</f>
-        <v/>
-      </c>
+      <c r="Q11" s="55" t="n"/>
       <c r="R11" s="51">
         <f>IF(H11=0,0,N11/(H11/(1+Supuestos!$B$26)))</f>
         <v/>
@@ -4386,10 +4115,7 @@
         <f>Costeo!F15</f>
         <v/>
       </c>
-      <c r="L12" s="45">
-        <f>Costeo!F15</f>
-        <v/>
-      </c>
+      <c r="L12" s="45" t="n"/>
       <c r="M12" s="52">
         <f>IF(H12=0,0,C12*Supuestos!$B$33+H12*Supuestos!$B$27*Supuestos!$C$33+H12/(1+Supuestos!$B$26)*Supuestos!$B$28)</f>
         <v/>
@@ -4398,18 +4124,12 @@
         <f>IF(H12=0,0,H12/(1+Supuestos!$B$26)-K12-M12)</f>
         <v/>
       </c>
-      <c r="O12" s="52">
-        <f>IF(H12=0,0,H12/(1+Supuestos!$B$26)-L12-M12)</f>
-        <v/>
-      </c>
+      <c r="O12" s="52" t="n"/>
       <c r="P12" s="55">
         <f>G12*N12</f>
         <v/>
       </c>
-      <c r="Q12" s="55">
-        <f>G12*O12</f>
-        <v/>
-      </c>
+      <c r="Q12" s="55" t="n"/>
       <c r="R12" s="51">
         <f>IF(H12=0,0,N12/(H12/(1+Supuestos!$B$26)))</f>
         <v/>
@@ -4466,10 +4186,7 @@
         <f>Costeo!B15</f>
         <v/>
       </c>
-      <c r="L13" s="45">
-        <f>Costeo!B15</f>
-        <v/>
-      </c>
+      <c r="L13" s="45" t="n"/>
       <c r="M13" s="52">
         <f>IF(H13=0,0,C13*Supuestos!$B$34+H13*Supuestos!$B$27*Supuestos!$C$34+H13/(1+Supuestos!$B$26)*Supuestos!$B$28)</f>
         <v/>
@@ -4478,18 +4195,12 @@
         <f>IF(H13=0,0,H13/(1+Supuestos!$B$26)-K13-M13)</f>
         <v/>
       </c>
-      <c r="O13" s="52">
-        <f>IF(H13=0,0,H13/(1+Supuestos!$B$26)-L13-M13)</f>
-        <v/>
-      </c>
+      <c r="O13" s="52" t="n"/>
       <c r="P13" s="55">
         <f>G13*N13</f>
         <v/>
       </c>
-      <c r="Q13" s="55">
-        <f>G13*O13</f>
-        <v/>
-      </c>
+      <c r="Q13" s="55" t="n"/>
       <c r="R13" s="51">
         <f>IF(H13=0,0,N13/(H13/(1+Supuestos!$B$26)))</f>
         <v/>
@@ -4546,10 +4257,7 @@
         <f>Costeo!C15</f>
         <v/>
       </c>
-      <c r="L14" s="45">
-        <f>Costeo!D15</f>
-        <v/>
-      </c>
+      <c r="L14" s="45" t="n"/>
       <c r="M14" s="52">
         <f>IF(H14=0,0,C14*Supuestos!$B$34+H14*Supuestos!$B$27*Supuestos!$C$34+H14/(1+Supuestos!$B$26)*Supuestos!$B$28)</f>
         <v/>
@@ -4558,18 +4266,12 @@
         <f>IF(H14=0,0,H14/(1+Supuestos!$B$26)-K14-M14)</f>
         <v/>
       </c>
-      <c r="O14" s="52">
-        <f>IF(H14=0,0,H14/(1+Supuestos!$B$26)-L14-M14)</f>
-        <v/>
-      </c>
+      <c r="O14" s="52" t="n"/>
       <c r="P14" s="55">
         <f>G14*N14</f>
         <v/>
       </c>
-      <c r="Q14" s="55">
-        <f>G14*O14</f>
-        <v/>
-      </c>
+      <c r="Q14" s="55" t="n"/>
       <c r="R14" s="51">
         <f>IF(H14=0,0,N14/(H14/(1+Supuestos!$B$26)))</f>
         <v/>
@@ -4626,10 +4328,7 @@
         <f>Costeo!E15</f>
         <v/>
       </c>
-      <c r="L15" s="45">
-        <f>Costeo!E15</f>
-        <v/>
-      </c>
+      <c r="L15" s="45" t="n"/>
       <c r="M15" s="52">
         <f>IF(H15=0,0,C15*Supuestos!$B$34+H15*Supuestos!$B$27*Supuestos!$C$34+H15/(1+Supuestos!$B$26)*Supuestos!$B$28)</f>
         <v/>
@@ -4638,18 +4337,12 @@
         <f>IF(H15=0,0,H15/(1+Supuestos!$B$26)-K15-M15)</f>
         <v/>
       </c>
-      <c r="O15" s="52">
-        <f>IF(H15=0,0,H15/(1+Supuestos!$B$26)-L15-M15)</f>
-        <v/>
-      </c>
+      <c r="O15" s="52" t="n"/>
       <c r="P15" s="55">
         <f>G15*N15</f>
         <v/>
       </c>
-      <c r="Q15" s="55">
-        <f>G15*O15</f>
-        <v/>
-      </c>
+      <c r="Q15" s="55" t="n"/>
       <c r="R15" s="51">
         <f>IF(H15=0,0,N15/(H15/(1+Supuestos!$B$26)))</f>
         <v/>
@@ -4706,10 +4399,7 @@
         <f>Costeo!F15</f>
         <v/>
       </c>
-      <c r="L16" s="45">
-        <f>Costeo!F15</f>
-        <v/>
-      </c>
+      <c r="L16" s="45" t="n"/>
       <c r="M16" s="52">
         <f>IF(H16=0,0,C16*Supuestos!$B$34+H16*Supuestos!$B$27*Supuestos!$C$34+H16/(1+Supuestos!$B$26)*Supuestos!$B$28)</f>
         <v/>
@@ -4718,18 +4408,12 @@
         <f>IF(H16=0,0,H16/(1+Supuestos!$B$26)-K16-M16)</f>
         <v/>
       </c>
-      <c r="O16" s="52">
-        <f>IF(H16=0,0,H16/(1+Supuestos!$B$26)-L16-M16)</f>
-        <v/>
-      </c>
+      <c r="O16" s="52" t="n"/>
       <c r="P16" s="55">
         <f>G16*N16</f>
         <v/>
       </c>
-      <c r="Q16" s="55">
-        <f>G16*O16</f>
-        <v/>
-      </c>
+      <c r="Q16" s="55" t="n"/>
       <c r="R16" s="51">
         <f>IF(H16=0,0,N16/(H16/(1+Supuestos!$B$26)))</f>
         <v/>
@@ -4786,10 +4470,7 @@
         <f>Costeo!B15</f>
         <v/>
       </c>
-      <c r="L17" s="45">
-        <f>Costeo!B15</f>
-        <v/>
-      </c>
+      <c r="L17" s="45" t="n"/>
       <c r="M17" s="52">
         <f>IF(H17=0,0,C17*Supuestos!$B$35+H17*Supuestos!$B$27*Supuestos!$C$35+H17/(1+Supuestos!$B$26)*Supuestos!$B$28)</f>
         <v/>
@@ -4798,18 +4479,12 @@
         <f>IF(H17=0,0,H17/(1+Supuestos!$B$26)-K17-M17)</f>
         <v/>
       </c>
-      <c r="O17" s="52">
-        <f>IF(H17=0,0,H17/(1+Supuestos!$B$26)-L17-M17)</f>
-        <v/>
-      </c>
+      <c r="O17" s="52" t="n"/>
       <c r="P17" s="55">
         <f>G17*N17</f>
         <v/>
       </c>
-      <c r="Q17" s="55">
-        <f>G17*O17</f>
-        <v/>
-      </c>
+      <c r="Q17" s="55" t="n"/>
       <c r="R17" s="51">
         <f>IF(H17=0,0,N17/(H17/(1+Supuestos!$B$26)))</f>
         <v/>
@@ -4866,10 +4541,7 @@
         <f>Costeo!C15</f>
         <v/>
       </c>
-      <c r="L18" s="45">
-        <f>Costeo!D15</f>
-        <v/>
-      </c>
+      <c r="L18" s="45" t="n"/>
       <c r="M18" s="52">
         <f>IF(H18=0,0,C18*Supuestos!$B$35+H18*Supuestos!$B$27*Supuestos!$C$35+H18/(1+Supuestos!$B$26)*Supuestos!$B$28)</f>
         <v/>
@@ -4878,18 +4550,12 @@
         <f>IF(H18=0,0,H18/(1+Supuestos!$B$26)-K18-M18)</f>
         <v/>
       </c>
-      <c r="O18" s="52">
-        <f>IF(H18=0,0,H18/(1+Supuestos!$B$26)-L18-M18)</f>
-        <v/>
-      </c>
+      <c r="O18" s="52" t="n"/>
       <c r="P18" s="55">
         <f>G18*N18</f>
         <v/>
       </c>
-      <c r="Q18" s="55">
-        <f>G18*O18</f>
-        <v/>
-      </c>
+      <c r="Q18" s="55" t="n"/>
       <c r="R18" s="51">
         <f>IF(H18=0,0,N18/(H18/(1+Supuestos!$B$26)))</f>
         <v/>
@@ -4946,10 +4612,7 @@
         <f>Costeo!E15</f>
         <v/>
       </c>
-      <c r="L19" s="45">
-        <f>Costeo!E15</f>
-        <v/>
-      </c>
+      <c r="L19" s="45" t="n"/>
       <c r="M19" s="52">
         <f>IF(H19=0,0,C19*Supuestos!$B$35+H19*Supuestos!$B$27*Supuestos!$C$35+H19/(1+Supuestos!$B$26)*Supuestos!$B$28)</f>
         <v/>
@@ -4958,18 +4621,12 @@
         <f>IF(H19=0,0,H19/(1+Supuestos!$B$26)-K19-M19)</f>
         <v/>
       </c>
-      <c r="O19" s="52">
-        <f>IF(H19=0,0,H19/(1+Supuestos!$B$26)-L19-M19)</f>
-        <v/>
-      </c>
+      <c r="O19" s="52" t="n"/>
       <c r="P19" s="55">
         <f>G19*N19</f>
         <v/>
       </c>
-      <c r="Q19" s="55">
-        <f>G19*O19</f>
-        <v/>
-      </c>
+      <c r="Q19" s="55" t="n"/>
       <c r="R19" s="51">
         <f>IF(H19=0,0,N19/(H19/(1+Supuestos!$B$26)))</f>
         <v/>
@@ -5026,10 +4683,7 @@
         <f>Costeo!F15</f>
         <v/>
       </c>
-      <c r="L20" s="45">
-        <f>Costeo!F15</f>
-        <v/>
-      </c>
+      <c r="L20" s="45" t="n"/>
       <c r="M20" s="52">
         <f>IF(H20=0,0,C20*Supuestos!$B$35+H20*Supuestos!$B$27*Supuestos!$C$35+H20/(1+Supuestos!$B$26)*Supuestos!$B$28)</f>
         <v/>
@@ -5038,18 +4692,12 @@
         <f>IF(H20=0,0,H20/(1+Supuestos!$B$26)-K20-M20)</f>
         <v/>
       </c>
-      <c r="O20" s="52">
-        <f>IF(H20=0,0,H20/(1+Supuestos!$B$26)-L20-M20)</f>
-        <v/>
-      </c>
+      <c r="O20" s="52" t="n"/>
       <c r="P20" s="55">
         <f>G20*N20</f>
         <v/>
       </c>
-      <c r="Q20" s="55">
-        <f>G20*O20</f>
-        <v/>
-      </c>
+      <c r="Q20" s="55" t="n"/>
       <c r="R20" s="51">
         <f>IF(H20=0,0,N20/(H20/(1+Supuestos!$B$26)))</f>
         <v/>
@@ -5106,10 +4754,7 @@
         <f>Costeo!B15</f>
         <v/>
       </c>
-      <c r="L21" s="45">
-        <f>Costeo!B15</f>
-        <v/>
-      </c>
+      <c r="L21" s="45" t="n"/>
       <c r="M21" s="52">
         <f>IF(H21=0,0,C21*Supuestos!$B$36+H21*Supuestos!$B$27*Supuestos!$C$36+H21/(1+Supuestos!$B$26)*Supuestos!$B$28)</f>
         <v/>
@@ -5118,18 +4763,12 @@
         <f>IF(H21=0,0,H21/(1+Supuestos!$B$26)-K21-M21)</f>
         <v/>
       </c>
-      <c r="O21" s="52">
-        <f>IF(H21=0,0,H21/(1+Supuestos!$B$26)-L21-M21)</f>
-        <v/>
-      </c>
+      <c r="O21" s="52" t="n"/>
       <c r="P21" s="55">
         <f>G21*N21</f>
         <v/>
       </c>
-      <c r="Q21" s="55">
-        <f>G21*O21</f>
-        <v/>
-      </c>
+      <c r="Q21" s="55" t="n"/>
       <c r="R21" s="51">
         <f>IF(H21=0,0,N21/(H21/(1+Supuestos!$B$26)))</f>
         <v/>
@@ -5186,10 +4825,7 @@
         <f>Costeo!C15</f>
         <v/>
       </c>
-      <c r="L22" s="45">
-        <f>Costeo!D15</f>
-        <v/>
-      </c>
+      <c r="L22" s="45" t="n"/>
       <c r="M22" s="52">
         <f>IF(H22=0,0,C22*Supuestos!$B$36+H22*Supuestos!$B$27*Supuestos!$C$36+H22/(1+Supuestos!$B$26)*Supuestos!$B$28)</f>
         <v/>
@@ -5198,18 +4834,12 @@
         <f>IF(H22=0,0,H22/(1+Supuestos!$B$26)-K22-M22)</f>
         <v/>
       </c>
-      <c r="O22" s="52">
-        <f>IF(H22=0,0,H22/(1+Supuestos!$B$26)-L22-M22)</f>
-        <v/>
-      </c>
+      <c r="O22" s="52" t="n"/>
       <c r="P22" s="55">
         <f>G22*N22</f>
         <v/>
       </c>
-      <c r="Q22" s="55">
-        <f>G22*O22</f>
-        <v/>
-      </c>
+      <c r="Q22" s="55" t="n"/>
       <c r="R22" s="51">
         <f>IF(H22=0,0,N22/(H22/(1+Supuestos!$B$26)))</f>
         <v/>
@@ -5266,10 +4896,7 @@
         <f>Costeo!E15</f>
         <v/>
       </c>
-      <c r="L23" s="45">
-        <f>Costeo!E15</f>
-        <v/>
-      </c>
+      <c r="L23" s="45" t="n"/>
       <c r="M23" s="52">
         <f>IF(H23=0,0,C23*Supuestos!$B$36+H23*Supuestos!$B$27*Supuestos!$C$36+H23/(1+Supuestos!$B$26)*Supuestos!$B$28)</f>
         <v/>
@@ -5278,18 +4905,12 @@
         <f>IF(H23=0,0,H23/(1+Supuestos!$B$26)-K23-M23)</f>
         <v/>
       </c>
-      <c r="O23" s="52">
-        <f>IF(H23=0,0,H23/(1+Supuestos!$B$26)-L23-M23)</f>
-        <v/>
-      </c>
+      <c r="O23" s="52" t="n"/>
       <c r="P23" s="55">
         <f>G23*N23</f>
         <v/>
       </c>
-      <c r="Q23" s="55">
-        <f>G23*O23</f>
-        <v/>
-      </c>
+      <c r="Q23" s="55" t="n"/>
       <c r="R23" s="51">
         <f>IF(H23=0,0,N23/(H23/(1+Supuestos!$B$26)))</f>
         <v/>
@@ -5346,10 +4967,7 @@
         <f>Costeo!F15</f>
         <v/>
       </c>
-      <c r="L24" s="45">
-        <f>Costeo!F15</f>
-        <v/>
-      </c>
+      <c r="L24" s="45" t="n"/>
       <c r="M24" s="52">
         <f>IF(H24=0,0,C24*Supuestos!$B$36+H24*Supuestos!$B$27*Supuestos!$C$36+H24/(1+Supuestos!$B$26)*Supuestos!$B$28)</f>
         <v/>
@@ -5358,18 +4976,12 @@
         <f>IF(H24=0,0,H24/(1+Supuestos!$B$26)-K24-M24)</f>
         <v/>
       </c>
-      <c r="O24" s="52">
-        <f>IF(H24=0,0,H24/(1+Supuestos!$B$26)-L24-M24)</f>
-        <v/>
-      </c>
+      <c r="O24" s="52" t="n"/>
       <c r="P24" s="55">
         <f>G24*N24</f>
         <v/>
       </c>
-      <c r="Q24" s="55">
-        <f>G24*O24</f>
-        <v/>
-      </c>
+      <c r="Q24" s="55" t="n"/>
       <c r="R24" s="51">
         <f>IF(H24=0,0,N24/(H24/(1+Supuestos!$B$26)))</f>
         <v/>
@@ -5401,10 +5013,7 @@
         <f>SUM(P5:P24)</f>
         <v/>
       </c>
-      <c r="Q25" s="50">
-        <f>SUM(Q5:Q24)</f>
-        <v/>
-      </c>
+      <c r="Q25" s="50" t="n"/>
     </row>
     <row r="28" ht="15" customHeight="1" s="39">
       <c r="A28" s="59" t="inlineStr">
@@ -5433,14 +5042,10 @@
       </c>
       <c r="C29" s="44" t="inlineStr">
         <is>
-          <t>Contribución — opción B</t>
-        </is>
-      </c>
-      <c r="D29" s="44" t="inlineStr">
-        <is>
-          <t>Contribución — opción C</t>
-        </is>
-      </c>
+          <t>Contribución</t>
+        </is>
+      </c>
+      <c r="D29" s="44" t="n"/>
       <c r="E29" s="44" t="inlineStr">
         <is>
           <t>Ingreso con IGV</t>
@@ -5451,11 +5056,7 @@
           <t>Contribución por unidad — B</t>
         </is>
       </c>
-      <c r="G29" s="44" t="inlineStr">
-        <is>
-          <t>Contribución por unidad — C</t>
-        </is>
-      </c>
+      <c r="G29" s="44" t="n"/>
       <c r="H29" s="44" t="inlineStr">
         <is>
           <t>Ingreso con IGV por unidad</t>
@@ -5476,10 +5077,7 @@
         <f>SUMIF($A$5:$A$24,A30,$P$5:$P$24)</f>
         <v/>
       </c>
-      <c r="D30" s="55">
-        <f>SUMIF($A$5:$A$24,A30,$Q$5:$Q$24)</f>
-        <v/>
-      </c>
+      <c r="D30" s="55" t="n"/>
       <c r="E30" s="55">
         <f>SUMIF($A$5:$A$24,A30,$I$5:$I$24)</f>
         <v/>
@@ -5488,10 +5086,7 @@
         <f>IF(B30=0,0,C30/B30)</f>
         <v/>
       </c>
-      <c r="G30" s="52">
-        <f>IF(B30=0,0,D30/B30)</f>
-        <v/>
-      </c>
+      <c r="G30" s="52" t="n"/>
       <c r="H30" s="52">
         <f>IF(B30=0,0,E30/B30)</f>
         <v/>
@@ -5511,10 +5106,7 @@
         <f>SUMIF($A$5:$A$24,A31,$P$5:$P$24)</f>
         <v/>
       </c>
-      <c r="D31" s="55">
-        <f>SUMIF($A$5:$A$24,A31,$Q$5:$Q$24)</f>
-        <v/>
-      </c>
+      <c r="D31" s="55" t="n"/>
       <c r="E31" s="55">
         <f>SUMIF($A$5:$A$24,A31,$I$5:$I$24)</f>
         <v/>
@@ -5523,10 +5115,7 @@
         <f>IF(B31=0,0,C31/B31)</f>
         <v/>
       </c>
-      <c r="G31" s="52">
-        <f>IF(B31=0,0,D31/B31)</f>
-        <v/>
-      </c>
+      <c r="G31" s="52" t="n"/>
       <c r="H31" s="52">
         <f>IF(B31=0,0,E31/B31)</f>
         <v/>
@@ -5546,10 +5135,7 @@
         <f>SUMIF($A$5:$A$24,A32,$P$5:$P$24)</f>
         <v/>
       </c>
-      <c r="D32" s="55">
-        <f>SUMIF($A$5:$A$24,A32,$Q$5:$Q$24)</f>
-        <v/>
-      </c>
+      <c r="D32" s="55" t="n"/>
       <c r="E32" s="55">
         <f>SUMIF($A$5:$A$24,A32,$I$5:$I$24)</f>
         <v/>
@@ -5558,10 +5144,7 @@
         <f>IF(B32=0,0,C32/B32)</f>
         <v/>
       </c>
-      <c r="G32" s="52">
-        <f>IF(B32=0,0,D32/B32)</f>
-        <v/>
-      </c>
+      <c r="G32" s="52" t="n"/>
       <c r="H32" s="52">
         <f>IF(B32=0,0,E32/B32)</f>
         <v/>
@@ -5581,10 +5164,7 @@
         <f>SUMIF($A$5:$A$24,A33,$P$5:$P$24)</f>
         <v/>
       </c>
-      <c r="D33" s="55">
-        <f>SUMIF($A$5:$A$24,A33,$Q$5:$Q$24)</f>
-        <v/>
-      </c>
+      <c r="D33" s="55" t="n"/>
       <c r="E33" s="55">
         <f>SUMIF($A$5:$A$24,A33,$I$5:$I$24)</f>
         <v/>
@@ -5593,10 +5173,7 @@
         <f>IF(B33=0,0,C33/B33)</f>
         <v/>
       </c>
-      <c r="G33" s="52">
-        <f>IF(B33=0,0,D33/B33)</f>
-        <v/>
-      </c>
+      <c r="G33" s="52" t="n"/>
       <c r="H33" s="52">
         <f>IF(B33=0,0,E33/B33)</f>
         <v/>
@@ -5616,10 +5193,7 @@
         <f>SUMIF($A$5:$A$24,A34,$P$5:$P$24)</f>
         <v/>
       </c>
-      <c r="D34" s="55">
-        <f>SUMIF($A$5:$A$24,A34,$Q$5:$Q$24)</f>
-        <v/>
-      </c>
+      <c r="D34" s="55" t="n"/>
       <c r="E34" s="55">
         <f>SUMIF($A$5:$A$24,A34,$I$5:$I$24)</f>
         <v/>
@@ -5628,10 +5202,7 @@
         <f>IF(B34=0,0,C34/B34)</f>
         <v/>
       </c>
-      <c r="G34" s="52">
-        <f>IF(B34=0,0,D34/B34)</f>
-        <v/>
-      </c>
+      <c r="G34" s="52" t="n"/>
       <c r="H34" s="52">
         <f>IF(B34=0,0,E34/B34)</f>
         <v/>
@@ -5651,10 +5222,7 @@
         <f>SUM(C30:C34)</f>
         <v/>
       </c>
-      <c r="D35" s="50">
-        <f>SUM(D30:D34)</f>
-        <v/>
-      </c>
+      <c r="D35" s="50" t="n"/>
       <c r="E35" s="50">
         <f>SUM(E30:E34)</f>
         <v/>
@@ -5663,10 +5231,7 @@
         <f>IF(B35=0,0,C35/B35)</f>
         <v/>
       </c>
-      <c r="G35" s="72">
-        <f>IF(B35=0,0,D35/B35)</f>
-        <v/>
-      </c>
+      <c r="G35" s="72" t="n"/>
       <c r="H35" s="72">
         <f>IF(B35=0,0,E35/B35)</f>
         <v/>
@@ -5709,14 +5274,10 @@
       </c>
       <c r="E38" s="44" t="inlineStr">
         <is>
-          <t>Contribución — opción B</t>
-        </is>
-      </c>
-      <c r="F38" s="44" t="inlineStr">
-        <is>
-          <t>Contribución — opción C</t>
-        </is>
-      </c>
+          <t>Contribución</t>
+        </is>
+      </c>
+      <c r="F38" s="44" t="n"/>
       <c r="G38" s="44" t="inlineStr">
         <is>
           <t>% de las unidades</t>
@@ -5746,10 +5307,7 @@
         <f>SUMIF($B$5:$B$24,A39,$P$5:$P$24)</f>
         <v/>
       </c>
-      <c r="F39" s="55">
-        <f>SUMIF($B$5:$B$24,A39,$Q$5:$Q$24)</f>
-        <v/>
-      </c>
+      <c r="F39" s="55" t="n"/>
       <c r="G39" s="51">
         <f>IF($F$25=0,0,B39/$F$25)</f>
         <v/>
@@ -5777,10 +5335,7 @@
         <f>SUMIF($B$5:$B$24,A40,$P$5:$P$24)</f>
         <v/>
       </c>
-      <c r="F40" s="55">
-        <f>SUMIF($B$5:$B$24,A40,$Q$5:$Q$24)</f>
-        <v/>
-      </c>
+      <c r="F40" s="55" t="n"/>
       <c r="G40" s="51">
         <f>IF($F$25=0,0,B40/$F$25)</f>
         <v/>
@@ -5808,10 +5363,7 @@
         <f>SUMIF($B$5:$B$24,A41,$P$5:$P$24)</f>
         <v/>
       </c>
-      <c r="F41" s="55">
-        <f>SUMIF($B$5:$B$24,A41,$Q$5:$Q$24)</f>
-        <v/>
-      </c>
+      <c r="F41" s="55" t="n"/>
       <c r="G41" s="51">
         <f>IF($F$25=0,0,B41/$F$25)</f>
         <v/>
@@ -5839,10 +5391,7 @@
         <f>SUMIF($B$5:$B$24,A42,$P$5:$P$24)</f>
         <v/>
       </c>
-      <c r="F42" s="55">
-        <f>SUMIF($B$5:$B$24,A42,$Q$5:$Q$24)</f>
-        <v/>
-      </c>
+      <c r="F42" s="55" t="n"/>
       <c r="G42" s="51">
         <f>IF($F$25=0,0,B42/$F$25)</f>
         <v/>
@@ -7928,7 +7477,7 @@
     <row r="31" ht="15" customHeight="1" s="39">
       <c r="A31" s="43" t="inlineStr">
         <is>
-          <t>Contribución con pack de 6 opción B</t>
+          <t>Contribución con pack de 6</t>
         </is>
       </c>
       <c r="B31" s="48">
@@ -7985,63 +7534,20 @@
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" s="39">
-      <c r="A32" s="43" t="inlineStr">
-        <is>
-          <t>Contribución con pack de 6 opción C</t>
-        </is>
-      </c>
-      <c r="B32" s="48">
-        <f>SUMPRODUCT(B$14:B$18,Proyeccion!$G$30:$G$34)</f>
-        <v/>
-      </c>
-      <c r="C32" s="48">
-        <f>SUMPRODUCT(C$14:C$18,Proyeccion!$G$30:$G$34)</f>
-        <v/>
-      </c>
-      <c r="D32" s="48">
-        <f>SUMPRODUCT(D$14:D$18,Proyeccion!$G$30:$G$34)</f>
-        <v/>
-      </c>
-      <c r="E32" s="48">
-        <f>SUMPRODUCT(E$14:E$18,Proyeccion!$G$30:$G$34)</f>
-        <v/>
-      </c>
-      <c r="F32" s="48">
-        <f>SUMPRODUCT(F$14:F$18,Proyeccion!$G$30:$G$34)</f>
-        <v/>
-      </c>
-      <c r="G32" s="48">
-        <f>SUMPRODUCT(G$14:G$18,Proyeccion!$G$30:$G$34)</f>
-        <v/>
-      </c>
-      <c r="H32" s="48">
-        <f>SUMPRODUCT(H$14:H$18,Proyeccion!$G$30:$G$34)</f>
-        <v/>
-      </c>
-      <c r="I32" s="48">
-        <f>SUMPRODUCT(I$14:I$18,Proyeccion!$G$30:$G$34)</f>
-        <v/>
-      </c>
-      <c r="J32" s="48">
-        <f>SUMPRODUCT(J$14:J$18,Proyeccion!$G$30:$G$34)</f>
-        <v/>
-      </c>
-      <c r="K32" s="48">
-        <f>SUMPRODUCT(K$14:K$18,Proyeccion!$G$30:$G$34)</f>
-        <v/>
-      </c>
-      <c r="L32" s="48">
-        <f>SUMPRODUCT(L$14:L$18,Proyeccion!$G$30:$G$34)</f>
-        <v/>
-      </c>
-      <c r="M32" s="48">
-        <f>SUMPRODUCT(M$14:M$18,Proyeccion!$G$30:$G$34)</f>
-        <v/>
-      </c>
-      <c r="N32" s="55">
-        <f>SUM(B32:M32)</f>
-        <v/>
-      </c>
+      <c r="A32" s="43" t="n"/>
+      <c r="B32" s="48" t="n"/>
+      <c r="C32" s="48" t="n"/>
+      <c r="D32" s="48" t="n"/>
+      <c r="E32" s="48" t="n"/>
+      <c r="F32" s="48" t="n"/>
+      <c r="G32" s="48" t="n"/>
+      <c r="H32" s="48" t="n"/>
+      <c r="I32" s="48" t="n"/>
+      <c r="J32" s="48" t="n"/>
+      <c r="K32" s="48" t="n"/>
+      <c r="L32" s="48" t="n"/>
+      <c r="M32" s="48" t="n"/>
+      <c r="N32" s="55" t="n"/>
     </row>
     <row r="33" ht="15" customHeight="1" s="39">
       <c r="A33" s="43" t="inlineStr">
@@ -8341,7 +7847,7 @@
     <row r="38" ht="15" customHeight="1" s="39">
       <c r="A38" s="49" t="inlineStr">
         <is>
-          <t>Resultado operativo — opción B</t>
+          <t>Resultado operativo</t>
         </is>
       </c>
       <c r="B38" s="50">
@@ -8398,68 +7904,25 @@
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" s="39">
-      <c r="A39" s="49" t="inlineStr">
-        <is>
-          <t>Resultado operativo — opción C</t>
-        </is>
-      </c>
-      <c r="B39" s="50">
-        <f>B32-SUM(B33:B37)</f>
-        <v/>
-      </c>
-      <c r="C39" s="50">
-        <f>C32-SUM(C33:C37)</f>
-        <v/>
-      </c>
-      <c r="D39" s="50">
-        <f>D32-SUM(D33:D37)</f>
-        <v/>
-      </c>
-      <c r="E39" s="50">
-        <f>E32-SUM(E33:E37)</f>
-        <v/>
-      </c>
-      <c r="F39" s="50">
-        <f>F32-SUM(F33:F37)</f>
-        <v/>
-      </c>
-      <c r="G39" s="50">
-        <f>G32-SUM(G33:G37)</f>
-        <v/>
-      </c>
-      <c r="H39" s="50">
-        <f>H32-SUM(H33:H37)</f>
-        <v/>
-      </c>
-      <c r="I39" s="50">
-        <f>I32-SUM(I33:I37)</f>
-        <v/>
-      </c>
-      <c r="J39" s="50">
-        <f>J32-SUM(J33:J37)</f>
-        <v/>
-      </c>
-      <c r="K39" s="50">
-        <f>K32-SUM(K33:K37)</f>
-        <v/>
-      </c>
-      <c r="L39" s="50">
-        <f>L32-SUM(L33:L37)</f>
-        <v/>
-      </c>
-      <c r="M39" s="50">
-        <f>M32-SUM(M33:M37)</f>
-        <v/>
-      </c>
-      <c r="N39" s="50">
-        <f>SUM(B39:M39)</f>
-        <v/>
-      </c>
+      <c r="A39" s="49" t="n"/>
+      <c r="B39" s="50" t="n"/>
+      <c r="C39" s="50" t="n"/>
+      <c r="D39" s="50" t="n"/>
+      <c r="E39" s="50" t="n"/>
+      <c r="F39" s="50" t="n"/>
+      <c r="G39" s="50" t="n"/>
+      <c r="H39" s="50" t="n"/>
+      <c r="I39" s="50" t="n"/>
+      <c r="J39" s="50" t="n"/>
+      <c r="K39" s="50" t="n"/>
+      <c r="L39" s="50" t="n"/>
+      <c r="M39" s="50" t="n"/>
+      <c r="N39" s="50" t="n"/>
     </row>
     <row r="40" ht="15" customHeight="1" s="39">
       <c r="A40" s="43" t="inlineStr">
         <is>
-          <t>Resultado acumulado — opción B</t>
+          <t>Resultado acumulado</t>
         </is>
       </c>
       <c r="B40" s="55">
@@ -8512,59 +7975,19 @@
       </c>
     </row>
     <row r="41" ht="15" customHeight="1" s="39">
-      <c r="A41" s="43" t="inlineStr">
-        <is>
-          <t>Resultado acumulado — opción C</t>
-        </is>
-      </c>
-      <c r="B41" s="55">
-        <f>B39</f>
-        <v/>
-      </c>
-      <c r="C41" s="55">
-        <f>B41+C39</f>
-        <v/>
-      </c>
-      <c r="D41" s="55">
-        <f>C41+D39</f>
-        <v/>
-      </c>
-      <c r="E41" s="55">
-        <f>D41+E39</f>
-        <v/>
-      </c>
-      <c r="F41" s="55">
-        <f>E41+F39</f>
-        <v/>
-      </c>
-      <c r="G41" s="55">
-        <f>F41+G39</f>
-        <v/>
-      </c>
-      <c r="H41" s="55">
-        <f>G41+H39</f>
-        <v/>
-      </c>
-      <c r="I41" s="55">
-        <f>H41+I39</f>
-        <v/>
-      </c>
-      <c r="J41" s="55">
-        <f>I41+J39</f>
-        <v/>
-      </c>
-      <c r="K41" s="55">
-        <f>J41+K39</f>
-        <v/>
-      </c>
-      <c r="L41" s="55">
-        <f>K41+L39</f>
-        <v/>
-      </c>
-      <c r="M41" s="55">
-        <f>L41+M39</f>
-        <v/>
-      </c>
+      <c r="A41" s="43" t="n"/>
+      <c r="B41" s="55" t="n"/>
+      <c r="C41" s="55" t="n"/>
+      <c r="D41" s="55" t="n"/>
+      <c r="E41" s="55" t="n"/>
+      <c r="F41" s="55" t="n"/>
+      <c r="G41" s="55" t="n"/>
+      <c r="H41" s="55" t="n"/>
+      <c r="I41" s="55" t="n"/>
+      <c r="J41" s="55" t="n"/>
+      <c r="K41" s="55" t="n"/>
+      <c r="L41" s="55" t="n"/>
+      <c r="M41" s="55" t="n"/>
     </row>
     <row r="42" ht="15" customHeight="1" s="39">
       <c r="A42" s="43" t="inlineStr">
@@ -9611,7 +9034,7 @@
     <row r="21" ht="15" customHeight="1" s="39">
       <c r="A21" s="59" t="inlineStr">
         <is>
-          <t>Resultado mensual del año 2 (S/ sin IGV, salvo la primera fila; pack de 6 opción B)</t>
+          <t>Resultado mensual del año 2 (S/ sin IGV, salvo la primera fila)</t>
         </is>
       </c>
       <c r="B21" s="60" t="n"/>

</xml_diff>